<commit_message>
removed explicit file reference in modelmetadata and updated the extraction file reference for ab initio metadata
</commit_message>
<xml_diff>
--- a/Schema/DB_scheme.xlsx
+++ b/Schema/DB_scheme.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aksam432/Documents/GitHub/WP3/Schema/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{572041DA-4B45-C440-AE73-E968EFC1EBAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2F0C3CC-1203-5842-9CDB-F68DFE78751F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="19980" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="852" uniqueCount="339">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="851" uniqueCount="338">
   <si>
     <t>PROJET :</t>
   </si>
@@ -102,9 +102,6 @@
   </si>
   <si>
     <t>Needed, by default for the moment</t>
-  </si>
-  <si>
-    <t>SimulationMetadata/File</t>
   </si>
   <si>
     <t>float</t>
@@ -637,9 +634,6 @@
     <t>Userform</t>
   </si>
   <si>
-    <t>ModelMetadata/File</t>
-  </si>
-  <si>
     <t>Metadata of the trained model.</t>
   </si>
   <si>
@@ -721,9 +715,6 @@
     <t>The description on choice of hyperparameter settings</t>
   </si>
   <si>
-    <t>The path to metadata file or downloadable link</t>
-  </si>
-  <si>
     <t>The cut-off radius of the model</t>
   </si>
   <si>
@@ -967,9 +958,6 @@
     <t>tar</t>
   </si>
   <si>
-    <t>configFilePath</t>
-  </si>
-  <si>
     <t>cutOffRadius</t>
   </si>
   <si>
@@ -1055,6 +1043,15 @@
   </si>
   <si>
     <t>The filled canonical form</t>
+  </si>
+  <si>
+    <t>metaDataFile</t>
+  </si>
+  <si>
+    <t>The file for ab initio metadata</t>
+  </si>
+  <si>
+    <t>Userform or metaDataFile</t>
   </si>
 </sst>
 </file>
@@ -2167,12 +2164,22 @@
     <xf numFmtId="49" fontId="1" fillId="11" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2185,16 +2192,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Excel Built-in 20% - Accent1" xfId="1" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
@@ -2648,21 +2645,21 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:14" ht="47" x14ac:dyDescent="0.55000000000000004">
-      <c r="B2" s="141" t="s">
+      <c r="B2" s="142" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="141"/>
-      <c r="D2" s="142" t="s">
-        <v>167</v>
-      </c>
-      <c r="E2" s="142"/>
-      <c r="F2" s="142"/>
-      <c r="G2" s="142"/>
-      <c r="H2" s="142"/>
-      <c r="I2" s="142"/>
-      <c r="J2" s="142"/>
-      <c r="K2" s="142"/>
-      <c r="L2" s="142"/>
+      <c r="C2" s="142"/>
+      <c r="D2" s="143" t="s">
+        <v>166</v>
+      </c>
+      <c r="E2" s="143"/>
+      <c r="F2" s="143"/>
+      <c r="G2" s="143"/>
+      <c r="H2" s="143"/>
+      <c r="I2" s="143"/>
+      <c r="J2" s="143"/>
+      <c r="K2" s="143"/>
+      <c r="L2" s="143"/>
     </row>
     <row r="4" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="5" spans="2:14" x14ac:dyDescent="0.2">
@@ -2705,7 +2702,7 @@
     </row>
     <row r="6" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B6" s="11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C6" s="12" t="s">
         <v>13</v>
@@ -2731,7 +2728,7 @@
     </row>
     <row r="7" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B7" s="11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C7" s="16" t="s">
         <v>17</v>
@@ -2749,12 +2746,12 @@
       <c r="H7" s="18"/>
       <c r="I7" s="18"/>
       <c r="J7" s="18" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="K7" s="18"/>
       <c r="L7" s="18"/>
       <c r="M7" s="16" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="N7" t="s">
         <v>19</v>
@@ -2762,10 +2759,10 @@
     </row>
     <row r="8" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B8" s="11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D8" s="17">
         <v>1</v>
@@ -2780,12 +2777,12 @@
       <c r="H8" s="18"/>
       <c r="I8" s="18"/>
       <c r="J8" s="18" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="K8" s="18"/>
       <c r="L8" s="18"/>
       <c r="M8" s="16" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="N8" t="s">
         <v>20</v>
@@ -2793,10 +2790,10 @@
     </row>
     <row r="9" spans="2:14" ht="17" x14ac:dyDescent="0.2">
       <c r="B9" s="11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C9" s="105" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D9" s="106">
         <v>120</v>
@@ -2811,33 +2808,33 @@
       <c r="H9" s="107"/>
       <c r="I9" s="107"/>
       <c r="J9" s="18" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="K9" s="107" t="s">
         <v>23</v>
       </c>
       <c r="L9" s="107" t="s">
+        <v>170</v>
+      </c>
+      <c r="M9" s="108" t="s">
         <v>171</v>
       </c>
-      <c r="M9" s="108" t="s">
-        <v>172</v>
-      </c>
       <c r="N9" s="104" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
     </row>
     <row r="10" spans="2:14" ht="17" x14ac:dyDescent="0.2">
       <c r="B10" s="11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C10" s="105" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="D10" s="106">
         <v>1</v>
       </c>
       <c r="E10" s="105" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F10" s="107" t="s">
         <v>15</v>
@@ -2846,29 +2843,29 @@
       <c r="H10" s="107"/>
       <c r="I10" s="107"/>
       <c r="J10" s="18" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="K10" s="107"/>
       <c r="L10" s="107"/>
       <c r="M10" s="108" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="N10" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="11" spans="2:14" ht="17" x14ac:dyDescent="0.2">
       <c r="B11" s="11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C11" s="105" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="D11" s="106">
         <v>1</v>
       </c>
       <c r="E11" s="105" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F11" s="107" t="s">
         <v>18</v>
@@ -2877,33 +2874,33 @@
       <c r="H11" s="107"/>
       <c r="I11" s="107"/>
       <c r="J11" s="18" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="K11" s="107" t="s">
         <v>23</v>
       </c>
       <c r="L11" s="107" t="s">
+        <v>191</v>
+      </c>
+      <c r="M11" s="108" t="s">
+        <v>202</v>
+      </c>
+      <c r="N11" s="104" t="s">
         <v>192</v>
-      </c>
-      <c r="M11" s="108" t="s">
-        <v>204</v>
-      </c>
-      <c r="N11" s="104" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="12" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B12" s="11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="D12" s="17">
         <v>1</v>
       </c>
       <c r="E12" s="16" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F12" s="18" t="s">
         <v>15</v>
@@ -2912,29 +2909,29 @@
       <c r="H12" s="18"/>
       <c r="I12" s="16"/>
       <c r="J12" s="18" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="K12" s="18"/>
       <c r="L12" s="18"/>
       <c r="M12" s="16" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="N12" s="115" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
     </row>
     <row r="13" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B13" s="11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="D13" s="17">
         <v>1</v>
       </c>
       <c r="E13" s="16" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F13" s="18" t="s">
         <v>18</v>
@@ -2943,27 +2940,27 @@
       <c r="H13" s="18"/>
       <c r="I13" s="16"/>
       <c r="J13" s="18" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="K13" s="18"/>
       <c r="L13" s="18"/>
       <c r="M13" s="16" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="N13" s="131"/>
     </row>
     <row r="14" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B14" s="11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="D14" s="17">
         <v>1</v>
       </c>
       <c r="E14" s="16" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F14" s="18" t="s">
         <v>18</v>
@@ -2972,24 +2969,24 @@
       <c r="H14" s="18"/>
       <c r="I14" s="16"/>
       <c r="J14" s="18" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="K14" s="18" t="s">
         <v>23</v>
       </c>
       <c r="L14" s="18" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="M14" s="16" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="15" spans="2:14" ht="17" x14ac:dyDescent="0.2">
       <c r="B15" s="11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C15" s="16" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="D15" s="17">
         <v>1</v>
@@ -3004,20 +3001,20 @@
       <c r="H15" s="18"/>
       <c r="I15" s="18"/>
       <c r="J15" s="18" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="K15" s="18"/>
       <c r="L15" s="18"/>
       <c r="M15" s="19" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="16" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B16" s="11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C16" s="16" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="D16" s="17">
         <v>1</v>
@@ -3032,20 +3029,20 @@
       <c r="H16" s="18"/>
       <c r="I16" s="16"/>
       <c r="J16" s="18" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="K16" s="18"/>
       <c r="L16" s="18"/>
       <c r="M16" s="16" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="17" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="B17" s="11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C17" s="16" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="D17" s="17">
         <v>1</v>
@@ -3060,12 +3057,12 @@
       <c r="H17" s="18"/>
       <c r="I17" s="18"/>
       <c r="J17" s="18" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="K17" s="18"/>
       <c r="L17" s="18"/>
       <c r="M17" s="21" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="N17" t="s">
         <v>20</v>
@@ -3073,10 +3070,10 @@
     </row>
     <row r="18" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="B18" s="11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C18" s="16" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="D18" s="17">
         <v>1</v>
@@ -3094,18 +3091,18 @@
       <c r="K18" s="18"/>
       <c r="L18" s="18"/>
       <c r="M18" s="19" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="N18" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B19" s="11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C19" s="16" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="D19" s="17">
         <v>1</v>
@@ -3119,32 +3116,30 @@
       <c r="G19" s="18"/>
       <c r="H19" s="18"/>
       <c r="I19" s="16" t="s">
-        <v>179</v>
-      </c>
-      <c r="J19" s="18" t="s">
-        <v>199</v>
-      </c>
+        <v>178</v>
+      </c>
+      <c r="J19" s="18"/>
       <c r="K19" s="18"/>
       <c r="L19" s="18"/>
       <c r="M19" s="16" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="N19" s="115" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="20" spans="1:14" s="109" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="B20" s="110" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C20" s="111" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="D20" s="112">
         <v>1</v>
       </c>
       <c r="E20" s="111" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F20" s="113" t="s">
         <v>15</v>
@@ -3153,30 +3148,30 @@
       <c r="H20" s="113"/>
       <c r="I20" s="113"/>
       <c r="J20" s="113" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="K20" s="113" t="s">
         <v>23</v>
       </c>
       <c r="L20" s="113" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="M20" s="114" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
     </row>
     <row r="21" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="B21" s="11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C21" s="16" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D21" s="17">
         <v>1</v>
       </c>
       <c r="E21" s="16" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F21" s="18" t="s">
         <v>18</v>
@@ -3185,16 +3180,16 @@
       <c r="H21" s="18"/>
       <c r="I21" s="18"/>
       <c r="J21" s="18" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="K21" s="18" t="s">
         <v>23</v>
       </c>
       <c r="L21" s="18" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="M21" s="19" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="N21" t="s">
         <v>24</v>
@@ -3202,10 +3197,10 @@
     </row>
     <row r="22" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B22" s="11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C22" s="16" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="D22" s="17">
         <v>1</v>
@@ -3219,13 +3214,13 @@
       <c r="G22" s="18"/>
       <c r="H22" s="18"/>
       <c r="I22" s="18" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="J22" s="18"/>
       <c r="K22" s="18"/>
       <c r="L22" s="18"/>
       <c r="M22" s="21" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="N22" t="s">
         <v>19</v>
@@ -3233,10 +3228,10 @@
     </row>
     <row r="23" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B23" s="11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C23" s="16" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="D23" s="17">
         <v>1</v>
@@ -3250,21 +3245,21 @@
       <c r="G23" s="18"/>
       <c r="H23" s="18"/>
       <c r="I23" s="18" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="J23" s="18"/>
       <c r="K23" s="18"/>
       <c r="L23" s="18"/>
       <c r="M23" s="21" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
     </row>
     <row r="24" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="B24" s="11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C24" s="16" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="D24" s="17">
         <v>1</v>
@@ -3278,13 +3273,13 @@
       <c r="G24" s="18"/>
       <c r="H24" s="18"/>
       <c r="I24" s="18" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="J24" s="18"/>
       <c r="K24" s="18"/>
       <c r="L24" s="18"/>
       <c r="M24" s="21" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="N24" t="s">
         <v>19</v>
@@ -3292,16 +3287,16 @@
     </row>
     <row r="25" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="B25" s="11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C25" s="16" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="D25" s="17">
         <v>1</v>
       </c>
       <c r="E25" s="16" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F25" s="18" t="s">
         <v>15</v>
@@ -3310,14 +3305,14 @@
       <c r="H25" s="18"/>
       <c r="I25" s="18"/>
       <c r="J25" s="18" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="K25" s="18"/>
       <c r="L25" s="18" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="M25" s="19" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="N25" t="s">
         <v>19</v>
@@ -3325,10 +3320,10 @@
     </row>
     <row r="26" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="B26" s="11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C26" s="16" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="D26" s="17">
         <v>10</v>
@@ -3343,23 +3338,23 @@
       <c r="H26" s="18"/>
       <c r="I26" s="18"/>
       <c r="J26" s="18" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="K26" s="18"/>
       <c r="L26" s="18"/>
       <c r="M26" s="19" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="N26" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
     </row>
     <row r="27" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="B27" s="11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C27" s="16" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="D27" s="17">
         <v>1</v>
@@ -3373,13 +3368,13 @@
       <c r="G27" s="18"/>
       <c r="H27" s="18"/>
       <c r="I27" s="18" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="J27" s="18"/>
       <c r="K27" s="18"/>
       <c r="L27" s="18"/>
       <c r="M27" s="19" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="N27" t="s">
         <v>19</v>
@@ -3387,16 +3382,16 @@
     </row>
     <row r="28" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="B28" s="11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C28" s="16" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="D28" s="17">
         <v>1</v>
       </c>
       <c r="E28" s="16" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="F28" s="18" t="s">
         <v>18</v>
@@ -3408,7 +3403,7 @@
       <c r="K28" s="18"/>
       <c r="L28" s="18"/>
       <c r="M28" s="19" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="N28" t="s">
         <v>19</v>
@@ -3416,30 +3411,30 @@
     </row>
     <row r="29" spans="1:14" s="139" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="B29" s="134" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C29" s="135" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="D29" s="136">
         <v>10</v>
       </c>
       <c r="E29" s="135" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F29" s="137" t="s">
         <v>18</v>
       </c>
       <c r="G29" s="137"/>
       <c r="H29" s="137" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="I29" s="137"/>
       <c r="J29" s="137"/>
       <c r="K29" s="137"/>
       <c r="L29" s="137"/>
       <c r="M29" s="140" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="N29" s="139" t="s">
         <v>20</v>
@@ -3447,10 +3442,10 @@
     </row>
     <row r="30" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="B30" s="11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C30" s="16" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="D30" s="17">
         <v>10</v>
@@ -3464,27 +3459,27 @@
       <c r="G30" s="18"/>
       <c r="H30" s="18"/>
       <c r="I30" s="18" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="J30" s="18"/>
       <c r="K30" s="18"/>
       <c r="L30" s="18"/>
       <c r="M30" s="19" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="N30" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
     </row>
     <row r="31" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="B31" s="11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C31" s="16" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="D31" s="17" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E31" s="16" t="s">
         <v>22</v>
@@ -3495,19 +3490,19 @@
       <c r="G31" s="18"/>
       <c r="H31" s="18"/>
       <c r="I31" s="18" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="J31" s="18"/>
       <c r="K31" s="18"/>
       <c r="L31" s="18"/>
       <c r="M31" s="21" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
     </row>
     <row r="32" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A32" s="22"/>
       <c r="B32" s="11" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C32" s="12" t="s">
         <v>13</v>
@@ -3534,10 +3529,10 @@
     <row r="33" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A33" s="22"/>
       <c r="B33" s="11" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C33" s="16" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D33" s="17">
         <v>1</v>
@@ -3552,12 +3547,12 @@
       <c r="H33" s="18"/>
       <c r="I33" s="23"/>
       <c r="J33" s="18" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="K33" s="18"/>
       <c r="L33" s="18"/>
       <c r="M33" s="19" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="N33" t="s">
         <v>19</v>
@@ -3566,225 +3561,227 @@
     <row r="34" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A34" s="22"/>
       <c r="B34" s="11" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C34" s="16" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="D34" s="17">
         <v>1</v>
       </c>
       <c r="E34" s="16" t="s">
-        <v>54</v>
+        <v>25</v>
       </c>
       <c r="F34" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="G34" s="18"/>
+      <c r="G34" s="18" t="s">
+        <v>28</v>
+      </c>
       <c r="H34" s="18"/>
       <c r="I34" s="23"/>
-      <c r="J34" s="18"/>
+      <c r="J34" s="18" t="s">
+        <v>197</v>
+      </c>
       <c r="K34" s="18"/>
       <c r="L34" s="18"/>
       <c r="M34" s="19" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
     </row>
     <row r="35" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A35" s="22"/>
       <c r="B35" s="11" t="s">
-        <v>179</v>
-      </c>
-      <c r="C35" s="16" t="s">
-        <v>310</v>
+        <v>178</v>
+      </c>
+      <c r="C35" s="132" t="s">
+        <v>307</v>
       </c>
       <c r="D35" s="17">
         <v>1</v>
       </c>
       <c r="E35" s="16" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F35" s="18" t="s">
         <v>18</v>
       </c>
       <c r="G35" s="18" t="s">
-        <v>29</v>
+        <v>278</v>
       </c>
       <c r="H35" s="18"/>
       <c r="I35" s="23"/>
       <c r="J35" s="18" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="K35" s="18"/>
       <c r="L35" s="18"/>
       <c r="M35" s="19" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
     </row>
     <row r="36" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A36" s="22"/>
       <c r="B36" s="11" t="s">
-        <v>179</v>
-      </c>
-      <c r="C36" s="132" t="s">
-        <v>311</v>
+        <v>178</v>
+      </c>
+      <c r="C36" s="5" t="s">
+        <v>308</v>
       </c>
       <c r="D36" s="17">
         <v>1</v>
       </c>
       <c r="E36" s="16" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F36" s="18" t="s">
         <v>18</v>
       </c>
       <c r="G36" s="18" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="H36" s="18"/>
-      <c r="I36" s="23"/>
+      <c r="I36" s="18"/>
       <c r="J36" s="18" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="K36" s="18"/>
       <c r="L36" s="18"/>
-      <c r="M36" s="19" t="s">
-        <v>229</v>
+      <c r="M36" s="21" t="s">
+        <v>226</v>
       </c>
     </row>
     <row r="37" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A37" s="22"/>
       <c r="B37" s="11" t="s">
-        <v>179</v>
-      </c>
-      <c r="C37" s="5" t="s">
-        <v>312</v>
+        <v>178</v>
+      </c>
+      <c r="C37" s="16" t="s">
+        <v>309</v>
       </c>
       <c r="D37" s="17">
         <v>1</v>
       </c>
       <c r="E37" s="16" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F37" s="18" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="G37" s="18" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="H37" s="18"/>
       <c r="I37" s="18"/>
       <c r="J37" s="18" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="K37" s="18"/>
       <c r="L37" s="18"/>
       <c r="M37" s="21" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="38" spans="1:14" ht="17" x14ac:dyDescent="0.2">
-      <c r="A38" s="22"/>
-      <c r="B38" s="11" t="s">
-        <v>179</v>
-      </c>
-      <c r="C38" s="16" t="s">
-        <v>313</v>
-      </c>
-      <c r="D38" s="17">
-        <v>1</v>
-      </c>
-      <c r="E38" s="16" t="s">
-        <v>26</v>
-      </c>
-      <c r="F38" s="18" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="38" spans="1:14" s="109" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A38" s="116"/>
+      <c r="B38" s="110" t="s">
+        <v>178</v>
+      </c>
+      <c r="C38" s="117" t="s">
+        <v>310</v>
+      </c>
+      <c r="D38" s="112">
+        <v>1</v>
+      </c>
+      <c r="E38" s="111" t="s">
+        <v>25</v>
+      </c>
+      <c r="F38" s="118" t="s">
         <v>15</v>
       </c>
       <c r="G38" s="18" t="s">
-        <v>280</v>
-      </c>
-      <c r="H38" s="18"/>
-      <c r="I38" s="18"/>
+        <v>277</v>
+      </c>
+      <c r="H38" s="113"/>
+      <c r="I38" s="113"/>
       <c r="J38" s="18" t="s">
-        <v>198</v>
-      </c>
-      <c r="K38" s="18"/>
-      <c r="L38" s="18"/>
+        <v>197</v>
+      </c>
+      <c r="K38" s="113"/>
+      <c r="L38" s="113"/>
       <c r="M38" s="21" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="39" spans="1:14" s="109" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A39" s="116"/>
+        <v>227</v>
+      </c>
+    </row>
+    <row r="39" spans="1:14" s="124" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A39" s="119"/>
       <c r="B39" s="110" t="s">
         <v>179</v>
       </c>
-      <c r="C39" s="117" t="s">
-        <v>314</v>
-      </c>
-      <c r="D39" s="112">
-        <v>1</v>
-      </c>
-      <c r="E39" s="111" t="s">
-        <v>26</v>
-      </c>
-      <c r="F39" s="118" t="s">
+      <c r="C39" s="121" t="s">
+        <v>13</v>
+      </c>
+      <c r="D39" s="122">
+        <v>1</v>
+      </c>
+      <c r="E39" s="121" t="s">
+        <v>14</v>
+      </c>
+      <c r="F39" s="123" t="s">
+        <v>18</v>
+      </c>
+      <c r="G39" s="123"/>
+      <c r="H39" s="123"/>
+      <c r="I39" s="123"/>
+      <c r="J39" s="123"/>
+      <c r="K39" s="123"/>
+      <c r="L39" s="123"/>
+      <c r="M39" s="20" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="40" spans="1:14" ht="17" x14ac:dyDescent="0.2">
+      <c r="A40" s="22"/>
+      <c r="B40" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="C40" s="16" t="s">
+        <v>223</v>
+      </c>
+      <c r="D40" s="17">
+        <v>1</v>
+      </c>
+      <c r="E40" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="F40" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="G39" s="18" t="s">
-        <v>280</v>
-      </c>
-      <c r="H39" s="113"/>
-      <c r="I39" s="113"/>
-      <c r="J39" s="18" t="s">
-        <v>198</v>
-      </c>
-      <c r="K39" s="113"/>
-      <c r="L39" s="113"/>
-      <c r="M39" s="21" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="40" spans="1:14" s="124" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A40" s="119"/>
-      <c r="B40" s="110" t="s">
-        <v>180</v>
-      </c>
-      <c r="C40" s="121" t="s">
-        <v>13</v>
-      </c>
-      <c r="D40" s="122">
-        <v>1</v>
-      </c>
-      <c r="E40" s="121" t="s">
-        <v>14</v>
-      </c>
-      <c r="F40" s="123" t="s">
-        <v>18</v>
-      </c>
-      <c r="G40" s="123"/>
-      <c r="H40" s="123"/>
-      <c r="I40" s="123"/>
-      <c r="J40" s="123"/>
-      <c r="K40" s="123"/>
-      <c r="L40" s="123"/>
-      <c r="M40" s="20" t="s">
-        <v>16</v>
+      <c r="G40" s="18"/>
+      <c r="H40" s="18"/>
+      <c r="I40" s="18"/>
+      <c r="J40" s="18" t="s">
+        <v>197</v>
+      </c>
+      <c r="K40" s="18"/>
+      <c r="L40" s="18"/>
+      <c r="M40" s="24" t="s">
+        <v>235</v>
       </c>
     </row>
     <row r="41" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A41" s="22"/>
       <c r="B41" s="11" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C41" s="16" t="s">
-        <v>225</v>
+        <v>168</v>
       </c>
       <c r="D41" s="17">
         <v>1</v>
       </c>
       <c r="E41" s="16" t="s">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="F41" s="18" t="s">
         <v>15</v>
@@ -3793,116 +3790,116 @@
       <c r="H41" s="18"/>
       <c r="I41" s="18"/>
       <c r="J41" s="18" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="K41" s="18"/>
       <c r="L41" s="18"/>
-      <c r="M41" s="24" t="s">
-        <v>238</v>
+      <c r="M41" s="19" t="s">
+        <v>236</v>
       </c>
     </row>
     <row r="42" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A42" s="22"/>
       <c r="B42" s="11" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C42" s="16" t="s">
-        <v>169</v>
+        <v>243</v>
       </c>
       <c r="D42" s="17">
         <v>1</v>
       </c>
       <c r="E42" s="16" t="s">
-        <v>30</v>
+        <v>62</v>
       </c>
       <c r="F42" s="18" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="G42" s="18"/>
       <c r="H42" s="18"/>
       <c r="I42" s="18"/>
       <c r="J42" s="18" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="K42" s="18"/>
-      <c r="L42" s="18"/>
+      <c r="L42" s="18" t="s">
+        <v>279</v>
+      </c>
       <c r="M42" s="19" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="43" spans="1:14" ht="17" x14ac:dyDescent="0.2">
-      <c r="A43" s="22"/>
-      <c r="B43" s="11" t="s">
-        <v>180</v>
-      </c>
-      <c r="C43" s="16" t="s">
-        <v>246</v>
-      </c>
-      <c r="D43" s="17">
-        <v>1</v>
-      </c>
-      <c r="E43" s="16" t="s">
-        <v>63</v>
-      </c>
-      <c r="F43" s="18" t="s">
-        <v>18</v>
-      </c>
-      <c r="G43" s="18"/>
-      <c r="H43" s="18"/>
-      <c r="I43" s="18"/>
-      <c r="J43" s="18" t="s">
-        <v>198</v>
-      </c>
-      <c r="K43" s="18"/>
-      <c r="L43" s="18" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="43" spans="1:14" s="139" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A43" s="133"/>
+      <c r="B43" s="134" t="s">
+        <v>179</v>
+      </c>
+      <c r="C43" s="135" t="s">
+        <v>311</v>
+      </c>
+      <c r="D43" s="136">
+        <v>1</v>
+      </c>
+      <c r="E43" s="135" t="s">
+        <v>332</v>
+      </c>
+      <c r="F43" s="137" t="s">
+        <v>18</v>
+      </c>
+      <c r="G43" s="137"/>
+      <c r="H43" s="137"/>
+      <c r="I43" s="137"/>
+      <c r="J43" s="137" t="s">
+        <v>197</v>
+      </c>
+      <c r="K43" s="137"/>
+      <c r="L43" s="137"/>
+      <c r="M43" s="138" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="44" spans="1:14" ht="17" x14ac:dyDescent="0.2">
+      <c r="A44" s="22"/>
+      <c r="B44" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="C44" s="16" t="s">
         <v>282</v>
       </c>
-      <c r="M43" s="19" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="44" spans="1:14" s="139" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A44" s="133"/>
-      <c r="B44" s="134" t="s">
-        <v>180</v>
-      </c>
-      <c r="C44" s="135" t="s">
-        <v>315</v>
-      </c>
-      <c r="D44" s="136">
-        <v>1</v>
-      </c>
-      <c r="E44" s="135" t="s">
-        <v>336</v>
-      </c>
-      <c r="F44" s="137" t="s">
-        <v>18</v>
-      </c>
-      <c r="G44" s="137"/>
-      <c r="H44" s="137"/>
-      <c r="I44" s="137"/>
-      <c r="J44" s="137" t="s">
-        <v>198</v>
-      </c>
-      <c r="K44" s="137"/>
-      <c r="L44" s="137"/>
-      <c r="M44" s="138" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="45" spans="1:14" ht="17" x14ac:dyDescent="0.2">
+      <c r="D44" s="17">
+        <v>5</v>
+      </c>
+      <c r="E44" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="F44" s="18" t="s">
+        <v>18</v>
+      </c>
+      <c r="G44" s="18"/>
+      <c r="H44" s="18"/>
+      <c r="I44" s="18"/>
+      <c r="J44" s="18" t="s">
+        <v>197</v>
+      </c>
+      <c r="K44" s="18"/>
+      <c r="L44" s="18"/>
+      <c r="M44" s="19" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="45" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A45" s="22"/>
       <c r="B45" s="11" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C45" s="16" t="s">
-        <v>285</v>
+        <v>312</v>
       </c>
       <c r="D45" s="17">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E45" s="16" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="F45" s="18" t="s">
         <v>18</v>
@@ -3911,232 +3908,229 @@
       <c r="H45" s="18"/>
       <c r="I45" s="18"/>
       <c r="J45" s="18" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="K45" s="18"/>
       <c r="L45" s="18"/>
-      <c r="M45" s="19" t="s">
-        <v>286</v>
+      <c r="M45" s="25" t="s">
+        <v>238</v>
       </c>
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A46" s="22"/>
       <c r="B46" s="11" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C46" s="16" t="s">
-        <v>316</v>
-      </c>
-      <c r="D46" s="17">
-        <v>1</v>
+        <v>27</v>
+      </c>
+      <c r="D46" s="17" t="s">
+        <v>172</v>
       </c>
       <c r="E46" s="16" t="s">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="F46" s="18" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="G46" s="18"/>
       <c r="H46" s="18"/>
       <c r="I46" s="18"/>
       <c r="J46" s="18" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="K46" s="18"/>
       <c r="L46" s="18"/>
       <c r="M46" s="25" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A47" s="22"/>
-      <c r="B47" s="11" t="s">
-        <v>180</v>
-      </c>
-      <c r="C47" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="D47" s="17" t="s">
-        <v>173</v>
-      </c>
-      <c r="E47" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="F47" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="G47" s="18"/>
-      <c r="H47" s="18"/>
-      <c r="I47" s="18"/>
+        <v>239</v>
+      </c>
+    </row>
+    <row r="47" spans="1:14" s="109" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B47" s="110" t="s">
+        <v>179</v>
+      </c>
+      <c r="C47" s="111" t="s">
+        <v>313</v>
+      </c>
+      <c r="D47" s="112">
+        <v>1</v>
+      </c>
+      <c r="E47" s="111" t="s">
+        <v>25</v>
+      </c>
+      <c r="F47" s="113" t="s">
+        <v>18</v>
+      </c>
+      <c r="G47" s="113" t="s">
+        <v>220</v>
+      </c>
+      <c r="H47" s="113"/>
+      <c r="I47" s="113"/>
       <c r="J47" s="18" t="s">
-        <v>198</v>
-      </c>
-      <c r="K47" s="18"/>
-      <c r="L47" s="18"/>
-      <c r="M47" s="25" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="48" spans="1:14" s="109" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B48" s="110" t="s">
-        <v>180</v>
-      </c>
-      <c r="C48" s="111" t="s">
-        <v>317</v>
-      </c>
-      <c r="D48" s="112">
-        <v>1</v>
-      </c>
-      <c r="E48" s="111" t="s">
-        <v>26</v>
-      </c>
-      <c r="F48" s="113" t="s">
-        <v>18</v>
-      </c>
-      <c r="G48" s="113" t="s">
-        <v>222</v>
-      </c>
-      <c r="H48" s="113"/>
-      <c r="I48" s="113"/>
+        <v>197</v>
+      </c>
+      <c r="K47" s="113"/>
+      <c r="L47" s="113"/>
+      <c r="M47" s="125" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="48" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B48" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="C48" s="16" t="s">
+        <v>314</v>
+      </c>
+      <c r="D48" s="17">
+        <v>1</v>
+      </c>
+      <c r="E48" s="16" t="s">
+        <v>25</v>
+      </c>
+      <c r="F48" s="18" t="s">
+        <v>18</v>
+      </c>
+      <c r="G48" s="18" t="s">
+        <v>220</v>
+      </c>
+      <c r="H48" s="18"/>
+      <c r="I48" s="18"/>
       <c r="J48" s="18" t="s">
-        <v>198</v>
-      </c>
-      <c r="K48" s="113"/>
-      <c r="L48" s="113"/>
-      <c r="M48" s="125" t="s">
-        <v>232</v>
+        <v>197</v>
+      </c>
+      <c r="K48" s="18"/>
+      <c r="L48" s="18"/>
+      <c r="M48" s="26" t="s">
+        <v>230</v>
       </c>
     </row>
     <row r="49" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B49" s="11" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C49" s="16" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="D49" s="17">
         <v>1</v>
       </c>
       <c r="E49" s="16" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F49" s="18" t="s">
         <v>18</v>
       </c>
       <c r="G49" s="18" t="s">
-        <v>222</v>
+        <v>234</v>
       </c>
       <c r="H49" s="18"/>
       <c r="I49" s="18"/>
       <c r="J49" s="18" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="K49" s="18"/>
       <c r="L49" s="18"/>
-      <c r="M49" s="26" t="s">
-        <v>233</v>
+      <c r="M49" s="16" t="s">
+        <v>231</v>
       </c>
     </row>
     <row r="50" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B50" s="11" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C50" s="16" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
       <c r="D50" s="17">
         <v>1</v>
       </c>
       <c r="E50" s="16" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F50" s="18" t="s">
         <v>18</v>
       </c>
       <c r="G50" s="18" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="H50" s="18"/>
       <c r="I50" s="18"/>
       <c r="J50" s="18" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="K50" s="18"/>
       <c r="L50" s="18"/>
-      <c r="M50" s="16" t="s">
-        <v>234</v>
+      <c r="M50" s="27" t="s">
+        <v>232</v>
       </c>
     </row>
     <row r="51" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B51" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="C51" s="16" t="s">
+        <v>317</v>
+      </c>
+      <c r="D51" s="17">
+        <v>1</v>
+      </c>
+      <c r="E51" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="F51" s="18" t="s">
+        <v>18</v>
+      </c>
+      <c r="G51" s="18"/>
+      <c r="H51" s="18"/>
+      <c r="I51" s="18" t="s">
         <v>180</v>
       </c>
-      <c r="C51" s="16" t="s">
-        <v>320</v>
-      </c>
-      <c r="D51" s="17">
-        <v>1</v>
-      </c>
-      <c r="E51" s="16" t="s">
-        <v>26</v>
-      </c>
-      <c r="F51" s="18" t="s">
-        <v>18</v>
-      </c>
-      <c r="G51" s="18" t="s">
-        <v>237</v>
-      </c>
-      <c r="H51" s="18"/>
-      <c r="I51" s="18"/>
-      <c r="J51" s="18" t="s">
-        <v>198</v>
-      </c>
+      <c r="J51" s="18"/>
       <c r="K51" s="18"/>
       <c r="L51" s="18"/>
       <c r="M51" s="27" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="52" spans="2:13" x14ac:dyDescent="0.2">
-      <c r="B52" s="11" t="s">
-        <v>180</v>
-      </c>
-      <c r="C52" s="16" t="s">
-        <v>321</v>
-      </c>
-      <c r="D52" s="17">
-        <v>1</v>
-      </c>
-      <c r="E52" s="16" t="s">
-        <v>22</v>
-      </c>
-      <c r="F52" s="18" t="s">
-        <v>18</v>
-      </c>
-      <c r="G52" s="18"/>
-      <c r="H52" s="18"/>
-      <c r="I52" s="18" t="s">
-        <v>181</v>
-      </c>
-      <c r="J52" s="18"/>
-      <c r="K52" s="18"/>
-      <c r="L52" s="18"/>
-      <c r="M52" s="27" t="s">
-        <v>236</v>
+        <v>233</v>
+      </c>
+    </row>
+    <row r="52" spans="2:13" s="139" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B52" s="134" t="s">
+        <v>179</v>
+      </c>
+      <c r="C52" s="135" t="s">
+        <v>335</v>
+      </c>
+      <c r="D52" s="136">
+        <v>1</v>
+      </c>
+      <c r="E52" s="135" t="s">
+        <v>53</v>
+      </c>
+      <c r="F52" s="137" t="s">
+        <v>15</v>
+      </c>
+      <c r="G52" s="137"/>
+      <c r="H52" s="137"/>
+      <c r="I52" s="137"/>
+      <c r="J52" s="137"/>
+      <c r="K52" s="137"/>
+      <c r="L52" s="137"/>
+      <c r="M52" s="141" t="s">
+        <v>336</v>
       </c>
     </row>
     <row r="53" spans="2:13" s="139" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B53" s="134" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C53" s="135" t="s">
-        <v>337</v>
+        <v>333</v>
       </c>
       <c r="D53" s="136">
         <v>1</v>
       </c>
       <c r="E53" s="135" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F53" s="137" t="s">
         <v>18</v>
@@ -4147,16 +4141,16 @@
       <c r="J53" s="137"/>
       <c r="K53" s="137"/>
       <c r="L53" s="137"/>
-      <c r="M53" s="150" t="s">
-        <v>338</v>
+      <c r="M53" s="141" t="s">
+        <v>334</v>
       </c>
     </row>
     <row r="54" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B54" s="11" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C54" s="16" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="D54" s="17">
         <v>1</v>
@@ -4170,27 +4164,27 @@
       <c r="G54" s="18"/>
       <c r="H54" s="18"/>
       <c r="I54" s="18" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="J54" s="18"/>
       <c r="K54" s="18"/>
       <c r="L54" s="18"/>
       <c r="M54" s="27" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
     </row>
     <row r="55" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B55" s="11" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C55" s="16" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="D55" s="17">
         <v>1</v>
       </c>
       <c r="E55" s="16" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="F55" s="18" t="s">
         <v>18</v>
@@ -4202,12 +4196,12 @@
       <c r="K55" s="18"/>
       <c r="L55" s="18"/>
       <c r="M55" s="27" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
     </row>
     <row r="56" spans="2:13" s="124" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="B56" s="120" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C56" s="121" t="s">
         <v>22</v>
@@ -4233,10 +4227,10 @@
     </row>
     <row r="57" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B57" s="11" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C57" s="16" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="D57" s="17">
         <v>1</v>
@@ -4251,20 +4245,20 @@
       <c r="H57" s="18"/>
       <c r="I57" s="18"/>
       <c r="J57" s="18" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="K57" s="18"/>
       <c r="L57" s="18"/>
       <c r="M57" s="16" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
     </row>
     <row r="58" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B58" s="11" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C58" s="16" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="D58" s="17">
         <v>1</v>
@@ -4279,26 +4273,26 @@
       <c r="H58" s="18"/>
       <c r="I58" s="18"/>
       <c r="J58" s="18" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="K58" s="18"/>
       <c r="L58" s="18"/>
       <c r="M58" s="27" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
     </row>
     <row r="59" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B59" s="11" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C59" s="16" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
       <c r="D59" s="17">
         <v>1</v>
       </c>
       <c r="E59" s="16" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F59" s="18" t="s">
         <v>18</v>
@@ -4307,28 +4301,28 @@
       <c r="H59" s="18"/>
       <c r="I59" s="18"/>
       <c r="J59" s="18" t="s">
-        <v>25</v>
+        <v>337</v>
       </c>
       <c r="K59" s="18"/>
       <c r="L59" s="18" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="M59" s="16" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
     </row>
     <row r="60" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B60" s="11" t="s">
+        <v>180</v>
+      </c>
+      <c r="C60" s="16" t="s">
         <v>181</v>
       </c>
-      <c r="C60" s="16" t="s">
-        <v>182</v>
-      </c>
       <c r="D60" s="17">
         <v>1</v>
       </c>
       <c r="E60" s="16" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F60" s="18" t="s">
         <v>15</v>
@@ -4337,86 +4331,86 @@
       <c r="H60" s="18"/>
       <c r="I60" s="18"/>
       <c r="J60" s="18" t="s">
-        <v>25</v>
+        <v>337</v>
       </c>
       <c r="K60" s="18"/>
       <c r="L60" s="18"/>
       <c r="M60" s="5" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
     </row>
     <row r="61" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B61" s="11" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C61" s="16" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="D61" s="17">
         <v>1</v>
       </c>
       <c r="E61" s="16" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F61" s="18" t="s">
         <v>15</v>
       </c>
       <c r="G61" s="18" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="H61" s="18"/>
       <c r="I61" s="18"/>
       <c r="J61" s="18" t="s">
-        <v>25</v>
+        <v>337</v>
       </c>
       <c r="K61" s="18"/>
       <c r="L61" s="18"/>
       <c r="M61" s="16" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
     </row>
     <row r="62" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B62" s="11" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C62" s="16" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="D62" s="17">
         <v>1</v>
       </c>
       <c r="E62" s="16" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F62" s="18" t="s">
         <v>15</v>
       </c>
       <c r="G62" s="18" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="H62" s="18"/>
       <c r="I62" s="18"/>
       <c r="J62" s="18" t="s">
-        <v>25</v>
+        <v>337</v>
       </c>
       <c r="K62" s="18"/>
       <c r="L62" s="18"/>
       <c r="M62" s="27" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
     </row>
     <row r="63" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B63" s="11" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C63" s="16" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D63" s="17">
         <v>1</v>
       </c>
       <c r="E63" s="16" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F63" s="18" t="s">
         <v>15</v>
@@ -4425,26 +4419,26 @@
       <c r="H63" s="18"/>
       <c r="I63" s="18"/>
       <c r="J63" s="18" t="s">
-        <v>25</v>
+        <v>337</v>
       </c>
       <c r="K63" s="18"/>
       <c r="L63" s="18"/>
       <c r="M63" s="16" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
     </row>
     <row r="64" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B64" s="11" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C64" s="16" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D64" s="17">
         <v>1</v>
       </c>
       <c r="E64" s="16" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F64" s="18" t="s">
         <v>15</v>
@@ -4453,26 +4447,26 @@
       <c r="H64" s="18"/>
       <c r="I64" s="18"/>
       <c r="J64" s="18" t="s">
-        <v>25</v>
+        <v>337</v>
       </c>
       <c r="K64" s="18"/>
       <c r="L64" s="18"/>
       <c r="M64" s="27" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
     </row>
     <row r="65" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B65" s="11" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C65" s="16" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D65" s="17">
         <v>1</v>
       </c>
       <c r="E65" s="16" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F65" s="18" t="s">
         <v>15</v>
@@ -4481,77 +4475,77 @@
       <c r="H65" s="18"/>
       <c r="I65" s="18"/>
       <c r="J65" s="18" t="s">
-        <v>25</v>
+        <v>337</v>
       </c>
       <c r="K65" s="18"/>
       <c r="L65" s="18"/>
       <c r="M65" s="16" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
     </row>
     <row r="66" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B66" s="11" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C66" s="16" t="s">
-        <v>326</v>
+        <v>322</v>
       </c>
       <c r="D66" s="17">
         <v>1</v>
       </c>
       <c r="E66" s="16" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F66" s="18" t="s">
         <v>15</v>
       </c>
       <c r="G66" s="18" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="H66" s="18"/>
       <c r="I66" s="18"/>
       <c r="J66" s="18" t="s">
-        <v>25</v>
+        <v>337</v>
       </c>
       <c r="K66" s="18"/>
       <c r="L66" s="18"/>
       <c r="M66" s="16" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
     </row>
     <row r="67" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B67" s="11" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C67" s="16" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
       <c r="D67" s="17">
         <v>1</v>
       </c>
       <c r="E67" s="16" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F67" s="18" t="s">
         <v>15</v>
       </c>
       <c r="G67" s="18" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="H67" s="18"/>
       <c r="I67" s="18"/>
       <c r="J67" s="18" t="s">
-        <v>25</v>
+        <v>337</v>
       </c>
       <c r="K67" s="18"/>
       <c r="L67" s="18"/>
       <c r="M67" s="16" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
     </row>
     <row r="68" spans="2:13" s="124" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="B68" s="110" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C68" s="121" t="s">
         <v>22</v>
@@ -4577,10 +4571,10 @@
     </row>
     <row r="69" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B69" s="11" t="s">
+        <v>185</v>
+      </c>
+      <c r="C69" s="16" t="s">
         <v>186</v>
-      </c>
-      <c r="C69" s="16" t="s">
-        <v>187</v>
       </c>
       <c r="D69" s="17">
         <v>1</v>
@@ -4598,12 +4592,12 @@
       <c r="K69" s="18"/>
       <c r="L69" s="18"/>
       <c r="M69" s="27" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
     </row>
     <row r="70" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B70" s="11" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C70" s="16" t="s">
         <v>12</v>
@@ -4624,15 +4618,15 @@
       <c r="K70" s="18"/>
       <c r="L70" s="18"/>
       <c r="M70" s="16" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
     </row>
     <row r="71" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B71" s="11" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C71" s="16" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="D71" s="17">
         <v>1</v>
@@ -4646,27 +4640,27 @@
       <c r="G71" s="18"/>
       <c r="H71" s="18"/>
       <c r="I71" s="18" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="J71" s="18"/>
       <c r="K71" s="18"/>
       <c r="L71" s="18"/>
       <c r="M71" s="16" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
     </row>
     <row r="72" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B72" s="11" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C72" s="16" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="D72" s="17">
         <v>1</v>
       </c>
       <c r="E72" s="16" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F72" s="18" t="s">
         <v>15</v>
@@ -4677,24 +4671,24 @@
       <c r="J72" s="18"/>
       <c r="K72" s="18"/>
       <c r="L72" s="18" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="M72" s="16" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
     </row>
     <row r="73" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B73" s="11" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C73" s="16" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="D73" s="17">
         <v>1</v>
       </c>
       <c r="E73" s="16" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F73" s="18" t="s">
         <v>15</v>
@@ -4706,15 +4700,15 @@
       <c r="K73" s="18"/>
       <c r="L73" s="18"/>
       <c r="M73" s="27" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
     </row>
     <row r="74" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B74" s="11" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C74" s="16" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="D74" s="17">
         <v>1</v>
@@ -4728,27 +4722,27 @@
       <c r="G74" s="18"/>
       <c r="H74" s="18"/>
       <c r="I74" s="18" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="J74" s="18"/>
       <c r="K74" s="18"/>
       <c r="L74" s="18"/>
       <c r="M74" s="16" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
     </row>
     <row r="75" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B75" s="11" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C75" s="16" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="D75" s="17">
         <v>1</v>
       </c>
       <c r="E75" s="16" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="F75" s="18" t="s">
         <v>15</v>
@@ -4760,12 +4754,12 @@
       <c r="K75" s="18"/>
       <c r="L75" s="18"/>
       <c r="M75" s="16" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
     </row>
     <row r="76" spans="2:13" s="126" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="B76" s="110" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C76" s="127" t="s">
         <v>22</v>
@@ -4791,10 +4785,10 @@
     </row>
     <row r="77" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B77" s="11" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C77" s="16" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="D77" s="17">
         <v>1</v>
@@ -4808,21 +4802,21 @@
       <c r="G77" s="18"/>
       <c r="H77" s="18"/>
       <c r="I77" s="18" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="J77" s="18"/>
       <c r="K77" s="18"/>
       <c r="L77" s="18"/>
       <c r="M77" s="16" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
     </row>
     <row r="78" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B78" s="11" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C78" s="16" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
       <c r="D78" s="17">
         <v>1</v>
@@ -4836,27 +4830,27 @@
       <c r="G78" s="18"/>
       <c r="H78" s="18"/>
       <c r="I78" s="18" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="J78" s="18"/>
       <c r="K78" s="18"/>
       <c r="L78" s="18"/>
       <c r="M78" s="16" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
     </row>
     <row r="79" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B79" s="11" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C79" s="16" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="D79" s="17">
         <v>1</v>
       </c>
       <c r="E79" s="16" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F79" s="18" t="s">
         <v>15</v>
@@ -4868,21 +4862,21 @@
       <c r="K79" s="18"/>
       <c r="L79" s="18"/>
       <c r="M79" s="16" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
     </row>
     <row r="80" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B80" s="11" t="s">
+        <v>187</v>
+      </c>
+      <c r="C80" s="16" t="s">
         <v>188</v>
       </c>
-      <c r="C80" s="16" t="s">
-        <v>189</v>
-      </c>
       <c r="D80" s="17">
         <v>1</v>
       </c>
       <c r="E80" s="16" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F80" s="18" t="s">
         <v>15</v>
@@ -4894,21 +4888,21 @@
       <c r="K80" s="18"/>
       <c r="L80" s="18"/>
       <c r="M80" s="27" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
     </row>
     <row r="81" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B81" s="11" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C81" s="16" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="D81" s="17">
         <v>1</v>
       </c>
       <c r="E81" s="16" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="F81" s="18" t="s">
         <v>15</v>
@@ -4920,12 +4914,12 @@
       <c r="K81" s="18"/>
       <c r="L81" s="18"/>
       <c r="M81" s="16" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
     </row>
     <row r="82" spans="2:13" s="126" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B82" s="110" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="C82" s="127" t="s">
         <v>22</v>
@@ -4951,10 +4945,10 @@
     </row>
     <row r="83" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B83" s="11" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="C83" s="16" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="D83" s="17">
         <v>1</v>
@@ -4969,20 +4963,20 @@
       <c r="H83" s="18"/>
       <c r="I83" s="18"/>
       <c r="J83" s="18" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="K83" s="18"/>
       <c r="L83" s="18"/>
       <c r="M83" s="16" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
     </row>
     <row r="84" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B84" s="11" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="C84" s="16" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="D84" s="17">
         <v>1</v>
@@ -4997,20 +4991,20 @@
       <c r="H84" s="18"/>
       <c r="I84" s="18"/>
       <c r="J84" s="18" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="K84" s="18"/>
       <c r="L84" s="18"/>
       <c r="M84" s="16" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
     </row>
     <row r="85" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B85" s="11" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="C85" s="16" t="s">
-        <v>334</v>
+        <v>330</v>
       </c>
       <c r="D85" s="17">
         <v>1</v>
@@ -5025,20 +5019,20 @@
       <c r="H85" s="18"/>
       <c r="I85" s="18"/>
       <c r="J85" s="18" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="K85" s="18"/>
       <c r="L85" s="18"/>
       <c r="M85" s="16" t="s">
-        <v>335</v>
+        <v>331</v>
       </c>
     </row>
     <row r="86" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B86" s="11" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="C86" s="16" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D86" s="17">
         <v>1</v>
@@ -5053,12 +5047,12 @@
       <c r="H86" s="18"/>
       <c r="I86" s="18"/>
       <c r="J86" s="18" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="K86" s="18"/>
       <c r="L86" s="18"/>
       <c r="M86" s="16" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
     </row>
   </sheetData>
@@ -5132,7 +5126,7 @@
     </row>
     <row r="3" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B3" s="31" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C3" s="32" t="s">
         <v>13</v>
@@ -5153,15 +5147,15 @@
       <c r="K3" s="34"/>
       <c r="L3" s="34"/>
       <c r="M3" s="35" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B4" s="36" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C4" s="37" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D4" s="38">
         <v>1</v>
@@ -5175,21 +5169,21 @@
       <c r="G4" s="39"/>
       <c r="H4" s="39"/>
       <c r="I4" s="39" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="J4" s="39"/>
       <c r="K4" s="39"/>
       <c r="L4" s="39"/>
       <c r="M4" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B5" s="36" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C5" s="37" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D5" s="38">
         <v>1</v>
@@ -5203,21 +5197,21 @@
       <c r="G5" s="39"/>
       <c r="H5" s="39"/>
       <c r="I5" s="39" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="J5" s="39"/>
       <c r="K5" s="39"/>
       <c r="L5" s="39"/>
       <c r="M5" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B6" s="36" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C6" s="37" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D6" s="38">
         <v>1</v>
@@ -5231,21 +5225,21 @@
       <c r="G6" s="39"/>
       <c r="H6" s="39"/>
       <c r="I6" s="39" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J6" s="39"/>
       <c r="K6" s="39"/>
       <c r="L6" s="39"/>
       <c r="M6" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="7" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B7" s="36" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C7" s="37" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D7" s="38">
         <v>1</v>
@@ -5259,21 +5253,21 @@
       <c r="G7" s="39"/>
       <c r="H7" s="39"/>
       <c r="I7" s="39" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="J7" s="39"/>
       <c r="K7" s="39"/>
       <c r="L7" s="39"/>
       <c r="M7" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="8" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B8" s="40" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C8" s="41" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D8" s="42">
         <v>1</v>
@@ -5287,21 +5281,21 @@
       <c r="G8" s="43"/>
       <c r="H8" s="43"/>
       <c r="I8" s="43" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="J8" s="43"/>
       <c r="K8" s="43"/>
       <c r="L8" s="43"/>
       <c r="M8" s="44" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="9" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B9" s="40" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C9" s="41" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D9" s="42">
         <v>500</v>
@@ -5315,18 +5309,18 @@
       <c r="G9" s="43"/>
       <c r="H9" s="43"/>
       <c r="I9" s="43" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="J9" s="43"/>
       <c r="K9" s="43"/>
       <c r="L9" s="43"/>
       <c r="M9" s="44" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="10" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B10" s="45" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C10" s="46" t="s">
         <v>13</v>
@@ -5347,43 +5341,43 @@
       <c r="K10" s="48"/>
       <c r="L10" s="48"/>
       <c r="M10" s="49" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="11" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B11" s="50" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C11" s="51" t="s">
+        <v>52</v>
+      </c>
+      <c r="D11" s="52">
+        <v>1</v>
+      </c>
+      <c r="E11" s="51" t="s">
         <v>53</v>
-      </c>
-      <c r="D11" s="52">
-        <v>1</v>
-      </c>
-      <c r="E11" s="51" t="s">
-        <v>54</v>
       </c>
       <c r="F11" s="53" t="s">
         <v>18</v>
       </c>
       <c r="G11" s="53"/>
       <c r="H11" s="53" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="I11" s="53"/>
       <c r="J11" s="53"/>
       <c r="K11" s="53"/>
       <c r="L11" s="53"/>
       <c r="M11" s="54" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="12" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B12" s="36" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C12" s="37" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D12" s="38">
         <v>1</v>
@@ -5398,20 +5392,20 @@
       <c r="H12" s="39"/>
       <c r="I12" s="39"/>
       <c r="J12" s="39" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="K12" s="39"/>
       <c r="L12" s="39"/>
       <c r="M12" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="13" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B13" s="36" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C13" s="37" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D13" s="38">
         <v>1</v>
@@ -5426,26 +5420,26 @@
       <c r="H13" s="39"/>
       <c r="I13" s="39"/>
       <c r="J13" s="39" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="K13" s="39"/>
       <c r="L13" s="39"/>
       <c r="M13" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="14" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B14" s="36" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C14" s="37" t="s">
+        <v>61</v>
+      </c>
+      <c r="D14" s="38">
+        <v>1</v>
+      </c>
+      <c r="E14" s="37" t="s">
         <v>62</v>
-      </c>
-      <c r="D14" s="38">
-        <v>1</v>
-      </c>
-      <c r="E14" s="37" t="s">
-        <v>63</v>
       </c>
       <c r="F14" s="39" t="s">
         <v>18</v>
@@ -5454,85 +5448,85 @@
       <c r="H14" s="39"/>
       <c r="I14" s="39"/>
       <c r="J14" s="39" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="K14" s="39" t="s">
         <v>23</v>
       </c>
       <c r="L14" s="39" t="s">
+        <v>63</v>
+      </c>
+      <c r="M14" s="2" t="s">
         <v>64</v>
-      </c>
-      <c r="M14" s="2" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="15" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B15" s="36" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C15" s="37" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D15" s="38">
         <v>1</v>
       </c>
       <c r="E15" s="37" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F15" s="39" t="s">
         <v>15</v>
       </c>
       <c r="G15" s="39" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="H15" s="39"/>
       <c r="I15" s="39"/>
       <c r="J15" s="39" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="K15" s="39" t="s">
+        <v>67</v>
+      </c>
+      <c r="L15" s="39" t="s">
         <v>68</v>
       </c>
-      <c r="L15" s="39" t="s">
+      <c r="M15" s="2" t="s">
         <v>69</v>
-      </c>
-      <c r="M15" s="2" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="16" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B16" s="55" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C16" s="56" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D16" s="57">
         <v>1</v>
       </c>
       <c r="E16" s="56" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F16" s="58" t="s">
         <v>15</v>
       </c>
       <c r="G16" s="58" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="H16" s="58"/>
       <c r="I16" s="58"/>
       <c r="J16" s="58" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="K16" s="58"/>
       <c r="L16" s="58"/>
       <c r="M16" s="59" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="17" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B17" s="60" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C17" s="61" t="s">
         <v>13</v>
@@ -5553,43 +5547,43 @@
       <c r="K17" s="63"/>
       <c r="L17" s="63"/>
       <c r="M17" s="64" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="18" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B18" s="50" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C18" s="51" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D18" s="52">
         <v>1</v>
       </c>
       <c r="E18" s="51" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F18" s="53" t="s">
         <v>18</v>
       </c>
       <c r="G18" s="53"/>
       <c r="H18" s="53" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="I18" s="53"/>
       <c r="J18" s="53"/>
       <c r="K18" s="53"/>
       <c r="L18" s="53"/>
       <c r="M18" s="54" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="19" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B19" s="36" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C19" s="37" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D19" s="38">
         <v>1</v>
@@ -5604,20 +5598,20 @@
       <c r="H19" s="39"/>
       <c r="I19" s="39"/>
       <c r="J19" s="39" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="K19" s="39"/>
       <c r="L19" s="39"/>
       <c r="M19" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="20" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B20" s="40" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C20" s="41" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D20" s="42">
         <v>1</v>
@@ -5632,17 +5626,17 @@
       <c r="H20" s="43"/>
       <c r="I20" s="43"/>
       <c r="J20" s="43" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="K20" s="43"/>
       <c r="L20" s="43"/>
       <c r="M20" s="44" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="21" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B21" s="45" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C21" s="46" t="s">
         <v>13</v>
@@ -5663,40 +5657,40 @@
       <c r="K21" s="48"/>
       <c r="L21" s="48"/>
       <c r="M21" s="49" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="22" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B22" s="65" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C22" s="66" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D22" s="67">
         <v>1</v>
       </c>
       <c r="E22" s="66" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F22" s="68" t="s">
         <v>18</v>
       </c>
       <c r="G22" s="68"/>
       <c r="H22" s="68" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="I22" s="68"/>
       <c r="J22" s="68"/>
       <c r="K22" s="68"/>
       <c r="L22" s="68"/>
       <c r="M22" s="69" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="23" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B23" s="60" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C23" s="61" t="s">
         <v>13</v>
@@ -5717,43 +5711,43 @@
       <c r="K23" s="63"/>
       <c r="L23" s="63"/>
       <c r="M23" s="64" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="24" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B24" s="50" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C24" s="51" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D24" s="52">
         <v>1</v>
       </c>
       <c r="E24" s="51" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F24" s="53" t="s">
         <v>18</v>
       </c>
       <c r="G24" s="53"/>
       <c r="H24" s="53" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="I24" s="53"/>
       <c r="J24" s="53"/>
       <c r="K24" s="53"/>
       <c r="L24" s="53"/>
       <c r="M24" s="54" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="25" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B25" s="40" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C25" s="41" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D25" s="42">
         <v>1</v>
@@ -5771,12 +5765,12 @@
       <c r="K25" s="43"/>
       <c r="L25" s="43"/>
       <c r="M25" s="44" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="26" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B26" s="45" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C26" s="46" t="s">
         <v>13</v>
@@ -5797,15 +5791,15 @@
       <c r="K26" s="48"/>
       <c r="L26" s="48"/>
       <c r="M26" s="49" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="27" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B27" s="36" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C27" s="37" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D27" s="38">
         <v>1</v>
@@ -5823,12 +5817,12 @@
       <c r="K27" s="39"/>
       <c r="L27" s="39"/>
       <c r="M27" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="28" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B28" s="36" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C28" s="37" t="s">
         <v>12</v>
@@ -5849,15 +5843,15 @@
       <c r="K28" s="39"/>
       <c r="L28" s="39"/>
       <c r="M28" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="29" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B29" s="36" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C29" s="37" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D29" s="38">
         <v>1</v>
@@ -5875,40 +5869,40 @@
       <c r="K29" s="39"/>
       <c r="L29" s="39"/>
       <c r="M29" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="30" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B30" s="65" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C30" s="66" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D30" s="67">
         <v>1</v>
       </c>
       <c r="E30" s="66" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F30" s="68" t="s">
         <v>18</v>
       </c>
       <c r="G30" s="68"/>
       <c r="H30" s="68" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="I30" s="68"/>
       <c r="J30" s="68"/>
       <c r="K30" s="68"/>
       <c r="L30" s="68"/>
       <c r="M30" s="69" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="31" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B31" s="70" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C31" s="71" t="s">
         <v>13</v>
@@ -5929,12 +5923,12 @@
       <c r="K31" s="73"/>
       <c r="L31" s="73"/>
       <c r="M31" s="74" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="32" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B32" s="60" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C32" s="61" t="s">
         <v>13</v>
@@ -5955,15 +5949,15 @@
       <c r="K32" s="63"/>
       <c r="L32" s="63"/>
       <c r="M32" s="64" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="33" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B33" s="36" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C33" s="37" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D33" s="38">
         <v>1</v>
@@ -5977,21 +5971,21 @@
       <c r="G33" s="39"/>
       <c r="H33" s="39"/>
       <c r="I33" s="39" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="J33" s="39"/>
       <c r="K33" s="39"/>
       <c r="L33" s="39"/>
       <c r="M33" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="34" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B34" s="36" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C34" s="37" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D34" s="38">
         <v>1</v>
@@ -6005,21 +5999,21 @@
       <c r="G34" s="39"/>
       <c r="H34" s="39"/>
       <c r="I34" s="39" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J34" s="39"/>
       <c r="K34" s="39"/>
       <c r="L34" s="39"/>
       <c r="M34" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="35" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B35" s="36" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C35" s="37" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D35" s="38">
         <v>1</v>
@@ -6033,21 +6027,21 @@
       <c r="G35" s="39"/>
       <c r="H35" s="39"/>
       <c r="I35" s="39" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="J35" s="39"/>
       <c r="K35" s="39"/>
       <c r="L35" s="39"/>
       <c r="M35" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="36" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B36" s="36" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C36" s="37" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D36" s="38">
         <v>10</v>
@@ -6061,33 +6055,33 @@
       <c r="G36" s="39"/>
       <c r="H36" s="39"/>
       <c r="I36" s="39" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="J36" s="39"/>
       <c r="K36" s="39"/>
       <c r="L36" s="39"/>
       <c r="M36" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="37" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B37" s="40" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C37" s="41" t="s">
+        <v>109</v>
+      </c>
+      <c r="D37" s="42">
+        <v>1</v>
+      </c>
+      <c r="E37" s="41" t="s">
+        <v>25</v>
+      </c>
+      <c r="F37" s="43" t="s">
+        <v>18</v>
+      </c>
+      <c r="G37" s="43" t="s">
         <v>110</v>
-      </c>
-      <c r="D37" s="42">
-        <v>1</v>
-      </c>
-      <c r="E37" s="41" t="s">
-        <v>26</v>
-      </c>
-      <c r="F37" s="43" t="s">
-        <v>18</v>
-      </c>
-      <c r="G37" s="43" t="s">
-        <v>111</v>
       </c>
       <c r="H37" s="43"/>
       <c r="I37" s="43"/>
@@ -6095,27 +6089,27 @@
       <c r="K37" s="43"/>
       <c r="L37" s="43"/>
       <c r="M37" s="44" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="38" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B38" s="40" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C38" s="41" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D38" s="42">
         <v>1</v>
       </c>
       <c r="E38" s="41" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F38" s="43" t="s">
         <v>18</v>
       </c>
       <c r="G38" s="43" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="H38" s="43"/>
       <c r="I38" s="43"/>
@@ -6123,27 +6117,27 @@
       <c r="K38" s="43"/>
       <c r="L38" s="43"/>
       <c r="M38" s="44" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="39" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B39" s="55" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C39" s="56" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D39" s="57">
         <v>1</v>
       </c>
       <c r="E39" s="56" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F39" s="58" t="s">
         <v>18</v>
       </c>
       <c r="G39" s="58" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="H39" s="58"/>
       <c r="I39" s="58"/>
@@ -6151,12 +6145,12 @@
       <c r="K39" s="58"/>
       <c r="L39" s="58"/>
       <c r="M39" s="59" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="40" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B40" s="60" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C40" s="61" t="s">
         <v>13</v>
@@ -6177,12 +6171,12 @@
       <c r="K40" s="63"/>
       <c r="L40" s="63"/>
       <c r="M40" s="64" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="41" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B41" s="36" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C41" s="37" t="s">
         <v>4</v>
@@ -6203,292 +6197,292 @@
       <c r="K41" s="39"/>
       <c r="L41" s="39"/>
       <c r="M41" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="42" spans="2:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B42" s="50" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C42" s="51" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D42" s="52">
         <v>1</v>
       </c>
       <c r="E42" s="51" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F42" s="53" t="s">
         <v>18</v>
       </c>
       <c r="G42" s="53"/>
       <c r="H42" s="53" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="I42" s="53"/>
       <c r="J42" s="53"/>
       <c r="K42" s="53"/>
       <c r="L42" s="53"/>
       <c r="M42" s="54" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="43" spans="2:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B43" s="75" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C43" s="76" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D43" s="77">
         <v>1</v>
       </c>
       <c r="E43" s="76" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F43" s="78" t="s">
         <v>15</v>
       </c>
       <c r="G43" s="78" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H43" s="78"/>
       <c r="I43" s="78"/>
       <c r="J43" s="78" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="K43" s="78"/>
       <c r="L43" s="78"/>
       <c r="M43" s="1" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="47" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B47" s="147" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="47" spans="2:13" x14ac:dyDescent="0.2">
-      <c r="B47" s="143" t="s">
+      <c r="C47" s="147"/>
+      <c r="D47" s="147"/>
+      <c r="E47" s="147"/>
+      <c r="F47" s="147"/>
+      <c r="H47" s="148" t="s">
         <v>126</v>
       </c>
-      <c r="C47" s="143"/>
-      <c r="D47" s="143"/>
-      <c r="E47" s="143"/>
-      <c r="F47" s="143"/>
-      <c r="H47" s="144" t="s">
-        <v>127</v>
-      </c>
-      <c r="I47" s="144"/>
+      <c r="I47" s="148"/>
     </row>
     <row r="48" spans="2:13" x14ac:dyDescent="0.2">
-      <c r="B48" s="143"/>
-      <c r="C48" s="143"/>
-      <c r="D48" s="143"/>
-      <c r="E48" s="143"/>
-      <c r="F48" s="143"/>
-      <c r="H48" s="144"/>
-      <c r="I48" s="144"/>
+      <c r="B48" s="147"/>
+      <c r="C48" s="147"/>
+      <c r="D48" s="147"/>
+      <c r="E48" s="147"/>
+      <c r="F48" s="147"/>
+      <c r="H48" s="148"/>
+      <c r="I48" s="148"/>
     </row>
     <row r="49" spans="2:9" ht="16" x14ac:dyDescent="0.2">
       <c r="B49" s="79" t="s">
+        <v>127</v>
+      </c>
+      <c r="C49" s="149" t="s">
+        <v>12</v>
+      </c>
+      <c r="D49" s="149"/>
+      <c r="E49" s="149"/>
+      <c r="F49" s="149"/>
+      <c r="H49" s="80" t="s">
         <v>128</v>
       </c>
-      <c r="C49" s="145" t="s">
-        <v>12</v>
-      </c>
-      <c r="D49" s="145"/>
-      <c r="E49" s="145"/>
-      <c r="F49" s="145"/>
-      <c r="H49" s="80" t="s">
+      <c r="I49" s="81" t="s">
         <v>129</v>
-      </c>
-      <c r="I49" s="81" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="50" spans="2:9" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B50" s="82" t="s">
         <v>1</v>
       </c>
-      <c r="C50" s="146" t="s">
+      <c r="C50" s="150" t="s">
+        <v>130</v>
+      </c>
+      <c r="D50" s="150"/>
+      <c r="E50" s="150"/>
+      <c r="F50" s="150"/>
+      <c r="H50" s="83" t="s">
+        <v>52</v>
+      </c>
+      <c r="I50" s="84" t="s">
         <v>131</v>
-      </c>
-      <c r="D50" s="146"/>
-      <c r="E50" s="146"/>
-      <c r="F50" s="146"/>
-      <c r="H50" s="83" t="s">
-        <v>53</v>
-      </c>
-      <c r="I50" s="84" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="51" spans="2:9" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B51" s="85" t="s">
         <v>2</v>
       </c>
-      <c r="C51" s="147" t="s">
+      <c r="C51" s="144" t="s">
+        <v>132</v>
+      </c>
+      <c r="D51" s="144"/>
+      <c r="E51" s="144"/>
+      <c r="F51" s="144"/>
+      <c r="H51" s="86" t="s">
+        <v>74</v>
+      </c>
+      <c r="I51" s="87" t="s">
         <v>133</v>
-      </c>
-      <c r="D51" s="147"/>
-      <c r="E51" s="147"/>
-      <c r="F51" s="147"/>
-      <c r="H51" s="86" t="s">
-        <v>75</v>
-      </c>
-      <c r="I51" s="87" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="52" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B52" s="85" t="s">
         <v>3</v>
       </c>
-      <c r="C52" s="147" t="s">
+      <c r="C52" s="144" t="s">
+        <v>134</v>
+      </c>
+      <c r="D52" s="144"/>
+      <c r="E52" s="144"/>
+      <c r="F52" s="144"/>
+      <c r="H52" s="88" t="s">
         <v>135</v>
       </c>
-      <c r="D52" s="147"/>
-      <c r="E52" s="147"/>
-      <c r="F52" s="147"/>
-      <c r="H52" s="88" t="s">
+      <c r="I52" s="89" t="s">
         <v>136</v>
-      </c>
-      <c r="I52" s="89" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="53" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B53" s="85" t="s">
         <v>4</v>
       </c>
-      <c r="C53" s="148" t="s">
+      <c r="C53" s="146" t="s">
+        <v>137</v>
+      </c>
+      <c r="D53" s="146"/>
+      <c r="E53" s="146"/>
+      <c r="F53" s="146"/>
+      <c r="H53" s="88" t="s">
+        <v>85</v>
+      </c>
+      <c r="I53" s="89" t="s">
         <v>138</v>
-      </c>
-      <c r="D53" s="148"/>
-      <c r="E53" s="148"/>
-      <c r="F53" s="148"/>
-      <c r="H53" s="88" t="s">
-        <v>86</v>
-      </c>
-      <c r="I53" s="89" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="54" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B54" s="85" t="s">
         <v>5</v>
       </c>
-      <c r="C54" s="147" t="s">
+      <c r="C54" s="144" t="s">
+        <v>139</v>
+      </c>
+      <c r="D54" s="144"/>
+      <c r="E54" s="144"/>
+      <c r="F54" s="144"/>
+      <c r="H54" s="88" t="s">
+        <v>59</v>
+      </c>
+      <c r="I54" s="89" t="s">
         <v>140</v>
-      </c>
-      <c r="D54" s="147"/>
-      <c r="E54" s="147"/>
-      <c r="F54" s="147"/>
-      <c r="H54" s="88" t="s">
-        <v>60</v>
-      </c>
-      <c r="I54" s="89" t="s">
-        <v>141</v>
       </c>
     </row>
     <row r="55" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B55" s="85" t="s">
         <v>6</v>
       </c>
-      <c r="C55" s="148" t="s">
+      <c r="C55" s="146" t="s">
+        <v>141</v>
+      </c>
+      <c r="D55" s="146"/>
+      <c r="E55" s="146"/>
+      <c r="F55" s="146"/>
+      <c r="H55" s="90" t="s">
+        <v>118</v>
+      </c>
+      <c r="I55" s="91" t="s">
         <v>142</v>
-      </c>
-      <c r="D55" s="148"/>
-      <c r="E55" s="148"/>
-      <c r="F55" s="148"/>
-      <c r="H55" s="90" t="s">
-        <v>119</v>
-      </c>
-      <c r="I55" s="91" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="56" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B56" s="85" t="s">
         <v>7</v>
       </c>
-      <c r="C56" s="147" t="s">
-        <v>144</v>
-      </c>
-      <c r="D56" s="147"/>
-      <c r="E56" s="147"/>
-      <c r="F56" s="147"/>
+      <c r="C56" s="144" t="s">
+        <v>143</v>
+      </c>
+      <c r="D56" s="144"/>
+      <c r="E56" s="144"/>
+      <c r="F56" s="144"/>
     </row>
     <row r="57" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B57" s="85" t="s">
         <v>8</v>
       </c>
-      <c r="C57" s="147" t="s">
-        <v>145</v>
-      </c>
-      <c r="D57" s="147"/>
-      <c r="E57" s="147"/>
-      <c r="F57" s="147"/>
+      <c r="C57" s="144" t="s">
+        <v>144</v>
+      </c>
+      <c r="D57" s="144"/>
+      <c r="E57" s="144"/>
+      <c r="F57" s="144"/>
     </row>
     <row r="58" spans="2:9" ht="45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B58" s="85" t="s">
         <v>9</v>
       </c>
-      <c r="C58" s="147" t="s">
-        <v>146</v>
-      </c>
-      <c r="D58" s="147"/>
-      <c r="E58" s="147"/>
-      <c r="F58" s="147"/>
+      <c r="C58" s="144" t="s">
+        <v>145</v>
+      </c>
+      <c r="D58" s="144"/>
+      <c r="E58" s="144"/>
+      <c r="F58" s="144"/>
     </row>
     <row r="59" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B59" s="85" t="s">
         <v>10</v>
       </c>
-      <c r="C59" s="147" t="s">
-        <v>147</v>
-      </c>
-      <c r="D59" s="147"/>
-      <c r="E59" s="147"/>
-      <c r="F59" s="147"/>
+      <c r="C59" s="144" t="s">
+        <v>146</v>
+      </c>
+      <c r="D59" s="144"/>
+      <c r="E59" s="144"/>
+      <c r="F59" s="144"/>
     </row>
     <row r="60" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B60" s="85" t="s">
         <v>11</v>
       </c>
-      <c r="C60" s="147" t="s">
-        <v>148</v>
-      </c>
-      <c r="D60" s="147"/>
-      <c r="E60" s="147"/>
-      <c r="F60" s="147"/>
+      <c r="C60" s="144" t="s">
+        <v>147</v>
+      </c>
+      <c r="D60" s="144"/>
+      <c r="E60" s="144"/>
+      <c r="F60" s="144"/>
     </row>
     <row r="61" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B61" s="92" t="s">
         <v>12</v>
       </c>
-      <c r="C61" s="149" t="s">
-        <v>149</v>
-      </c>
-      <c r="D61" s="149"/>
-      <c r="E61" s="149"/>
-      <c r="F61" s="149"/>
+      <c r="C61" s="145" t="s">
+        <v>148</v>
+      </c>
+      <c r="D61" s="145"/>
+      <c r="E61" s="145"/>
+      <c r="F61" s="145"/>
     </row>
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="EAttMbwrYpwG6akiV7biz2nw7wlXtTooCxJogsSt7negKq0wKQ9sygPbVeHZ99cgmdNfAtLu9NnPC64y/Uaw7A==" saltValue="FJhchlgDftI44klS+XpFDg==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="15">
+    <mergeCell ref="B47:F48"/>
+    <mergeCell ref="H47:I48"/>
+    <mergeCell ref="C49:F49"/>
+    <mergeCell ref="C50:F50"/>
+    <mergeCell ref="C51:F51"/>
+    <mergeCell ref="C52:F52"/>
+    <mergeCell ref="C53:F53"/>
+    <mergeCell ref="C54:F54"/>
+    <mergeCell ref="C55:F55"/>
+    <mergeCell ref="C56:F56"/>
     <mergeCell ref="C57:F57"/>
     <mergeCell ref="C58:F58"/>
     <mergeCell ref="C59:F59"/>
     <mergeCell ref="C60:F60"/>
     <mergeCell ref="C61:F61"/>
-    <mergeCell ref="C52:F52"/>
-    <mergeCell ref="C53:F53"/>
-    <mergeCell ref="C54:F54"/>
-    <mergeCell ref="C55:F55"/>
-    <mergeCell ref="C56:F56"/>
-    <mergeCell ref="B47:F48"/>
-    <mergeCell ref="H47:I48"/>
-    <mergeCell ref="C49:F49"/>
-    <mergeCell ref="C50:F50"/>
-    <mergeCell ref="C51:F51"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -6541,30 +6535,30 @@
   <sheetData>
     <row r="4" spans="3:6" x14ac:dyDescent="0.2">
       <c r="C4" s="93" t="s">
+        <v>149</v>
+      </c>
+      <c r="D4" s="94" t="s">
         <v>150</v>
       </c>
-      <c r="D4" s="94" t="s">
+      <c r="E4" s="93" t="s">
         <v>151</v>
       </c>
-      <c r="E4" s="93" t="s">
+      <c r="F4" s="93" t="s">
         <v>152</v>
-      </c>
-      <c r="F4" s="93" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="5" spans="3:6" x14ac:dyDescent="0.2">
       <c r="C5" s="95" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D5" s="96" t="s">
         <v>18</v>
       </c>
       <c r="E5" s="97" t="s">
+        <v>153</v>
+      </c>
+      <c r="F5" s="98" t="s">
         <v>154</v>
-      </c>
-      <c r="F5" s="98" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="6" spans="3:6" x14ac:dyDescent="0.2">
@@ -6575,63 +6569,63 @@
         <v>15</v>
       </c>
       <c r="E6" s="101" t="s">
+        <v>155</v>
+      </c>
+      <c r="F6" s="102" t="s">
         <v>156</v>
-      </c>
-      <c r="F6" s="102" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="7" spans="3:6" x14ac:dyDescent="0.2">
       <c r="C7" s="99" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E7" s="101" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="8" spans="3:6" x14ac:dyDescent="0.2">
       <c r="C8" s="99" t="s">
+        <v>158</v>
+      </c>
+      <c r="E8" s="101" t="s">
         <v>159</v>
-      </c>
-      <c r="E8" s="101" t="s">
-        <v>160</v>
       </c>
     </row>
     <row r="9" spans="3:6" x14ac:dyDescent="0.2">
       <c r="C9" s="99" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E9" s="101" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="10" spans="3:6" x14ac:dyDescent="0.2">
       <c r="C10" s="99" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E10" s="101" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="11" spans="3:6" x14ac:dyDescent="0.2">
       <c r="C11" s="99" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E11" s="101" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="12" spans="3:6" x14ac:dyDescent="0.2">
       <c r="C12" s="99" t="s">
+        <v>162</v>
+      </c>
+      <c r="E12" s="101" t="s">
         <v>163</v>
-      </c>
-      <c r="E12" s="101" t="s">
-        <v>164</v>
       </c>
     </row>
     <row r="13" spans="3:6" x14ac:dyDescent="0.2">
       <c r="C13" s="99" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E13" s="101" t="s">
         <v>23</v>
@@ -6639,7 +6633,7 @@
     </row>
     <row r="14" spans="3:6" x14ac:dyDescent="0.2">
       <c r="C14" s="99" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="15" spans="3:6" x14ac:dyDescent="0.2">
@@ -6654,7 +6648,7 @@
     </row>
     <row r="17" spans="3:3" x14ac:dyDescent="0.2">
       <c r="C17" s="103" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Capacity of  Filereferences attribute in collection Model  changed to 1 from n
</commit_message>
<xml_diff>
--- a/Schema/DB_scheme.xlsx
+++ b/Schema/DB_scheme.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DIADEM\Data\WP3 - MLIP\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aksam432/Documents/GitHub/WP3/Schema/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDC0B31B-51A8-498E-9270-FA68C550618A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27C364D0-E05D-2142-93F1-F6DA897FDE11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="23260" windowHeight="12460" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Schéma à compléter" sheetId="1" r:id="rId1"/>
@@ -19,9 +19,6 @@
   </sheets>
   <calcPr calcId="0"/>
   <extLst>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
     </ext>
@@ -30,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="895" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="894" uniqueCount="325">
   <si>
     <t>PROJET :</t>
   </si>
@@ -1747,7 +1744,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="190">
+  <cellXfs count="178">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2036,15 +2033,6 @@
     <xf numFmtId="49" fontId="5" fillId="8" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="4" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2063,22 +2051,19 @@
     <xf numFmtId="49" fontId="5" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="5" fillId="3" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -2107,16 +2092,9 @@
     <xf numFmtId="49" fontId="5" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="49" fontId="4" fillId="6" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2195,23 +2173,10 @@
     <xf numFmtId="49" fontId="5" fillId="5" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="5" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -2243,10 +2208,10 @@
     <xf numFmtId="49" fontId="5" fillId="10" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2255,6 +2220,15 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2266,15 +2240,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2414,7 +2379,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -2711,45 +2676,45 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A2:N97"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.88671875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="2.88671875" customWidth="1"/>
-    <col min="2" max="2" width="23.88671875" customWidth="1"/>
-    <col min="3" max="3" width="23.44140625" style="3" customWidth="1"/>
-    <col min="4" max="4" width="8.88671875" style="4" customWidth="1"/>
+    <col min="1" max="1" width="2.83203125" customWidth="1"/>
+    <col min="2" max="2" width="23.83203125" customWidth="1"/>
+    <col min="3" max="3" width="23.5" style="3" customWidth="1"/>
+    <col min="4" max="4" width="8.83203125" style="4" customWidth="1"/>
     <col min="5" max="5" width="12.33203125" style="3" customWidth="1"/>
-    <col min="6" max="6" width="9.44140625" customWidth="1"/>
-    <col min="7" max="7" width="14.88671875" customWidth="1"/>
+    <col min="6" max="6" width="9.5" customWidth="1"/>
+    <col min="7" max="7" width="14.83203125" customWidth="1"/>
     <col min="8" max="8" width="10.33203125" customWidth="1"/>
-    <col min="9" max="9" width="28.109375" customWidth="1"/>
+    <col min="9" max="9" width="28.1640625" customWidth="1"/>
     <col min="10" max="10" width="26.33203125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="15.6640625" customWidth="1"/>
-    <col min="12" max="12" width="39.109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="39.1640625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="88.33203125" style="5" customWidth="1"/>
-    <col min="14" max="14" width="57.88671875" style="134" customWidth="1"/>
-    <col min="15" max="15" width="30.88671875" customWidth="1"/>
-    <col min="1023" max="1024" width="11.44140625" customWidth="1"/>
+    <col min="14" max="14" width="57.83203125" customWidth="1"/>
+    <col min="15" max="15" width="30.83203125" customWidth="1"/>
+    <col min="1023" max="1024" width="11.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:14" ht="46.2" x14ac:dyDescent="0.85">
-      <c r="B2" s="181" t="s">
+    <row r="2" spans="2:14" ht="47" x14ac:dyDescent="0.55000000000000004">
+      <c r="B2" s="169" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="181"/>
-      <c r="D2" s="182" t="s">
+      <c r="C2" s="169"/>
+      <c r="D2" s="170" t="s">
         <v>316</v>
       </c>
-      <c r="E2" s="182"/>
-      <c r="F2" s="182"/>
-      <c r="G2" s="182"/>
-      <c r="H2" s="182"/>
-      <c r="I2" s="182"/>
-      <c r="J2" s="182"/>
-      <c r="K2" s="182"/>
-      <c r="L2" s="182"/>
-    </row>
-    <row r="4" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="5" spans="2:14" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E2" s="170"/>
+      <c r="F2" s="170"/>
+      <c r="G2" s="170"/>
+      <c r="H2" s="170"/>
+      <c r="I2" s="170"/>
+      <c r="J2" s="170"/>
+      <c r="K2" s="170"/>
+      <c r="L2" s="170"/>
+    </row>
+    <row r="4" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="5" spans="2:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B5" s="6" t="s">
         <v>1</v>
       </c>
@@ -2787,85 +2752,85 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B6" s="109" t="s">
+    <row r="6" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B6" s="106" t="s">
         <v>55</v>
       </c>
-      <c r="C6" s="110" t="s">
+      <c r="C6" s="107" t="s">
         <v>13</v>
       </c>
-      <c r="D6" s="111">
-        <v>1</v>
-      </c>
-      <c r="E6" s="110" t="s">
+      <c r="D6" s="108">
+        <v>1</v>
+      </c>
+      <c r="E6" s="107" t="s">
         <v>14</v>
       </c>
-      <c r="F6" s="112" t="s">
-        <v>18</v>
-      </c>
-      <c r="G6" s="112"/>
-      <c r="H6" s="112"/>
-      <c r="I6" s="112"/>
-      <c r="J6" s="112"/>
-      <c r="K6" s="112"/>
-      <c r="L6" s="112"/>
-      <c r="M6" s="113" t="s">
+      <c r="F6" s="109" t="s">
+        <v>18</v>
+      </c>
+      <c r="G6" s="109"/>
+      <c r="H6" s="109"/>
+      <c r="I6" s="109"/>
+      <c r="J6" s="109"/>
+      <c r="K6" s="109"/>
+      <c r="L6" s="109"/>
+      <c r="M6" s="110" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B7" s="135" t="s">
+    <row r="7" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B7" s="128" t="s">
         <v>55</v>
       </c>
-      <c r="C7" s="136" t="s">
+      <c r="C7" s="129" t="s">
         <v>300</v>
       </c>
-      <c r="D7" s="137">
-        <v>1</v>
-      </c>
-      <c r="E7" s="136" t="s">
+      <c r="D7" s="130">
+        <v>1</v>
+      </c>
+      <c r="E7" s="129" t="s">
         <v>14</v>
       </c>
-      <c r="F7" s="138" t="s">
-        <v>18</v>
-      </c>
-      <c r="G7" s="138"/>
-      <c r="H7" s="138"/>
-      <c r="I7" s="138"/>
-      <c r="J7" s="138"/>
-      <c r="K7" s="138"/>
-      <c r="L7" s="138"/>
-      <c r="M7" s="139" t="s">
+      <c r="F7" s="131" t="s">
+        <v>18</v>
+      </c>
+      <c r="G7" s="131"/>
+      <c r="H7" s="131"/>
+      <c r="I7" s="131"/>
+      <c r="J7" s="131"/>
+      <c r="K7" s="131"/>
+      <c r="L7" s="131"/>
+      <c r="M7" s="132" t="s">
         <v>302</v>
       </c>
     </row>
-    <row r="8" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B8" s="135" t="s">
+    <row r="8" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B8" s="128" t="s">
         <v>55</v>
       </c>
-      <c r="C8" s="136" t="s">
+      <c r="C8" s="129" t="s">
         <v>301</v>
       </c>
-      <c r="D8" s="137">
-        <v>1</v>
-      </c>
-      <c r="E8" s="136" t="s">
+      <c r="D8" s="130">
+        <v>1</v>
+      </c>
+      <c r="E8" s="129" t="s">
         <v>19</v>
       </c>
-      <c r="F8" s="138" t="s">
-        <v>18</v>
-      </c>
-      <c r="G8" s="138"/>
-      <c r="H8" s="138"/>
-      <c r="I8" s="138"/>
-      <c r="J8" s="138"/>
-      <c r="K8" s="138"/>
-      <c r="L8" s="138"/>
-      <c r="M8" s="139" t="s">
+      <c r="F8" s="131" t="s">
+        <v>18</v>
+      </c>
+      <c r="G8" s="131"/>
+      <c r="H8" s="131"/>
+      <c r="I8" s="131"/>
+      <c r="J8" s="131"/>
+      <c r="K8" s="131"/>
+      <c r="L8" s="131"/>
+      <c r="M8" s="132" t="s">
         <v>303</v>
       </c>
     </row>
-    <row r="9" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B9" s="11" t="s">
         <v>55</v>
       </c>
@@ -2884,16 +2849,16 @@
       <c r="G9" s="14"/>
       <c r="H9" s="14"/>
       <c r="I9" s="14"/>
-      <c r="J9" s="108" t="s">
+      <c r="J9" s="14" t="s">
         <v>299</v>
       </c>
       <c r="K9" s="14"/>
       <c r="L9" s="14"/>
-      <c r="M9" s="114" t="s">
+      <c r="M9" s="111" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="10" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B10" s="11" t="s">
         <v>55</v>
       </c>
@@ -2912,49 +2877,49 @@
       <c r="G10" s="14"/>
       <c r="H10" s="14"/>
       <c r="I10" s="14"/>
-      <c r="J10" s="108" t="s">
+      <c r="J10" s="14" t="s">
         <v>299</v>
       </c>
       <c r="K10" s="14"/>
       <c r="L10" s="14"/>
-      <c r="M10" s="114" t="s">
+      <c r="M10" s="111" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="11" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B11" s="106" t="s">
+    <row r="11" spans="2:14" ht="17" x14ac:dyDescent="0.2">
+      <c r="B11" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="C11" s="107" t="s">
+      <c r="C11" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="D11" s="133">
+      <c r="D11" s="13">
         <v>118</v>
       </c>
-      <c r="E11" s="107" t="s">
+      <c r="E11" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="F11" s="108" t="s">
-        <v>18</v>
-      </c>
-      <c r="G11" s="108"/>
-      <c r="H11" s="108"/>
-      <c r="I11" s="108"/>
-      <c r="J11" s="108" t="s">
+      <c r="F11" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="G11" s="14"/>
+      <c r="H11" s="14"/>
+      <c r="I11" s="14"/>
+      <c r="J11" s="14" t="s">
         <v>299</v>
       </c>
-      <c r="K11" s="108" t="s">
+      <c r="K11" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="L11" s="108" t="s">
+      <c r="L11" s="14" t="s">
         <v>295</v>
       </c>
-      <c r="M11" s="115" t="s">
+      <c r="M11" s="112" t="s">
         <v>165</v>
       </c>
-      <c r="N11" s="179"/>
-    </row>
-    <row r="12" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="N11" s="167"/>
+    </row>
+    <row r="12" spans="2:14" ht="17" x14ac:dyDescent="0.2">
       <c r="B12" s="11" t="s">
         <v>55</v>
       </c>
@@ -2973,16 +2938,16 @@
       <c r="G12" s="95"/>
       <c r="H12" s="95"/>
       <c r="I12" s="95"/>
-      <c r="J12" s="108" t="s">
+      <c r="J12" s="14" t="s">
         <v>299</v>
       </c>
       <c r="K12" s="95"/>
       <c r="L12" s="95"/>
-      <c r="M12" s="116" t="s">
+      <c r="M12" s="113" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="13" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:14" ht="17" x14ac:dyDescent="0.2">
       <c r="B13" s="11" t="s">
         <v>55</v>
       </c>
@@ -3001,7 +2966,7 @@
       <c r="G13" s="95"/>
       <c r="H13" s="95"/>
       <c r="I13" s="95"/>
-      <c r="J13" s="108" t="s">
+      <c r="J13" s="14" t="s">
         <v>299</v>
       </c>
       <c r="K13" s="95" t="s">
@@ -3010,12 +2975,12 @@
       <c r="L13" s="95" t="s">
         <v>180</v>
       </c>
-      <c r="M13" s="116" t="s">
+      <c r="M13" s="113" t="s">
         <v>186</v>
       </c>
-      <c r="N13" s="179"/>
-    </row>
-    <row r="14" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="N13" s="167"/>
+    </row>
+    <row r="14" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B14" s="11" t="s">
         <v>55</v>
       </c>
@@ -3025,7 +2990,7 @@
       <c r="D14" s="13">
         <v>1</v>
       </c>
-      <c r="E14" s="107" t="s">
+      <c r="E14" s="12" t="s">
         <v>25</v>
       </c>
       <c r="F14" s="14" t="s">
@@ -3034,17 +2999,17 @@
       <c r="G14" s="14"/>
       <c r="H14" s="14"/>
       <c r="I14" s="12"/>
-      <c r="J14" s="108" t="s">
+      <c r="J14" s="14" t="s">
         <v>299</v>
       </c>
       <c r="K14" s="14"/>
       <c r="L14" s="14"/>
-      <c r="M14" s="114" t="s">
+      <c r="M14" s="111" t="s">
         <v>237</v>
       </c>
-      <c r="N14" s="179"/>
-    </row>
-    <row r="15" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="N14" s="167"/>
+    </row>
+    <row r="15" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B15" s="11" t="s">
         <v>55</v>
       </c>
@@ -3063,17 +3028,17 @@
       <c r="G15" s="14"/>
       <c r="H15" s="14"/>
       <c r="I15" s="12"/>
-      <c r="J15" s="108" t="s">
+      <c r="J15" s="14" t="s">
         <v>299</v>
       </c>
       <c r="K15" s="14"/>
       <c r="L15" s="14"/>
-      <c r="M15" s="114" t="s">
+      <c r="M15" s="111" t="s">
         <v>240</v>
       </c>
-      <c r="N15" s="180"/>
-    </row>
-    <row r="16" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="N15" s="168"/>
+    </row>
+    <row r="16" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B16" s="11" t="s">
         <v>55</v>
       </c>
@@ -3092,7 +3057,7 @@
       <c r="G16" s="14"/>
       <c r="H16" s="14"/>
       <c r="I16" s="12"/>
-      <c r="J16" s="108" t="s">
+      <c r="J16" s="14" t="s">
         <v>299</v>
       </c>
       <c r="K16" s="14" t="s">
@@ -3101,11 +3066,11 @@
       <c r="L16" s="14" t="s">
         <v>167</v>
       </c>
-      <c r="M16" s="114" t="s">
+      <c r="M16" s="111" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="B17" s="11" t="s">
         <v>55</v>
       </c>
@@ -3124,16 +3089,16 @@
       <c r="G17" s="14"/>
       <c r="H17" s="14"/>
       <c r="I17" s="14"/>
-      <c r="J17" s="108" t="s">
+      <c r="J17" s="14" t="s">
         <v>299</v>
       </c>
       <c r="K17" s="14"/>
       <c r="L17" s="14"/>
-      <c r="M17" s="117" t="s">
+      <c r="M17" s="112" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B18" s="11" t="s">
         <v>55</v>
       </c>
@@ -3143,7 +3108,7 @@
       <c r="D18" s="13">
         <v>1</v>
       </c>
-      <c r="E18" s="107" t="s">
+      <c r="E18" s="12" t="s">
         <v>161</v>
       </c>
       <c r="F18" s="14" t="s">
@@ -3152,16 +3117,16 @@
       <c r="G18" s="14"/>
       <c r="H18" s="14"/>
       <c r="I18" s="12"/>
-      <c r="J18" s="108" t="s">
+      <c r="J18" s="14" t="s">
         <v>299</v>
       </c>
       <c r="K18" s="14"/>
       <c r="L18" s="14"/>
-      <c r="M18" s="114" t="s">
+      <c r="M18" s="111" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="B19" s="11" t="s">
         <v>55</v>
       </c>
@@ -3180,42 +3145,42 @@
       <c r="G19" s="14"/>
       <c r="H19" s="14"/>
       <c r="I19" s="14"/>
-      <c r="J19" s="108" t="s">
+      <c r="J19" s="14" t="s">
         <v>299</v>
       </c>
       <c r="K19" s="14"/>
       <c r="L19" s="14"/>
-      <c r="M19" s="118" t="s">
+      <c r="M19" s="114" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="B20" s="174" t="s">
+    <row r="20" spans="1:14" ht="17" x14ac:dyDescent="0.2">
+      <c r="B20" s="162" t="s">
         <v>55</v>
       </c>
-      <c r="C20" s="175" t="s">
+      <c r="C20" s="163" t="s">
         <v>249</v>
       </c>
-      <c r="D20" s="176">
-        <v>1</v>
-      </c>
-      <c r="E20" s="175" t="s">
+      <c r="D20" s="164">
+        <v>1</v>
+      </c>
+      <c r="E20" s="163" t="s">
         <v>14</v>
       </c>
-      <c r="F20" s="177" t="s">
-        <v>18</v>
-      </c>
-      <c r="G20" s="177"/>
-      <c r="H20" s="177"/>
-      <c r="I20" s="177"/>
-      <c r="J20" s="177"/>
-      <c r="K20" s="177"/>
-      <c r="L20" s="177"/>
-      <c r="M20" s="178" t="s">
+      <c r="F20" s="165" t="s">
+        <v>18</v>
+      </c>
+      <c r="G20" s="165"/>
+      <c r="H20" s="165"/>
+      <c r="I20" s="165"/>
+      <c r="J20" s="165"/>
+      <c r="K20" s="165"/>
+      <c r="L20" s="165"/>
+      <c r="M20" s="166" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B21" s="11" t="s">
         <v>55</v>
       </c>
@@ -3236,15 +3201,15 @@
       <c r="I21" s="14" t="s">
         <v>170</v>
       </c>
-      <c r="J21" s="108"/>
+      <c r="J21" s="14"/>
       <c r="K21" s="14"/>
       <c r="L21" s="14"/>
-      <c r="M21" s="114" t="s">
+      <c r="M21" s="111" t="s">
         <v>184</v>
       </c>
-      <c r="N21" s="179"/>
-    </row>
-    <row r="22" spans="1:14" s="96" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="N21" s="167"/>
+    </row>
+    <row r="22" spans="1:14" s="96" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="B22" s="97" t="s">
         <v>55</v>
       </c>
@@ -3263,7 +3228,7 @@
       <c r="G22" s="100"/>
       <c r="H22" s="100"/>
       <c r="I22" s="100"/>
-      <c r="J22" s="108" t="s">
+      <c r="J22" s="14" t="s">
         <v>299</v>
       </c>
       <c r="K22" s="100" t="s">
@@ -3272,12 +3237,12 @@
       <c r="L22" s="105" t="s">
         <v>296</v>
       </c>
-      <c r="M22" s="119" t="s">
+      <c r="M22" s="115" t="s">
         <v>185</v>
       </c>
-      <c r="N22" s="134"/>
-    </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="N22"/>
+    </row>
+    <row r="23" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="B23" s="11" t="s">
         <v>55</v>
       </c>
@@ -3296,7 +3261,7 @@
       <c r="G23" s="14"/>
       <c r="H23" s="14"/>
       <c r="I23" s="14"/>
-      <c r="J23" s="108" t="s">
+      <c r="J23" s="14" t="s">
         <v>299</v>
       </c>
       <c r="K23" s="14" t="s">
@@ -3305,11 +3270,11 @@
       <c r="L23" s="14" t="s">
         <v>182</v>
       </c>
-      <c r="M23" s="117" t="s">
+      <c r="M23" s="112" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="24" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B24" s="11" t="s">
         <v>55</v>
       </c>
@@ -3333,11 +3298,11 @@
       <c r="J24" s="14"/>
       <c r="K24" s="14"/>
       <c r="L24" s="14"/>
-      <c r="M24" s="118" t="s">
+      <c r="M24" s="114" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="25" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B25" s="11" t="s">
         <v>55</v>
       </c>
@@ -3361,11 +3326,11 @@
       <c r="J25" s="14"/>
       <c r="K25" s="14"/>
       <c r="L25" s="14"/>
-      <c r="M25" s="118" t="s">
+      <c r="M25" s="114" t="s">
         <v>238</v>
       </c>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="B26" s="11" t="s">
         <v>55</v>
       </c>
@@ -3389,11 +3354,11 @@
       <c r="J26" s="14"/>
       <c r="K26" s="14"/>
       <c r="L26" s="14"/>
-      <c r="M26" s="118" t="s">
+      <c r="M26" s="114" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="B27" s="11" t="s">
         <v>55</v>
       </c>
@@ -3412,7 +3377,7 @@
       <c r="G27" s="14"/>
       <c r="H27" s="14"/>
       <c r="I27" s="14"/>
-      <c r="J27" s="108" t="s">
+      <c r="J27" s="14" t="s">
         <v>299</v>
       </c>
       <c r="K27" s="14" t="s">
@@ -3421,176 +3386,176 @@
       <c r="L27" s="14" t="s">
         <v>183</v>
       </c>
-      <c r="M27" s="117" t="s">
+      <c r="M27" s="112" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="B28" s="106" t="s">
+    <row r="28" spans="1:14" ht="17" x14ac:dyDescent="0.2">
+      <c r="B28" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="C28" s="107" t="s">
+      <c r="C28" s="12" t="s">
         <v>256</v>
       </c>
-      <c r="D28" s="133">
+      <c r="D28" s="13">
         <v>10</v>
       </c>
-      <c r="E28" s="107" t="s">
+      <c r="E28" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="F28" s="108" t="s">
+      <c r="F28" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="G28" s="108"/>
-      <c r="H28" s="108"/>
-      <c r="I28" s="108"/>
-      <c r="J28" s="108" t="s">
+      <c r="G28" s="14"/>
+      <c r="H28" s="14"/>
+      <c r="I28" s="14"/>
+      <c r="J28" s="14" t="s">
         <v>299</v>
       </c>
-      <c r="K28" s="108"/>
-      <c r="L28" s="108"/>
-      <c r="M28" s="115" t="s">
+      <c r="K28" s="14"/>
+      <c r="L28" s="14"/>
+      <c r="M28" s="112" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="29" spans="1:14" s="134" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="140" t="s">
+    <row r="29" spans="1:14" ht="17" x14ac:dyDescent="0.2">
+      <c r="B29" s="133" t="s">
         <v>55</v>
       </c>
-      <c r="C29" s="141" t="s">
+      <c r="C29" s="134" t="s">
         <v>257</v>
       </c>
-      <c r="D29" s="142" t="s">
-        <v>317</v>
-      </c>
-      <c r="E29" s="141" t="s">
+      <c r="D29" s="135">
+        <v>1</v>
+      </c>
+      <c r="E29" s="134" t="s">
         <v>49</v>
       </c>
-      <c r="F29" s="143" t="s">
-        <v>18</v>
-      </c>
-      <c r="G29" s="143"/>
-      <c r="H29" s="143" t="s">
+      <c r="F29" s="136" t="s">
+        <v>18</v>
+      </c>
+      <c r="G29" s="136"/>
+      <c r="H29" s="136" t="s">
         <v>259</v>
       </c>
-      <c r="I29" s="143"/>
-      <c r="J29" s="143"/>
-      <c r="K29" s="143"/>
-      <c r="L29" s="143"/>
-      <c r="M29" s="144" t="s">
+      <c r="I29" s="136"/>
+      <c r="J29" s="136"/>
+      <c r="K29" s="136"/>
+      <c r="L29" s="136"/>
+      <c r="M29" s="137" t="s">
         <v>194</v>
       </c>
     </row>
-    <row r="30" spans="1:14" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B30" s="146" t="s">
+    <row r="30" spans="1:14" ht="18" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B30" s="139" t="s">
         <v>55</v>
       </c>
-      <c r="C30" s="147" t="s">
+      <c r="C30" s="140" t="s">
         <v>258</v>
       </c>
-      <c r="D30" s="148">
+      <c r="D30" s="141">
         <v>10</v>
       </c>
-      <c r="E30" s="147" t="s">
+      <c r="E30" s="140" t="s">
         <v>20</v>
       </c>
-      <c r="F30" s="149" t="s">
-        <v>18</v>
-      </c>
-      <c r="G30" s="149"/>
-      <c r="H30" s="149"/>
-      <c r="I30" s="149" t="s">
+      <c r="F30" s="142" t="s">
+        <v>18</v>
+      </c>
+      <c r="G30" s="142"/>
+      <c r="H30" s="142"/>
+      <c r="I30" s="142" t="s">
         <v>298</v>
       </c>
-      <c r="J30" s="149"/>
-      <c r="K30" s="149"/>
-      <c r="L30" s="149"/>
-      <c r="M30" s="150" t="s">
+      <c r="J30" s="142"/>
+      <c r="K30" s="142"/>
+      <c r="L30" s="142"/>
+      <c r="M30" s="143" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="31" spans="1:14" ht="16.2" thickTop="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:14" ht="18" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A31" s="15"/>
-      <c r="B31" s="135" t="s">
+      <c r="B31" s="128" t="s">
         <v>170</v>
       </c>
-      <c r="C31" s="136" t="s">
+      <c r="C31" s="129" t="s">
         <v>13</v>
       </c>
-      <c r="D31" s="137">
-        <v>1</v>
-      </c>
-      <c r="E31" s="136" t="s">
+      <c r="D31" s="130">
+        <v>1</v>
+      </c>
+      <c r="E31" s="129" t="s">
         <v>14</v>
       </c>
-      <c r="F31" s="138" t="s">
-        <v>18</v>
-      </c>
-      <c r="G31" s="138"/>
-      <c r="H31" s="138"/>
-      <c r="I31" s="138"/>
-      <c r="J31" s="138"/>
-      <c r="K31" s="138"/>
-      <c r="L31" s="138"/>
-      <c r="M31" s="145" t="s">
+      <c r="F31" s="131" t="s">
+        <v>18</v>
+      </c>
+      <c r="G31" s="131"/>
+      <c r="H31" s="131"/>
+      <c r="I31" s="131"/>
+      <c r="J31" s="131"/>
+      <c r="K31" s="131"/>
+      <c r="L31" s="131"/>
+      <c r="M31" s="138" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A32" s="15"/>
-      <c r="B32" s="135" t="s">
+      <c r="B32" s="128" t="s">
         <v>170</v>
       </c>
-      <c r="C32" s="136" t="s">
+      <c r="C32" s="129" t="s">
         <v>300</v>
       </c>
-      <c r="D32" s="137">
-        <v>1</v>
-      </c>
-      <c r="E32" s="136" t="s">
+      <c r="D32" s="130">
+        <v>1</v>
+      </c>
+      <c r="E32" s="129" t="s">
         <v>14</v>
       </c>
-      <c r="F32" s="138" t="s">
-        <v>18</v>
-      </c>
-      <c r="G32" s="138"/>
-      <c r="H32" s="138"/>
-      <c r="I32" s="138"/>
-      <c r="J32" s="138"/>
-      <c r="K32" s="138"/>
-      <c r="L32" s="138"/>
-      <c r="M32" s="145" t="s">
+      <c r="F32" s="131" t="s">
+        <v>18</v>
+      </c>
+      <c r="G32" s="131"/>
+      <c r="H32" s="131"/>
+      <c r="I32" s="131"/>
+      <c r="J32" s="131"/>
+      <c r="K32" s="131"/>
+      <c r="L32" s="131"/>
+      <c r="M32" s="138" t="s">
         <v>302</v>
       </c>
     </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A33" s="15"/>
-      <c r="B33" s="135" t="s">
+      <c r="B33" s="128" t="s">
         <v>170</v>
       </c>
-      <c r="C33" s="136" t="s">
+      <c r="C33" s="129" t="s">
         <v>301</v>
       </c>
-      <c r="D33" s="137">
-        <v>1</v>
-      </c>
-      <c r="E33" s="136" t="s">
+      <c r="D33" s="130">
+        <v>1</v>
+      </c>
+      <c r="E33" s="129" t="s">
         <v>19</v>
       </c>
-      <c r="F33" s="138" t="s">
-        <v>18</v>
-      </c>
-      <c r="G33" s="138"/>
-      <c r="H33" s="138"/>
-      <c r="I33" s="138"/>
-      <c r="J33" s="138"/>
-      <c r="K33" s="138"/>
-      <c r="L33" s="138"/>
-      <c r="M33" s="145" t="s">
+      <c r="F33" s="131" t="s">
+        <v>18</v>
+      </c>
+      <c r="G33" s="131"/>
+      <c r="H33" s="131"/>
+      <c r="I33" s="131"/>
+      <c r="J33" s="131"/>
+      <c r="K33" s="131"/>
+      <c r="L33" s="131"/>
+      <c r="M33" s="138" t="s">
         <v>303</v>
       </c>
     </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A34" s="15"/>
       <c r="B34" s="11" t="s">
         <v>170</v>
@@ -3610,16 +3575,16 @@
       <c r="G34" s="14"/>
       <c r="H34" s="14"/>
       <c r="I34" s="16"/>
-      <c r="J34" s="108" t="s">
+      <c r="J34" s="14" t="s">
         <v>299</v>
       </c>
       <c r="K34" s="14"/>
       <c r="L34" s="14"/>
-      <c r="M34" s="117" t="s">
+      <c r="M34" s="112" t="s">
         <v>198</v>
       </c>
     </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A35" s="15"/>
       <c r="B35" s="11" t="s">
         <v>170</v>
@@ -3636,17 +3601,17 @@
       <c r="F35" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="G35" s="108"/>
+      <c r="G35" s="14"/>
       <c r="H35" s="14"/>
       <c r="I35" s="16"/>
       <c r="J35" s="14"/>
       <c r="K35" s="14"/>
       <c r="L35" s="14"/>
-      <c r="M35" s="115" t="s">
+      <c r="M35" s="112" t="s">
         <v>306</v>
       </c>
     </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A36" s="15"/>
       <c r="B36" s="11" t="s">
         <v>170</v>
@@ -3663,17 +3628,17 @@
       <c r="F36" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="G36" s="108"/>
+      <c r="G36" s="14"/>
       <c r="H36" s="14"/>
       <c r="I36" s="16"/>
       <c r="J36" s="14"/>
       <c r="K36" s="14"/>
       <c r="L36" s="14"/>
-      <c r="M36" s="115" t="s">
+      <c r="M36" s="112" t="s">
         <v>305</v>
       </c>
     </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A37" s="15"/>
       <c r="B37" s="11" t="s">
         <v>170</v>
@@ -3695,21 +3660,21 @@
       </c>
       <c r="H37" s="14"/>
       <c r="I37" s="16"/>
-      <c r="J37" s="108" t="s">
+      <c r="J37" s="14" t="s">
         <v>299</v>
       </c>
       <c r="K37" s="14"/>
       <c r="L37" s="14"/>
-      <c r="M37" s="117" t="s">
+      <c r="M37" s="112" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A38" s="15"/>
       <c r="B38" s="11" t="s">
         <v>170</v>
       </c>
-      <c r="C38" s="120" t="s">
+      <c r="C38" s="116" t="s">
         <v>261</v>
       </c>
       <c r="D38" s="13">
@@ -3726,21 +3691,21 @@
       </c>
       <c r="H38" s="14"/>
       <c r="I38" s="16"/>
-      <c r="J38" s="108" t="s">
+      <c r="J38" s="14" t="s">
         <v>299</v>
       </c>
       <c r="K38" s="14"/>
       <c r="L38" s="14"/>
-      <c r="M38" s="117" t="s">
+      <c r="M38" s="112" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A39" s="15"/>
       <c r="B39" s="11" t="s">
         <v>170</v>
       </c>
-      <c r="C39" s="151" t="s">
+      <c r="C39" s="144" t="s">
         <v>262</v>
       </c>
       <c r="D39" s="13">
@@ -3757,16 +3722,16 @@
       </c>
       <c r="H39" s="14"/>
       <c r="I39" s="14"/>
-      <c r="J39" s="108" t="s">
+      <c r="J39" s="14" t="s">
         <v>299</v>
       </c>
       <c r="K39" s="14"/>
       <c r="L39" s="14"/>
-      <c r="M39" s="118" t="s">
+      <c r="M39" s="114" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="40" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A40" s="15"/>
       <c r="B40" s="11" t="s">
         <v>170</v>
@@ -3788,130 +3753,130 @@
       </c>
       <c r="H40" s="14"/>
       <c r="I40" s="14"/>
-      <c r="J40" s="108" t="s">
+      <c r="J40" s="14" t="s">
         <v>299</v>
       </c>
       <c r="K40" s="14"/>
       <c r="L40" s="14"/>
-      <c r="M40" s="118" t="s">
+      <c r="M40" s="114" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="41" spans="1:14" s="96" customFormat="1" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:14" s="96" customFormat="1" ht="18" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A41" s="101"/>
-      <c r="B41" s="155" t="s">
+      <c r="B41" s="148" t="s">
         <v>170</v>
       </c>
-      <c r="C41" s="156" t="s">
+      <c r="C41" s="149" t="s">
         <v>264</v>
       </c>
-      <c r="D41" s="157">
-        <v>1</v>
-      </c>
-      <c r="E41" s="158" t="s">
+      <c r="D41" s="150">
+        <v>1</v>
+      </c>
+      <c r="E41" s="151" t="s">
         <v>22</v>
       </c>
-      <c r="F41" s="159" t="s">
+      <c r="F41" s="152" t="s">
         <v>15</v>
       </c>
-      <c r="G41" s="149" t="s">
+      <c r="G41" s="142" t="s">
         <v>320</v>
       </c>
-      <c r="H41" s="160"/>
-      <c r="I41" s="160"/>
-      <c r="J41" s="161" t="s">
+      <c r="H41" s="153"/>
+      <c r="I41" s="153"/>
+      <c r="J41" s="142" t="s">
         <v>299</v>
       </c>
-      <c r="K41" s="160"/>
-      <c r="L41" s="160"/>
-      <c r="M41" s="162" t="s">
+      <c r="K41" s="153"/>
+      <c r="L41" s="153"/>
+      <c r="M41" s="154" t="s">
         <v>201</v>
       </c>
-      <c r="N41" s="134"/>
-    </row>
-    <row r="42" spans="1:14" s="96" customFormat="1" ht="16.2" thickTop="1" x14ac:dyDescent="0.3">
+      <c r="N41"/>
+    </row>
+    <row r="42" spans="1:14" s="96" customFormat="1" ht="18" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A42" s="101"/>
-      <c r="B42" s="135" t="s">
+      <c r="B42" s="128" t="s">
         <v>297</v>
       </c>
-      <c r="C42" s="152" t="s">
+      <c r="C42" s="145" t="s">
         <v>13</v>
       </c>
-      <c r="D42" s="153">
-        <v>1</v>
-      </c>
-      <c r="E42" s="152" t="s">
+      <c r="D42" s="146">
+        <v>1</v>
+      </c>
+      <c r="E42" s="145" t="s">
         <v>14</v>
       </c>
-      <c r="F42" s="154" t="s">
-        <v>18</v>
-      </c>
-      <c r="G42" s="154"/>
-      <c r="H42" s="154"/>
-      <c r="I42" s="154"/>
-      <c r="J42" s="154"/>
-      <c r="K42" s="154"/>
-      <c r="L42" s="154"/>
-      <c r="M42" s="168" t="s">
+      <c r="F42" s="147" t="s">
+        <v>18</v>
+      </c>
+      <c r="G42" s="147"/>
+      <c r="H42" s="147"/>
+      <c r="I42" s="147"/>
+      <c r="J42" s="147"/>
+      <c r="K42" s="147"/>
+      <c r="L42" s="147"/>
+      <c r="M42" s="156" t="s">
         <v>16</v>
       </c>
-      <c r="N42" s="134"/>
-    </row>
-    <row r="43" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="N42"/>
+    </row>
+    <row r="43" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A43" s="15"/>
-      <c r="B43" s="135" t="s">
+      <c r="B43" s="128" t="s">
         <v>297</v>
       </c>
-      <c r="C43" s="136" t="s">
+      <c r="C43" s="129" t="s">
         <v>300</v>
       </c>
-      <c r="D43" s="137">
-        <v>1</v>
-      </c>
-      <c r="E43" s="136" t="s">
+      <c r="D43" s="130">
+        <v>1</v>
+      </c>
+      <c r="E43" s="129" t="s">
         <v>14</v>
       </c>
-      <c r="F43" s="138" t="s">
-        <v>18</v>
-      </c>
-      <c r="G43" s="138"/>
-      <c r="H43" s="138"/>
-      <c r="I43" s="138"/>
-      <c r="J43" s="138"/>
-      <c r="K43" s="138"/>
-      <c r="L43" s="138"/>
-      <c r="M43" s="145" t="s">
+      <c r="F43" s="131" t="s">
+        <v>18</v>
+      </c>
+      <c r="G43" s="131"/>
+      <c r="H43" s="131"/>
+      <c r="I43" s="131"/>
+      <c r="J43" s="131"/>
+      <c r="K43" s="131"/>
+      <c r="L43" s="131"/>
+      <c r="M43" s="138" t="s">
         <v>302</v>
       </c>
     </row>
-    <row r="44" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A44" s="15"/>
-      <c r="B44" s="135" t="s">
+      <c r="B44" s="128" t="s">
         <v>297</v>
       </c>
-      <c r="C44" s="136" t="s">
+      <c r="C44" s="129" t="s">
         <v>301</v>
       </c>
-      <c r="D44" s="137">
-        <v>1</v>
-      </c>
-      <c r="E44" s="136" t="s">
+      <c r="D44" s="130">
+        <v>1</v>
+      </c>
+      <c r="E44" s="129" t="s">
         <v>19</v>
       </c>
-      <c r="F44" s="138" t="s">
-        <v>18</v>
-      </c>
-      <c r="G44" s="138"/>
-      <c r="H44" s="138"/>
-      <c r="I44" s="138"/>
-      <c r="J44" s="138"/>
-      <c r="K44" s="138"/>
-      <c r="L44" s="138"/>
-      <c r="M44" s="145" t="s">
+      <c r="F44" s="131" t="s">
+        <v>18</v>
+      </c>
+      <c r="G44" s="131"/>
+      <c r="H44" s="131"/>
+      <c r="I44" s="131"/>
+      <c r="J44" s="131"/>
+      <c r="K44" s="131"/>
+      <c r="L44" s="131"/>
+      <c r="M44" s="138" t="s">
         <v>303</v>
       </c>
     </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A45" s="15"/>
       <c r="B45" s="11" t="s">
         <v>297</v>
@@ -3931,16 +3896,16 @@
       <c r="G45" s="14"/>
       <c r="H45" s="14"/>
       <c r="I45" s="14"/>
-      <c r="J45" s="108" t="s">
+      <c r="J45" s="14" t="s">
         <v>299</v>
       </c>
       <c r="K45" s="14"/>
       <c r="L45" s="14"/>
-      <c r="M45" s="121" t="s">
+      <c r="M45" s="117" t="s">
         <v>207</v>
       </c>
     </row>
-    <row r="46" spans="1:14" s="96" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:14" s="96" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A46" s="101"/>
       <c r="B46" s="97" t="s">
         <v>297</v>
@@ -3948,7 +3913,7 @@
       <c r="C46" s="102" t="s">
         <v>163</v>
       </c>
-      <c r="D46" s="169">
+      <c r="D46" s="157">
         <v>1</v>
       </c>
       <c r="E46" s="102" t="s">
@@ -3965,12 +3930,12 @@
       </c>
       <c r="K46" s="103"/>
       <c r="L46" s="103"/>
-      <c r="M46" s="170" t="s">
+      <c r="M46" s="158" t="s">
         <v>208</v>
       </c>
-      <c r="N46" s="134"/>
-    </row>
-    <row r="47" spans="1:14" s="96" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="N46"/>
+    </row>
+    <row r="47" spans="1:14" s="96" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A47" s="101"/>
       <c r="B47" s="97" t="s">
         <v>297</v>
@@ -3978,7 +3943,7 @@
       <c r="C47" s="102" t="s">
         <v>211</v>
       </c>
-      <c r="D47" s="169">
+      <c r="D47" s="157">
         <v>1</v>
       </c>
       <c r="E47" s="102" t="s">
@@ -3999,68 +3964,68 @@
       <c r="L47" s="103" t="s">
         <v>236</v>
       </c>
-      <c r="M47" s="170" t="s">
+      <c r="M47" s="158" t="s">
         <v>210</v>
       </c>
-      <c r="N47" s="134"/>
-    </row>
-    <row r="48" spans="1:14" s="134" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="163"/>
-      <c r="B48" s="106" t="s">
+      <c r="N47"/>
+    </row>
+    <row r="48" spans="1:14" ht="17" x14ac:dyDescent="0.2">
+      <c r="A48" s="15"/>
+      <c r="B48" s="11" t="s">
         <v>297</v>
       </c>
-      <c r="C48" s="107" t="s">
+      <c r="C48" s="12" t="s">
         <v>285</v>
       </c>
-      <c r="D48" s="133">
-        <v>1</v>
-      </c>
-      <c r="E48" s="107" t="s">
+      <c r="D48" s="13">
+        <v>1</v>
+      </c>
+      <c r="E48" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="F48" s="108" t="s">
+      <c r="F48" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="G48" s="108"/>
-      <c r="H48" s="108"/>
-      <c r="I48" s="108"/>
-      <c r="J48" s="108"/>
-      <c r="K48" s="108"/>
-      <c r="L48" s="108"/>
-      <c r="M48" s="115" t="s">
+      <c r="G48" s="14"/>
+      <c r="H48" s="14"/>
+      <c r="I48" s="14"/>
+      <c r="J48" s="14"/>
+      <c r="K48" s="14"/>
+      <c r="L48" s="14"/>
+      <c r="M48" s="112" t="s">
         <v>310</v>
       </c>
     </row>
-    <row r="49" spans="1:14" s="134" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="163"/>
-      <c r="B49" s="106" t="s">
+    <row r="49" spans="1:14" ht="17" x14ac:dyDescent="0.2">
+      <c r="A49" s="15"/>
+      <c r="B49" s="11" t="s">
         <v>297</v>
       </c>
-      <c r="C49" s="107" t="s">
+      <c r="C49" s="12" t="s">
         <v>308</v>
       </c>
-      <c r="D49" s="133">
-        <v>1</v>
-      </c>
-      <c r="E49" s="107" t="s">
+      <c r="D49" s="13">
+        <v>1</v>
+      </c>
+      <c r="E49" s="12" t="s">
         <v>161</v>
       </c>
-      <c r="F49" s="108" t="s">
+      <c r="F49" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="G49" s="108"/>
-      <c r="H49" s="108"/>
-      <c r="I49" s="108"/>
-      <c r="J49" s="108" t="s">
+      <c r="G49" s="14"/>
+      <c r="H49" s="14"/>
+      <c r="I49" s="14"/>
+      <c r="J49" s="14" t="s">
         <v>299</v>
       </c>
-      <c r="K49" s="108"/>
-      <c r="L49" s="108"/>
-      <c r="M49" s="115" t="s">
+      <c r="K49" s="14"/>
+      <c r="L49" s="14"/>
+      <c r="M49" s="112" t="s">
         <v>309</v>
       </c>
     </row>
-    <row r="50" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A50" s="15"/>
       <c r="B50" s="11" t="s">
         <v>297</v>
@@ -4080,16 +4045,16 @@
       <c r="G50" s="14"/>
       <c r="H50" s="14"/>
       <c r="I50" s="14"/>
-      <c r="J50" s="108" t="s">
+      <c r="J50" s="14" t="s">
         <v>299</v>
       </c>
       <c r="K50" s="14"/>
       <c r="L50" s="14"/>
-      <c r="M50" s="117" t="s">
+      <c r="M50" s="112" t="s">
         <v>311</v>
       </c>
     </row>
-    <row r="51" spans="1:14" s="96" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:14" s="96" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A51" s="15"/>
       <c r="B51" s="11" t="s">
         <v>297</v>
@@ -4109,17 +4074,17 @@
       <c r="G51" s="14"/>
       <c r="H51" s="14"/>
       <c r="I51" s="14"/>
-      <c r="J51" s="108" t="s">
+      <c r="J51" s="14" t="s">
         <v>299</v>
       </c>
       <c r="K51" s="14"/>
       <c r="L51" s="14"/>
-      <c r="M51" s="122" t="s">
+      <c r="M51" s="118" t="s">
         <v>209</v>
       </c>
-      <c r="N51" s="134"/>
-    </row>
-    <row r="52" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="N51"/>
+    </row>
+    <row r="52" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A52" s="15"/>
       <c r="B52" s="11" t="s">
         <v>297</v>
@@ -4139,16 +4104,16 @@
       <c r="G52" s="14"/>
       <c r="H52" s="14"/>
       <c r="I52" s="14"/>
-      <c r="J52" s="108" t="s">
+      <c r="J52" s="14" t="s">
         <v>299</v>
       </c>
       <c r="K52" s="14"/>
       <c r="L52" s="14"/>
-      <c r="M52" s="122" t="s">
+      <c r="M52" s="118" t="s">
         <v>312</v>
       </c>
     </row>
-    <row r="53" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A53" s="96"/>
       <c r="B53" s="11" t="s">
         <v>297</v>
@@ -4170,16 +4135,16 @@
       </c>
       <c r="H53" s="100"/>
       <c r="I53" s="100"/>
-      <c r="J53" s="108" t="s">
+      <c r="J53" s="14" t="s">
         <v>299</v>
       </c>
       <c r="K53" s="100"/>
       <c r="L53" s="100"/>
-      <c r="M53" s="123" t="s">
+      <c r="M53" s="119" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="54" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B54" s="11" t="s">
         <v>297</v>
       </c>
@@ -4200,16 +4165,16 @@
       </c>
       <c r="H54" s="14"/>
       <c r="I54" s="14"/>
-      <c r="J54" s="108" t="s">
+      <c r="J54" s="14" t="s">
         <v>299</v>
       </c>
       <c r="K54" s="14"/>
       <c r="L54" s="14"/>
-      <c r="M54" s="124" t="s">
+      <c r="M54" s="120" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="55" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B55" s="11" t="s">
         <v>297</v>
       </c>
@@ -4230,23 +4195,23 @@
       </c>
       <c r="H55" s="14"/>
       <c r="I55" s="14"/>
-      <c r="J55" s="108" t="s">
+      <c r="J55" s="14" t="s">
         <v>299</v>
       </c>
       <c r="K55" s="14"/>
       <c r="L55" s="14"/>
-      <c r="M55" s="114" t="s">
+      <c r="M55" s="111" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="56" spans="1:14" s="96" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:14" s="96" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B56" s="97" t="s">
         <v>297</v>
       </c>
       <c r="C56" s="102" t="s">
         <v>269</v>
       </c>
-      <c r="D56" s="169">
+      <c r="D56" s="157">
         <v>1</v>
       </c>
       <c r="E56" s="102" t="s">
@@ -4265,12 +4230,12 @@
       </c>
       <c r="K56" s="103"/>
       <c r="L56" s="103"/>
-      <c r="M56" s="171" t="s">
+      <c r="M56" s="159" t="s">
         <v>205</v>
       </c>
-      <c r="N56" s="134"/>
-    </row>
-    <row r="57" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="N56"/>
+    </row>
+    <row r="57" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B57" s="11" t="s">
         <v>297</v>
       </c>
@@ -4294,119 +4259,119 @@
       <c r="J57" s="14"/>
       <c r="K57" s="14"/>
       <c r="L57" s="14"/>
-      <c r="M57" s="125" t="s">
+      <c r="M57" s="121" t="s">
         <v>206</v>
       </c>
     </row>
-    <row r="58" spans="1:14" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A58" s="96"/>
-      <c r="B58" s="164" t="s">
+      <c r="B58" s="139" t="s">
         <v>297</v>
       </c>
-      <c r="C58" s="165" t="s">
+      <c r="C58" s="140" t="s">
         <v>283</v>
       </c>
-      <c r="D58" s="166">
-        <v>1</v>
-      </c>
-      <c r="E58" s="165" t="s">
+      <c r="D58" s="141">
+        <v>1</v>
+      </c>
+      <c r="E58" s="140" t="s">
         <v>49</v>
       </c>
-      <c r="F58" s="161" t="s">
-        <v>18</v>
-      </c>
-      <c r="G58" s="161"/>
-      <c r="H58" s="161"/>
-      <c r="I58" s="161"/>
-      <c r="J58" s="161"/>
-      <c r="K58" s="161"/>
-      <c r="L58" s="161"/>
-      <c r="M58" s="167" t="s">
+      <c r="F58" s="142" t="s">
+        <v>18</v>
+      </c>
+      <c r="G58" s="142"/>
+      <c r="H58" s="142"/>
+      <c r="I58" s="142"/>
+      <c r="J58" s="142"/>
+      <c r="K58" s="142"/>
+      <c r="L58" s="142"/>
+      <c r="M58" s="155" t="s">
         <v>284</v>
       </c>
     </row>
-    <row r="59" spans="1:14" ht="16.2" thickTop="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:14" ht="18" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A59" s="101"/>
-      <c r="B59" s="135" t="s">
+      <c r="B59" s="128" t="s">
         <v>171</v>
       </c>
-      <c r="C59" s="152" t="s">
+      <c r="C59" s="145" t="s">
         <v>13</v>
       </c>
-      <c r="D59" s="153">
-        <v>1</v>
-      </c>
-      <c r="E59" s="152" t="s">
+      <c r="D59" s="146">
+        <v>1</v>
+      </c>
+      <c r="E59" s="145" t="s">
         <v>14</v>
       </c>
-      <c r="F59" s="154" t="s">
-        <v>18</v>
-      </c>
-      <c r="G59" s="154"/>
-      <c r="H59" s="154"/>
-      <c r="I59" s="154"/>
-      <c r="J59" s="154"/>
-      <c r="K59" s="154"/>
-      <c r="L59" s="154"/>
-      <c r="M59" s="168" t="s">
+      <c r="F59" s="147" t="s">
+        <v>18</v>
+      </c>
+      <c r="G59" s="147"/>
+      <c r="H59" s="147"/>
+      <c r="I59" s="147"/>
+      <c r="J59" s="147"/>
+      <c r="K59" s="147"/>
+      <c r="L59" s="147"/>
+      <c r="M59" s="156" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="60" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A60" s="15"/>
-      <c r="B60" s="135" t="s">
+      <c r="B60" s="128" t="s">
         <v>171</v>
       </c>
-      <c r="C60" s="136" t="s">
+      <c r="C60" s="129" t="s">
         <v>300</v>
       </c>
-      <c r="D60" s="137">
-        <v>1</v>
-      </c>
-      <c r="E60" s="136" t="s">
+      <c r="D60" s="130">
+        <v>1</v>
+      </c>
+      <c r="E60" s="129" t="s">
         <v>14</v>
       </c>
-      <c r="F60" s="138" t="s">
-        <v>18</v>
-      </c>
-      <c r="G60" s="138"/>
-      <c r="H60" s="138"/>
-      <c r="I60" s="138"/>
-      <c r="J60" s="138"/>
-      <c r="K60" s="138"/>
-      <c r="L60" s="138"/>
-      <c r="M60" s="145" t="s">
+      <c r="F60" s="131" t="s">
+        <v>18</v>
+      </c>
+      <c r="G60" s="131"/>
+      <c r="H60" s="131"/>
+      <c r="I60" s="131"/>
+      <c r="J60" s="131"/>
+      <c r="K60" s="131"/>
+      <c r="L60" s="131"/>
+      <c r="M60" s="138" t="s">
         <v>302</v>
       </c>
     </row>
-    <row r="61" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A61" s="15"/>
-      <c r="B61" s="135" t="s">
+      <c r="B61" s="128" t="s">
         <v>171</v>
       </c>
-      <c r="C61" s="136" t="s">
+      <c r="C61" s="129" t="s">
         <v>301</v>
       </c>
-      <c r="D61" s="137">
-        <v>1</v>
-      </c>
-      <c r="E61" s="136" t="s">
+      <c r="D61" s="130">
+        <v>1</v>
+      </c>
+      <c r="E61" s="129" t="s">
         <v>19</v>
       </c>
-      <c r="F61" s="138" t="s">
-        <v>18</v>
-      </c>
-      <c r="G61" s="138"/>
-      <c r="H61" s="138"/>
-      <c r="I61" s="138"/>
-      <c r="J61" s="138"/>
-      <c r="K61" s="138"/>
-      <c r="L61" s="138"/>
-      <c r="M61" s="145" t="s">
+      <c r="F61" s="131" t="s">
+        <v>18</v>
+      </c>
+      <c r="G61" s="131"/>
+      <c r="H61" s="131"/>
+      <c r="I61" s="131"/>
+      <c r="J61" s="131"/>
+      <c r="K61" s="131"/>
+      <c r="L61" s="131"/>
+      <c r="M61" s="138" t="s">
         <v>303</v>
       </c>
     </row>
-    <row r="62" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B62" s="11" t="s">
         <v>171</v>
       </c>
@@ -4425,16 +4390,16 @@
       <c r="G62" s="14"/>
       <c r="H62" s="14"/>
       <c r="I62" s="14"/>
-      <c r="J62" s="108" t="s">
+      <c r="J62" s="14" t="s">
         <v>299</v>
       </c>
       <c r="K62" s="14"/>
       <c r="L62" s="14"/>
-      <c r="M62" s="114" t="s">
+      <c r="M62" s="111" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="63" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B63" s="11" t="s">
         <v>171</v>
       </c>
@@ -4453,16 +4418,16 @@
       <c r="G63" s="14"/>
       <c r="H63" s="14"/>
       <c r="I63" s="14"/>
-      <c r="J63" s="108" t="s">
+      <c r="J63" s="14" t="s">
         <v>299</v>
       </c>
       <c r="K63" s="14"/>
       <c r="L63" s="14"/>
-      <c r="M63" s="125" t="s">
+      <c r="M63" s="121" t="s">
         <v>214</v>
       </c>
     </row>
-    <row r="64" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B64" s="11" t="s">
         <v>171</v>
       </c>
@@ -4481,14 +4446,14 @@
       <c r="G64" s="14"/>
       <c r="H64" s="14"/>
       <c r="I64" s="14"/>
-      <c r="J64" s="108"/>
+      <c r="J64" s="14"/>
       <c r="K64" s="14"/>
       <c r="L64" s="14"/>
-      <c r="M64" s="171" t="s">
+      <c r="M64" s="159" t="s">
         <v>288</v>
       </c>
     </row>
-    <row r="65" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B65" s="11" t="s">
         <v>171</v>
       </c>
@@ -4507,7 +4472,7 @@
       <c r="G65" s="14"/>
       <c r="H65" s="14"/>
       <c r="I65" s="14"/>
-      <c r="J65" s="108" t="s">
+      <c r="J65" s="14" t="s">
         <v>287</v>
       </c>
       <c r="K65" s="14" t="s">
@@ -4516,11 +4481,11 @@
       <c r="L65" s="14" t="s">
         <v>313</v>
       </c>
-      <c r="M65" s="114" t="s">
+      <c r="M65" s="111" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="66" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B66" s="11" t="s">
         <v>171</v>
       </c>
@@ -4539,16 +4504,16 @@
       <c r="G66" s="14"/>
       <c r="H66" s="14"/>
       <c r="I66" s="14"/>
-      <c r="J66" s="108" t="s">
+      <c r="J66" s="14" t="s">
         <v>287</v>
       </c>
       <c r="K66" s="14"/>
       <c r="L66" s="14"/>
-      <c r="M66" s="126" t="s">
+      <c r="M66" s="122" t="s">
         <v>216</v>
       </c>
     </row>
-    <row r="67" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B67" s="11" t="s">
         <v>171</v>
       </c>
@@ -4569,16 +4534,16 @@
       </c>
       <c r="H67" s="14"/>
       <c r="I67" s="14"/>
-      <c r="J67" s="108" t="s">
+      <c r="J67" s="14" t="s">
         <v>287</v>
       </c>
       <c r="K67" s="14"/>
       <c r="L67" s="14"/>
-      <c r="M67" s="114" t="s">
+      <c r="M67" s="111" t="s">
         <v>217</v>
       </c>
     </row>
-    <row r="68" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B68" s="11" t="s">
         <v>171</v>
       </c>
@@ -4599,23 +4564,23 @@
       </c>
       <c r="H68" s="14"/>
       <c r="I68" s="14"/>
-      <c r="J68" s="108" t="s">
+      <c r="J68" s="14" t="s">
         <v>287</v>
       </c>
       <c r="K68" s="14"/>
       <c r="L68" s="14"/>
-      <c r="M68" s="125" t="s">
+      <c r="M68" s="121" t="s">
         <v>218</v>
       </c>
     </row>
-    <row r="69" spans="1:14" s="96" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:14" s="96" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B69" s="97" t="s">
         <v>171</v>
       </c>
       <c r="C69" s="102" t="s">
         <v>173</v>
       </c>
-      <c r="D69" s="169">
+      <c r="D69" s="157">
         <v>1</v>
       </c>
       <c r="E69" s="102" t="s">
@@ -4632,12 +4597,12 @@
       </c>
       <c r="K69" s="103"/>
       <c r="L69" s="103"/>
-      <c r="M69" s="173" t="s">
+      <c r="M69" s="161" t="s">
         <v>219</v>
       </c>
-      <c r="N69" s="134"/>
-    </row>
-    <row r="70" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="N69"/>
+    </row>
+    <row r="70" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B70" s="11" t="s">
         <v>171</v>
       </c>
@@ -4656,16 +4621,16 @@
       <c r="G70" s="14"/>
       <c r="H70" s="14"/>
       <c r="I70" s="14"/>
-      <c r="J70" s="108" t="s">
+      <c r="J70" s="14" t="s">
         <v>287</v>
       </c>
       <c r="K70" s="14"/>
       <c r="L70" s="14"/>
-      <c r="M70" s="125" t="s">
+      <c r="M70" s="121" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="71" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B71" s="11" t="s">
         <v>171</v>
       </c>
@@ -4684,16 +4649,16 @@
       <c r="G71" s="14"/>
       <c r="H71" s="14"/>
       <c r="I71" s="14"/>
-      <c r="J71" s="108" t="s">
+      <c r="J71" s="14" t="s">
         <v>287</v>
       </c>
       <c r="K71" s="14"/>
       <c r="L71" s="14"/>
-      <c r="M71" s="114" t="s">
+      <c r="M71" s="111" t="s">
         <v>223</v>
       </c>
     </row>
-    <row r="72" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B72" s="11" t="s">
         <v>171</v>
       </c>
@@ -4714,127 +4679,127 @@
       </c>
       <c r="H72" s="14"/>
       <c r="I72" s="14"/>
-      <c r="J72" s="108" t="s">
+      <c r="J72" s="14" t="s">
         <v>287</v>
       </c>
       <c r="K72" s="14"/>
       <c r="L72" s="14"/>
-      <c r="M72" s="114" t="s">
+      <c r="M72" s="111" t="s">
         <v>220</v>
       </c>
     </row>
-    <row r="73" spans="1:14" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B73" s="146" t="s">
+    <row r="73" spans="1:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B73" s="139" t="s">
         <v>171</v>
       </c>
-      <c r="C73" s="147" t="s">
+      <c r="C73" s="140" t="s">
         <v>275</v>
       </c>
-      <c r="D73" s="148">
-        <v>1</v>
-      </c>
-      <c r="E73" s="147" t="s">
+      <c r="D73" s="141">
+        <v>1</v>
+      </c>
+      <c r="E73" s="140" t="s">
         <v>22</v>
       </c>
-      <c r="F73" s="149" t="s">
+      <c r="F73" s="142" t="s">
         <v>15</v>
       </c>
-      <c r="G73" s="149" t="s">
+      <c r="G73" s="142" t="s">
         <v>324</v>
       </c>
-      <c r="H73" s="149"/>
-      <c r="I73" s="149"/>
-      <c r="J73" s="161" t="s">
+      <c r="H73" s="142"/>
+      <c r="I73" s="142"/>
+      <c r="J73" s="142" t="s">
         <v>287</v>
       </c>
-      <c r="K73" s="149"/>
-      <c r="L73" s="149"/>
-      <c r="M73" s="172" t="s">
+      <c r="K73" s="142"/>
+      <c r="L73" s="142"/>
+      <c r="M73" s="160" t="s">
         <v>221</v>
       </c>
     </row>
-    <row r="74" spans="1:14" ht="16.2" thickTop="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:14" ht="18" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A74" s="96"/>
-      <c r="B74" s="135" t="s">
+      <c r="B74" s="128" t="s">
         <v>176</v>
       </c>
-      <c r="C74" s="152" t="s">
+      <c r="C74" s="145" t="s">
         <v>13</v>
       </c>
-      <c r="D74" s="153">
-        <v>1</v>
-      </c>
-      <c r="E74" s="152" t="s">
+      <c r="D74" s="146">
+        <v>1</v>
+      </c>
+      <c r="E74" s="145" t="s">
         <v>14</v>
       </c>
-      <c r="F74" s="154" t="s">
+      <c r="F74" s="147" t="s">
         <v>15</v>
       </c>
-      <c r="G74" s="154"/>
-      <c r="H74" s="154"/>
-      <c r="I74" s="154"/>
-      <c r="J74" s="154"/>
-      <c r="K74" s="154"/>
-      <c r="L74" s="154"/>
-      <c r="M74" s="145" t="s">
+      <c r="G74" s="147"/>
+      <c r="H74" s="147"/>
+      <c r="I74" s="147"/>
+      <c r="J74" s="147"/>
+      <c r="K74" s="147"/>
+      <c r="L74" s="147"/>
+      <c r="M74" s="138" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="75" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A75" s="101"/>
-      <c r="B75" s="135" t="s">
+      <c r="B75" s="128" t="s">
         <v>176</v>
       </c>
-      <c r="C75" s="136" t="s">
+      <c r="C75" s="129" t="s">
         <v>300</v>
       </c>
-      <c r="D75" s="137">
-        <v>1</v>
-      </c>
-      <c r="E75" s="136" t="s">
+      <c r="D75" s="130">
+        <v>1</v>
+      </c>
+      <c r="E75" s="129" t="s">
         <v>14</v>
       </c>
-      <c r="F75" s="138" t="s">
-        <v>18</v>
-      </c>
-      <c r="G75" s="138"/>
-      <c r="H75" s="138"/>
-      <c r="I75" s="138"/>
-      <c r="J75" s="138"/>
-      <c r="K75" s="138"/>
-      <c r="L75" s="138"/>
-      <c r="M75" s="145" t="s">
+      <c r="F75" s="131" t="s">
+        <v>18</v>
+      </c>
+      <c r="G75" s="131"/>
+      <c r="H75" s="131"/>
+      <c r="I75" s="131"/>
+      <c r="J75" s="131"/>
+      <c r="K75" s="131"/>
+      <c r="L75" s="131"/>
+      <c r="M75" s="138" t="s">
         <v>302</v>
       </c>
     </row>
-    <row r="76" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A76" s="101"/>
-      <c r="B76" s="135" t="s">
+      <c r="B76" s="128" t="s">
         <v>176</v>
       </c>
-      <c r="C76" s="136" t="s">
+      <c r="C76" s="129" t="s">
         <v>301</v>
       </c>
-      <c r="D76" s="137">
-        <v>1</v>
-      </c>
-      <c r="E76" s="136" t="s">
+      <c r="D76" s="130">
+        <v>1</v>
+      </c>
+      <c r="E76" s="129" t="s">
         <v>19</v>
       </c>
-      <c r="F76" s="138" t="s">
-        <v>18</v>
-      </c>
-      <c r="G76" s="138"/>
-      <c r="H76" s="138"/>
-      <c r="I76" s="138"/>
-      <c r="J76" s="138"/>
-      <c r="K76" s="138"/>
-      <c r="L76" s="138"/>
-      <c r="M76" s="145" t="s">
+      <c r="F76" s="131" t="s">
+        <v>18</v>
+      </c>
+      <c r="G76" s="131"/>
+      <c r="H76" s="131"/>
+      <c r="I76" s="131"/>
+      <c r="J76" s="131"/>
+      <c r="K76" s="131"/>
+      <c r="L76" s="131"/>
+      <c r="M76" s="138" t="s">
         <v>303</v>
       </c>
     </row>
-    <row r="77" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A77" s="96"/>
       <c r="B77" s="11" t="s">
         <v>176</v>
@@ -4859,11 +4824,11 @@
       </c>
       <c r="K77" s="14"/>
       <c r="L77" s="14"/>
-      <c r="M77" s="125" t="s">
+      <c r="M77" s="121" t="s">
         <v>227</v>
       </c>
     </row>
-    <row r="78" spans="1:14" s="96" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:14" s="96" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B78" s="11" t="s">
         <v>176</v>
       </c>
@@ -4887,12 +4852,12 @@
       </c>
       <c r="K78" s="14"/>
       <c r="L78" s="14"/>
-      <c r="M78" s="114" t="s">
+      <c r="M78" s="111" t="s">
         <v>228</v>
       </c>
-      <c r="N78" s="134"/>
-    </row>
-    <row r="79" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="N78"/>
+    </row>
+    <row r="79" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A79" s="96"/>
       <c r="B79" s="11" t="s">
         <v>176</v>
@@ -4917,11 +4882,11 @@
       <c r="J79" s="14"/>
       <c r="K79" s="14"/>
       <c r="L79" s="14"/>
-      <c r="M79" s="114" t="s">
+      <c r="M79" s="111" t="s">
         <v>229</v>
       </c>
     </row>
-    <row r="80" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A80" s="96"/>
       <c r="B80" s="97" t="s">
         <v>176</v>
@@ -4929,7 +4894,7 @@
       <c r="C80" s="102" t="s">
         <v>277</v>
       </c>
-      <c r="D80" s="169">
+      <c r="D80" s="157">
         <v>1</v>
       </c>
       <c r="E80" s="102" t="s">
@@ -4950,11 +4915,11 @@
       <c r="L80" s="103" t="s">
         <v>235</v>
       </c>
-      <c r="M80" s="173" t="s">
+      <c r="M80" s="161" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="81" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A81" s="96"/>
       <c r="B81" s="11" t="s">
         <v>176</v>
@@ -4979,121 +4944,121 @@
       </c>
       <c r="K81" s="14"/>
       <c r="L81" s="14"/>
-      <c r="M81" s="125" t="s">
+      <c r="M81" s="121" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="82" spans="1:14" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A82" s="96"/>
-      <c r="B82" s="146" t="s">
+      <c r="B82" s="139" t="s">
         <v>176</v>
       </c>
-      <c r="C82" s="147" t="s">
+      <c r="C82" s="140" t="s">
         <v>286</v>
       </c>
-      <c r="D82" s="148">
-        <v>1</v>
-      </c>
-      <c r="E82" s="147" t="s">
+      <c r="D82" s="141">
+        <v>1</v>
+      </c>
+      <c r="E82" s="140" t="s">
         <v>49</v>
       </c>
-      <c r="F82" s="149" t="s">
-        <v>18</v>
-      </c>
-      <c r="G82" s="149"/>
-      <c r="H82" s="149" t="s">
+      <c r="F82" s="142" t="s">
+        <v>18</v>
+      </c>
+      <c r="G82" s="142"/>
+      <c r="H82" s="142" t="s">
         <v>292</v>
       </c>
-      <c r="I82" s="149"/>
-      <c r="J82" s="149"/>
-      <c r="K82" s="149"/>
-      <c r="L82" s="149"/>
-      <c r="M82" s="172" t="s">
+      <c r="I82" s="142"/>
+      <c r="J82" s="142"/>
+      <c r="K82" s="142"/>
+      <c r="L82" s="142"/>
+      <c r="M82" s="160" t="s">
         <v>314</v>
       </c>
     </row>
-    <row r="83" spans="1:14" s="96" customFormat="1" ht="16.2" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B83" s="135" t="s">
+    <row r="83" spans="1:14" s="96" customFormat="1" ht="18" thickTop="1" x14ac:dyDescent="0.2">
+      <c r="B83" s="128" t="s">
         <v>289</v>
       </c>
-      <c r="C83" s="152" t="s">
+      <c r="C83" s="145" t="s">
         <v>13</v>
       </c>
-      <c r="D83" s="153">
-        <v>1</v>
-      </c>
-      <c r="E83" s="152" t="s">
+      <c r="D83" s="146">
+        <v>1</v>
+      </c>
+      <c r="E83" s="145" t="s">
         <v>14</v>
       </c>
-      <c r="F83" s="154" t="s">
+      <c r="F83" s="147" t="s">
         <v>15</v>
       </c>
-      <c r="G83" s="154"/>
-      <c r="H83" s="154"/>
-      <c r="I83" s="154"/>
-      <c r="J83" s="154"/>
-      <c r="K83" s="154"/>
-      <c r="L83" s="154"/>
-      <c r="M83" s="145" t="s">
+      <c r="G83" s="147"/>
+      <c r="H83" s="147"/>
+      <c r="I83" s="147"/>
+      <c r="J83" s="147"/>
+      <c r="K83" s="147"/>
+      <c r="L83" s="147"/>
+      <c r="M83" s="138" t="s">
         <v>16</v>
       </c>
-      <c r="N83" s="134"/>
-    </row>
-    <row r="84" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="N83"/>
+    </row>
+    <row r="84" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A84" s="15"/>
-      <c r="B84" s="135" t="s">
+      <c r="B84" s="128" t="s">
         <v>289</v>
       </c>
-      <c r="C84" s="136" t="s">
+      <c r="C84" s="129" t="s">
         <v>300</v>
       </c>
-      <c r="D84" s="137">
-        <v>1</v>
-      </c>
-      <c r="E84" s="136" t="s">
+      <c r="D84" s="130">
+        <v>1</v>
+      </c>
+      <c r="E84" s="129" t="s">
         <v>14</v>
       </c>
-      <c r="F84" s="138" t="s">
-        <v>18</v>
-      </c>
-      <c r="G84" s="138"/>
-      <c r="H84" s="138"/>
-      <c r="I84" s="138"/>
-      <c r="J84" s="138"/>
-      <c r="K84" s="138"/>
-      <c r="L84" s="138"/>
-      <c r="M84" s="145" t="s">
+      <c r="F84" s="131" t="s">
+        <v>18</v>
+      </c>
+      <c r="G84" s="131"/>
+      <c r="H84" s="131"/>
+      <c r="I84" s="131"/>
+      <c r="J84" s="131"/>
+      <c r="K84" s="131"/>
+      <c r="L84" s="131"/>
+      <c r="M84" s="138" t="s">
         <v>302</v>
       </c>
     </row>
-    <row r="85" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A85" s="15"/>
-      <c r="B85" s="135" t="s">
+      <c r="B85" s="128" t="s">
         <v>289</v>
       </c>
-      <c r="C85" s="136" t="s">
+      <c r="C85" s="129" t="s">
         <v>301</v>
       </c>
-      <c r="D85" s="137">
-        <v>1</v>
-      </c>
-      <c r="E85" s="136" t="s">
+      <c r="D85" s="130">
+        <v>1</v>
+      </c>
+      <c r="E85" s="129" t="s">
         <v>19</v>
       </c>
-      <c r="F85" s="138" t="s">
-        <v>18</v>
-      </c>
-      <c r="G85" s="138"/>
-      <c r="H85" s="138"/>
-      <c r="I85" s="138"/>
-      <c r="J85" s="138"/>
-      <c r="K85" s="138"/>
-      <c r="L85" s="138"/>
-      <c r="M85" s="145" t="s">
+      <c r="F85" s="131" t="s">
+        <v>18</v>
+      </c>
+      <c r="G85" s="131"/>
+      <c r="H85" s="131"/>
+      <c r="I85" s="131"/>
+      <c r="J85" s="131"/>
+      <c r="K85" s="131"/>
+      <c r="L85" s="131"/>
+      <c r="M85" s="138" t="s">
         <v>303</v>
       </c>
     </row>
-    <row r="86" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B86" s="97" t="s">
         <v>289</v>
       </c>
@@ -5117,11 +5082,11 @@
       <c r="J86" s="14"/>
       <c r="K86" s="14"/>
       <c r="L86" s="14"/>
-      <c r="M86" s="114" t="s">
+      <c r="M86" s="111" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="87" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A87" s="96"/>
       <c r="B87" s="97" t="s">
         <v>289</v>
@@ -5129,7 +5094,7 @@
       <c r="C87" s="102" t="s">
         <v>280</v>
       </c>
-      <c r="D87" s="169">
+      <c r="D87" s="157">
         <v>1</v>
       </c>
       <c r="E87" s="102" t="s">
@@ -5146,11 +5111,11 @@
       <c r="J87" s="103"/>
       <c r="K87" s="103"/>
       <c r="L87" s="103"/>
-      <c r="M87" s="173" t="s">
+      <c r="M87" s="161" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="88" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B88" s="97" t="s">
         <v>289</v>
       </c>
@@ -5160,7 +5125,7 @@
       <c r="D88" s="13">
         <v>1</v>
       </c>
-      <c r="E88" s="107" t="s">
+      <c r="E88" s="12" t="s">
         <v>26</v>
       </c>
       <c r="F88" s="14" t="s">
@@ -5174,11 +5139,11 @@
       </c>
       <c r="K88" s="14"/>
       <c r="L88" s="14"/>
-      <c r="M88" s="114" t="s">
+      <c r="M88" s="111" t="s">
         <v>291</v>
       </c>
     </row>
-    <row r="89" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B89" s="97" t="s">
         <v>289</v>
       </c>
@@ -5202,120 +5167,120 @@
       </c>
       <c r="K89" s="14"/>
       <c r="L89" s="14"/>
-      <c r="M89" s="125" t="s">
+      <c r="M89" s="121" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="90" spans="1:14" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B90" s="155" t="s">
+    <row r="90" spans="1:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B90" s="148" t="s">
         <v>289</v>
       </c>
-      <c r="C90" s="147" t="s">
+      <c r="C90" s="140" t="s">
         <v>286</v>
       </c>
-      <c r="D90" s="148">
-        <v>1</v>
-      </c>
-      <c r="E90" s="147" t="s">
+      <c r="D90" s="141">
+        <v>1</v>
+      </c>
+      <c r="E90" s="140" t="s">
         <v>49</v>
       </c>
-      <c r="F90" s="149" t="s">
-        <v>18</v>
-      </c>
-      <c r="G90" s="149"/>
-      <c r="H90" s="149" t="s">
+      <c r="F90" s="142" t="s">
+        <v>18</v>
+      </c>
+      <c r="G90" s="142"/>
+      <c r="H90" s="142" t="s">
         <v>292</v>
       </c>
-      <c r="I90" s="149"/>
-      <c r="J90" s="149"/>
-      <c r="K90" s="149"/>
-      <c r="L90" s="149"/>
-      <c r="M90" s="172" t="s">
+      <c r="I90" s="142"/>
+      <c r="J90" s="142"/>
+      <c r="K90" s="142"/>
+      <c r="L90" s="142"/>
+      <c r="M90" s="160" t="s">
         <v>315</v>
       </c>
     </row>
-    <row r="91" spans="1:14" ht="16.2" thickTop="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:14" ht="17" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A91" s="104"/>
-      <c r="B91" s="135" t="s">
+      <c r="B91" s="128" t="s">
         <v>298</v>
       </c>
-      <c r="C91" s="152" t="s">
+      <c r="C91" s="145" t="s">
         <v>13</v>
       </c>
-      <c r="D91" s="153">
-        <v>1</v>
-      </c>
-      <c r="E91" s="152" t="s">
+      <c r="D91" s="146">
+        <v>1</v>
+      </c>
+      <c r="E91" s="145" t="s">
         <v>14</v>
       </c>
-      <c r="F91" s="154" t="s">
+      <c r="F91" s="147" t="s">
         <v>15</v>
       </c>
-      <c r="G91" s="154"/>
-      <c r="H91" s="154"/>
-      <c r="I91" s="154"/>
-      <c r="J91" s="154"/>
-      <c r="K91" s="154"/>
-      <c r="L91" s="154"/>
-      <c r="M91" s="139" t="s">
+      <c r="G91" s="147"/>
+      <c r="H91" s="147"/>
+      <c r="I91" s="147"/>
+      <c r="J91" s="147"/>
+      <c r="K91" s="147"/>
+      <c r="L91" s="147"/>
+      <c r="M91" s="132" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="92" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A92" s="15"/>
-      <c r="B92" s="135" t="s">
+      <c r="B92" s="128" t="s">
         <v>298</v>
       </c>
-      <c r="C92" s="136" t="s">
+      <c r="C92" s="129" t="s">
         <v>300</v>
       </c>
-      <c r="D92" s="137">
-        <v>1</v>
-      </c>
-      <c r="E92" s="136" t="s">
+      <c r="D92" s="130">
+        <v>1</v>
+      </c>
+      <c r="E92" s="129" t="s">
         <v>14</v>
       </c>
-      <c r="F92" s="138" t="s">
-        <v>18</v>
-      </c>
-      <c r="G92" s="138"/>
-      <c r="H92" s="138"/>
-      <c r="I92" s="138"/>
-      <c r="J92" s="138"/>
-      <c r="K92" s="138"/>
-      <c r="L92" s="138"/>
-      <c r="M92" s="145" t="s">
+      <c r="F92" s="131" t="s">
+        <v>18</v>
+      </c>
+      <c r="G92" s="131"/>
+      <c r="H92" s="131"/>
+      <c r="I92" s="131"/>
+      <c r="J92" s="131"/>
+      <c r="K92" s="131"/>
+      <c r="L92" s="131"/>
+      <c r="M92" s="138" t="s">
         <v>302</v>
       </c>
     </row>
-    <row r="93" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A93" s="15"/>
-      <c r="B93" s="135" t="s">
+      <c r="B93" s="128" t="s">
         <v>298</v>
       </c>
-      <c r="C93" s="136" t="s">
+      <c r="C93" s="129" t="s">
         <v>301</v>
       </c>
-      <c r="D93" s="137">
-        <v>1</v>
-      </c>
-      <c r="E93" s="136" t="s">
+      <c r="D93" s="130">
+        <v>1</v>
+      </c>
+      <c r="E93" s="129" t="s">
         <v>19</v>
       </c>
-      <c r="F93" s="138" t="s">
-        <v>18</v>
-      </c>
-      <c r="G93" s="138"/>
-      <c r="H93" s="138"/>
-      <c r="I93" s="138"/>
-      <c r="J93" s="138"/>
-      <c r="K93" s="138"/>
-      <c r="L93" s="138"/>
-      <c r="M93" s="145" t="s">
+      <c r="F93" s="131" t="s">
+        <v>18</v>
+      </c>
+      <c r="G93" s="131"/>
+      <c r="H93" s="131"/>
+      <c r="I93" s="131"/>
+      <c r="J93" s="131"/>
+      <c r="K93" s="131"/>
+      <c r="L93" s="131"/>
+      <c r="M93" s="138" t="s">
         <v>303</v>
       </c>
     </row>
-    <row r="94" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B94" s="11" t="s">
         <v>298</v>
       </c>
@@ -5334,16 +5299,16 @@
       <c r="G94" s="14"/>
       <c r="H94" s="14"/>
       <c r="I94" s="14"/>
-      <c r="J94" s="108" t="s">
+      <c r="J94" s="14" t="s">
         <v>299</v>
       </c>
       <c r="K94" s="14"/>
       <c r="L94" s="14"/>
-      <c r="M94" s="114" t="s">
+      <c r="M94" s="111" t="s">
         <v>224</v>
       </c>
     </row>
-    <row r="95" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B95" s="11" t="s">
         <v>298</v>
       </c>
@@ -5362,16 +5327,16 @@
       <c r="G95" s="14"/>
       <c r="H95" s="14"/>
       <c r="I95" s="14"/>
-      <c r="J95" s="108" t="s">
+      <c r="J95" s="14" t="s">
         <v>299</v>
       </c>
       <c r="K95" s="14"/>
       <c r="L95" s="14"/>
-      <c r="M95" s="114" t="s">
+      <c r="M95" s="111" t="s">
         <v>225</v>
       </c>
     </row>
-    <row r="96" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B96" s="11" t="s">
         <v>298</v>
       </c>
@@ -5390,40 +5355,40 @@
       <c r="G96" s="14"/>
       <c r="H96" s="14"/>
       <c r="I96" s="14"/>
-      <c r="J96" s="108" t="s">
+      <c r="J96" s="14" t="s">
         <v>299</v>
       </c>
       <c r="K96" s="14"/>
       <c r="L96" s="14"/>
-      <c r="M96" s="114" t="s">
+      <c r="M96" s="111" t="s">
         <v>282</v>
       </c>
     </row>
-    <row r="97" spans="2:13" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B97" s="127" t="s">
+    <row r="97" spans="2:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B97" s="123" t="s">
         <v>298</v>
       </c>
-      <c r="C97" s="128" t="s">
+      <c r="C97" s="124" t="s">
         <v>161</v>
       </c>
-      <c r="D97" s="129">
-        <v>1</v>
-      </c>
-      <c r="E97" s="128" t="s">
+      <c r="D97" s="125">
+        <v>1</v>
+      </c>
+      <c r="E97" s="124" t="s">
         <v>14</v>
       </c>
-      <c r="F97" s="130" t="s">
+      <c r="F97" s="126" t="s">
         <v>15</v>
       </c>
-      <c r="G97" s="130"/>
-      <c r="H97" s="130"/>
-      <c r="I97" s="130"/>
-      <c r="J97" s="131" t="s">
+      <c r="G97" s="126"/>
+      <c r="H97" s="126"/>
+      <c r="I97" s="126"/>
+      <c r="J97" s="126" t="s">
         <v>299</v>
       </c>
-      <c r="K97" s="130"/>
-      <c r="L97" s="130"/>
-      <c r="M97" s="132" t="s">
+      <c r="K97" s="126"/>
+      <c r="L97" s="126"/>
+      <c r="M97" s="127" t="s">
         <v>226</v>
       </c>
     </row>
@@ -5440,25 +5405,25 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="B1:M61"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="2.88671875" customWidth="1"/>
-    <col min="2" max="2" width="34.109375" customWidth="1"/>
-    <col min="3" max="3" width="24.88671875" style="3" customWidth="1"/>
+    <col min="1" max="1" width="2.83203125" customWidth="1"/>
+    <col min="2" max="2" width="34.1640625" customWidth="1"/>
+    <col min="3" max="3" width="24.83203125" style="3" customWidth="1"/>
     <col min="4" max="4" width="9" style="3" customWidth="1"/>
-    <col min="5" max="5" width="9.44140625" style="3" customWidth="1"/>
-    <col min="6" max="6" width="9.44140625" customWidth="1"/>
+    <col min="5" max="5" width="9.5" style="3" customWidth="1"/>
+    <col min="6" max="6" width="9.5" customWidth="1"/>
     <col min="7" max="7" width="5" customWidth="1"/>
-    <col min="8" max="8" width="26.44140625" customWidth="1"/>
-    <col min="9" max="9" width="34.88671875" customWidth="1"/>
+    <col min="8" max="8" width="26.5" customWidth="1"/>
+    <col min="9" max="9" width="34.83203125" customWidth="1"/>
     <col min="10" max="10" width="31" customWidth="1"/>
-    <col min="11" max="11" width="15.88671875" customWidth="1"/>
-    <col min="12" max="12" width="22.44140625" customWidth="1"/>
-    <col min="13" max="13" width="96.88671875" customWidth="1"/>
+    <col min="11" max="11" width="15.83203125" customWidth="1"/>
+    <col min="12" max="12" width="22.5" customWidth="1"/>
+    <col min="13" max="13" width="96.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:13" ht="9.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="2:13" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:13" ht="9.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="2" spans="2:13" ht="16" x14ac:dyDescent="0.2">
       <c r="B2" s="17" t="s">
         <v>1</v>
       </c>
@@ -5496,7 +5461,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B3" s="20" t="s">
         <v>27</v>
       </c>
@@ -5522,7 +5487,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="4" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B4" s="25" t="s">
         <v>27</v>
       </c>
@@ -5550,7 +5515,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B5" s="25" t="s">
         <v>27</v>
       </c>
@@ -5578,7 +5543,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="6" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B6" s="25" t="s">
         <v>27</v>
       </c>
@@ -5606,7 +5571,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="7" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B7" s="25" t="s">
         <v>27</v>
       </c>
@@ -5634,7 +5599,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="8" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B8" s="29" t="s">
         <v>27</v>
       </c>
@@ -5662,7 +5627,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="9" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B9" s="29" t="s">
         <v>27</v>
       </c>
@@ -5690,7 +5655,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="10" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B10" s="34" t="s">
         <v>30</v>
       </c>
@@ -5716,7 +5681,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="11" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B11" s="39" t="s">
         <v>30</v>
       </c>
@@ -5744,7 +5709,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="12" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B12" s="25" t="s">
         <v>30</v>
       </c>
@@ -5772,7 +5737,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="13" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B13" s="25" t="s">
         <v>30</v>
       </c>
@@ -5800,7 +5765,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="14" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B14" s="25" t="s">
         <v>30</v>
       </c>
@@ -5832,7 +5797,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="15" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B15" s="25" t="s">
         <v>30</v>
       </c>
@@ -5866,7 +5831,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="16" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B16" s="44" t="s">
         <v>30</v>
       </c>
@@ -5896,7 +5861,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="17" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B17" s="49" t="s">
         <v>33</v>
       </c>
@@ -5922,7 +5887,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="18" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B18" s="39" t="s">
         <v>33</v>
       </c>
@@ -5950,7 +5915,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="19" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B19" s="25" t="s">
         <v>33</v>
       </c>
@@ -5978,7 +5943,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="20" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B20" s="29" t="s">
         <v>33</v>
       </c>
@@ -6006,7 +5971,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="21" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B21" s="34" t="s">
         <v>36</v>
       </c>
@@ -6032,7 +5997,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="22" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B22" s="54" t="s">
         <v>36</v>
       </c>
@@ -6060,7 +6025,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="23" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B23" s="49" t="s">
         <v>39</v>
       </c>
@@ -6086,7 +6051,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="24" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B24" s="39" t="s">
         <v>39</v>
       </c>
@@ -6114,7 +6079,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="25" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B25" s="29" t="s">
         <v>39</v>
       </c>
@@ -6140,7 +6105,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="26" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B26" s="34" t="s">
         <v>86</v>
       </c>
@@ -6166,7 +6131,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="27" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B27" s="25" t="s">
         <v>86</v>
       </c>
@@ -6192,7 +6157,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="28" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B28" s="25" t="s">
         <v>86</v>
       </c>
@@ -6218,7 +6183,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="29" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B29" s="25" t="s">
         <v>86</v>
       </c>
@@ -6244,7 +6209,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="30" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B30" s="54" t="s">
         <v>86</v>
       </c>
@@ -6272,7 +6237,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="31" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B31" s="59" t="s">
         <v>42</v>
       </c>
@@ -6298,7 +6263,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="32" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B32" s="49" t="s">
         <v>45</v>
       </c>
@@ -6324,7 +6289,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="33" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B33" s="25" t="s">
         <v>45</v>
       </c>
@@ -6352,7 +6317,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="34" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B34" s="25" t="s">
         <v>45</v>
       </c>
@@ -6380,7 +6345,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="35" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B35" s="25" t="s">
         <v>45</v>
       </c>
@@ -6408,7 +6373,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="36" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B36" s="25" t="s">
         <v>45</v>
       </c>
@@ -6436,7 +6401,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="37" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B37" s="29" t="s">
         <v>45</v>
       </c>
@@ -6464,7 +6429,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="38" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B38" s="29" t="s">
         <v>45</v>
       </c>
@@ -6492,7 +6457,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="39" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B39" s="44" t="s">
         <v>45</v>
       </c>
@@ -6520,7 +6485,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="40" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B40" s="49" t="s">
         <v>103</v>
       </c>
@@ -6546,7 +6511,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="41" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B41" s="25" t="s">
         <v>103</v>
       </c>
@@ -6572,7 +6537,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="42" spans="2:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B42" s="39" t="s">
         <v>103</v>
       </c>
@@ -6600,7 +6565,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="43" spans="2:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B43" s="64" t="s">
         <v>103</v>
       </c>
@@ -6630,38 +6595,38 @@
         <v>120</v>
       </c>
     </row>
-    <row r="47" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B47" s="183" t="s">
+    <row r="47" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B47" s="174" t="s">
         <v>121</v>
       </c>
-      <c r="C47" s="183"/>
-      <c r="D47" s="183"/>
-      <c r="E47" s="183"/>
-      <c r="F47" s="183"/>
-      <c r="H47" s="184" t="s">
+      <c r="C47" s="174"/>
+      <c r="D47" s="174"/>
+      <c r="E47" s="174"/>
+      <c r="F47" s="174"/>
+      <c r="H47" s="175" t="s">
         <v>122</v>
       </c>
-      <c r="I47" s="184"/>
-    </row>
-    <row r="48" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B48" s="183"/>
-      <c r="C48" s="183"/>
-      <c r="D48" s="183"/>
-      <c r="E48" s="183"/>
-      <c r="F48" s="183"/>
-      <c r="H48" s="184"/>
-      <c r="I48" s="184"/>
-    </row>
-    <row r="49" spans="2:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="I47" s="175"/>
+    </row>
+    <row r="48" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B48" s="174"/>
+      <c r="C48" s="174"/>
+      <c r="D48" s="174"/>
+      <c r="E48" s="174"/>
+      <c r="F48" s="174"/>
+      <c r="H48" s="175"/>
+      <c r="I48" s="175"/>
+    </row>
+    <row r="49" spans="2:9" ht="16" x14ac:dyDescent="0.2">
       <c r="B49" s="68" t="s">
         <v>123</v>
       </c>
-      <c r="C49" s="185" t="s">
+      <c r="C49" s="176" t="s">
         <v>12</v>
       </c>
-      <c r="D49" s="185"/>
-      <c r="E49" s="185"/>
-      <c r="F49" s="185"/>
+      <c r="D49" s="176"/>
+      <c r="E49" s="176"/>
+      <c r="F49" s="176"/>
       <c r="H49" s="69" t="s">
         <v>124</v>
       </c>
@@ -6669,16 +6634,16 @@
         <v>125</v>
       </c>
     </row>
-    <row r="50" spans="2:9" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:9" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B50" s="71" t="s">
         <v>1</v>
       </c>
-      <c r="C50" s="186" t="s">
+      <c r="C50" s="177" t="s">
         <v>126</v>
       </c>
-      <c r="D50" s="186"/>
-      <c r="E50" s="186"/>
-      <c r="F50" s="186"/>
+      <c r="D50" s="177"/>
+      <c r="E50" s="177"/>
+      <c r="F50" s="177"/>
       <c r="H50" s="72" t="s">
         <v>48</v>
       </c>
@@ -6686,16 +6651,16 @@
         <v>127</v>
       </c>
     </row>
-    <row r="51" spans="2:9" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:9" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B51" s="74" t="s">
         <v>2</v>
       </c>
-      <c r="C51" s="187" t="s">
+      <c r="C51" s="171" t="s">
         <v>128</v>
       </c>
-      <c r="D51" s="187"/>
-      <c r="E51" s="187"/>
-      <c r="F51" s="187"/>
+      <c r="D51" s="171"/>
+      <c r="E51" s="171"/>
+      <c r="F51" s="171"/>
       <c r="H51" s="75" t="s">
         <v>70</v>
       </c>
@@ -6703,16 +6668,16 @@
         <v>129</v>
       </c>
     </row>
-    <row r="52" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B52" s="74" t="s">
         <v>3</v>
       </c>
-      <c r="C52" s="187" t="s">
+      <c r="C52" s="171" t="s">
         <v>130</v>
       </c>
-      <c r="D52" s="187"/>
-      <c r="E52" s="187"/>
-      <c r="F52" s="187"/>
+      <c r="D52" s="171"/>
+      <c r="E52" s="171"/>
+      <c r="F52" s="171"/>
       <c r="H52" s="77" t="s">
         <v>131</v>
       </c>
@@ -6720,16 +6685,16 @@
         <v>132</v>
       </c>
     </row>
-    <row r="53" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="53" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B53" s="74" t="s">
         <v>4</v>
       </c>
-      <c r="C53" s="188" t="s">
+      <c r="C53" s="173" t="s">
         <v>133</v>
       </c>
-      <c r="D53" s="188"/>
-      <c r="E53" s="188"/>
-      <c r="F53" s="188"/>
+      <c r="D53" s="173"/>
+      <c r="E53" s="173"/>
+      <c r="F53" s="173"/>
       <c r="H53" s="77" t="s">
         <v>81</v>
       </c>
@@ -6737,16 +6702,16 @@
         <v>134</v>
       </c>
     </row>
-    <row r="54" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B54" s="74" t="s">
         <v>5</v>
       </c>
-      <c r="C54" s="187" t="s">
+      <c r="C54" s="171" t="s">
         <v>135</v>
       </c>
-      <c r="D54" s="187"/>
-      <c r="E54" s="187"/>
-      <c r="F54" s="187"/>
+      <c r="D54" s="171"/>
+      <c r="E54" s="171"/>
+      <c r="F54" s="171"/>
       <c r="H54" s="77" t="s">
         <v>55</v>
       </c>
@@ -6754,16 +6719,16 @@
         <v>136</v>
       </c>
     </row>
-    <row r="55" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="55" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B55" s="74" t="s">
         <v>6</v>
       </c>
-      <c r="C55" s="188" t="s">
+      <c r="C55" s="173" t="s">
         <v>137</v>
       </c>
-      <c r="D55" s="188"/>
-      <c r="E55" s="188"/>
-      <c r="F55" s="188"/>
+      <c r="D55" s="173"/>
+      <c r="E55" s="173"/>
+      <c r="F55" s="173"/>
       <c r="H55" s="79" t="s">
         <v>114</v>
       </c>
@@ -6771,90 +6736,90 @@
         <v>138</v>
       </c>
     </row>
-    <row r="56" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B56" s="74" t="s">
         <v>7</v>
       </c>
-      <c r="C56" s="187" t="s">
+      <c r="C56" s="171" t="s">
         <v>139</v>
       </c>
-      <c r="D56" s="187"/>
-      <c r="E56" s="187"/>
-      <c r="F56" s="187"/>
-    </row>
-    <row r="57" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D56" s="171"/>
+      <c r="E56" s="171"/>
+      <c r="F56" s="171"/>
+    </row>
+    <row r="57" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B57" s="74" t="s">
         <v>8</v>
       </c>
-      <c r="C57" s="187" t="s">
+      <c r="C57" s="171" t="s">
         <v>140</v>
       </c>
-      <c r="D57" s="187"/>
-      <c r="E57" s="187"/>
-      <c r="F57" s="187"/>
-    </row>
-    <row r="58" spans="2:9" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D57" s="171"/>
+      <c r="E57" s="171"/>
+      <c r="F57" s="171"/>
+    </row>
+    <row r="58" spans="2:9" ht="45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B58" s="74" t="s">
         <v>9</v>
       </c>
-      <c r="C58" s="187" t="s">
+      <c r="C58" s="171" t="s">
         <v>141</v>
       </c>
-      <c r="D58" s="187"/>
-      <c r="E58" s="187"/>
-      <c r="F58" s="187"/>
-    </row>
-    <row r="59" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D58" s="171"/>
+      <c r="E58" s="171"/>
+      <c r="F58" s="171"/>
+    </row>
+    <row r="59" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B59" s="74" t="s">
         <v>10</v>
       </c>
-      <c r="C59" s="187" t="s">
+      <c r="C59" s="171" t="s">
         <v>142</v>
       </c>
-      <c r="D59" s="187"/>
-      <c r="E59" s="187"/>
-      <c r="F59" s="187"/>
-    </row>
-    <row r="60" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D59" s="171"/>
+      <c r="E59" s="171"/>
+      <c r="F59" s="171"/>
+    </row>
+    <row r="60" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B60" s="74" t="s">
         <v>11</v>
       </c>
-      <c r="C60" s="187" t="s">
+      <c r="C60" s="171" t="s">
         <v>143</v>
       </c>
-      <c r="D60" s="187"/>
-      <c r="E60" s="187"/>
-      <c r="F60" s="187"/>
-    </row>
-    <row r="61" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="D60" s="171"/>
+      <c r="E60" s="171"/>
+      <c r="F60" s="171"/>
+    </row>
+    <row r="61" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B61" s="81" t="s">
         <v>12</v>
       </c>
-      <c r="C61" s="189" t="s">
+      <c r="C61" s="172" t="s">
         <v>144</v>
       </c>
-      <c r="D61" s="189"/>
-      <c r="E61" s="189"/>
-      <c r="F61" s="189"/>
+      <c r="D61" s="172"/>
+      <c r="E61" s="172"/>
+      <c r="F61" s="172"/>
     </row>
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="EAttMbwrYpwG6akiV7biz2nw7wlXtTooCxJogsSt7negKq0wKQ9sygPbVeHZ99cgmdNfAtLu9NnPC64y/Uaw7A==" saltValue="FJhchlgDftI44klS+XpFDg==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="15">
+    <mergeCell ref="B47:F48"/>
+    <mergeCell ref="H47:I48"/>
+    <mergeCell ref="C49:F49"/>
+    <mergeCell ref="C50:F50"/>
+    <mergeCell ref="C51:F51"/>
+    <mergeCell ref="C52:F52"/>
+    <mergeCell ref="C53:F53"/>
+    <mergeCell ref="C54:F54"/>
+    <mergeCell ref="C55:F55"/>
+    <mergeCell ref="C56:F56"/>
     <mergeCell ref="C57:F57"/>
     <mergeCell ref="C58:F58"/>
     <mergeCell ref="C59:F59"/>
     <mergeCell ref="C60:F60"/>
     <mergeCell ref="C61:F61"/>
-    <mergeCell ref="C52:F52"/>
-    <mergeCell ref="C53:F53"/>
-    <mergeCell ref="C54:F54"/>
-    <mergeCell ref="C55:F55"/>
-    <mergeCell ref="C56:F56"/>
-    <mergeCell ref="B47:F48"/>
-    <mergeCell ref="H47:I48"/>
-    <mergeCell ref="C49:F49"/>
-    <mergeCell ref="C50:F50"/>
-    <mergeCell ref="C51:F51"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -6898,14 +6863,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="C4:F17"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="13.6640625" customWidth="1"/>
-    <col min="4" max="4" width="16.88671875" customWidth="1"/>
-    <col min="5" max="5" width="22.88671875" customWidth="1"/>
+    <col min="4" max="4" width="16.83203125" customWidth="1"/>
+    <col min="5" max="5" width="22.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="3:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="3:6" x14ac:dyDescent="0.2">
       <c r="C4" s="82" t="s">
         <v>145</v>
       </c>
@@ -6919,7 +6884,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="5" spans="3:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="3:6" x14ac:dyDescent="0.2">
       <c r="C5" s="84" t="s">
         <v>26</v>
       </c>
@@ -6933,7 +6898,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="6" spans="3:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="3:6" x14ac:dyDescent="0.2">
       <c r="C6" s="88" t="s">
         <v>19</v>
       </c>
@@ -6947,7 +6912,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="7" spans="3:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="3:6" x14ac:dyDescent="0.2">
       <c r="C7" s="88" t="s">
         <v>25</v>
       </c>
@@ -6955,7 +6920,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="8" spans="3:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="3:6" x14ac:dyDescent="0.2">
       <c r="C8" s="88" t="s">
         <v>154</v>
       </c>
@@ -6963,7 +6928,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="9" spans="3:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="3:6" x14ac:dyDescent="0.2">
       <c r="C9" s="88" t="s">
         <v>58</v>
       </c>
@@ -6971,7 +6936,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="10" spans="3:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="3:6" x14ac:dyDescent="0.2">
       <c r="C10" s="88" t="s">
         <v>49</v>
       </c>
@@ -6979,7 +6944,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="11" spans="3:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="3:6" x14ac:dyDescent="0.2">
       <c r="C11" s="88" t="s">
         <v>22</v>
       </c>
@@ -6987,7 +6952,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="12" spans="3:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="3:6" x14ac:dyDescent="0.2">
       <c r="C12" s="88" t="s">
         <v>158</v>
       </c>
@@ -6995,7 +6960,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="13" spans="3:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="3:6" x14ac:dyDescent="0.2">
       <c r="C13" s="88" t="s">
         <v>23</v>
       </c>
@@ -7003,22 +6968,22 @@
         <v>21</v>
       </c>
     </row>
-    <row r="14" spans="3:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="3:6" x14ac:dyDescent="0.2">
       <c r="C14" s="88" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="15" spans="3:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="3:6" x14ac:dyDescent="0.2">
       <c r="C15" s="88" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="16" spans="3:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="3:6" x14ac:dyDescent="0.2">
       <c r="C16" s="88" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="17" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="3:3" x14ac:dyDescent="0.2">
       <c r="C17" s="92" t="s">
         <v>161</v>
       </c>

</xml_diff>

<commit_message>
DBschema: More options for base MLIPs
</commit_message>
<xml_diff>
--- a/Schema/DB_scheme.xlsx
+++ b/Schema/DB_scheme.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aksam432/Documents/GitHub/WP3/Schema/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27C364D0-E05D-2142-93F1-F6DA897FDE11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4666AC5F-0E88-404D-BAF9-C88D9B8D12B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="23260" windowHeight="12460" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -580,9 +580,6 @@
     <t>MLIP is trained from scratch or is it a fine tuned model</t>
   </si>
   <si>
-    <t>['n2p2','MACE','Custom']</t>
-  </si>
-  <si>
     <t>prediction</t>
   </si>
   <si>
@@ -1013,6 +1010,9 @@
   </si>
   <si>
     <t>eV/A</t>
+  </si>
+  <si>
+    <t>['n2p2','ANI','GAP','SOAP','MTP','ACE','NequIP','Allegro','DeepMD','M3GNet','CHGNet','SevenNet','OrbNet',MACE','Custom']</t>
   </si>
 </sst>
 </file>
@@ -2220,26 +2220,26 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="31" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="31" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2702,7 +2702,7 @@
       </c>
       <c r="C2" s="169"/>
       <c r="D2" s="170" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="E2" s="170"/>
       <c r="F2" s="170"/>
@@ -2783,7 +2783,7 @@
         <v>55</v>
       </c>
       <c r="C7" s="129" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="D7" s="130">
         <v>1</v>
@@ -2801,7 +2801,7 @@
       <c r="K7" s="131"/>
       <c r="L7" s="131"/>
       <c r="M7" s="132" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="8" spans="2:14" x14ac:dyDescent="0.2">
@@ -2809,7 +2809,7 @@
         <v>55</v>
       </c>
       <c r="C8" s="129" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="D8" s="130">
         <v>1</v>
@@ -2827,7 +2827,7 @@
       <c r="K8" s="131"/>
       <c r="L8" s="131"/>
       <c r="M8" s="132" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="9" spans="2:14" x14ac:dyDescent="0.2">
@@ -2850,7 +2850,7 @@
       <c r="H9" s="14"/>
       <c r="I9" s="14"/>
       <c r="J9" s="14" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="K9" s="14"/>
       <c r="L9" s="14"/>
@@ -2878,7 +2878,7 @@
       <c r="H10" s="14"/>
       <c r="I10" s="14"/>
       <c r="J10" s="14" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="K10" s="14"/>
       <c r="L10" s="14"/>
@@ -2906,13 +2906,13 @@
       <c r="H11" s="14"/>
       <c r="I11" s="14"/>
       <c r="J11" s="14" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="K11" s="14" t="s">
         <v>21</v>
       </c>
       <c r="L11" s="14" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="M11" s="112" t="s">
         <v>165</v>
@@ -2924,7 +2924,7 @@
         <v>55</v>
       </c>
       <c r="C12" s="93" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="D12" s="94">
         <v>1</v>
@@ -2939,7 +2939,7 @@
       <c r="H12" s="95"/>
       <c r="I12" s="95"/>
       <c r="J12" s="14" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="K12" s="95"/>
       <c r="L12" s="95"/>
@@ -2952,7 +2952,7 @@
         <v>55</v>
       </c>
       <c r="C13" s="93" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="D13" s="94">
         <v>1</v>
@@ -2967,16 +2967,16 @@
       <c r="H13" s="95"/>
       <c r="I13" s="95"/>
       <c r="J13" s="14" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="K13" s="95" t="s">
         <v>21</v>
       </c>
       <c r="L13" s="95" t="s">
-        <v>180</v>
+        <v>324</v>
       </c>
       <c r="M13" s="113" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="N13" s="167"/>
     </row>
@@ -2985,7 +2985,7 @@
         <v>55</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="D14" s="13">
         <v>1</v>
@@ -3000,12 +3000,12 @@
       <c r="H14" s="14"/>
       <c r="I14" s="12"/>
       <c r="J14" s="14" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="K14" s="14"/>
       <c r="L14" s="14"/>
       <c r="M14" s="111" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="N14" s="167"/>
     </row>
@@ -3014,7 +3014,7 @@
         <v>55</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="D15" s="13">
         <v>1</v>
@@ -3029,12 +3029,12 @@
       <c r="H15" s="14"/>
       <c r="I15" s="12"/>
       <c r="J15" s="14" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="K15" s="14"/>
       <c r="L15" s="14"/>
       <c r="M15" s="111" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="N15" s="168"/>
     </row>
@@ -3043,7 +3043,7 @@
         <v>55</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="D16" s="13">
         <v>1</v>
@@ -3058,7 +3058,7 @@
       <c r="H16" s="14"/>
       <c r="I16" s="12"/>
       <c r="J16" s="14" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="K16" s="14" t="s">
         <v>21</v>
@@ -3075,7 +3075,7 @@
         <v>55</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="D17" s="13">
         <v>1</v>
@@ -3090,7 +3090,7 @@
       <c r="H17" s="14"/>
       <c r="I17" s="14"/>
       <c r="J17" s="14" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="K17" s="14"/>
       <c r="L17" s="14"/>
@@ -3103,7 +3103,7 @@
         <v>55</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="D18" s="13">
         <v>1</v>
@@ -3118,7 +3118,7 @@
       <c r="H18" s="14"/>
       <c r="I18" s="12"/>
       <c r="J18" s="14" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="K18" s="14"/>
       <c r="L18" s="14"/>
@@ -3131,7 +3131,7 @@
         <v>55</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="D19" s="13">
         <v>1</v>
@@ -3146,12 +3146,12 @@
       <c r="H19" s="14"/>
       <c r="I19" s="14"/>
       <c r="J19" s="14" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="K19" s="14"/>
       <c r="L19" s="14"/>
       <c r="M19" s="114" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="20" spans="1:14" ht="17" x14ac:dyDescent="0.2">
@@ -3159,7 +3159,7 @@
         <v>55</v>
       </c>
       <c r="C20" s="163" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D20" s="164">
         <v>1</v>
@@ -3177,7 +3177,7 @@
       <c r="K20" s="165"/>
       <c r="L20" s="165"/>
       <c r="M20" s="166" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.2">
@@ -3185,7 +3185,7 @@
         <v>55</v>
       </c>
       <c r="C21" s="12" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="D21" s="13">
         <v>1</v>
@@ -3205,7 +3205,7 @@
       <c r="K21" s="14"/>
       <c r="L21" s="14"/>
       <c r="M21" s="111" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="N21" s="167"/>
     </row>
@@ -3214,7 +3214,7 @@
         <v>55</v>
       </c>
       <c r="C22" s="98" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="D22" s="99">
         <v>1</v>
@@ -3229,16 +3229,16 @@
       <c r="H22" s="100"/>
       <c r="I22" s="100"/>
       <c r="J22" s="14" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="K22" s="100" t="s">
         <v>21</v>
       </c>
       <c r="L22" s="105" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="M22" s="115" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="N22"/>
     </row>
@@ -3247,7 +3247,7 @@
         <v>55</v>
       </c>
       <c r="C23" s="12" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D23" s="13">
         <v>1</v>
@@ -3262,16 +3262,16 @@
       <c r="H23" s="14"/>
       <c r="I23" s="14"/>
       <c r="J23" s="14" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="K23" s="14" t="s">
         <v>21</v>
       </c>
       <c r="L23" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="M23" s="112" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="24" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -3279,7 +3279,7 @@
         <v>55</v>
       </c>
       <c r="C24" s="12" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="D24" s="13">
         <v>1</v>
@@ -3293,13 +3293,13 @@
       <c r="G24" s="14"/>
       <c r="H24" s="14"/>
       <c r="I24" s="14" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="J24" s="14"/>
       <c r="K24" s="14"/>
       <c r="L24" s="14"/>
       <c r="M24" s="114" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="25" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -3307,7 +3307,7 @@
         <v>55</v>
       </c>
       <c r="C25" s="12" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D25" s="13">
         <v>1</v>
@@ -3321,13 +3321,13 @@
       <c r="G25" s="14"/>
       <c r="H25" s="14"/>
       <c r="I25" s="14" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="J25" s="14"/>
       <c r="K25" s="14"/>
       <c r="L25" s="14"/>
       <c r="M25" s="114" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="26" spans="1:14" ht="17" x14ac:dyDescent="0.2">
@@ -3335,7 +3335,7 @@
         <v>55</v>
       </c>
       <c r="C26" s="12" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="D26" s="13">
         <v>1</v>
@@ -3349,13 +3349,13 @@
       <c r="G26" s="14"/>
       <c r="H26" s="14"/>
       <c r="I26" s="14" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="J26" s="14"/>
       <c r="K26" s="14"/>
       <c r="L26" s="14"/>
       <c r="M26" s="114" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="27" spans="1:14" ht="17" x14ac:dyDescent="0.2">
@@ -3363,7 +3363,7 @@
         <v>55</v>
       </c>
       <c r="C27" s="12" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="D27" s="13">
         <v>1</v>
@@ -3378,16 +3378,16 @@
       <c r="H27" s="14"/>
       <c r="I27" s="14"/>
       <c r="J27" s="14" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="K27" s="14" t="s">
         <v>21</v>
       </c>
       <c r="L27" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="M27" s="112" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="28" spans="1:14" ht="17" x14ac:dyDescent="0.2">
@@ -3395,7 +3395,7 @@
         <v>55</v>
       </c>
       <c r="C28" s="12" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="D28" s="13">
         <v>10</v>
@@ -3410,12 +3410,12 @@
       <c r="H28" s="14"/>
       <c r="I28" s="14"/>
       <c r="J28" s="14" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="K28" s="14"/>
       <c r="L28" s="14"/>
       <c r="M28" s="112" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="29" spans="1:14" ht="17" x14ac:dyDescent="0.2">
@@ -3423,7 +3423,7 @@
         <v>55</v>
       </c>
       <c r="C29" s="134" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="D29" s="135">
         <v>1</v>
@@ -3436,14 +3436,14 @@
       </c>
       <c r="G29" s="136"/>
       <c r="H29" s="136" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="I29" s="136"/>
       <c r="J29" s="136"/>
       <c r="K29" s="136"/>
       <c r="L29" s="136"/>
       <c r="M29" s="137" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="30" spans="1:14" ht="18" thickBot="1" x14ac:dyDescent="0.25">
@@ -3451,7 +3451,7 @@
         <v>55</v>
       </c>
       <c r="C30" s="140" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="D30" s="141">
         <v>10</v>
@@ -3465,13 +3465,13 @@
       <c r="G30" s="142"/>
       <c r="H30" s="142"/>
       <c r="I30" s="142" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="J30" s="142"/>
       <c r="K30" s="142"/>
       <c r="L30" s="142"/>
       <c r="M30" s="143" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="31" spans="1:14" ht="18" thickTop="1" x14ac:dyDescent="0.2">
@@ -3507,7 +3507,7 @@
         <v>170</v>
       </c>
       <c r="C32" s="129" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="D32" s="130">
         <v>1</v>
@@ -3525,7 +3525,7 @@
       <c r="K32" s="131"/>
       <c r="L32" s="131"/>
       <c r="M32" s="138" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="33" spans="1:14" ht="17" x14ac:dyDescent="0.2">
@@ -3534,7 +3534,7 @@
         <v>170</v>
       </c>
       <c r="C33" s="129" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="D33" s="130">
         <v>1</v>
@@ -3552,7 +3552,7 @@
       <c r="K33" s="131"/>
       <c r="L33" s="131"/>
       <c r="M33" s="138" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="34" spans="1:14" ht="17" x14ac:dyDescent="0.2">
@@ -3576,12 +3576,12 @@
       <c r="H34" s="14"/>
       <c r="I34" s="16"/>
       <c r="J34" s="14" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="K34" s="14"/>
       <c r="L34" s="14"/>
       <c r="M34" s="112" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="35" spans="1:14" ht="17" x14ac:dyDescent="0.2">
@@ -3590,7 +3590,7 @@
         <v>170</v>
       </c>
       <c r="C35" s="12" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="D35" s="13">
         <v>1</v>
@@ -3608,7 +3608,7 @@
       <c r="K35" s="14"/>
       <c r="L35" s="14"/>
       <c r="M35" s="112" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="36" spans="1:14" ht="17" x14ac:dyDescent="0.2">
@@ -3617,7 +3617,7 @@
         <v>170</v>
       </c>
       <c r="C36" s="12" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="D36" s="13">
         <v>1</v>
@@ -3635,7 +3635,7 @@
       <c r="K36" s="14"/>
       <c r="L36" s="14"/>
       <c r="M36" s="112" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="37" spans="1:14" ht="17" x14ac:dyDescent="0.2">
@@ -3644,7 +3644,7 @@
         <v>170</v>
       </c>
       <c r="C37" s="12" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="D37" s="13">
         <v>1</v>
@@ -3656,17 +3656,17 @@
         <v>18</v>
       </c>
       <c r="G37" s="14" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="H37" s="14"/>
       <c r="I37" s="16"/>
       <c r="J37" s="14" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="K37" s="14"/>
       <c r="L37" s="14"/>
       <c r="M37" s="112" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="38" spans="1:14" ht="17" x14ac:dyDescent="0.2">
@@ -3675,7 +3675,7 @@
         <v>170</v>
       </c>
       <c r="C38" s="116" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="D38" s="13">
         <v>1</v>
@@ -3687,17 +3687,17 @@
         <v>18</v>
       </c>
       <c r="G38" s="14" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="H38" s="14"/>
       <c r="I38" s="16"/>
       <c r="J38" s="14" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="K38" s="14"/>
       <c r="L38" s="14"/>
       <c r="M38" s="112" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="39" spans="1:14" ht="17" x14ac:dyDescent="0.2">
@@ -3706,7 +3706,7 @@
         <v>170</v>
       </c>
       <c r="C39" s="144" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="D39" s="13">
         <v>1</v>
@@ -3718,17 +3718,17 @@
         <v>18</v>
       </c>
       <c r="G39" s="14" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="H39" s="14"/>
       <c r="I39" s="14"/>
       <c r="J39" s="14" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="K39" s="14"/>
       <c r="L39" s="14"/>
       <c r="M39" s="114" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="40" spans="1:14" ht="17" x14ac:dyDescent="0.2">
@@ -3737,7 +3737,7 @@
         <v>170</v>
       </c>
       <c r="C40" s="12" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="D40" s="13">
         <v>1</v>
@@ -3749,17 +3749,17 @@
         <v>15</v>
       </c>
       <c r="G40" s="14" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H40" s="14"/>
       <c r="I40" s="14"/>
       <c r="J40" s="14" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="K40" s="14"/>
       <c r="L40" s="14"/>
       <c r="M40" s="114" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="41" spans="1:14" s="96" customFormat="1" ht="18" thickBot="1" x14ac:dyDescent="0.25">
@@ -3768,7 +3768,7 @@
         <v>170</v>
       </c>
       <c r="C41" s="149" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D41" s="150">
         <v>1</v>
@@ -3780,24 +3780,24 @@
         <v>15</v>
       </c>
       <c r="G41" s="142" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H41" s="153"/>
       <c r="I41" s="153"/>
       <c r="J41" s="142" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="K41" s="153"/>
       <c r="L41" s="153"/>
       <c r="M41" s="154" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="N41"/>
     </row>
     <row r="42" spans="1:14" s="96" customFormat="1" ht="18" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A42" s="101"/>
       <c r="B42" s="128" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C42" s="145" t="s">
         <v>13</v>
@@ -3825,10 +3825,10 @@
     <row r="43" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A43" s="15"/>
       <c r="B43" s="128" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C43" s="129" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="D43" s="130">
         <v>1</v>
@@ -3846,16 +3846,16 @@
       <c r="K43" s="131"/>
       <c r="L43" s="131"/>
       <c r="M43" s="138" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="44" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A44" s="15"/>
       <c r="B44" s="128" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C44" s="129" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="D44" s="130">
         <v>1</v>
@@ -3873,16 +3873,16 @@
       <c r="K44" s="131"/>
       <c r="L44" s="131"/>
       <c r="M44" s="138" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="45" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A45" s="15"/>
       <c r="B45" s="11" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C45" s="12" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="D45" s="13">
         <v>1</v>
@@ -3897,18 +3897,18 @@
       <c r="H45" s="14"/>
       <c r="I45" s="14"/>
       <c r="J45" s="14" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="K45" s="14"/>
       <c r="L45" s="14"/>
       <c r="M45" s="117" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="46" spans="1:14" s="96" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A46" s="101"/>
       <c r="B46" s="97" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C46" s="102" t="s">
         <v>163</v>
@@ -3926,22 +3926,22 @@
       <c r="H46" s="103"/>
       <c r="I46" s="103"/>
       <c r="J46" s="103" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="K46" s="103"/>
       <c r="L46" s="103"/>
       <c r="M46" s="158" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="N46"/>
     </row>
     <row r="47" spans="1:14" s="96" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A47" s="101"/>
       <c r="B47" s="97" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C47" s="102" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D47" s="157">
         <v>1</v>
@@ -3956,26 +3956,26 @@
       <c r="H47" s="103"/>
       <c r="I47" s="103"/>
       <c r="J47" s="103" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="K47" s="103" t="s">
         <v>21</v>
       </c>
       <c r="L47" s="103" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="M47" s="158" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="N47"/>
     </row>
     <row r="48" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A48" s="15"/>
       <c r="B48" s="11" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C48" s="12" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="D48" s="13">
         <v>1</v>
@@ -3993,16 +3993,16 @@
       <c r="K48" s="14"/>
       <c r="L48" s="14"/>
       <c r="M48" s="112" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="49" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A49" s="15"/>
       <c r="B49" s="11" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C49" s="12" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="D49" s="13">
         <v>1</v>
@@ -4017,21 +4017,21 @@
       <c r="H49" s="14"/>
       <c r="I49" s="14"/>
       <c r="J49" s="14" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="K49" s="14"/>
       <c r="L49" s="14"/>
       <c r="M49" s="112" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="50" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A50" s="15"/>
       <c r="B50" s="11" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C50" s="12" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="D50" s="13">
         <v>5</v>
@@ -4046,21 +4046,21 @@
       <c r="H50" s="14"/>
       <c r="I50" s="14"/>
       <c r="J50" s="14" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="K50" s="14"/>
       <c r="L50" s="14"/>
       <c r="M50" s="112" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
     <row r="51" spans="1:14" s="96" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A51" s="15"/>
       <c r="B51" s="11" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C51" s="12" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D51" s="13">
         <v>1</v>
@@ -4075,25 +4075,25 @@
       <c r="H51" s="14"/>
       <c r="I51" s="14"/>
       <c r="J51" s="14" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="K51" s="14"/>
       <c r="L51" s="14"/>
       <c r="M51" s="118" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="N51"/>
     </row>
     <row r="52" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A52" s="15"/>
       <c r="B52" s="11" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C52" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D52" s="13" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="E52" s="12" t="s">
         <v>14</v>
@@ -4105,21 +4105,21 @@
       <c r="H52" s="14"/>
       <c r="I52" s="14"/>
       <c r="J52" s="14" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="K52" s="14"/>
       <c r="L52" s="14"/>
       <c r="M52" s="118" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="53" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A53" s="96"/>
       <c r="B53" s="11" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C53" s="98" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D53" s="99">
         <v>1</v>
@@ -4131,25 +4131,25 @@
         <v>18</v>
       </c>
       <c r="G53" s="100" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="H53" s="100"/>
       <c r="I53" s="100"/>
       <c r="J53" s="14" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="K53" s="100"/>
       <c r="L53" s="100"/>
       <c r="M53" s="119" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="54" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B54" s="11" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C54" s="12" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D54" s="13">
         <v>1</v>
@@ -4161,25 +4161,25 @@
         <v>18</v>
       </c>
       <c r="G54" s="14" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="H54" s="14"/>
       <c r="I54" s="14"/>
       <c r="J54" s="14" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="K54" s="14"/>
       <c r="L54" s="14"/>
       <c r="M54" s="120" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="55" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B55" s="11" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C55" s="12" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D55" s="13">
         <v>1</v>
@@ -4191,25 +4191,25 @@
         <v>18</v>
       </c>
       <c r="G55" s="14" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="H55" s="14"/>
       <c r="I55" s="14"/>
       <c r="J55" s="14" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="K55" s="14"/>
       <c r="L55" s="14"/>
       <c r="M55" s="111" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="56" spans="1:14" s="96" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B56" s="97" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C56" s="102" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="D56" s="157">
         <v>1</v>
@@ -4221,26 +4221,26 @@
         <v>18</v>
       </c>
       <c r="G56" s="103" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="H56" s="103"/>
       <c r="I56" s="103"/>
       <c r="J56" s="103" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="K56" s="103"/>
       <c r="L56" s="103"/>
       <c r="M56" s="159" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="N56"/>
     </row>
     <row r="57" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B57" s="11" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C57" s="12" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="D57" s="13">
         <v>1</v>
@@ -4260,16 +4260,16 @@
       <c r="K57" s="14"/>
       <c r="L57" s="14"/>
       <c r="M57" s="121" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="58" spans="1:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A58" s="96"/>
       <c r="B58" s="139" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C58" s="140" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="D58" s="141">
         <v>1</v>
@@ -4287,7 +4287,7 @@
       <c r="K58" s="142"/>
       <c r="L58" s="142"/>
       <c r="M58" s="155" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="59" spans="1:14" ht="18" thickTop="1" x14ac:dyDescent="0.2">
@@ -4323,7 +4323,7 @@
         <v>171</v>
       </c>
       <c r="C60" s="129" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="D60" s="130">
         <v>1</v>
@@ -4341,7 +4341,7 @@
       <c r="K60" s="131"/>
       <c r="L60" s="131"/>
       <c r="M60" s="138" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="61" spans="1:14" ht="17" x14ac:dyDescent="0.2">
@@ -4350,7 +4350,7 @@
         <v>171</v>
       </c>
       <c r="C61" s="129" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="D61" s="130">
         <v>1</v>
@@ -4368,7 +4368,7 @@
       <c r="K61" s="131"/>
       <c r="L61" s="131"/>
       <c r="M61" s="138" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="62" spans="1:14" x14ac:dyDescent="0.2">
@@ -4376,7 +4376,7 @@
         <v>171</v>
       </c>
       <c r="C62" s="12" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="D62" s="13">
         <v>1</v>
@@ -4391,12 +4391,12 @@
       <c r="H62" s="14"/>
       <c r="I62" s="14"/>
       <c r="J62" s="14" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="K62" s="14"/>
       <c r="L62" s="14"/>
       <c r="M62" s="111" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="63" spans="1:14" x14ac:dyDescent="0.2">
@@ -4404,7 +4404,7 @@
         <v>171</v>
       </c>
       <c r="C63" s="12" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="D63" s="13">
         <v>1</v>
@@ -4419,12 +4419,12 @@
       <c r="H63" s="14"/>
       <c r="I63" s="14"/>
       <c r="J63" s="14" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="K63" s="14"/>
       <c r="L63" s="14"/>
       <c r="M63" s="121" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="64" spans="1:14" x14ac:dyDescent="0.2">
@@ -4432,7 +4432,7 @@
         <v>171</v>
       </c>
       <c r="C64" s="12" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="D64" s="13">
         <v>1</v>
@@ -4450,7 +4450,7 @@
       <c r="K64" s="14"/>
       <c r="L64" s="14"/>
       <c r="M64" s="159" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="65" spans="1:14" x14ac:dyDescent="0.2">
@@ -4458,7 +4458,7 @@
         <v>171</v>
       </c>
       <c r="C65" s="12" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="D65" s="13">
         <v>1</v>
@@ -4473,16 +4473,16 @@
       <c r="H65" s="14"/>
       <c r="I65" s="14"/>
       <c r="J65" s="14" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="K65" s="14" t="s">
         <v>21</v>
       </c>
       <c r="L65" s="14" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="M65" s="111" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="66" spans="1:14" x14ac:dyDescent="0.2">
@@ -4505,12 +4505,12 @@
       <c r="H66" s="14"/>
       <c r="I66" s="14"/>
       <c r="J66" s="14" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="K66" s="14"/>
       <c r="L66" s="14"/>
       <c r="M66" s="122" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="67" spans="1:14" x14ac:dyDescent="0.2">
@@ -4518,7 +4518,7 @@
         <v>171</v>
       </c>
       <c r="C67" s="12" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="D67" s="13">
         <v>1</v>
@@ -4530,17 +4530,17 @@
         <v>15</v>
       </c>
       <c r="G67" s="14" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="H67" s="14"/>
       <c r="I67" s="14"/>
       <c r="J67" s="14" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="K67" s="14"/>
       <c r="L67" s="14"/>
       <c r="M67" s="111" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="68" spans="1:14" x14ac:dyDescent="0.2">
@@ -4548,7 +4548,7 @@
         <v>171</v>
       </c>
       <c r="C68" s="12" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="D68" s="13">
         <v>1</v>
@@ -4560,17 +4560,17 @@
         <v>15</v>
       </c>
       <c r="G68" s="14" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="H68" s="14"/>
       <c r="I68" s="14"/>
       <c r="J68" s="14" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="K68" s="14"/>
       <c r="L68" s="14"/>
       <c r="M68" s="121" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="69" spans="1:14" s="96" customFormat="1" x14ac:dyDescent="0.2">
@@ -4593,12 +4593,12 @@
       <c r="H69" s="103"/>
       <c r="I69" s="103"/>
       <c r="J69" s="103" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="K69" s="103"/>
       <c r="L69" s="103"/>
       <c r="M69" s="161" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="N69"/>
     </row>
@@ -4622,12 +4622,12 @@
       <c r="H70" s="14"/>
       <c r="I70" s="14"/>
       <c r="J70" s="14" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="K70" s="14"/>
       <c r="L70" s="14"/>
       <c r="M70" s="121" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="71" spans="1:14" x14ac:dyDescent="0.2">
@@ -4650,12 +4650,12 @@
       <c r="H71" s="14"/>
       <c r="I71" s="14"/>
       <c r="J71" s="14" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="K71" s="14"/>
       <c r="L71" s="14"/>
       <c r="M71" s="111" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="72" spans="1:14" x14ac:dyDescent="0.2">
@@ -4663,7 +4663,7 @@
         <v>171</v>
       </c>
       <c r="C72" s="12" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="D72" s="13">
         <v>1</v>
@@ -4675,17 +4675,17 @@
         <v>15</v>
       </c>
       <c r="G72" s="14" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="H72" s="14"/>
       <c r="I72" s="14"/>
       <c r="J72" s="14" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="K72" s="14"/>
       <c r="L72" s="14"/>
       <c r="M72" s="111" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="73" spans="1:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -4693,7 +4693,7 @@
         <v>171</v>
       </c>
       <c r="C73" s="140" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="D73" s="141">
         <v>1</v>
@@ -4705,17 +4705,17 @@
         <v>15</v>
       </c>
       <c r="G73" s="142" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="H73" s="142"/>
       <c r="I73" s="142"/>
       <c r="J73" s="142" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="K73" s="142"/>
       <c r="L73" s="142"/>
       <c r="M73" s="160" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="74" spans="1:14" ht="18" thickTop="1" x14ac:dyDescent="0.2">
@@ -4751,7 +4751,7 @@
         <v>176</v>
       </c>
       <c r="C75" s="129" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="D75" s="130">
         <v>1</v>
@@ -4769,7 +4769,7 @@
       <c r="K75" s="131"/>
       <c r="L75" s="131"/>
       <c r="M75" s="138" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="76" spans="1:14" ht="17" x14ac:dyDescent="0.2">
@@ -4778,7 +4778,7 @@
         <v>176</v>
       </c>
       <c r="C76" s="129" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="D76" s="130">
         <v>1</v>
@@ -4796,7 +4796,7 @@
       <c r="K76" s="131"/>
       <c r="L76" s="131"/>
       <c r="M76" s="138" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="77" spans="1:14" x14ac:dyDescent="0.2">
@@ -4820,12 +4820,12 @@
       <c r="H77" s="14"/>
       <c r="I77" s="14"/>
       <c r="J77" s="14" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="K77" s="14"/>
       <c r="L77" s="14"/>
       <c r="M77" s="121" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="78" spans="1:14" s="96" customFormat="1" x14ac:dyDescent="0.2">
@@ -4848,12 +4848,12 @@
       <c r="H78" s="14"/>
       <c r="I78" s="14"/>
       <c r="J78" s="14" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="K78" s="14"/>
       <c r="L78" s="14"/>
       <c r="M78" s="111" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="N78"/>
     </row>
@@ -4863,7 +4863,7 @@
         <v>176</v>
       </c>
       <c r="C79" s="12" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="D79" s="13">
         <v>1</v>
@@ -4877,13 +4877,13 @@
       <c r="G79" s="14"/>
       <c r="H79" s="14"/>
       <c r="I79" s="14" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="J79" s="14"/>
       <c r="K79" s="14"/>
       <c r="L79" s="14"/>
       <c r="M79" s="111" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="80" spans="1:14" x14ac:dyDescent="0.2">
@@ -4892,7 +4892,7 @@
         <v>176</v>
       </c>
       <c r="C80" s="102" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="D80" s="157">
         <v>1</v>
@@ -4907,16 +4907,16 @@
       <c r="H80" s="103"/>
       <c r="I80" s="103"/>
       <c r="J80" s="103" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="K80" s="103" t="s">
         <v>21</v>
       </c>
       <c r="L80" s="103" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="M80" s="161" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="81" spans="1:14" x14ac:dyDescent="0.2">
@@ -4925,7 +4925,7 @@
         <v>176</v>
       </c>
       <c r="C81" s="12" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="D81" s="13">
         <v>1</v>
@@ -4940,12 +4940,12 @@
       <c r="H81" s="14"/>
       <c r="I81" s="14"/>
       <c r="J81" s="14" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="K81" s="14"/>
       <c r="L81" s="14"/>
       <c r="M81" s="121" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="82" spans="1:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -4954,7 +4954,7 @@
         <v>176</v>
       </c>
       <c r="C82" s="140" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="D82" s="141">
         <v>1</v>
@@ -4967,19 +4967,19 @@
       </c>
       <c r="G82" s="142"/>
       <c r="H82" s="142" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="I82" s="142"/>
       <c r="J82" s="142"/>
       <c r="K82" s="142"/>
       <c r="L82" s="142"/>
       <c r="M82" s="160" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="83" spans="1:14" s="96" customFormat="1" ht="18" thickTop="1" x14ac:dyDescent="0.2">
       <c r="B83" s="128" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C83" s="145" t="s">
         <v>13</v>
@@ -5007,10 +5007,10 @@
     <row r="84" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A84" s="15"/>
       <c r="B84" s="128" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C84" s="129" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="D84" s="130">
         <v>1</v>
@@ -5028,16 +5028,16 @@
       <c r="K84" s="131"/>
       <c r="L84" s="131"/>
       <c r="M84" s="138" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="85" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A85" s="15"/>
       <c r="B85" s="128" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C85" s="129" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="D85" s="130">
         <v>1</v>
@@ -5055,15 +5055,15 @@
       <c r="K85" s="131"/>
       <c r="L85" s="131"/>
       <c r="M85" s="138" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="86" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B86" s="97" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C86" s="12" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="D86" s="13">
         <v>1</v>
@@ -5083,16 +5083,16 @@
       <c r="K86" s="14"/>
       <c r="L86" s="14"/>
       <c r="M86" s="111" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="87" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A87" s="96"/>
       <c r="B87" s="97" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C87" s="102" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="D87" s="157">
         <v>1</v>
@@ -5112,15 +5112,15 @@
       <c r="K87" s="103"/>
       <c r="L87" s="103"/>
       <c r="M87" s="161" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="88" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B88" s="97" t="s">
+        <v>288</v>
+      </c>
+      <c r="C88" s="12" t="s">
         <v>289</v>
-      </c>
-      <c r="C88" s="12" t="s">
-        <v>290</v>
       </c>
       <c r="D88" s="13">
         <v>1</v>
@@ -5135,17 +5135,17 @@
       <c r="H88" s="14"/>
       <c r="I88" s="14"/>
       <c r="J88" s="14" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="K88" s="14"/>
       <c r="L88" s="14"/>
       <c r="M88" s="111" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="89" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B89" s="97" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C89" s="12" t="s">
         <v>178</v>
@@ -5163,20 +5163,20 @@
       <c r="H89" s="14"/>
       <c r="I89" s="14"/>
       <c r="J89" s="14" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="K89" s="14"/>
       <c r="L89" s="14"/>
       <c r="M89" s="121" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="90" spans="1:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B90" s="148" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C90" s="140" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="D90" s="141">
         <v>1</v>
@@ -5189,20 +5189,20 @@
       </c>
       <c r="G90" s="142"/>
       <c r="H90" s="142" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="I90" s="142"/>
       <c r="J90" s="142"/>
       <c r="K90" s="142"/>
       <c r="L90" s="142"/>
       <c r="M90" s="160" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="91" spans="1:14" ht="17" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A91" s="104"/>
       <c r="B91" s="128" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C91" s="145" t="s">
         <v>13</v>
@@ -5229,10 +5229,10 @@
     <row r="92" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A92" s="15"/>
       <c r="B92" s="128" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C92" s="129" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="D92" s="130">
         <v>1</v>
@@ -5250,16 +5250,16 @@
       <c r="K92" s="131"/>
       <c r="L92" s="131"/>
       <c r="M92" s="138" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="93" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A93" s="15"/>
       <c r="B93" s="128" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C93" s="129" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="D93" s="130">
         <v>1</v>
@@ -5277,15 +5277,15 @@
       <c r="K93" s="131"/>
       <c r="L93" s="131"/>
       <c r="M93" s="138" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="94" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B94" s="11" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C94" s="12" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="D94" s="13">
         <v>1</v>
@@ -5300,20 +5300,20 @@
       <c r="H94" s="14"/>
       <c r="I94" s="14"/>
       <c r="J94" s="14" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="K94" s="14"/>
       <c r="L94" s="14"/>
       <c r="M94" s="111" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="95" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B95" s="11" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C95" s="12" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="D95" s="13">
         <v>1</v>
@@ -5328,20 +5328,20 @@
       <c r="H95" s="14"/>
       <c r="I95" s="14"/>
       <c r="J95" s="14" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="K95" s="14"/>
       <c r="L95" s="14"/>
       <c r="M95" s="111" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="96" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B96" s="11" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C96" s="12" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="D96" s="13">
         <v>1</v>
@@ -5356,17 +5356,17 @@
       <c r="H96" s="14"/>
       <c r="I96" s="14"/>
       <c r="J96" s="14" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="K96" s="14"/>
       <c r="L96" s="14"/>
       <c r="M96" s="111" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="97" spans="2:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B97" s="123" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C97" s="124" t="s">
         <v>161</v>
@@ -5384,12 +5384,12 @@
       <c r="H97" s="126"/>
       <c r="I97" s="126"/>
       <c r="J97" s="126" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="K97" s="126"/>
       <c r="L97" s="126"/>
       <c r="M97" s="127" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
   </sheetData>
@@ -6596,37 +6596,37 @@
       </c>
     </row>
     <row r="47" spans="2:13" x14ac:dyDescent="0.2">
-      <c r="B47" s="174" t="s">
+      <c r="B47" s="171" t="s">
         <v>121</v>
       </c>
-      <c r="C47" s="174"/>
-      <c r="D47" s="174"/>
-      <c r="E47" s="174"/>
-      <c r="F47" s="174"/>
-      <c r="H47" s="175" t="s">
+      <c r="C47" s="171"/>
+      <c r="D47" s="171"/>
+      <c r="E47" s="171"/>
+      <c r="F47" s="171"/>
+      <c r="H47" s="172" t="s">
         <v>122</v>
       </c>
-      <c r="I47" s="175"/>
+      <c r="I47" s="172"/>
     </row>
     <row r="48" spans="2:13" x14ac:dyDescent="0.2">
-      <c r="B48" s="174"/>
-      <c r="C48" s="174"/>
-      <c r="D48" s="174"/>
-      <c r="E48" s="174"/>
-      <c r="F48" s="174"/>
-      <c r="H48" s="175"/>
-      <c r="I48" s="175"/>
+      <c r="B48" s="171"/>
+      <c r="C48" s="171"/>
+      <c r="D48" s="171"/>
+      <c r="E48" s="171"/>
+      <c r="F48" s="171"/>
+      <c r="H48" s="172"/>
+      <c r="I48" s="172"/>
     </row>
     <row r="49" spans="2:9" ht="16" x14ac:dyDescent="0.2">
       <c r="B49" s="68" t="s">
         <v>123</v>
       </c>
-      <c r="C49" s="176" t="s">
+      <c r="C49" s="173" t="s">
         <v>12</v>
       </c>
-      <c r="D49" s="176"/>
-      <c r="E49" s="176"/>
-      <c r="F49" s="176"/>
+      <c r="D49" s="173"/>
+      <c r="E49" s="173"/>
+      <c r="F49" s="173"/>
       <c r="H49" s="69" t="s">
         <v>124</v>
       </c>
@@ -6638,12 +6638,12 @@
       <c r="B50" s="71" t="s">
         <v>1</v>
       </c>
-      <c r="C50" s="177" t="s">
+      <c r="C50" s="174" t="s">
         <v>126</v>
       </c>
-      <c r="D50" s="177"/>
-      <c r="E50" s="177"/>
-      <c r="F50" s="177"/>
+      <c r="D50" s="174"/>
+      <c r="E50" s="174"/>
+      <c r="F50" s="174"/>
       <c r="H50" s="72" t="s">
         <v>48</v>
       </c>
@@ -6655,12 +6655,12 @@
       <c r="B51" s="74" t="s">
         <v>2</v>
       </c>
-      <c r="C51" s="171" t="s">
+      <c r="C51" s="175" t="s">
         <v>128</v>
       </c>
-      <c r="D51" s="171"/>
-      <c r="E51" s="171"/>
-      <c r="F51" s="171"/>
+      <c r="D51" s="175"/>
+      <c r="E51" s="175"/>
+      <c r="F51" s="175"/>
       <c r="H51" s="75" t="s">
         <v>70</v>
       </c>
@@ -6672,12 +6672,12 @@
       <c r="B52" s="74" t="s">
         <v>3</v>
       </c>
-      <c r="C52" s="171" t="s">
+      <c r="C52" s="175" t="s">
         <v>130</v>
       </c>
-      <c r="D52" s="171"/>
-      <c r="E52" s="171"/>
-      <c r="F52" s="171"/>
+      <c r="D52" s="175"/>
+      <c r="E52" s="175"/>
+      <c r="F52" s="175"/>
       <c r="H52" s="77" t="s">
         <v>131</v>
       </c>
@@ -6689,12 +6689,12 @@
       <c r="B53" s="74" t="s">
         <v>4</v>
       </c>
-      <c r="C53" s="173" t="s">
+      <c r="C53" s="176" t="s">
         <v>133</v>
       </c>
-      <c r="D53" s="173"/>
-      <c r="E53" s="173"/>
-      <c r="F53" s="173"/>
+      <c r="D53" s="176"/>
+      <c r="E53" s="176"/>
+      <c r="F53" s="176"/>
       <c r="H53" s="77" t="s">
         <v>81</v>
       </c>
@@ -6706,12 +6706,12 @@
       <c r="B54" s="74" t="s">
         <v>5</v>
       </c>
-      <c r="C54" s="171" t="s">
+      <c r="C54" s="175" t="s">
         <v>135</v>
       </c>
-      <c r="D54" s="171"/>
-      <c r="E54" s="171"/>
-      <c r="F54" s="171"/>
+      <c r="D54" s="175"/>
+      <c r="E54" s="175"/>
+      <c r="F54" s="175"/>
       <c r="H54" s="77" t="s">
         <v>55</v>
       </c>
@@ -6723,12 +6723,12 @@
       <c r="B55" s="74" t="s">
         <v>6</v>
       </c>
-      <c r="C55" s="173" t="s">
+      <c r="C55" s="176" t="s">
         <v>137</v>
       </c>
-      <c r="D55" s="173"/>
-      <c r="E55" s="173"/>
-      <c r="F55" s="173"/>
+      <c r="D55" s="176"/>
+      <c r="E55" s="176"/>
+      <c r="F55" s="176"/>
       <c r="H55" s="79" t="s">
         <v>114</v>
       </c>
@@ -6740,86 +6740,86 @@
       <c r="B56" s="74" t="s">
         <v>7</v>
       </c>
-      <c r="C56" s="171" t="s">
+      <c r="C56" s="175" t="s">
         <v>139</v>
       </c>
-      <c r="D56" s="171"/>
-      <c r="E56" s="171"/>
-      <c r="F56" s="171"/>
+      <c r="D56" s="175"/>
+      <c r="E56" s="175"/>
+      <c r="F56" s="175"/>
     </row>
     <row r="57" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B57" s="74" t="s">
         <v>8</v>
       </c>
-      <c r="C57" s="171" t="s">
+      <c r="C57" s="175" t="s">
         <v>140</v>
       </c>
-      <c r="D57" s="171"/>
-      <c r="E57" s="171"/>
-      <c r="F57" s="171"/>
+      <c r="D57" s="175"/>
+      <c r="E57" s="175"/>
+      <c r="F57" s="175"/>
     </row>
     <row r="58" spans="2:9" ht="45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B58" s="74" t="s">
         <v>9</v>
       </c>
-      <c r="C58" s="171" t="s">
+      <c r="C58" s="175" t="s">
         <v>141</v>
       </c>
-      <c r="D58" s="171"/>
-      <c r="E58" s="171"/>
-      <c r="F58" s="171"/>
+      <c r="D58" s="175"/>
+      <c r="E58" s="175"/>
+      <c r="F58" s="175"/>
     </row>
     <row r="59" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B59" s="74" t="s">
         <v>10</v>
       </c>
-      <c r="C59" s="171" t="s">
+      <c r="C59" s="175" t="s">
         <v>142</v>
       </c>
-      <c r="D59" s="171"/>
-      <c r="E59" s="171"/>
-      <c r="F59" s="171"/>
+      <c r="D59" s="175"/>
+      <c r="E59" s="175"/>
+      <c r="F59" s="175"/>
     </row>
     <row r="60" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B60" s="74" t="s">
         <v>11</v>
       </c>
-      <c r="C60" s="171" t="s">
+      <c r="C60" s="175" t="s">
         <v>143</v>
       </c>
-      <c r="D60" s="171"/>
-      <c r="E60" s="171"/>
-      <c r="F60" s="171"/>
+      <c r="D60" s="175"/>
+      <c r="E60" s="175"/>
+      <c r="F60" s="175"/>
     </row>
     <row r="61" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B61" s="81" t="s">
         <v>12</v>
       </c>
-      <c r="C61" s="172" t="s">
+      <c r="C61" s="177" t="s">
         <v>144</v>
       </c>
-      <c r="D61" s="172"/>
-      <c r="E61" s="172"/>
-      <c r="F61" s="172"/>
+      <c r="D61" s="177"/>
+      <c r="E61" s="177"/>
+      <c r="F61" s="177"/>
     </row>
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="EAttMbwrYpwG6akiV7biz2nw7wlXtTooCxJogsSt7negKq0wKQ9sygPbVeHZ99cgmdNfAtLu9NnPC64y/Uaw7A==" saltValue="FJhchlgDftI44klS+XpFDg==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="15">
+    <mergeCell ref="C57:F57"/>
+    <mergeCell ref="C58:F58"/>
+    <mergeCell ref="C59:F59"/>
+    <mergeCell ref="C60:F60"/>
+    <mergeCell ref="C61:F61"/>
+    <mergeCell ref="C52:F52"/>
+    <mergeCell ref="C53:F53"/>
+    <mergeCell ref="C54:F54"/>
+    <mergeCell ref="C55:F55"/>
+    <mergeCell ref="C56:F56"/>
     <mergeCell ref="B47:F48"/>
     <mergeCell ref="H47:I48"/>
     <mergeCell ref="C49:F49"/>
     <mergeCell ref="C50:F50"/>
     <mergeCell ref="C51:F51"/>
-    <mergeCell ref="C52:F52"/>
-    <mergeCell ref="C53:F53"/>
-    <mergeCell ref="C54:F54"/>
-    <mergeCell ref="C55:F55"/>
-    <mergeCell ref="C56:F56"/>
-    <mergeCell ref="C57:F57"/>
-    <mergeCell ref="C58:F58"/>
-    <mergeCell ref="C59:F59"/>
-    <mergeCell ref="C60:F60"/>
-    <mergeCell ref="C61:F61"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
DBschema: PET and GRACE added for model types
</commit_message>
<xml_diff>
--- a/Schema/DB_scheme.xlsx
+++ b/Schema/DB_scheme.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aksam432/Documents/GitHub/WP3/Schema/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4666AC5F-0E88-404D-BAF9-C88D9B8D12B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29C1E736-913C-DE4B-8CA0-22F16931EE37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="23260" windowHeight="12460" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1012,7 +1012,7 @@
     <t>eV/A</t>
   </si>
   <si>
-    <t>['n2p2','ANI','GAP','SOAP','MTP','ACE','NequIP','Allegro','DeepMD','M3GNet','CHGNet','SevenNet','OrbNet',MACE','Custom']</t>
+    <t>[ 'DeepMD','n2p2','ANI','GAP','SOAP','MTP','ACE', 'NequIP', 'Allegro', 'M3GNet', 'CHGNet', 'SevenNet', 'OrbNet', 'MACE', 'GRACE', 'PET', 'Custom']</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
TrainingStrategy added an option for unknown for cases were models are just validated and not trained
</commit_message>
<xml_diff>
--- a/Schema/DB_scheme.xlsx
+++ b/Schema/DB_scheme.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aksam432/Documents/GitHub/WP3/Schema/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29C1E736-913C-DE4B-8CA0-22F16931EE37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{756BB8CF-28BA-9246-8632-C022C8E45FEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="23260" windowHeight="12460" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38400" yWindow="500" windowWidth="21600" windowHeight="37900" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Schéma à compléter" sheetId="1" r:id="rId1"/>
@@ -541,9 +541,6 @@
     <t>The total number of elements covered by the MLIP</t>
   </si>
   <si>
-    <t>['scratch','fine-tune']</t>
-  </si>
-  <si>
     <t>Version of software used</t>
   </si>
   <si>
@@ -1012,7 +1009,10 @@
     <t>eV/A</t>
   </si>
   <si>
-    <t>[ 'DeepMD','n2p2','ANI','GAP','SOAP','MTP','ACE', 'NequIP', 'Allegro', 'M3GNet', 'CHGNet', 'SevenNet', 'OrbNet', 'MACE', 'GRACE', 'PET', 'Custom']</t>
+    <t>[ 'DeepMD','HDNNP','ANI','GAP','SOAP','MTP','ACE', 'NequIP', 'Allegro', 'M3GNet', 'CHGNet', 'SevenNet', 'OrbNet', 'MACE', 'GRACE', 'PET', 'Custom']</t>
+  </si>
+  <si>
+    <t>['scratch','fine-tune','unknown']</t>
   </si>
 </sst>
 </file>
@@ -2220,6 +2220,15 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2231,15 +2240,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2702,7 +2702,7 @@
       </c>
       <c r="C2" s="169"/>
       <c r="D2" s="170" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="E2" s="170"/>
       <c r="F2" s="170"/>
@@ -2783,7 +2783,7 @@
         <v>55</v>
       </c>
       <c r="C7" s="129" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D7" s="130">
         <v>1</v>
@@ -2801,7 +2801,7 @@
       <c r="K7" s="131"/>
       <c r="L7" s="131"/>
       <c r="M7" s="132" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="8" spans="2:14" x14ac:dyDescent="0.2">
@@ -2809,7 +2809,7 @@
         <v>55</v>
       </c>
       <c r="C8" s="129" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="D8" s="130">
         <v>1</v>
@@ -2827,7 +2827,7 @@
       <c r="K8" s="131"/>
       <c r="L8" s="131"/>
       <c r="M8" s="132" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="9" spans="2:14" x14ac:dyDescent="0.2">
@@ -2850,7 +2850,7 @@
       <c r="H9" s="14"/>
       <c r="I9" s="14"/>
       <c r="J9" s="14" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="K9" s="14"/>
       <c r="L9" s="14"/>
@@ -2878,7 +2878,7 @@
       <c r="H10" s="14"/>
       <c r="I10" s="14"/>
       <c r="J10" s="14" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="K10" s="14"/>
       <c r="L10" s="14"/>
@@ -2906,13 +2906,13 @@
       <c r="H11" s="14"/>
       <c r="I11" s="14"/>
       <c r="J11" s="14" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="K11" s="14" t="s">
         <v>21</v>
       </c>
       <c r="L11" s="14" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="M11" s="112" t="s">
         <v>165</v>
@@ -2924,7 +2924,7 @@
         <v>55</v>
       </c>
       <c r="C12" s="93" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="D12" s="94">
         <v>1</v>
@@ -2939,7 +2939,7 @@
       <c r="H12" s="95"/>
       <c r="I12" s="95"/>
       <c r="J12" s="14" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="K12" s="95"/>
       <c r="L12" s="95"/>
@@ -2952,7 +2952,7 @@
         <v>55</v>
       </c>
       <c r="C13" s="93" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="D13" s="94">
         <v>1</v>
@@ -2967,16 +2967,16 @@
       <c r="H13" s="95"/>
       <c r="I13" s="95"/>
       <c r="J13" s="14" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="K13" s="95" t="s">
         <v>21</v>
       </c>
       <c r="L13" s="95" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="M13" s="113" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="N13" s="167"/>
     </row>
@@ -2985,71 +2985,74 @@
         <v>55</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="D14" s="13">
         <v>1</v>
       </c>
       <c r="E14" s="12" t="s">
-        <v>25</v>
+        <v>58</v>
       </c>
       <c r="F14" s="14" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="G14" s="14"/>
       <c r="H14" s="14"/>
       <c r="I14" s="12"/>
       <c r="J14" s="14" t="s">
-        <v>298</v>
-      </c>
-      <c r="K14" s="14"/>
-      <c r="L14" s="14"/>
+        <v>297</v>
+      </c>
+      <c r="K14" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="L14" s="14" t="s">
+        <v>324</v>
+      </c>
       <c r="M14" s="111" t="s">
-        <v>236</v>
-      </c>
-      <c r="N14" s="167"/>
+        <v>178</v>
+      </c>
     </row>
     <row r="15" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B15" s="11" t="s">
         <v>55</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>243</v>
+        <v>239</v>
       </c>
       <c r="D15" s="13">
         <v>1</v>
       </c>
       <c r="E15" s="12" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F15" s="14" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="G15" s="14"/>
       <c r="H15" s="14"/>
       <c r="I15" s="12"/>
       <c r="J15" s="14" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="K15" s="14"/>
       <c r="L15" s="14"/>
       <c r="M15" s="111" t="s">
-        <v>239</v>
-      </c>
-      <c r="N15" s="168"/>
+        <v>235</v>
+      </c>
+      <c r="N15" s="167"/>
     </row>
     <row r="16" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B16" s="11" t="s">
         <v>55</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="D16" s="13">
         <v>1</v>
       </c>
       <c r="E16" s="12" t="s">
-        <v>58</v>
+        <v>26</v>
       </c>
       <c r="F16" s="14" t="s">
         <v>18</v>
@@ -3058,24 +3061,21 @@
       <c r="H16" s="14"/>
       <c r="I16" s="12"/>
       <c r="J16" s="14" t="s">
-        <v>298</v>
-      </c>
-      <c r="K16" s="14" t="s">
-        <v>21</v>
-      </c>
-      <c r="L16" s="14" t="s">
-        <v>167</v>
-      </c>
+        <v>297</v>
+      </c>
+      <c r="K16" s="14"/>
+      <c r="L16" s="14"/>
       <c r="M16" s="111" t="s">
-        <v>179</v>
-      </c>
+        <v>238</v>
+      </c>
+      <c r="N16" s="168"/>
     </row>
     <row r="17" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="B17" s="11" t="s">
         <v>55</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="D17" s="13">
         <v>1</v>
@@ -3090,12 +3090,12 @@
       <c r="H17" s="14"/>
       <c r="I17" s="14"/>
       <c r="J17" s="14" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="K17" s="14"/>
       <c r="L17" s="14"/>
       <c r="M17" s="112" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.2">
@@ -3103,7 +3103,7 @@
         <v>55</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="D18" s="13">
         <v>1</v>
@@ -3118,12 +3118,12 @@
       <c r="H18" s="14"/>
       <c r="I18" s="12"/>
       <c r="J18" s="14" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="K18" s="14"/>
       <c r="L18" s="14"/>
       <c r="M18" s="111" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="19" spans="1:14" ht="17" x14ac:dyDescent="0.2">
@@ -3131,7 +3131,7 @@
         <v>55</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="D19" s="13">
         <v>1</v>
@@ -3146,12 +3146,12 @@
       <c r="H19" s="14"/>
       <c r="I19" s="14"/>
       <c r="J19" s="14" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="K19" s="14"/>
       <c r="L19" s="14"/>
       <c r="M19" s="114" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="20" spans="1:14" ht="17" x14ac:dyDescent="0.2">
@@ -3159,7 +3159,7 @@
         <v>55</v>
       </c>
       <c r="C20" s="163" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="D20" s="164">
         <v>1</v>
@@ -3177,7 +3177,7 @@
       <c r="K20" s="165"/>
       <c r="L20" s="165"/>
       <c r="M20" s="166" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.2">
@@ -3185,7 +3185,7 @@
         <v>55</v>
       </c>
       <c r="C21" s="12" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D21" s="13">
         <v>1</v>
@@ -3199,13 +3199,13 @@
       <c r="G21" s="14"/>
       <c r="H21" s="14"/>
       <c r="I21" s="14" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="J21" s="14"/>
       <c r="K21" s="14"/>
       <c r="L21" s="14"/>
       <c r="M21" s="111" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="N21" s="167"/>
     </row>
@@ -3214,7 +3214,7 @@
         <v>55</v>
       </c>
       <c r="C22" s="98" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="D22" s="99">
         <v>1</v>
@@ -3229,16 +3229,16 @@
       <c r="H22" s="100"/>
       <c r="I22" s="100"/>
       <c r="J22" s="14" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="K22" s="100" t="s">
         <v>21</v>
       </c>
       <c r="L22" s="105" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="M22" s="115" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="N22"/>
     </row>
@@ -3247,7 +3247,7 @@
         <v>55</v>
       </c>
       <c r="C23" s="12" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D23" s="13">
         <v>1</v>
@@ -3262,16 +3262,16 @@
       <c r="H23" s="14"/>
       <c r="I23" s="14"/>
       <c r="J23" s="14" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="K23" s="14" t="s">
         <v>21</v>
       </c>
       <c r="L23" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="M23" s="112" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="24" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -3279,7 +3279,7 @@
         <v>55</v>
       </c>
       <c r="C24" s="12" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="D24" s="13">
         <v>1</v>
@@ -3293,13 +3293,13 @@
       <c r="G24" s="14"/>
       <c r="H24" s="14"/>
       <c r="I24" s="14" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="J24" s="14"/>
       <c r="K24" s="14"/>
       <c r="L24" s="14"/>
       <c r="M24" s="114" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="25" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -3307,7 +3307,7 @@
         <v>55</v>
       </c>
       <c r="C25" s="12" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="D25" s="13">
         <v>1</v>
@@ -3321,13 +3321,13 @@
       <c r="G25" s="14"/>
       <c r="H25" s="14"/>
       <c r="I25" s="14" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="J25" s="14"/>
       <c r="K25" s="14"/>
       <c r="L25" s="14"/>
       <c r="M25" s="114" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="26" spans="1:14" ht="17" x14ac:dyDescent="0.2">
@@ -3335,7 +3335,7 @@
         <v>55</v>
       </c>
       <c r="C26" s="12" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D26" s="13">
         <v>1</v>
@@ -3349,13 +3349,13 @@
       <c r="G26" s="14"/>
       <c r="H26" s="14"/>
       <c r="I26" s="14" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="J26" s="14"/>
       <c r="K26" s="14"/>
       <c r="L26" s="14"/>
       <c r="M26" s="114" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="27" spans="1:14" ht="17" x14ac:dyDescent="0.2">
@@ -3363,7 +3363,7 @@
         <v>55</v>
       </c>
       <c r="C27" s="12" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="D27" s="13">
         <v>1</v>
@@ -3378,16 +3378,16 @@
       <c r="H27" s="14"/>
       <c r="I27" s="14"/>
       <c r="J27" s="14" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="K27" s="14" t="s">
         <v>21</v>
       </c>
       <c r="L27" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="M27" s="112" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="28" spans="1:14" ht="17" x14ac:dyDescent="0.2">
@@ -3395,7 +3395,7 @@
         <v>55</v>
       </c>
       <c r="C28" s="12" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="D28" s="13">
         <v>10</v>
@@ -3410,12 +3410,12 @@
       <c r="H28" s="14"/>
       <c r="I28" s="14"/>
       <c r="J28" s="14" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="K28" s="14"/>
       <c r="L28" s="14"/>
       <c r="M28" s="112" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="29" spans="1:14" ht="17" x14ac:dyDescent="0.2">
@@ -3423,7 +3423,7 @@
         <v>55</v>
       </c>
       <c r="C29" s="134" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="D29" s="135">
         <v>1</v>
@@ -3436,14 +3436,14 @@
       </c>
       <c r="G29" s="136"/>
       <c r="H29" s="136" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="I29" s="136"/>
       <c r="J29" s="136"/>
       <c r="K29" s="136"/>
       <c r="L29" s="136"/>
       <c r="M29" s="137" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="30" spans="1:14" ht="18" thickBot="1" x14ac:dyDescent="0.25">
@@ -3451,7 +3451,7 @@
         <v>55</v>
       </c>
       <c r="C30" s="140" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="D30" s="141">
         <v>10</v>
@@ -3465,19 +3465,19 @@
       <c r="G30" s="142"/>
       <c r="H30" s="142"/>
       <c r="I30" s="142" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="J30" s="142"/>
       <c r="K30" s="142"/>
       <c r="L30" s="142"/>
       <c r="M30" s="143" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="31" spans="1:14" ht="18" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A31" s="15"/>
       <c r="B31" s="128" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C31" s="129" t="s">
         <v>13</v>
@@ -3504,10 +3504,10 @@
     <row r="32" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A32" s="15"/>
       <c r="B32" s="128" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C32" s="129" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D32" s="130">
         <v>1</v>
@@ -3525,16 +3525,16 @@
       <c r="K32" s="131"/>
       <c r="L32" s="131"/>
       <c r="M32" s="138" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="33" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A33" s="15"/>
       <c r="B33" s="128" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C33" s="129" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="D33" s="130">
         <v>1</v>
@@ -3552,13 +3552,13 @@
       <c r="K33" s="131"/>
       <c r="L33" s="131"/>
       <c r="M33" s="138" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="34" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A34" s="15"/>
       <c r="B34" s="11" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C34" s="12" t="s">
         <v>163</v>
@@ -3576,21 +3576,21 @@
       <c r="H34" s="14"/>
       <c r="I34" s="16"/>
       <c r="J34" s="14" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="K34" s="14"/>
       <c r="L34" s="14"/>
       <c r="M34" s="112" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="35" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A35" s="15"/>
       <c r="B35" s="11" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C35" s="12" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="D35" s="13">
         <v>1</v>
@@ -3608,16 +3608,16 @@
       <c r="K35" s="14"/>
       <c r="L35" s="14"/>
       <c r="M35" s="112" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="36" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A36" s="15"/>
       <c r="B36" s="11" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C36" s="12" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="D36" s="13">
         <v>1</v>
@@ -3635,16 +3635,16 @@
       <c r="K36" s="14"/>
       <c r="L36" s="14"/>
       <c r="M36" s="112" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="37" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A37" s="15"/>
       <c r="B37" s="11" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C37" s="12" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="D37" s="13">
         <v>1</v>
@@ -3656,26 +3656,26 @@
         <v>18</v>
       </c>
       <c r="G37" s="14" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="H37" s="14"/>
       <c r="I37" s="16"/>
       <c r="J37" s="14" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="K37" s="14"/>
       <c r="L37" s="14"/>
       <c r="M37" s="112" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="38" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A38" s="15"/>
       <c r="B38" s="11" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C38" s="116" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="D38" s="13">
         <v>1</v>
@@ -3687,26 +3687,26 @@
         <v>18</v>
       </c>
       <c r="G38" s="14" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="H38" s="14"/>
       <c r="I38" s="16"/>
       <c r="J38" s="14" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="K38" s="14"/>
       <c r="L38" s="14"/>
       <c r="M38" s="112" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="39" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A39" s="15"/>
       <c r="B39" s="11" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C39" s="144" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="D39" s="13">
         <v>1</v>
@@ -3718,26 +3718,26 @@
         <v>18</v>
       </c>
       <c r="G39" s="14" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="H39" s="14"/>
       <c r="I39" s="14"/>
       <c r="J39" s="14" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="K39" s="14"/>
       <c r="L39" s="14"/>
       <c r="M39" s="114" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="40" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A40" s="15"/>
       <c r="B40" s="11" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C40" s="12" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="D40" s="13">
         <v>1</v>
@@ -3749,26 +3749,26 @@
         <v>15</v>
       </c>
       <c r="G40" s="14" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="H40" s="14"/>
       <c r="I40" s="14"/>
       <c r="J40" s="14" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="K40" s="14"/>
       <c r="L40" s="14"/>
       <c r="M40" s="114" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="41" spans="1:14" s="96" customFormat="1" ht="18" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A41" s="101"/>
       <c r="B41" s="148" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C41" s="149" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="D41" s="150">
         <v>1</v>
@@ -3780,24 +3780,24 @@
         <v>15</v>
       </c>
       <c r="G41" s="142" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="H41" s="153"/>
       <c r="I41" s="153"/>
       <c r="J41" s="142" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="K41" s="153"/>
       <c r="L41" s="153"/>
       <c r="M41" s="154" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="N41"/>
     </row>
     <row r="42" spans="1:14" s="96" customFormat="1" ht="18" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A42" s="101"/>
       <c r="B42" s="128" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C42" s="145" t="s">
         <v>13</v>
@@ -3825,10 +3825,10 @@
     <row r="43" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A43" s="15"/>
       <c r="B43" s="128" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C43" s="129" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D43" s="130">
         <v>1</v>
@@ -3846,16 +3846,16 @@
       <c r="K43" s="131"/>
       <c r="L43" s="131"/>
       <c r="M43" s="138" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="44" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A44" s="15"/>
       <c r="B44" s="128" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C44" s="129" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="D44" s="130">
         <v>1</v>
@@ -3873,16 +3873,16 @@
       <c r="K44" s="131"/>
       <c r="L44" s="131"/>
       <c r="M44" s="138" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="45" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A45" s="15"/>
       <c r="B45" s="11" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C45" s="12" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="D45" s="13">
         <v>1</v>
@@ -3897,18 +3897,18 @@
       <c r="H45" s="14"/>
       <c r="I45" s="14"/>
       <c r="J45" s="14" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="K45" s="14"/>
       <c r="L45" s="14"/>
       <c r="M45" s="117" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="46" spans="1:14" s="96" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A46" s="101"/>
       <c r="B46" s="97" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C46" s="102" t="s">
         <v>163</v>
@@ -3926,22 +3926,22 @@
       <c r="H46" s="103"/>
       <c r="I46" s="103"/>
       <c r="J46" s="103" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="K46" s="103"/>
       <c r="L46" s="103"/>
       <c r="M46" s="158" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="N46"/>
     </row>
     <row r="47" spans="1:14" s="96" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A47" s="101"/>
       <c r="B47" s="97" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C47" s="102" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D47" s="157">
         <v>1</v>
@@ -3956,26 +3956,26 @@
       <c r="H47" s="103"/>
       <c r="I47" s="103"/>
       <c r="J47" s="103" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="K47" s="103" t="s">
         <v>21</v>
       </c>
       <c r="L47" s="103" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="M47" s="158" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="N47"/>
     </row>
     <row r="48" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A48" s="15"/>
       <c r="B48" s="11" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C48" s="12" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="D48" s="13">
         <v>1</v>
@@ -3993,16 +3993,16 @@
       <c r="K48" s="14"/>
       <c r="L48" s="14"/>
       <c r="M48" s="112" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="49" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A49" s="15"/>
       <c r="B49" s="11" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C49" s="12" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="D49" s="13">
         <v>1</v>
@@ -4017,21 +4017,21 @@
       <c r="H49" s="14"/>
       <c r="I49" s="14"/>
       <c r="J49" s="14" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="K49" s="14"/>
       <c r="L49" s="14"/>
       <c r="M49" s="112" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="50" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A50" s="15"/>
       <c r="B50" s="11" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C50" s="12" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="D50" s="13">
         <v>5</v>
@@ -4046,21 +4046,21 @@
       <c r="H50" s="14"/>
       <c r="I50" s="14"/>
       <c r="J50" s="14" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="K50" s="14"/>
       <c r="L50" s="14"/>
       <c r="M50" s="112" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="51" spans="1:14" s="96" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A51" s="15"/>
       <c r="B51" s="11" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C51" s="12" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D51" s="13">
         <v>1</v>
@@ -4075,25 +4075,25 @@
       <c r="H51" s="14"/>
       <c r="I51" s="14"/>
       <c r="J51" s="14" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="K51" s="14"/>
       <c r="L51" s="14"/>
       <c r="M51" s="118" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="N51"/>
     </row>
     <row r="52" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A52" s="15"/>
       <c r="B52" s="11" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C52" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D52" s="13" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="E52" s="12" t="s">
         <v>14</v>
@@ -4105,21 +4105,21 @@
       <c r="H52" s="14"/>
       <c r="I52" s="14"/>
       <c r="J52" s="14" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="K52" s="14"/>
       <c r="L52" s="14"/>
       <c r="M52" s="118" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
     <row r="53" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A53" s="96"/>
       <c r="B53" s="11" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C53" s="98" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D53" s="99">
         <v>1</v>
@@ -4131,25 +4131,25 @@
         <v>18</v>
       </c>
       <c r="G53" s="100" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H53" s="100"/>
       <c r="I53" s="100"/>
       <c r="J53" s="14" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="K53" s="100"/>
       <c r="L53" s="100"/>
       <c r="M53" s="119" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="54" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B54" s="11" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C54" s="12" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D54" s="13">
         <v>1</v>
@@ -4161,25 +4161,25 @@
         <v>18</v>
       </c>
       <c r="G54" s="14" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H54" s="14"/>
       <c r="I54" s="14"/>
       <c r="J54" s="14" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="K54" s="14"/>
       <c r="L54" s="14"/>
       <c r="M54" s="120" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="55" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B55" s="11" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C55" s="12" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D55" s="13">
         <v>1</v>
@@ -4191,25 +4191,25 @@
         <v>18</v>
       </c>
       <c r="G55" s="14" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="H55" s="14"/>
       <c r="I55" s="14"/>
       <c r="J55" s="14" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="K55" s="14"/>
       <c r="L55" s="14"/>
       <c r="M55" s="111" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="56" spans="1:14" s="96" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B56" s="97" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C56" s="102" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D56" s="157">
         <v>1</v>
@@ -4221,26 +4221,26 @@
         <v>18</v>
       </c>
       <c r="G56" s="103" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="H56" s="103"/>
       <c r="I56" s="103"/>
       <c r="J56" s="103" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="K56" s="103"/>
       <c r="L56" s="103"/>
       <c r="M56" s="159" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="N56"/>
     </row>
     <row r="57" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B57" s="11" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C57" s="12" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="D57" s="13">
         <v>1</v>
@@ -4254,22 +4254,22 @@
       <c r="G57" s="14"/>
       <c r="H57" s="14"/>
       <c r="I57" s="14" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="J57" s="14"/>
       <c r="K57" s="14"/>
       <c r="L57" s="14"/>
       <c r="M57" s="121" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="58" spans="1:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A58" s="96"/>
       <c r="B58" s="139" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C58" s="140" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="D58" s="141">
         <v>1</v>
@@ -4287,13 +4287,13 @@
       <c r="K58" s="142"/>
       <c r="L58" s="142"/>
       <c r="M58" s="155" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="59" spans="1:14" ht="18" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A59" s="101"/>
       <c r="B59" s="128" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C59" s="145" t="s">
         <v>13</v>
@@ -4320,10 +4320,10 @@
     <row r="60" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A60" s="15"/>
       <c r="B60" s="128" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C60" s="129" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D60" s="130">
         <v>1</v>
@@ -4341,16 +4341,16 @@
       <c r="K60" s="131"/>
       <c r="L60" s="131"/>
       <c r="M60" s="138" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="61" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A61" s="15"/>
       <c r="B61" s="128" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C61" s="129" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="D61" s="130">
         <v>1</v>
@@ -4368,15 +4368,15 @@
       <c r="K61" s="131"/>
       <c r="L61" s="131"/>
       <c r="M61" s="138" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="62" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B62" s="11" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C62" s="12" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D62" s="13">
         <v>1</v>
@@ -4391,20 +4391,20 @@
       <c r="H62" s="14"/>
       <c r="I62" s="14"/>
       <c r="J62" s="14" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="K62" s="14"/>
       <c r="L62" s="14"/>
       <c r="M62" s="111" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="63" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B63" s="11" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C63" s="12" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D63" s="13">
         <v>1</v>
@@ -4419,20 +4419,20 @@
       <c r="H63" s="14"/>
       <c r="I63" s="14"/>
       <c r="J63" s="14" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="K63" s="14"/>
       <c r="L63" s="14"/>
       <c r="M63" s="121" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="64" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B64" s="11" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C64" s="12" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="D64" s="13">
         <v>1</v>
@@ -4450,15 +4450,15 @@
       <c r="K64" s="14"/>
       <c r="L64" s="14"/>
       <c r="M64" s="159" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="65" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B65" s="11" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C65" s="12" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="D65" s="13">
         <v>1</v>
@@ -4473,24 +4473,24 @@
       <c r="H65" s="14"/>
       <c r="I65" s="14"/>
       <c r="J65" s="14" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="K65" s="14" t="s">
         <v>21</v>
       </c>
       <c r="L65" s="14" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="M65" s="111" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="66" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B66" s="11" t="s">
+        <v>170</v>
+      </c>
+      <c r="C66" s="12" t="s">
         <v>171</v>
-      </c>
-      <c r="C66" s="12" t="s">
-        <v>172</v>
       </c>
       <c r="D66" s="13">
         <v>1</v>
@@ -4505,20 +4505,20 @@
       <c r="H66" s="14"/>
       <c r="I66" s="14"/>
       <c r="J66" s="14" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="K66" s="14"/>
       <c r="L66" s="14"/>
       <c r="M66" s="122" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="67" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B67" s="11" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C67" s="12" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="D67" s="13">
         <v>1</v>
@@ -4530,25 +4530,25 @@
         <v>15</v>
       </c>
       <c r="G67" s="14" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="H67" s="14"/>
       <c r="I67" s="14"/>
       <c r="J67" s="14" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="K67" s="14"/>
       <c r="L67" s="14"/>
       <c r="M67" s="111" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="68" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B68" s="11" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C68" s="12" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="D68" s="13">
         <v>1</v>
@@ -4560,25 +4560,25 @@
         <v>15</v>
       </c>
       <c r="G68" s="14" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="H68" s="14"/>
       <c r="I68" s="14"/>
       <c r="J68" s="14" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="K68" s="14"/>
       <c r="L68" s="14"/>
       <c r="M68" s="121" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="69" spans="1:14" s="96" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B69" s="97" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C69" s="102" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D69" s="157">
         <v>1</v>
@@ -4593,21 +4593,21 @@
       <c r="H69" s="103"/>
       <c r="I69" s="103"/>
       <c r="J69" s="103" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="K69" s="103"/>
       <c r="L69" s="103"/>
       <c r="M69" s="161" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="N69"/>
     </row>
     <row r="70" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B70" s="11" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C70" s="12" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D70" s="13">
         <v>1</v>
@@ -4622,20 +4622,20 @@
       <c r="H70" s="14"/>
       <c r="I70" s="14"/>
       <c r="J70" s="14" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="K70" s="14"/>
       <c r="L70" s="14"/>
       <c r="M70" s="121" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="71" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B71" s="11" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C71" s="12" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D71" s="13">
         <v>1</v>
@@ -4650,20 +4650,20 @@
       <c r="H71" s="14"/>
       <c r="I71" s="14"/>
       <c r="J71" s="14" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="K71" s="14"/>
       <c r="L71" s="14"/>
       <c r="M71" s="111" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="72" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B72" s="11" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C72" s="12" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="D72" s="13">
         <v>1</v>
@@ -4675,25 +4675,25 @@
         <v>15</v>
       </c>
       <c r="G72" s="14" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="H72" s="14"/>
       <c r="I72" s="14"/>
       <c r="J72" s="14" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="K72" s="14"/>
       <c r="L72" s="14"/>
       <c r="M72" s="111" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="73" spans="1:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B73" s="139" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C73" s="140" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="D73" s="141">
         <v>1</v>
@@ -4705,23 +4705,23 @@
         <v>15</v>
       </c>
       <c r="G73" s="142" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="H73" s="142"/>
       <c r="I73" s="142"/>
       <c r="J73" s="142" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="K73" s="142"/>
       <c r="L73" s="142"/>
       <c r="M73" s="160" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="74" spans="1:14" ht="18" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A74" s="96"/>
       <c r="B74" s="128" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C74" s="145" t="s">
         <v>13</v>
@@ -4748,10 +4748,10 @@
     <row r="75" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A75" s="101"/>
       <c r="B75" s="128" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C75" s="129" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D75" s="130">
         <v>1</v>
@@ -4769,16 +4769,16 @@
       <c r="K75" s="131"/>
       <c r="L75" s="131"/>
       <c r="M75" s="138" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="76" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A76" s="101"/>
       <c r="B76" s="128" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C76" s="129" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="D76" s="130">
         <v>1</v>
@@ -4796,16 +4796,16 @@
       <c r="K76" s="131"/>
       <c r="L76" s="131"/>
       <c r="M76" s="138" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="77" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A77" s="96"/>
       <c r="B77" s="11" t="s">
+        <v>175</v>
+      </c>
+      <c r="C77" s="12" t="s">
         <v>176</v>
-      </c>
-      <c r="C77" s="12" t="s">
-        <v>177</v>
       </c>
       <c r="D77" s="13">
         <v>1</v>
@@ -4820,17 +4820,17 @@
       <c r="H77" s="14"/>
       <c r="I77" s="14"/>
       <c r="J77" s="14" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="K77" s="14"/>
       <c r="L77" s="14"/>
       <c r="M77" s="121" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="78" spans="1:14" s="96" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B78" s="11" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C78" s="12" t="s">
         <v>12</v>
@@ -4848,22 +4848,22 @@
       <c r="H78" s="14"/>
       <c r="I78" s="14"/>
       <c r="J78" s="14" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="K78" s="14"/>
       <c r="L78" s="14"/>
       <c r="M78" s="111" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="N78"/>
     </row>
     <row r="79" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A79" s="96"/>
       <c r="B79" s="11" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C79" s="12" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="D79" s="13">
         <v>1</v>
@@ -4877,22 +4877,22 @@
       <c r="G79" s="14"/>
       <c r="H79" s="14"/>
       <c r="I79" s="14" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="J79" s="14"/>
       <c r="K79" s="14"/>
       <c r="L79" s="14"/>
       <c r="M79" s="111" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="80" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A80" s="96"/>
       <c r="B80" s="97" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C80" s="102" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="D80" s="157">
         <v>1</v>
@@ -4907,25 +4907,25 @@
       <c r="H80" s="103"/>
       <c r="I80" s="103"/>
       <c r="J80" s="103" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="K80" s="103" t="s">
         <v>21</v>
       </c>
       <c r="L80" s="103" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="M80" s="161" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="81" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A81" s="96"/>
       <c r="B81" s="11" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C81" s="12" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="D81" s="13">
         <v>1</v>
@@ -4940,21 +4940,21 @@
       <c r="H81" s="14"/>
       <c r="I81" s="14"/>
       <c r="J81" s="14" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="K81" s="14"/>
       <c r="L81" s="14"/>
       <c r="M81" s="121" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="82" spans="1:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A82" s="96"/>
       <c r="B82" s="139" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C82" s="140" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="D82" s="141">
         <v>1</v>
@@ -4967,19 +4967,19 @@
       </c>
       <c r="G82" s="142"/>
       <c r="H82" s="142" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="I82" s="142"/>
       <c r="J82" s="142"/>
       <c r="K82" s="142"/>
       <c r="L82" s="142"/>
       <c r="M82" s="160" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="83" spans="1:14" s="96" customFormat="1" ht="18" thickTop="1" x14ac:dyDescent="0.2">
       <c r="B83" s="128" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C83" s="145" t="s">
         <v>13</v>
@@ -5007,10 +5007,10 @@
     <row r="84" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A84" s="15"/>
       <c r="B84" s="128" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C84" s="129" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D84" s="130">
         <v>1</v>
@@ -5028,16 +5028,16 @@
       <c r="K84" s="131"/>
       <c r="L84" s="131"/>
       <c r="M84" s="138" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="85" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A85" s="15"/>
       <c r="B85" s="128" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C85" s="129" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="D85" s="130">
         <v>1</v>
@@ -5055,15 +5055,15 @@
       <c r="K85" s="131"/>
       <c r="L85" s="131"/>
       <c r="M85" s="138" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="86" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B86" s="97" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C86" s="12" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="D86" s="13">
         <v>1</v>
@@ -5083,16 +5083,16 @@
       <c r="K86" s="14"/>
       <c r="L86" s="14"/>
       <c r="M86" s="111" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="87" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A87" s="96"/>
       <c r="B87" s="97" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C87" s="102" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="D87" s="157">
         <v>1</v>
@@ -5106,21 +5106,21 @@
       <c r="G87" s="103"/>
       <c r="H87" s="103"/>
       <c r="I87" s="103" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="J87" s="103"/>
       <c r="K87" s="103"/>
       <c r="L87" s="103"/>
       <c r="M87" s="161" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="88" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B88" s="97" t="s">
+        <v>287</v>
+      </c>
+      <c r="C88" s="12" t="s">
         <v>288</v>
-      </c>
-      <c r="C88" s="12" t="s">
-        <v>289</v>
       </c>
       <c r="D88" s="13">
         <v>1</v>
@@ -5135,20 +5135,20 @@
       <c r="H88" s="14"/>
       <c r="I88" s="14"/>
       <c r="J88" s="14" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="K88" s="14"/>
       <c r="L88" s="14"/>
       <c r="M88" s="111" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="89" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B89" s="97" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C89" s="12" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="D89" s="13">
         <v>1</v>
@@ -5163,20 +5163,20 @@
       <c r="H89" s="14"/>
       <c r="I89" s="14"/>
       <c r="J89" s="14" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="K89" s="14"/>
       <c r="L89" s="14"/>
       <c r="M89" s="121" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="90" spans="1:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B90" s="148" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C90" s="140" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="D90" s="141">
         <v>1</v>
@@ -5189,20 +5189,20 @@
       </c>
       <c r="G90" s="142"/>
       <c r="H90" s="142" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="I90" s="142"/>
       <c r="J90" s="142"/>
       <c r="K90" s="142"/>
       <c r="L90" s="142"/>
       <c r="M90" s="160" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="91" spans="1:14" ht="17" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A91" s="104"/>
       <c r="B91" s="128" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C91" s="145" t="s">
         <v>13</v>
@@ -5229,10 +5229,10 @@
     <row r="92" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A92" s="15"/>
       <c r="B92" s="128" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C92" s="129" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D92" s="130">
         <v>1</v>
@@ -5250,16 +5250,16 @@
       <c r="K92" s="131"/>
       <c r="L92" s="131"/>
       <c r="M92" s="138" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="93" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A93" s="15"/>
       <c r="B93" s="128" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C93" s="129" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="D93" s="130">
         <v>1</v>
@@ -5277,15 +5277,15 @@
       <c r="K93" s="131"/>
       <c r="L93" s="131"/>
       <c r="M93" s="138" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="94" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B94" s="11" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C94" s="12" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D94" s="13">
         <v>1</v>
@@ -5300,20 +5300,20 @@
       <c r="H94" s="14"/>
       <c r="I94" s="14"/>
       <c r="J94" s="14" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="K94" s="14"/>
       <c r="L94" s="14"/>
       <c r="M94" s="111" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="95" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B95" s="11" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C95" s="12" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D95" s="13">
         <v>1</v>
@@ -5328,20 +5328,20 @@
       <c r="H95" s="14"/>
       <c r="I95" s="14"/>
       <c r="J95" s="14" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="K95" s="14"/>
       <c r="L95" s="14"/>
       <c r="M95" s="111" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="96" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B96" s="11" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C96" s="12" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="D96" s="13">
         <v>1</v>
@@ -5356,17 +5356,17 @@
       <c r="H96" s="14"/>
       <c r="I96" s="14"/>
       <c r="J96" s="14" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="K96" s="14"/>
       <c r="L96" s="14"/>
       <c r="M96" s="111" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="97" spans="2:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B97" s="123" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C97" s="124" t="s">
         <v>161</v>
@@ -5384,12 +5384,12 @@
       <c r="H97" s="126"/>
       <c r="I97" s="126"/>
       <c r="J97" s="126" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="K97" s="126"/>
       <c r="L97" s="126"/>
       <c r="M97" s="127" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
   </sheetData>
@@ -6596,37 +6596,37 @@
       </c>
     </row>
     <row r="47" spans="2:13" x14ac:dyDescent="0.2">
-      <c r="B47" s="171" t="s">
+      <c r="B47" s="174" t="s">
         <v>121</v>
       </c>
-      <c r="C47" s="171"/>
-      <c r="D47" s="171"/>
-      <c r="E47" s="171"/>
-      <c r="F47" s="171"/>
-      <c r="H47" s="172" t="s">
+      <c r="C47" s="174"/>
+      <c r="D47" s="174"/>
+      <c r="E47" s="174"/>
+      <c r="F47" s="174"/>
+      <c r="H47" s="175" t="s">
         <v>122</v>
       </c>
-      <c r="I47" s="172"/>
+      <c r="I47" s="175"/>
     </row>
     <row r="48" spans="2:13" x14ac:dyDescent="0.2">
-      <c r="B48" s="171"/>
-      <c r="C48" s="171"/>
-      <c r="D48" s="171"/>
-      <c r="E48" s="171"/>
-      <c r="F48" s="171"/>
-      <c r="H48" s="172"/>
-      <c r="I48" s="172"/>
+      <c r="B48" s="174"/>
+      <c r="C48" s="174"/>
+      <c r="D48" s="174"/>
+      <c r="E48" s="174"/>
+      <c r="F48" s="174"/>
+      <c r="H48" s="175"/>
+      <c r="I48" s="175"/>
     </row>
     <row r="49" spans="2:9" ht="16" x14ac:dyDescent="0.2">
       <c r="B49" s="68" t="s">
         <v>123</v>
       </c>
-      <c r="C49" s="173" t="s">
+      <c r="C49" s="176" t="s">
         <v>12</v>
       </c>
-      <c r="D49" s="173"/>
-      <c r="E49" s="173"/>
-      <c r="F49" s="173"/>
+      <c r="D49" s="176"/>
+      <c r="E49" s="176"/>
+      <c r="F49" s="176"/>
       <c r="H49" s="69" t="s">
         <v>124</v>
       </c>
@@ -6638,12 +6638,12 @@
       <c r="B50" s="71" t="s">
         <v>1</v>
       </c>
-      <c r="C50" s="174" t="s">
+      <c r="C50" s="177" t="s">
         <v>126</v>
       </c>
-      <c r="D50" s="174"/>
-      <c r="E50" s="174"/>
-      <c r="F50" s="174"/>
+      <c r="D50" s="177"/>
+      <c r="E50" s="177"/>
+      <c r="F50" s="177"/>
       <c r="H50" s="72" t="s">
         <v>48</v>
       </c>
@@ -6655,12 +6655,12 @@
       <c r="B51" s="74" t="s">
         <v>2</v>
       </c>
-      <c r="C51" s="175" t="s">
+      <c r="C51" s="171" t="s">
         <v>128</v>
       </c>
-      <c r="D51" s="175"/>
-      <c r="E51" s="175"/>
-      <c r="F51" s="175"/>
+      <c r="D51" s="171"/>
+      <c r="E51" s="171"/>
+      <c r="F51" s="171"/>
       <c r="H51" s="75" t="s">
         <v>70</v>
       </c>
@@ -6672,12 +6672,12 @@
       <c r="B52" s="74" t="s">
         <v>3</v>
       </c>
-      <c r="C52" s="175" t="s">
+      <c r="C52" s="171" t="s">
         <v>130</v>
       </c>
-      <c r="D52" s="175"/>
-      <c r="E52" s="175"/>
-      <c r="F52" s="175"/>
+      <c r="D52" s="171"/>
+      <c r="E52" s="171"/>
+      <c r="F52" s="171"/>
       <c r="H52" s="77" t="s">
         <v>131</v>
       </c>
@@ -6689,12 +6689,12 @@
       <c r="B53" s="74" t="s">
         <v>4</v>
       </c>
-      <c r="C53" s="176" t="s">
+      <c r="C53" s="173" t="s">
         <v>133</v>
       </c>
-      <c r="D53" s="176"/>
-      <c r="E53" s="176"/>
-      <c r="F53" s="176"/>
+      <c r="D53" s="173"/>
+      <c r="E53" s="173"/>
+      <c r="F53" s="173"/>
       <c r="H53" s="77" t="s">
         <v>81</v>
       </c>
@@ -6706,12 +6706,12 @@
       <c r="B54" s="74" t="s">
         <v>5</v>
       </c>
-      <c r="C54" s="175" t="s">
+      <c r="C54" s="171" t="s">
         <v>135</v>
       </c>
-      <c r="D54" s="175"/>
-      <c r="E54" s="175"/>
-      <c r="F54" s="175"/>
+      <c r="D54" s="171"/>
+      <c r="E54" s="171"/>
+      <c r="F54" s="171"/>
       <c r="H54" s="77" t="s">
         <v>55</v>
       </c>
@@ -6723,12 +6723,12 @@
       <c r="B55" s="74" t="s">
         <v>6</v>
       </c>
-      <c r="C55" s="176" t="s">
+      <c r="C55" s="173" t="s">
         <v>137</v>
       </c>
-      <c r="D55" s="176"/>
-      <c r="E55" s="176"/>
-      <c r="F55" s="176"/>
+      <c r="D55" s="173"/>
+      <c r="E55" s="173"/>
+      <c r="F55" s="173"/>
       <c r="H55" s="79" t="s">
         <v>114</v>
       </c>
@@ -6740,86 +6740,86 @@
       <c r="B56" s="74" t="s">
         <v>7</v>
       </c>
-      <c r="C56" s="175" t="s">
+      <c r="C56" s="171" t="s">
         <v>139</v>
       </c>
-      <c r="D56" s="175"/>
-      <c r="E56" s="175"/>
-      <c r="F56" s="175"/>
+      <c r="D56" s="171"/>
+      <c r="E56" s="171"/>
+      <c r="F56" s="171"/>
     </row>
     <row r="57" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B57" s="74" t="s">
         <v>8</v>
       </c>
-      <c r="C57" s="175" t="s">
+      <c r="C57" s="171" t="s">
         <v>140</v>
       </c>
-      <c r="D57" s="175"/>
-      <c r="E57" s="175"/>
-      <c r="F57" s="175"/>
+      <c r="D57" s="171"/>
+      <c r="E57" s="171"/>
+      <c r="F57" s="171"/>
     </row>
     <row r="58" spans="2:9" ht="45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B58" s="74" t="s">
         <v>9</v>
       </c>
-      <c r="C58" s="175" t="s">
+      <c r="C58" s="171" t="s">
         <v>141</v>
       </c>
-      <c r="D58" s="175"/>
-      <c r="E58" s="175"/>
-      <c r="F58" s="175"/>
+      <c r="D58" s="171"/>
+      <c r="E58" s="171"/>
+      <c r="F58" s="171"/>
     </row>
     <row r="59" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B59" s="74" t="s">
         <v>10</v>
       </c>
-      <c r="C59" s="175" t="s">
+      <c r="C59" s="171" t="s">
         <v>142</v>
       </c>
-      <c r="D59" s="175"/>
-      <c r="E59" s="175"/>
-      <c r="F59" s="175"/>
+      <c r="D59" s="171"/>
+      <c r="E59" s="171"/>
+      <c r="F59" s="171"/>
     </row>
     <row r="60" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B60" s="74" t="s">
         <v>11</v>
       </c>
-      <c r="C60" s="175" t="s">
+      <c r="C60" s="171" t="s">
         <v>143</v>
       </c>
-      <c r="D60" s="175"/>
-      <c r="E60" s="175"/>
-      <c r="F60" s="175"/>
+      <c r="D60" s="171"/>
+      <c r="E60" s="171"/>
+      <c r="F60" s="171"/>
     </row>
     <row r="61" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B61" s="81" t="s">
         <v>12</v>
       </c>
-      <c r="C61" s="177" t="s">
+      <c r="C61" s="172" t="s">
         <v>144</v>
       </c>
-      <c r="D61" s="177"/>
-      <c r="E61" s="177"/>
-      <c r="F61" s="177"/>
+      <c r="D61" s="172"/>
+      <c r="E61" s="172"/>
+      <c r="F61" s="172"/>
     </row>
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="EAttMbwrYpwG6akiV7biz2nw7wlXtTooCxJogsSt7negKq0wKQ9sygPbVeHZ99cgmdNfAtLu9NnPC64y/Uaw7A==" saltValue="FJhchlgDftI44klS+XpFDg==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="15">
+    <mergeCell ref="B47:F48"/>
+    <mergeCell ref="H47:I48"/>
+    <mergeCell ref="C49:F49"/>
+    <mergeCell ref="C50:F50"/>
+    <mergeCell ref="C51:F51"/>
+    <mergeCell ref="C52:F52"/>
+    <mergeCell ref="C53:F53"/>
+    <mergeCell ref="C54:F54"/>
+    <mergeCell ref="C55:F55"/>
+    <mergeCell ref="C56:F56"/>
     <mergeCell ref="C57:F57"/>
     <mergeCell ref="C58:F58"/>
     <mergeCell ref="C59:F59"/>
     <mergeCell ref="C60:F60"/>
     <mergeCell ref="C61:F61"/>
-    <mergeCell ref="C52:F52"/>
-    <mergeCell ref="C53:F53"/>
-    <mergeCell ref="C54:F54"/>
-    <mergeCell ref="C55:F55"/>
-    <mergeCell ref="C56:F56"/>
-    <mergeCell ref="B47:F48"/>
-    <mergeCell ref="H47:I48"/>
-    <mergeCell ref="C49:F49"/>
-    <mergeCell ref="C50:F50"/>
-    <mergeCell ref="C51:F51"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
ModelType chaged to  ModelArchitecture
</commit_message>
<xml_diff>
--- a/Schema/DB_scheme.xlsx
+++ b/Schema/DB_scheme.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aksam432/Documents/GitHub/WP3/Schema/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{756BB8CF-28BA-9246-8632-C022C8E45FEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5144DA8-3ECF-6C44-BE35-F374456A1E86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38400" yWindow="500" windowWidth="21600" windowHeight="37900" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -763,9 +763,6 @@
     <t>noOfElements</t>
   </si>
   <si>
-    <t>modelType</t>
-  </si>
-  <si>
     <t>longRangeInteraction</t>
   </si>
   <si>
@@ -1013,6 +1010,9 @@
   </si>
   <si>
     <t>['scratch','fine-tune','unknown']</t>
+  </si>
+  <si>
+    <t>modelArchitecture</t>
   </si>
 </sst>
 </file>
@@ -2220,26 +2220,26 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="31" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="31" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2702,7 +2702,7 @@
       </c>
       <c r="C2" s="169"/>
       <c r="D2" s="170" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="E2" s="170"/>
       <c r="F2" s="170"/>
@@ -2783,7 +2783,7 @@
         <v>55</v>
       </c>
       <c r="C7" s="129" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="D7" s="130">
         <v>1</v>
@@ -2801,7 +2801,7 @@
       <c r="K7" s="131"/>
       <c r="L7" s="131"/>
       <c r="M7" s="132" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="8" spans="2:14" x14ac:dyDescent="0.2">
@@ -2809,7 +2809,7 @@
         <v>55</v>
       </c>
       <c r="C8" s="129" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D8" s="130">
         <v>1</v>
@@ -2827,7 +2827,7 @@
       <c r="K8" s="131"/>
       <c r="L8" s="131"/>
       <c r="M8" s="132" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="9" spans="2:14" x14ac:dyDescent="0.2">
@@ -2850,7 +2850,7 @@
       <c r="H9" s="14"/>
       <c r="I9" s="14"/>
       <c r="J9" s="14" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="K9" s="14"/>
       <c r="L9" s="14"/>
@@ -2878,7 +2878,7 @@
       <c r="H10" s="14"/>
       <c r="I10" s="14"/>
       <c r="J10" s="14" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="K10" s="14"/>
       <c r="L10" s="14"/>
@@ -2906,13 +2906,13 @@
       <c r="H11" s="14"/>
       <c r="I11" s="14"/>
       <c r="J11" s="14" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="K11" s="14" t="s">
         <v>21</v>
       </c>
       <c r="L11" s="14" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="M11" s="112" t="s">
         <v>165</v>
@@ -2939,7 +2939,7 @@
       <c r="H12" s="95"/>
       <c r="I12" s="95"/>
       <c r="J12" s="14" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="K12" s="95"/>
       <c r="L12" s="95"/>
@@ -2952,7 +2952,7 @@
         <v>55</v>
       </c>
       <c r="C13" s="93" t="s">
-        <v>241</v>
+        <v>324</v>
       </c>
       <c r="D13" s="94">
         <v>1</v>
@@ -2967,13 +2967,13 @@
       <c r="H13" s="95"/>
       <c r="I13" s="95"/>
       <c r="J13" s="14" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="K13" s="95" t="s">
         <v>21</v>
       </c>
       <c r="L13" s="95" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="M13" s="113" t="s">
         <v>184</v>
@@ -2985,7 +2985,7 @@
         <v>55</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="D14" s="13">
         <v>1</v>
@@ -3000,13 +3000,13 @@
       <c r="H14" s="14"/>
       <c r="I14" s="12"/>
       <c r="J14" s="14" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="K14" s="14" t="s">
         <v>21</v>
       </c>
       <c r="L14" s="14" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="M14" s="111" t="s">
         <v>178</v>
@@ -3032,7 +3032,7 @@
       <c r="H15" s="14"/>
       <c r="I15" s="12"/>
       <c r="J15" s="14" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="K15" s="14"/>
       <c r="L15" s="14"/>
@@ -3046,7 +3046,7 @@
         <v>55</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="D16" s="13">
         <v>1</v>
@@ -3061,7 +3061,7 @@
       <c r="H16" s="14"/>
       <c r="I16" s="12"/>
       <c r="J16" s="14" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="K16" s="14"/>
       <c r="L16" s="14"/>
@@ -3075,7 +3075,7 @@
         <v>55</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="D17" s="13">
         <v>1</v>
@@ -3090,7 +3090,7 @@
       <c r="H17" s="14"/>
       <c r="I17" s="14"/>
       <c r="J17" s="14" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="K17" s="14"/>
       <c r="L17" s="14"/>
@@ -3103,7 +3103,7 @@
         <v>55</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="D18" s="13">
         <v>1</v>
@@ -3118,7 +3118,7 @@
       <c r="H18" s="14"/>
       <c r="I18" s="12"/>
       <c r="J18" s="14" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="K18" s="14"/>
       <c r="L18" s="14"/>
@@ -3131,7 +3131,7 @@
         <v>55</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="D19" s="13">
         <v>1</v>
@@ -3146,7 +3146,7 @@
       <c r="H19" s="14"/>
       <c r="I19" s="14"/>
       <c r="J19" s="14" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="K19" s="14"/>
       <c r="L19" s="14"/>
@@ -3159,7 +3159,7 @@
         <v>55</v>
       </c>
       <c r="C20" s="163" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="D20" s="164">
         <v>1</v>
@@ -3185,7 +3185,7 @@
         <v>55</v>
       </c>
       <c r="C21" s="12" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="D21" s="13">
         <v>1</v>
@@ -3214,7 +3214,7 @@
         <v>55</v>
       </c>
       <c r="C22" s="98" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D22" s="99">
         <v>1</v>
@@ -3229,13 +3229,13 @@
       <c r="H22" s="100"/>
       <c r="I22" s="100"/>
       <c r="J22" s="14" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="K22" s="100" t="s">
         <v>21</v>
       </c>
       <c r="L22" s="105" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="M22" s="115" t="s">
         <v>183</v>
@@ -3262,7 +3262,7 @@
       <c r="H23" s="14"/>
       <c r="I23" s="14"/>
       <c r="J23" s="14" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="K23" s="14" t="s">
         <v>21</v>
@@ -3279,7 +3279,7 @@
         <v>55</v>
       </c>
       <c r="C24" s="12" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="D24" s="13">
         <v>1</v>
@@ -3293,7 +3293,7 @@
       <c r="G24" s="14"/>
       <c r="H24" s="14"/>
       <c r="I24" s="14" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="J24" s="14"/>
       <c r="K24" s="14"/>
@@ -3307,7 +3307,7 @@
         <v>55</v>
       </c>
       <c r="C25" s="12" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="D25" s="13">
         <v>1</v>
@@ -3321,7 +3321,7 @@
       <c r="G25" s="14"/>
       <c r="H25" s="14"/>
       <c r="I25" s="14" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="J25" s="14"/>
       <c r="K25" s="14"/>
@@ -3335,7 +3335,7 @@
         <v>55</v>
       </c>
       <c r="C26" s="12" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="D26" s="13">
         <v>1</v>
@@ -3349,7 +3349,7 @@
       <c r="G26" s="14"/>
       <c r="H26" s="14"/>
       <c r="I26" s="14" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="J26" s="14"/>
       <c r="K26" s="14"/>
@@ -3363,7 +3363,7 @@
         <v>55</v>
       </c>
       <c r="C27" s="12" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D27" s="13">
         <v>1</v>
@@ -3378,7 +3378,7 @@
       <c r="H27" s="14"/>
       <c r="I27" s="14"/>
       <c r="J27" s="14" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="K27" s="14" t="s">
         <v>21</v>
@@ -3395,7 +3395,7 @@
         <v>55</v>
       </c>
       <c r="C28" s="12" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="D28" s="13">
         <v>10</v>
@@ -3410,7 +3410,7 @@
       <c r="H28" s="14"/>
       <c r="I28" s="14"/>
       <c r="J28" s="14" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="K28" s="14"/>
       <c r="L28" s="14"/>
@@ -3423,7 +3423,7 @@
         <v>55</v>
       </c>
       <c r="C29" s="134" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="D29" s="135">
         <v>1</v>
@@ -3436,7 +3436,7 @@
       </c>
       <c r="G29" s="136"/>
       <c r="H29" s="136" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="I29" s="136"/>
       <c r="J29" s="136"/>
@@ -3451,7 +3451,7 @@
         <v>55</v>
       </c>
       <c r="C30" s="140" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="D30" s="141">
         <v>10</v>
@@ -3465,7 +3465,7 @@
       <c r="G30" s="142"/>
       <c r="H30" s="142"/>
       <c r="I30" s="142" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="J30" s="142"/>
       <c r="K30" s="142"/>
@@ -3507,7 +3507,7 @@
         <v>169</v>
       </c>
       <c r="C32" s="129" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="D32" s="130">
         <v>1</v>
@@ -3525,7 +3525,7 @@
       <c r="K32" s="131"/>
       <c r="L32" s="131"/>
       <c r="M32" s="138" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="33" spans="1:14" ht="17" x14ac:dyDescent="0.2">
@@ -3534,7 +3534,7 @@
         <v>169</v>
       </c>
       <c r="C33" s="129" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D33" s="130">
         <v>1</v>
@@ -3552,7 +3552,7 @@
       <c r="K33" s="131"/>
       <c r="L33" s="131"/>
       <c r="M33" s="138" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="34" spans="1:14" ht="17" x14ac:dyDescent="0.2">
@@ -3576,7 +3576,7 @@
       <c r="H34" s="14"/>
       <c r="I34" s="16"/>
       <c r="J34" s="14" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="K34" s="14"/>
       <c r="L34" s="14"/>
@@ -3590,7 +3590,7 @@
         <v>169</v>
       </c>
       <c r="C35" s="12" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="D35" s="13">
         <v>1</v>
@@ -3608,7 +3608,7 @@
       <c r="K35" s="14"/>
       <c r="L35" s="14"/>
       <c r="M35" s="112" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="36" spans="1:14" ht="17" x14ac:dyDescent="0.2">
@@ -3617,7 +3617,7 @@
         <v>169</v>
       </c>
       <c r="C36" s="12" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="D36" s="13">
         <v>1</v>
@@ -3635,7 +3635,7 @@
       <c r="K36" s="14"/>
       <c r="L36" s="14"/>
       <c r="M36" s="112" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="37" spans="1:14" ht="17" x14ac:dyDescent="0.2">
@@ -3644,7 +3644,7 @@
         <v>169</v>
       </c>
       <c r="C37" s="12" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="D37" s="13">
         <v>1</v>
@@ -3656,12 +3656,12 @@
         <v>18</v>
       </c>
       <c r="G37" s="14" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="H37" s="14"/>
       <c r="I37" s="16"/>
       <c r="J37" s="14" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="K37" s="14"/>
       <c r="L37" s="14"/>
@@ -3675,7 +3675,7 @@
         <v>169</v>
       </c>
       <c r="C38" s="116" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="D38" s="13">
         <v>1</v>
@@ -3687,12 +3687,12 @@
         <v>18</v>
       </c>
       <c r="G38" s="14" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="H38" s="14"/>
       <c r="I38" s="16"/>
       <c r="J38" s="14" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="K38" s="14"/>
       <c r="L38" s="14"/>
@@ -3706,7 +3706,7 @@
         <v>169</v>
       </c>
       <c r="C39" s="144" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="D39" s="13">
         <v>1</v>
@@ -3718,12 +3718,12 @@
         <v>18</v>
       </c>
       <c r="G39" s="14" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="H39" s="14"/>
       <c r="I39" s="14"/>
       <c r="J39" s="14" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="K39" s="14"/>
       <c r="L39" s="14"/>
@@ -3737,7 +3737,7 @@
         <v>169</v>
       </c>
       <c r="C40" s="12" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="D40" s="13">
         <v>1</v>
@@ -3749,12 +3749,12 @@
         <v>15</v>
       </c>
       <c r="G40" s="14" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="H40" s="14"/>
       <c r="I40" s="14"/>
       <c r="J40" s="14" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="K40" s="14"/>
       <c r="L40" s="14"/>
@@ -3768,7 +3768,7 @@
         <v>169</v>
       </c>
       <c r="C41" s="149" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="D41" s="150">
         <v>1</v>
@@ -3780,12 +3780,12 @@
         <v>15</v>
       </c>
       <c r="G41" s="142" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="H41" s="153"/>
       <c r="I41" s="153"/>
       <c r="J41" s="142" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="K41" s="153"/>
       <c r="L41" s="153"/>
@@ -3797,7 +3797,7 @@
     <row r="42" spans="1:14" s="96" customFormat="1" ht="18" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A42" s="101"/>
       <c r="B42" s="128" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C42" s="145" t="s">
         <v>13</v>
@@ -3825,10 +3825,10 @@
     <row r="43" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A43" s="15"/>
       <c r="B43" s="128" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C43" s="129" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="D43" s="130">
         <v>1</v>
@@ -3846,16 +3846,16 @@
       <c r="K43" s="131"/>
       <c r="L43" s="131"/>
       <c r="M43" s="138" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="44" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A44" s="15"/>
       <c r="B44" s="128" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C44" s="129" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D44" s="130">
         <v>1</v>
@@ -3873,13 +3873,13 @@
       <c r="K44" s="131"/>
       <c r="L44" s="131"/>
       <c r="M44" s="138" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="45" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A45" s="15"/>
       <c r="B45" s="11" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C45" s="12" t="s">
         <v>195</v>
@@ -3897,7 +3897,7 @@
       <c r="H45" s="14"/>
       <c r="I45" s="14"/>
       <c r="J45" s="14" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="K45" s="14"/>
       <c r="L45" s="14"/>
@@ -3908,7 +3908,7 @@
     <row r="46" spans="1:14" s="96" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A46" s="101"/>
       <c r="B46" s="97" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C46" s="102" t="s">
         <v>163</v>
@@ -3926,7 +3926,7 @@
       <c r="H46" s="103"/>
       <c r="I46" s="103"/>
       <c r="J46" s="103" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="K46" s="103"/>
       <c r="L46" s="103"/>
@@ -3938,7 +3938,7 @@
     <row r="47" spans="1:14" s="96" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A47" s="101"/>
       <c r="B47" s="97" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C47" s="102" t="s">
         <v>209</v>
@@ -3956,7 +3956,7 @@
       <c r="H47" s="103"/>
       <c r="I47" s="103"/>
       <c r="J47" s="103" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="K47" s="103" t="s">
         <v>21</v>
@@ -3972,10 +3972,10 @@
     <row r="48" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A48" s="15"/>
       <c r="B48" s="11" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C48" s="12" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="D48" s="13">
         <v>1</v>
@@ -3993,16 +3993,16 @@
       <c r="K48" s="14"/>
       <c r="L48" s="14"/>
       <c r="M48" s="112" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="49" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A49" s="15"/>
       <c r="B49" s="11" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C49" s="12" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="D49" s="13">
         <v>1</v>
@@ -4017,18 +4017,18 @@
       <c r="H49" s="14"/>
       <c r="I49" s="14"/>
       <c r="J49" s="14" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="K49" s="14"/>
       <c r="L49" s="14"/>
       <c r="M49" s="112" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="50" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A50" s="15"/>
       <c r="B50" s="11" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C50" s="12" t="s">
         <v>237</v>
@@ -4046,21 +4046,21 @@
       <c r="H50" s="14"/>
       <c r="I50" s="14"/>
       <c r="J50" s="14" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="K50" s="14"/>
       <c r="L50" s="14"/>
       <c r="M50" s="112" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="51" spans="1:14" s="96" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A51" s="15"/>
       <c r="B51" s="11" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C51" s="12" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="D51" s="13">
         <v>1</v>
@@ -4075,7 +4075,7 @@
       <c r="H51" s="14"/>
       <c r="I51" s="14"/>
       <c r="J51" s="14" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="K51" s="14"/>
       <c r="L51" s="14"/>
@@ -4087,13 +4087,13 @@
     <row r="52" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A52" s="15"/>
       <c r="B52" s="11" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C52" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D52" s="13" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="E52" s="12" t="s">
         <v>14</v>
@@ -4105,21 +4105,21 @@
       <c r="H52" s="14"/>
       <c r="I52" s="14"/>
       <c r="J52" s="14" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="K52" s="14"/>
       <c r="L52" s="14"/>
       <c r="M52" s="118" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="53" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A53" s="96"/>
       <c r="B53" s="11" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C53" s="98" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D53" s="99">
         <v>1</v>
@@ -4131,12 +4131,12 @@
         <v>18</v>
       </c>
       <c r="G53" s="100" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="H53" s="100"/>
       <c r="I53" s="100"/>
       <c r="J53" s="14" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="K53" s="100"/>
       <c r="L53" s="100"/>
@@ -4146,10 +4146,10 @@
     </row>
     <row r="54" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B54" s="11" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C54" s="12" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D54" s="13">
         <v>1</v>
@@ -4161,12 +4161,12 @@
         <v>18</v>
       </c>
       <c r="G54" s="14" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="H54" s="14"/>
       <c r="I54" s="14"/>
       <c r="J54" s="14" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="K54" s="14"/>
       <c r="L54" s="14"/>
@@ -4176,10 +4176,10 @@
     </row>
     <row r="55" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B55" s="11" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C55" s="12" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D55" s="13">
         <v>1</v>
@@ -4191,12 +4191,12 @@
         <v>18</v>
       </c>
       <c r="G55" s="14" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H55" s="14"/>
       <c r="I55" s="14"/>
       <c r="J55" s="14" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="K55" s="14"/>
       <c r="L55" s="14"/>
@@ -4206,10 +4206,10 @@
     </row>
     <row r="56" spans="1:14" s="96" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B56" s="97" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C56" s="102" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D56" s="157">
         <v>1</v>
@@ -4221,12 +4221,12 @@
         <v>18</v>
       </c>
       <c r="G56" s="103" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H56" s="103"/>
       <c r="I56" s="103"/>
       <c r="J56" s="103" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="K56" s="103"/>
       <c r="L56" s="103"/>
@@ -4237,10 +4237,10 @@
     </row>
     <row r="57" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B57" s="11" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C57" s="12" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D57" s="13">
         <v>1</v>
@@ -4266,10 +4266,10 @@
     <row r="58" spans="1:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A58" s="96"/>
       <c r="B58" s="139" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C58" s="140" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="D58" s="141">
         <v>1</v>
@@ -4287,7 +4287,7 @@
       <c r="K58" s="142"/>
       <c r="L58" s="142"/>
       <c r="M58" s="155" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="59" spans="1:14" ht="18" thickTop="1" x14ac:dyDescent="0.2">
@@ -4323,7 +4323,7 @@
         <v>170</v>
       </c>
       <c r="C60" s="129" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="D60" s="130">
         <v>1</v>
@@ -4341,7 +4341,7 @@
       <c r="K60" s="131"/>
       <c r="L60" s="131"/>
       <c r="M60" s="138" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="61" spans="1:14" ht="17" x14ac:dyDescent="0.2">
@@ -4350,7 +4350,7 @@
         <v>170</v>
       </c>
       <c r="C61" s="129" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D61" s="130">
         <v>1</v>
@@ -4368,7 +4368,7 @@
       <c r="K61" s="131"/>
       <c r="L61" s="131"/>
       <c r="M61" s="138" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="62" spans="1:14" x14ac:dyDescent="0.2">
@@ -4391,7 +4391,7 @@
       <c r="H62" s="14"/>
       <c r="I62" s="14"/>
       <c r="J62" s="14" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="K62" s="14"/>
       <c r="L62" s="14"/>
@@ -4419,7 +4419,7 @@
       <c r="H63" s="14"/>
       <c r="I63" s="14"/>
       <c r="J63" s="14" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="K63" s="14"/>
       <c r="L63" s="14"/>
@@ -4432,7 +4432,7 @@
         <v>170</v>
       </c>
       <c r="C64" s="12" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="D64" s="13">
         <v>1</v>
@@ -4450,7 +4450,7 @@
       <c r="K64" s="14"/>
       <c r="L64" s="14"/>
       <c r="M64" s="159" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="65" spans="1:14" x14ac:dyDescent="0.2">
@@ -4458,7 +4458,7 @@
         <v>170</v>
       </c>
       <c r="C65" s="12" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="D65" s="13">
         <v>1</v>
@@ -4473,13 +4473,13 @@
       <c r="H65" s="14"/>
       <c r="I65" s="14"/>
       <c r="J65" s="14" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="K65" s="14" t="s">
         <v>21</v>
       </c>
       <c r="L65" s="14" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="M65" s="111" t="s">
         <v>213</v>
@@ -4505,7 +4505,7 @@
       <c r="H66" s="14"/>
       <c r="I66" s="14"/>
       <c r="J66" s="14" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="K66" s="14"/>
       <c r="L66" s="14"/>
@@ -4518,7 +4518,7 @@
         <v>170</v>
       </c>
       <c r="C67" s="12" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="D67" s="13">
         <v>1</v>
@@ -4530,12 +4530,12 @@
         <v>15</v>
       </c>
       <c r="G67" s="14" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="H67" s="14"/>
       <c r="I67" s="14"/>
       <c r="J67" s="14" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="K67" s="14"/>
       <c r="L67" s="14"/>
@@ -4548,7 +4548,7 @@
         <v>170</v>
       </c>
       <c r="C68" s="12" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="D68" s="13">
         <v>1</v>
@@ -4560,12 +4560,12 @@
         <v>15</v>
       </c>
       <c r="G68" s="14" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="H68" s="14"/>
       <c r="I68" s="14"/>
       <c r="J68" s="14" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="K68" s="14"/>
       <c r="L68" s="14"/>
@@ -4593,7 +4593,7 @@
       <c r="H69" s="103"/>
       <c r="I69" s="103"/>
       <c r="J69" s="103" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="K69" s="103"/>
       <c r="L69" s="103"/>
@@ -4622,7 +4622,7 @@
       <c r="H70" s="14"/>
       <c r="I70" s="14"/>
       <c r="J70" s="14" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="K70" s="14"/>
       <c r="L70" s="14"/>
@@ -4650,7 +4650,7 @@
       <c r="H71" s="14"/>
       <c r="I71" s="14"/>
       <c r="J71" s="14" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="K71" s="14"/>
       <c r="L71" s="14"/>
@@ -4663,7 +4663,7 @@
         <v>170</v>
       </c>
       <c r="C72" s="12" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="D72" s="13">
         <v>1</v>
@@ -4675,12 +4675,12 @@
         <v>15</v>
       </c>
       <c r="G72" s="14" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="H72" s="14"/>
       <c r="I72" s="14"/>
       <c r="J72" s="14" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="K72" s="14"/>
       <c r="L72" s="14"/>
@@ -4693,7 +4693,7 @@
         <v>170</v>
       </c>
       <c r="C73" s="140" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="D73" s="141">
         <v>1</v>
@@ -4705,12 +4705,12 @@
         <v>15</v>
       </c>
       <c r="G73" s="142" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="H73" s="142"/>
       <c r="I73" s="142"/>
       <c r="J73" s="142" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="K73" s="142"/>
       <c r="L73" s="142"/>
@@ -4751,7 +4751,7 @@
         <v>175</v>
       </c>
       <c r="C75" s="129" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="D75" s="130">
         <v>1</v>
@@ -4769,7 +4769,7 @@
       <c r="K75" s="131"/>
       <c r="L75" s="131"/>
       <c r="M75" s="138" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="76" spans="1:14" ht="17" x14ac:dyDescent="0.2">
@@ -4778,7 +4778,7 @@
         <v>175</v>
       </c>
       <c r="C76" s="129" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D76" s="130">
         <v>1</v>
@@ -4796,7 +4796,7 @@
       <c r="K76" s="131"/>
       <c r="L76" s="131"/>
       <c r="M76" s="138" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="77" spans="1:14" x14ac:dyDescent="0.2">
@@ -4820,7 +4820,7 @@
       <c r="H77" s="14"/>
       <c r="I77" s="14"/>
       <c r="J77" s="14" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="K77" s="14"/>
       <c r="L77" s="14"/>
@@ -4848,7 +4848,7 @@
       <c r="H78" s="14"/>
       <c r="I78" s="14"/>
       <c r="J78" s="14" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="K78" s="14"/>
       <c r="L78" s="14"/>
@@ -4863,7 +4863,7 @@
         <v>175</v>
       </c>
       <c r="C79" s="12" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="D79" s="13">
         <v>1</v>
@@ -4877,7 +4877,7 @@
       <c r="G79" s="14"/>
       <c r="H79" s="14"/>
       <c r="I79" s="14" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="J79" s="14"/>
       <c r="K79" s="14"/>
@@ -4892,7 +4892,7 @@
         <v>175</v>
       </c>
       <c r="C80" s="102" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="D80" s="157">
         <v>1</v>
@@ -4907,7 +4907,7 @@
       <c r="H80" s="103"/>
       <c r="I80" s="103"/>
       <c r="J80" s="103" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="K80" s="103" t="s">
         <v>21</v>
@@ -4925,7 +4925,7 @@
         <v>175</v>
       </c>
       <c r="C81" s="12" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="D81" s="13">
         <v>1</v>
@@ -4940,7 +4940,7 @@
       <c r="H81" s="14"/>
       <c r="I81" s="14"/>
       <c r="J81" s="14" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="K81" s="14"/>
       <c r="L81" s="14"/>
@@ -4954,7 +4954,7 @@
         <v>175</v>
       </c>
       <c r="C82" s="140" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="D82" s="141">
         <v>1</v>
@@ -4967,19 +4967,19 @@
       </c>
       <c r="G82" s="142"/>
       <c r="H82" s="142" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="I82" s="142"/>
       <c r="J82" s="142"/>
       <c r="K82" s="142"/>
       <c r="L82" s="142"/>
       <c r="M82" s="160" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="83" spans="1:14" s="96" customFormat="1" ht="18" thickTop="1" x14ac:dyDescent="0.2">
       <c r="B83" s="128" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="C83" s="145" t="s">
         <v>13</v>
@@ -5007,10 +5007,10 @@
     <row r="84" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A84" s="15"/>
       <c r="B84" s="128" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="C84" s="129" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="D84" s="130">
         <v>1</v>
@@ -5028,16 +5028,16 @@
       <c r="K84" s="131"/>
       <c r="L84" s="131"/>
       <c r="M84" s="138" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="85" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A85" s="15"/>
       <c r="B85" s="128" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="C85" s="129" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D85" s="130">
         <v>1</v>
@@ -5055,15 +5055,15 @@
       <c r="K85" s="131"/>
       <c r="L85" s="131"/>
       <c r="M85" s="138" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="86" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B86" s="97" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="C86" s="12" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="D86" s="13">
         <v>1</v>
@@ -5089,10 +5089,10 @@
     <row r="87" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A87" s="96"/>
       <c r="B87" s="97" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="C87" s="102" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="D87" s="157">
         <v>1</v>
@@ -5117,10 +5117,10 @@
     </row>
     <row r="88" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B88" s="97" t="s">
+        <v>286</v>
+      </c>
+      <c r="C88" s="12" t="s">
         <v>287</v>
-      </c>
-      <c r="C88" s="12" t="s">
-        <v>288</v>
       </c>
       <c r="D88" s="13">
         <v>1</v>
@@ -5135,17 +5135,17 @@
       <c r="H88" s="14"/>
       <c r="I88" s="14"/>
       <c r="J88" s="14" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="K88" s="14"/>
       <c r="L88" s="14"/>
       <c r="M88" s="111" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="89" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B89" s="97" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="C89" s="12" t="s">
         <v>177</v>
@@ -5163,7 +5163,7 @@
       <c r="H89" s="14"/>
       <c r="I89" s="14"/>
       <c r="J89" s="14" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="K89" s="14"/>
       <c r="L89" s="14"/>
@@ -5173,10 +5173,10 @@
     </row>
     <row r="90" spans="1:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B90" s="148" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="C90" s="140" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="D90" s="141">
         <v>1</v>
@@ -5189,20 +5189,20 @@
       </c>
       <c r="G90" s="142"/>
       <c r="H90" s="142" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="I90" s="142"/>
       <c r="J90" s="142"/>
       <c r="K90" s="142"/>
       <c r="L90" s="142"/>
       <c r="M90" s="160" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="91" spans="1:14" ht="17" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A91" s="104"/>
       <c r="B91" s="128" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C91" s="145" t="s">
         <v>13</v>
@@ -5229,10 +5229,10 @@
     <row r="92" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A92" s="15"/>
       <c r="B92" s="128" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C92" s="129" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="D92" s="130">
         <v>1</v>
@@ -5250,16 +5250,16 @@
       <c r="K92" s="131"/>
       <c r="L92" s="131"/>
       <c r="M92" s="138" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="93" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A93" s="15"/>
       <c r="B93" s="128" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C93" s="129" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D93" s="130">
         <v>1</v>
@@ -5277,12 +5277,12 @@
       <c r="K93" s="131"/>
       <c r="L93" s="131"/>
       <c r="M93" s="138" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="94" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B94" s="11" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C94" s="12" t="s">
         <v>210</v>
@@ -5300,7 +5300,7 @@
       <c r="H94" s="14"/>
       <c r="I94" s="14"/>
       <c r="J94" s="14" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="K94" s="14"/>
       <c r="L94" s="14"/>
@@ -5310,7 +5310,7 @@
     </row>
     <row r="95" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B95" s="11" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C95" s="12" t="s">
         <v>194</v>
@@ -5328,7 +5328,7 @@
       <c r="H95" s="14"/>
       <c r="I95" s="14"/>
       <c r="J95" s="14" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="K95" s="14"/>
       <c r="L95" s="14"/>
@@ -5338,10 +5338,10 @@
     </row>
     <row r="96" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B96" s="11" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C96" s="12" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="D96" s="13">
         <v>1</v>
@@ -5356,17 +5356,17 @@
       <c r="H96" s="14"/>
       <c r="I96" s="14"/>
       <c r="J96" s="14" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="K96" s="14"/>
       <c r="L96" s="14"/>
       <c r="M96" s="111" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="97" spans="2:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B97" s="123" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C97" s="124" t="s">
         <v>161</v>
@@ -5384,7 +5384,7 @@
       <c r="H97" s="126"/>
       <c r="I97" s="126"/>
       <c r="J97" s="126" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="K97" s="126"/>
       <c r="L97" s="126"/>
@@ -6596,37 +6596,37 @@
       </c>
     </row>
     <row r="47" spans="2:13" x14ac:dyDescent="0.2">
-      <c r="B47" s="174" t="s">
+      <c r="B47" s="171" t="s">
         <v>121</v>
       </c>
-      <c r="C47" s="174"/>
-      <c r="D47" s="174"/>
-      <c r="E47" s="174"/>
-      <c r="F47" s="174"/>
-      <c r="H47" s="175" t="s">
+      <c r="C47" s="171"/>
+      <c r="D47" s="171"/>
+      <c r="E47" s="171"/>
+      <c r="F47" s="171"/>
+      <c r="H47" s="172" t="s">
         <v>122</v>
       </c>
-      <c r="I47" s="175"/>
+      <c r="I47" s="172"/>
     </row>
     <row r="48" spans="2:13" x14ac:dyDescent="0.2">
-      <c r="B48" s="174"/>
-      <c r="C48" s="174"/>
-      <c r="D48" s="174"/>
-      <c r="E48" s="174"/>
-      <c r="F48" s="174"/>
-      <c r="H48" s="175"/>
-      <c r="I48" s="175"/>
+      <c r="B48" s="171"/>
+      <c r="C48" s="171"/>
+      <c r="D48" s="171"/>
+      <c r="E48" s="171"/>
+      <c r="F48" s="171"/>
+      <c r="H48" s="172"/>
+      <c r="I48" s="172"/>
     </row>
     <row r="49" spans="2:9" ht="16" x14ac:dyDescent="0.2">
       <c r="B49" s="68" t="s">
         <v>123</v>
       </c>
-      <c r="C49" s="176" t="s">
+      <c r="C49" s="173" t="s">
         <v>12</v>
       </c>
-      <c r="D49" s="176"/>
-      <c r="E49" s="176"/>
-      <c r="F49" s="176"/>
+      <c r="D49" s="173"/>
+      <c r="E49" s="173"/>
+      <c r="F49" s="173"/>
       <c r="H49" s="69" t="s">
         <v>124</v>
       </c>
@@ -6638,12 +6638,12 @@
       <c r="B50" s="71" t="s">
         <v>1</v>
       </c>
-      <c r="C50" s="177" t="s">
+      <c r="C50" s="174" t="s">
         <v>126</v>
       </c>
-      <c r="D50" s="177"/>
-      <c r="E50" s="177"/>
-      <c r="F50" s="177"/>
+      <c r="D50" s="174"/>
+      <c r="E50" s="174"/>
+      <c r="F50" s="174"/>
       <c r="H50" s="72" t="s">
         <v>48</v>
       </c>
@@ -6655,12 +6655,12 @@
       <c r="B51" s="74" t="s">
         <v>2</v>
       </c>
-      <c r="C51" s="171" t="s">
+      <c r="C51" s="175" t="s">
         <v>128</v>
       </c>
-      <c r="D51" s="171"/>
-      <c r="E51" s="171"/>
-      <c r="F51" s="171"/>
+      <c r="D51" s="175"/>
+      <c r="E51" s="175"/>
+      <c r="F51" s="175"/>
       <c r="H51" s="75" t="s">
         <v>70</v>
       </c>
@@ -6672,12 +6672,12 @@
       <c r="B52" s="74" t="s">
         <v>3</v>
       </c>
-      <c r="C52" s="171" t="s">
+      <c r="C52" s="175" t="s">
         <v>130</v>
       </c>
-      <c r="D52" s="171"/>
-      <c r="E52" s="171"/>
-      <c r="F52" s="171"/>
+      <c r="D52" s="175"/>
+      <c r="E52" s="175"/>
+      <c r="F52" s="175"/>
       <c r="H52" s="77" t="s">
         <v>131</v>
       </c>
@@ -6689,12 +6689,12 @@
       <c r="B53" s="74" t="s">
         <v>4</v>
       </c>
-      <c r="C53" s="173" t="s">
+      <c r="C53" s="176" t="s">
         <v>133</v>
       </c>
-      <c r="D53" s="173"/>
-      <c r="E53" s="173"/>
-      <c r="F53" s="173"/>
+      <c r="D53" s="176"/>
+      <c r="E53" s="176"/>
+      <c r="F53" s="176"/>
       <c r="H53" s="77" t="s">
         <v>81</v>
       </c>
@@ -6706,12 +6706,12 @@
       <c r="B54" s="74" t="s">
         <v>5</v>
       </c>
-      <c r="C54" s="171" t="s">
+      <c r="C54" s="175" t="s">
         <v>135</v>
       </c>
-      <c r="D54" s="171"/>
-      <c r="E54" s="171"/>
-      <c r="F54" s="171"/>
+      <c r="D54" s="175"/>
+      <c r="E54" s="175"/>
+      <c r="F54" s="175"/>
       <c r="H54" s="77" t="s">
         <v>55</v>
       </c>
@@ -6723,12 +6723,12 @@
       <c r="B55" s="74" t="s">
         <v>6</v>
       </c>
-      <c r="C55" s="173" t="s">
+      <c r="C55" s="176" t="s">
         <v>137</v>
       </c>
-      <c r="D55" s="173"/>
-      <c r="E55" s="173"/>
-      <c r="F55" s="173"/>
+      <c r="D55" s="176"/>
+      <c r="E55" s="176"/>
+      <c r="F55" s="176"/>
       <c r="H55" s="79" t="s">
         <v>114</v>
       </c>
@@ -6740,86 +6740,86 @@
       <c r="B56" s="74" t="s">
         <v>7</v>
       </c>
-      <c r="C56" s="171" t="s">
+      <c r="C56" s="175" t="s">
         <v>139</v>
       </c>
-      <c r="D56" s="171"/>
-      <c r="E56" s="171"/>
-      <c r="F56" s="171"/>
+      <c r="D56" s="175"/>
+      <c r="E56" s="175"/>
+      <c r="F56" s="175"/>
     </row>
     <row r="57" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B57" s="74" t="s">
         <v>8</v>
       </c>
-      <c r="C57" s="171" t="s">
+      <c r="C57" s="175" t="s">
         <v>140</v>
       </c>
-      <c r="D57" s="171"/>
-      <c r="E57" s="171"/>
-      <c r="F57" s="171"/>
+      <c r="D57" s="175"/>
+      <c r="E57" s="175"/>
+      <c r="F57" s="175"/>
     </row>
     <row r="58" spans="2:9" ht="45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B58" s="74" t="s">
         <v>9</v>
       </c>
-      <c r="C58" s="171" t="s">
+      <c r="C58" s="175" t="s">
         <v>141</v>
       </c>
-      <c r="D58" s="171"/>
-      <c r="E58" s="171"/>
-      <c r="F58" s="171"/>
+      <c r="D58" s="175"/>
+      <c r="E58" s="175"/>
+      <c r="F58" s="175"/>
     </row>
     <row r="59" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B59" s="74" t="s">
         <v>10</v>
       </c>
-      <c r="C59" s="171" t="s">
+      <c r="C59" s="175" t="s">
         <v>142</v>
       </c>
-      <c r="D59" s="171"/>
-      <c r="E59" s="171"/>
-      <c r="F59" s="171"/>
+      <c r="D59" s="175"/>
+      <c r="E59" s="175"/>
+      <c r="F59" s="175"/>
     </row>
     <row r="60" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B60" s="74" t="s">
         <v>11</v>
       </c>
-      <c r="C60" s="171" t="s">
+      <c r="C60" s="175" t="s">
         <v>143</v>
       </c>
-      <c r="D60" s="171"/>
-      <c r="E60" s="171"/>
-      <c r="F60" s="171"/>
+      <c r="D60" s="175"/>
+      <c r="E60" s="175"/>
+      <c r="F60" s="175"/>
     </row>
     <row r="61" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B61" s="81" t="s">
         <v>12</v>
       </c>
-      <c r="C61" s="172" t="s">
+      <c r="C61" s="177" t="s">
         <v>144</v>
       </c>
-      <c r="D61" s="172"/>
-      <c r="E61" s="172"/>
-      <c r="F61" s="172"/>
+      <c r="D61" s="177"/>
+      <c r="E61" s="177"/>
+      <c r="F61" s="177"/>
     </row>
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="EAttMbwrYpwG6akiV7biz2nw7wlXtTooCxJogsSt7negKq0wKQ9sygPbVeHZ99cgmdNfAtLu9NnPC64y/Uaw7A==" saltValue="FJhchlgDftI44klS+XpFDg==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="15">
+    <mergeCell ref="C57:F57"/>
+    <mergeCell ref="C58:F58"/>
+    <mergeCell ref="C59:F59"/>
+    <mergeCell ref="C60:F60"/>
+    <mergeCell ref="C61:F61"/>
+    <mergeCell ref="C52:F52"/>
+    <mergeCell ref="C53:F53"/>
+    <mergeCell ref="C54:F54"/>
+    <mergeCell ref="C55:F55"/>
+    <mergeCell ref="C56:F56"/>
     <mergeCell ref="B47:F48"/>
     <mergeCell ref="H47:I48"/>
     <mergeCell ref="C49:F49"/>
     <mergeCell ref="C50:F50"/>
     <mergeCell ref="C51:F51"/>
-    <mergeCell ref="C52:F52"/>
-    <mergeCell ref="C53:F53"/>
-    <mergeCell ref="C54:F54"/>
-    <mergeCell ref="C55:F55"/>
-    <mergeCell ref="C56:F56"/>
-    <mergeCell ref="C57:F57"/>
-    <mergeCell ref="C58:F58"/>
-    <mergeCell ref="C59:F59"/>
-    <mergeCell ref="C60:F60"/>
-    <mergeCell ref="C61:F61"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
New row for modelSize
</commit_message>
<xml_diff>
--- a/Schema/DB_scheme.xlsx
+++ b/Schema/DB_scheme.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aksam432/Documents/GitHub/WP3/Schema/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5144DA8-3ECF-6C44-BE35-F374456A1E86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D71973B3-3252-2C4F-A288-93CF822A0E52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38400" yWindow="500" windowWidth="21600" windowHeight="37900" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="894" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="900" uniqueCount="327">
   <si>
     <t>PROJET :</t>
   </si>
@@ -1013,6 +1013,12 @@
   </si>
   <si>
     <t>modelArchitecture</t>
+  </si>
+  <si>
+    <t>modelSize</t>
+  </si>
+  <si>
+    <t>The number of parameters in the model</t>
   </si>
 </sst>
 </file>
@@ -1744,7 +1750,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="178">
+  <cellXfs count="179">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2239,6 +2245,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2675,7 +2684,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:N97"/>
+  <dimension ref="A2:N98"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2.83203125" customWidth="1"/>
@@ -2980,53 +2989,50 @@
       </c>
       <c r="N13" s="167"/>
     </row>
-    <row r="14" spans="2:14" x14ac:dyDescent="0.2">
+    <row r="14" spans="2:14" ht="17" x14ac:dyDescent="0.2">
       <c r="B14" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="C14" s="12" t="s">
-        <v>242</v>
-      </c>
-      <c r="D14" s="13">
-        <v>1</v>
-      </c>
-      <c r="E14" s="12" t="s">
-        <v>58</v>
-      </c>
-      <c r="F14" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="G14" s="14"/>
-      <c r="H14" s="14"/>
-      <c r="I14" s="12"/>
+      <c r="C14" s="93" t="s">
+        <v>325</v>
+      </c>
+      <c r="D14" s="94">
+        <v>1</v>
+      </c>
+      <c r="E14" s="93" t="s">
+        <v>14</v>
+      </c>
+      <c r="F14" s="95" t="s">
+        <v>18</v>
+      </c>
+      <c r="G14" s="95"/>
+      <c r="H14" s="95"/>
+      <c r="I14" s="95"/>
       <c r="J14" s="14" t="s">
         <v>296</v>
       </c>
-      <c r="K14" s="14" t="s">
-        <v>21</v>
-      </c>
-      <c r="L14" s="14" t="s">
-        <v>323</v>
-      </c>
-      <c r="M14" s="111" t="s">
-        <v>178</v>
-      </c>
+      <c r="K14" s="95"/>
+      <c r="L14" s="95"/>
+      <c r="M14" s="113" t="s">
+        <v>326</v>
+      </c>
+      <c r="N14" s="178"/>
     </row>
     <row r="15" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B15" s="11" t="s">
         <v>55</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="D15" s="13">
         <v>1</v>
       </c>
       <c r="E15" s="12" t="s">
-        <v>25</v>
+        <v>58</v>
       </c>
       <c r="F15" s="14" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="G15" s="14"/>
       <c r="H15" s="14"/>
@@ -3034,28 +3040,31 @@
       <c r="J15" s="14" t="s">
         <v>296</v>
       </c>
-      <c r="K15" s="14"/>
-      <c r="L15" s="14"/>
+      <c r="K15" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="L15" s="14" t="s">
+        <v>323</v>
+      </c>
       <c r="M15" s="111" t="s">
-        <v>235</v>
-      </c>
-      <c r="N15" s="167"/>
+        <v>178</v>
+      </c>
     </row>
     <row r="16" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B16" s="11" t="s">
         <v>55</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="D16" s="13">
         <v>1</v>
       </c>
       <c r="E16" s="12" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F16" s="14" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="G16" s="14"/>
       <c r="H16" s="14"/>
@@ -3066,240 +3075,241 @@
       <c r="K16" s="14"/>
       <c r="L16" s="14"/>
       <c r="M16" s="111" t="s">
-        <v>238</v>
-      </c>
-      <c r="N16" s="168"/>
-    </row>
-    <row r="17" spans="1:14" ht="17" x14ac:dyDescent="0.2">
+        <v>235</v>
+      </c>
+      <c r="N16" s="167"/>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B17" s="11" t="s">
         <v>55</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="D17" s="13">
         <v>1</v>
       </c>
       <c r="E17" s="12" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="F17" s="14" t="s">
         <v>18</v>
       </c>
       <c r="G17" s="14"/>
       <c r="H17" s="14"/>
-      <c r="I17" s="14"/>
+      <c r="I17" s="12"/>
       <c r="J17" s="14" t="s">
         <v>296</v>
       </c>
       <c r="K17" s="14"/>
       <c r="L17" s="14"/>
-      <c r="M17" s="112" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="M17" s="111" t="s">
+        <v>238</v>
+      </c>
+      <c r="N17" s="168"/>
+    </row>
+    <row r="18" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="B18" s="11" t="s">
         <v>55</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="D18" s="13">
         <v>1</v>
       </c>
       <c r="E18" s="12" t="s">
-        <v>161</v>
+        <v>14</v>
       </c>
       <c r="F18" s="14" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="G18" s="14"/>
       <c r="H18" s="14"/>
-      <c r="I18" s="12"/>
+      <c r="I18" s="14"/>
       <c r="J18" s="14" t="s">
         <v>296</v>
       </c>
       <c r="K18" s="14"/>
       <c r="L18" s="14"/>
-      <c r="M18" s="111" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="19" spans="1:14" ht="17" x14ac:dyDescent="0.2">
+      <c r="M18" s="112" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B19" s="11" t="s">
         <v>55</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="D19" s="13">
         <v>1</v>
       </c>
       <c r="E19" s="12" t="s">
-        <v>14</v>
+        <v>161</v>
       </c>
       <c r="F19" s="14" t="s">
         <v>15</v>
       </c>
       <c r="G19" s="14"/>
       <c r="H19" s="14"/>
-      <c r="I19" s="14"/>
+      <c r="I19" s="12"/>
       <c r="J19" s="14" t="s">
         <v>296</v>
       </c>
       <c r="K19" s="14"/>
       <c r="L19" s="14"/>
-      <c r="M19" s="114" t="s">
+      <c r="M19" s="111" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" ht="17" x14ac:dyDescent="0.2">
+      <c r="B20" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="C20" s="12" t="s">
+        <v>245</v>
+      </c>
+      <c r="D20" s="13">
+        <v>1</v>
+      </c>
+      <c r="E20" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="F20" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="G20" s="14"/>
+      <c r="H20" s="14"/>
+      <c r="I20" s="14"/>
+      <c r="J20" s="14" t="s">
+        <v>296</v>
+      </c>
+      <c r="K20" s="14"/>
+      <c r="L20" s="14"/>
+      <c r="M20" s="114" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="20" spans="1:14" ht="17" x14ac:dyDescent="0.2">
-      <c r="B20" s="162" t="s">
+    <row r="21" spans="1:14" ht="17" x14ac:dyDescent="0.2">
+      <c r="B21" s="162" t="s">
         <v>55</v>
       </c>
-      <c r="C20" s="163" t="s">
+      <c r="C21" s="163" t="s">
         <v>246</v>
       </c>
-      <c r="D20" s="164">
-        <v>1</v>
-      </c>
-      <c r="E20" s="163" t="s">
+      <c r="D21" s="164">
+        <v>1</v>
+      </c>
+      <c r="E21" s="163" t="s">
         <v>14</v>
       </c>
-      <c r="F20" s="165" t="s">
-        <v>18</v>
-      </c>
-      <c r="G20" s="165"/>
-      <c r="H20" s="165"/>
-      <c r="I20" s="165"/>
-      <c r="J20" s="165"/>
-      <c r="K20" s="165"/>
-      <c r="L20" s="165"/>
-      <c r="M20" s="166" t="s">
+      <c r="F21" s="165" t="s">
+        <v>18</v>
+      </c>
+      <c r="G21" s="165"/>
+      <c r="H21" s="165"/>
+      <c r="I21" s="165"/>
+      <c r="J21" s="165"/>
+      <c r="K21" s="165"/>
+      <c r="L21" s="165"/>
+      <c r="M21" s="166" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="B21" s="11" t="s">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B22" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="C21" s="12" t="s">
+      <c r="C22" s="12" t="s">
         <v>247</v>
       </c>
-      <c r="D21" s="13">
-        <v>1</v>
-      </c>
-      <c r="E21" s="12" t="s">
+      <c r="D22" s="13">
+        <v>1</v>
+      </c>
+      <c r="E22" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="F21" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="G21" s="14"/>
-      <c r="H21" s="14"/>
-      <c r="I21" s="14" t="s">
+      <c r="F22" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="G22" s="14"/>
+      <c r="H22" s="14"/>
+      <c r="I22" s="14" t="s">
         <v>169</v>
       </c>
-      <c r="J21" s="14"/>
-      <c r="K21" s="14"/>
-      <c r="L21" s="14"/>
-      <c r="M21" s="111" t="s">
+      <c r="J22" s="14"/>
+      <c r="K22" s="14"/>
+      <c r="L22" s="14"/>
+      <c r="M22" s="111" t="s">
         <v>182</v>
       </c>
-      <c r="N21" s="167"/>
-    </row>
-    <row r="22" spans="1:14" s="96" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="B22" s="97" t="s">
+      <c r="N22" s="167"/>
+    </row>
+    <row r="23" spans="1:14" s="96" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="B23" s="97" t="s">
         <v>55</v>
       </c>
-      <c r="C22" s="98" t="s">
+      <c r="C23" s="98" t="s">
         <v>248</v>
       </c>
-      <c r="D22" s="99">
-        <v>1</v>
-      </c>
-      <c r="E22" s="98" t="s">
+      <c r="D23" s="99">
+        <v>1</v>
+      </c>
+      <c r="E23" s="98" t="s">
         <v>58</v>
       </c>
-      <c r="F22" s="100" t="s">
+      <c r="F23" s="100" t="s">
         <v>15</v>
       </c>
-      <c r="G22" s="100"/>
-      <c r="H22" s="100"/>
-      <c r="I22" s="100"/>
-      <c r="J22" s="14" t="s">
-        <v>296</v>
-      </c>
-      <c r="K22" s="100" t="s">
-        <v>21</v>
-      </c>
-      <c r="L22" s="105" t="s">
-        <v>293</v>
-      </c>
-      <c r="M22" s="115" t="s">
-        <v>183</v>
-      </c>
-      <c r="N22"/>
-    </row>
-    <row r="23" spans="1:14" ht="17" x14ac:dyDescent="0.2">
-      <c r="B23" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="C23" s="12" t="s">
-        <v>179</v>
-      </c>
-      <c r="D23" s="13">
-        <v>1</v>
-      </c>
-      <c r="E23" s="12" t="s">
-        <v>58</v>
-      </c>
-      <c r="F23" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="G23" s="14"/>
-      <c r="H23" s="14"/>
-      <c r="I23" s="14"/>
+      <c r="G23" s="100"/>
+      <c r="H23" s="100"/>
+      <c r="I23" s="100"/>
       <c r="J23" s="14" t="s">
         <v>296</v>
       </c>
-      <c r="K23" s="14" t="s">
+      <c r="K23" s="100" t="s">
         <v>21</v>
       </c>
-      <c r="L23" s="14" t="s">
-        <v>180</v>
-      </c>
-      <c r="M23" s="112" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="24" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L23" s="105" t="s">
+        <v>293</v>
+      </c>
+      <c r="M23" s="115" t="s">
+        <v>183</v>
+      </c>
+      <c r="N23"/>
+    </row>
+    <row r="24" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="B24" s="11" t="s">
         <v>55</v>
       </c>
       <c r="C24" s="12" t="s">
-        <v>249</v>
+        <v>179</v>
       </c>
       <c r="D24" s="13">
         <v>1</v>
       </c>
       <c r="E24" s="12" t="s">
-        <v>20</v>
+        <v>58</v>
       </c>
       <c r="F24" s="14" t="s">
         <v>18</v>
       </c>
       <c r="G24" s="14"/>
       <c r="H24" s="14"/>
-      <c r="I24" s="14" t="s">
-        <v>294</v>
-      </c>
-      <c r="J24" s="14"/>
-      <c r="K24" s="14"/>
-      <c r="L24" s="14"/>
-      <c r="M24" s="114" t="s">
-        <v>188</v>
+      <c r="I24" s="14"/>
+      <c r="J24" s="14" t="s">
+        <v>296</v>
+      </c>
+      <c r="K24" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="L24" s="14" t="s">
+        <v>180</v>
+      </c>
+      <c r="M24" s="112" t="s">
+        <v>187</v>
       </c>
     </row>
     <row r="25" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -3307,7 +3317,7 @@
         <v>55</v>
       </c>
       <c r="C25" s="12" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="D25" s="13">
         <v>1</v>
@@ -3316,7 +3326,7 @@
         <v>20</v>
       </c>
       <c r="F25" s="14" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="G25" s="14"/>
       <c r="H25" s="14"/>
@@ -3327,15 +3337,15 @@
       <c r="K25" s="14"/>
       <c r="L25" s="14"/>
       <c r="M25" s="114" t="s">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="26" spans="1:14" ht="17" x14ac:dyDescent="0.2">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B26" s="11" t="s">
         <v>55</v>
       </c>
       <c r="C26" s="12" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="D26" s="13">
         <v>1</v>
@@ -3355,7 +3365,7 @@
       <c r="K26" s="14"/>
       <c r="L26" s="14"/>
       <c r="M26" s="114" t="s">
-        <v>189</v>
+        <v>236</v>
       </c>
     </row>
     <row r="27" spans="1:14" ht="17" x14ac:dyDescent="0.2">
@@ -3363,31 +3373,27 @@
         <v>55</v>
       </c>
       <c r="C27" s="12" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="D27" s="13">
         <v>1</v>
       </c>
       <c r="E27" s="12" t="s">
-        <v>58</v>
+        <v>20</v>
       </c>
       <c r="F27" s="14" t="s">
         <v>15</v>
       </c>
       <c r="G27" s="14"/>
       <c r="H27" s="14"/>
-      <c r="I27" s="14"/>
-      <c r="J27" s="14" t="s">
-        <v>296</v>
-      </c>
-      <c r="K27" s="14" t="s">
-        <v>21</v>
-      </c>
-      <c r="L27" s="14" t="s">
-        <v>181</v>
-      </c>
-      <c r="M27" s="112" t="s">
-        <v>190</v>
+      <c r="I27" s="14" t="s">
+        <v>294</v>
+      </c>
+      <c r="J27" s="14"/>
+      <c r="K27" s="14"/>
+      <c r="L27" s="14"/>
+      <c r="M27" s="114" t="s">
+        <v>189</v>
       </c>
     </row>
     <row r="28" spans="1:14" ht="17" x14ac:dyDescent="0.2">
@@ -3395,13 +3401,13 @@
         <v>55</v>
       </c>
       <c r="C28" s="12" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D28" s="13">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="E28" s="12" t="s">
-        <v>14</v>
+        <v>58</v>
       </c>
       <c r="F28" s="14" t="s">
         <v>15</v>
@@ -3412,102 +3418,107 @@
       <c r="J28" s="14" t="s">
         <v>296</v>
       </c>
-      <c r="K28" s="14"/>
-      <c r="L28" s="14"/>
+      <c r="K28" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="L28" s="14" t="s">
+        <v>181</v>
+      </c>
       <c r="M28" s="112" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14" ht="17" x14ac:dyDescent="0.2">
+      <c r="B29" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="C29" s="12" t="s">
+        <v>253</v>
+      </c>
+      <c r="D29" s="13">
+        <v>10</v>
+      </c>
+      <c r="E29" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="F29" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="G29" s="14"/>
+      <c r="H29" s="14"/>
+      <c r="I29" s="14"/>
+      <c r="J29" s="14" t="s">
+        <v>296</v>
+      </c>
+      <c r="K29" s="14"/>
+      <c r="L29" s="14"/>
+      <c r="M29" s="112" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="29" spans="1:14" ht="17" x14ac:dyDescent="0.2">
-      <c r="B29" s="133" t="s">
+    <row r="30" spans="1:14" ht="17" x14ac:dyDescent="0.2">
+      <c r="B30" s="133" t="s">
         <v>55</v>
       </c>
-      <c r="C29" s="134" t="s">
+      <c r="C30" s="134" t="s">
         <v>254</v>
       </c>
-      <c r="D29" s="135">
-        <v>1</v>
-      </c>
-      <c r="E29" s="134" t="s">
+      <c r="D30" s="135">
+        <v>1</v>
+      </c>
+      <c r="E30" s="134" t="s">
         <v>49</v>
       </c>
-      <c r="F29" s="136" t="s">
-        <v>18</v>
-      </c>
-      <c r="G29" s="136"/>
-      <c r="H29" s="136" t="s">
+      <c r="F30" s="136" t="s">
+        <v>18</v>
+      </c>
+      <c r="G30" s="136"/>
+      <c r="H30" s="136" t="s">
         <v>256</v>
       </c>
-      <c r="I29" s="136"/>
-      <c r="J29" s="136"/>
-      <c r="K29" s="136"/>
-      <c r="L29" s="136"/>
-      <c r="M29" s="137" t="s">
+      <c r="I30" s="136"/>
+      <c r="J30" s="136"/>
+      <c r="K30" s="136"/>
+      <c r="L30" s="136"/>
+      <c r="M30" s="137" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="30" spans="1:14" ht="18" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B30" s="139" t="s">
+    <row r="31" spans="1:14" ht="18" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B31" s="139" t="s">
         <v>55</v>
       </c>
-      <c r="C30" s="140" t="s">
+      <c r="C31" s="140" t="s">
         <v>255</v>
       </c>
-      <c r="D30" s="141">
+      <c r="D31" s="141">
         <v>10</v>
       </c>
-      <c r="E30" s="140" t="s">
+      <c r="E31" s="140" t="s">
         <v>20</v>
       </c>
-      <c r="F30" s="142" t="s">
-        <v>18</v>
-      </c>
-      <c r="G30" s="142"/>
-      <c r="H30" s="142"/>
-      <c r="I30" s="142" t="s">
+      <c r="F31" s="142" t="s">
+        <v>18</v>
+      </c>
+      <c r="G31" s="142"/>
+      <c r="H31" s="142"/>
+      <c r="I31" s="142" t="s">
         <v>295</v>
       </c>
-      <c r="J30" s="142"/>
-      <c r="K30" s="142"/>
-      <c r="L30" s="142"/>
-      <c r="M30" s="143" t="s">
+      <c r="J31" s="142"/>
+      <c r="K31" s="142"/>
+      <c r="L31" s="142"/>
+      <c r="M31" s="143" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="31" spans="1:14" ht="18" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="15"/>
-      <c r="B31" s="128" t="s">
-        <v>169</v>
-      </c>
-      <c r="C31" s="129" t="s">
-        <v>13</v>
-      </c>
-      <c r="D31" s="130">
-        <v>1</v>
-      </c>
-      <c r="E31" s="129" t="s">
-        <v>14</v>
-      </c>
-      <c r="F31" s="131" t="s">
-        <v>18</v>
-      </c>
-      <c r="G31" s="131"/>
-      <c r="H31" s="131"/>
-      <c r="I31" s="131"/>
-      <c r="J31" s="131"/>
-      <c r="K31" s="131"/>
-      <c r="L31" s="131"/>
-      <c r="M31" s="138" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="32" spans="1:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:14" ht="18" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A32" s="15"/>
       <c r="B32" s="128" t="s">
         <v>169</v>
       </c>
       <c r="C32" s="129" t="s">
-        <v>297</v>
+        <v>13</v>
       </c>
       <c r="D32" s="130">
         <v>1</v>
@@ -3525,7 +3536,7 @@
       <c r="K32" s="131"/>
       <c r="L32" s="131"/>
       <c r="M32" s="138" t="s">
-        <v>299</v>
+        <v>16</v>
       </c>
     </row>
     <row r="33" spans="1:14" ht="17" x14ac:dyDescent="0.2">
@@ -3534,13 +3545,13 @@
         <v>169</v>
       </c>
       <c r="C33" s="129" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="D33" s="130">
         <v>1</v>
       </c>
       <c r="E33" s="129" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="F33" s="131" t="s">
         <v>18</v>
@@ -3552,36 +3563,34 @@
       <c r="K33" s="131"/>
       <c r="L33" s="131"/>
       <c r="M33" s="138" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="34" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A34" s="15"/>
-      <c r="B34" s="11" t="s">
+      <c r="B34" s="128" t="s">
         <v>169</v>
       </c>
-      <c r="C34" s="12" t="s">
-        <v>163</v>
-      </c>
-      <c r="D34" s="13">
-        <v>1</v>
-      </c>
-      <c r="E34" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="F34" s="14" t="s">
-        <v>15</v>
-      </c>
-      <c r="G34" s="14"/>
-      <c r="H34" s="14"/>
-      <c r="I34" s="16"/>
-      <c r="J34" s="14" t="s">
-        <v>296</v>
-      </c>
-      <c r="K34" s="14"/>
-      <c r="L34" s="14"/>
-      <c r="M34" s="112" t="s">
-        <v>196</v>
+      <c r="C34" s="129" t="s">
+        <v>298</v>
+      </c>
+      <c r="D34" s="130">
+        <v>1</v>
+      </c>
+      <c r="E34" s="129" t="s">
+        <v>19</v>
+      </c>
+      <c r="F34" s="131" t="s">
+        <v>18</v>
+      </c>
+      <c r="G34" s="131"/>
+      <c r="H34" s="131"/>
+      <c r="I34" s="131"/>
+      <c r="J34" s="131"/>
+      <c r="K34" s="131"/>
+      <c r="L34" s="131"/>
+      <c r="M34" s="138" t="s">
+        <v>300</v>
       </c>
     </row>
     <row r="35" spans="1:14" ht="17" x14ac:dyDescent="0.2">
@@ -3590,13 +3599,13 @@
         <v>169</v>
       </c>
       <c r="C35" s="12" t="s">
-        <v>304</v>
+        <v>163</v>
       </c>
       <c r="D35" s="13">
         <v>1</v>
       </c>
       <c r="E35" s="12" t="s">
-        <v>49</v>
+        <v>14</v>
       </c>
       <c r="F35" s="14" t="s">
         <v>15</v>
@@ -3604,11 +3613,13 @@
       <c r="G35" s="14"/>
       <c r="H35" s="14"/>
       <c r="I35" s="16"/>
-      <c r="J35" s="14"/>
+      <c r="J35" s="14" t="s">
+        <v>296</v>
+      </c>
       <c r="K35" s="14"/>
       <c r="L35" s="14"/>
       <c r="M35" s="112" t="s">
-        <v>303</v>
+        <v>196</v>
       </c>
     </row>
     <row r="36" spans="1:14" ht="17" x14ac:dyDescent="0.2">
@@ -3617,13 +3628,13 @@
         <v>169</v>
       </c>
       <c r="C36" s="12" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="D36" s="13">
         <v>1</v>
       </c>
       <c r="E36" s="12" t="s">
-        <v>161</v>
+        <v>49</v>
       </c>
       <c r="F36" s="14" t="s">
         <v>15</v>
@@ -3635,7 +3646,7 @@
       <c r="K36" s="14"/>
       <c r="L36" s="14"/>
       <c r="M36" s="112" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
     </row>
     <row r="37" spans="1:14" ht="17" x14ac:dyDescent="0.2">
@@ -3644,29 +3655,25 @@
         <v>169</v>
       </c>
       <c r="C37" s="12" t="s">
-        <v>257</v>
+        <v>301</v>
       </c>
       <c r="D37" s="13">
         <v>1</v>
       </c>
       <c r="E37" s="12" t="s">
-        <v>22</v>
+        <v>161</v>
       </c>
       <c r="F37" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="G37" s="14" t="s">
-        <v>315</v>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="G37" s="14"/>
       <c r="H37" s="14"/>
       <c r="I37" s="16"/>
-      <c r="J37" s="14" t="s">
-        <v>296</v>
-      </c>
+      <c r="J37" s="14"/>
       <c r="K37" s="14"/>
       <c r="L37" s="14"/>
       <c r="M37" s="112" t="s">
-        <v>197</v>
+        <v>302</v>
       </c>
     </row>
     <row r="38" spans="1:14" ht="17" x14ac:dyDescent="0.2">
@@ -3674,8 +3681,8 @@
       <c r="B38" s="11" t="s">
         <v>169</v>
       </c>
-      <c r="C38" s="116" t="s">
-        <v>258</v>
+      <c r="C38" s="12" t="s">
+        <v>257</v>
       </c>
       <c r="D38" s="13">
         <v>1</v>
@@ -3687,7 +3694,7 @@
         <v>18</v>
       </c>
       <c r="G38" s="14" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="H38" s="14"/>
       <c r="I38" s="16"/>
@@ -3697,7 +3704,7 @@
       <c r="K38" s="14"/>
       <c r="L38" s="14"/>
       <c r="M38" s="112" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="39" spans="1:14" ht="17" x14ac:dyDescent="0.2">
@@ -3705,8 +3712,8 @@
       <c r="B39" s="11" t="s">
         <v>169</v>
       </c>
-      <c r="C39" s="144" t="s">
-        <v>259</v>
+      <c r="C39" s="116" t="s">
+        <v>258</v>
       </c>
       <c r="D39" s="13">
         <v>1</v>
@@ -3721,13 +3728,13 @@
         <v>316</v>
       </c>
       <c r="H39" s="14"/>
-      <c r="I39" s="14"/>
+      <c r="I39" s="16"/>
       <c r="J39" s="14" t="s">
         <v>296</v>
       </c>
       <c r="K39" s="14"/>
       <c r="L39" s="14"/>
-      <c r="M39" s="114" t="s">
+      <c r="M39" s="112" t="s">
         <v>198</v>
       </c>
     </row>
@@ -3736,8 +3743,8 @@
       <c r="B40" s="11" t="s">
         <v>169</v>
       </c>
-      <c r="C40" s="12" t="s">
-        <v>260</v>
+      <c r="C40" s="144" t="s">
+        <v>259</v>
       </c>
       <c r="D40" s="13">
         <v>1</v>
@@ -3746,10 +3753,10 @@
         <v>22</v>
       </c>
       <c r="F40" s="14" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="G40" s="14" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="H40" s="14"/>
       <c r="I40" s="14"/>
@@ -3759,95 +3766,99 @@
       <c r="K40" s="14"/>
       <c r="L40" s="14"/>
       <c r="M40" s="114" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="41" spans="1:14" ht="17" x14ac:dyDescent="0.2">
+      <c r="A41" s="15"/>
+      <c r="B41" s="11" t="s">
+        <v>169</v>
+      </c>
+      <c r="C41" s="12" t="s">
+        <v>260</v>
+      </c>
+      <c r="D41" s="13">
+        <v>1</v>
+      </c>
+      <c r="E41" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="F41" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="G41" s="14" t="s">
+        <v>317</v>
+      </c>
+      <c r="H41" s="14"/>
+      <c r="I41" s="14"/>
+      <c r="J41" s="14" t="s">
+        <v>296</v>
+      </c>
+      <c r="K41" s="14"/>
+      <c r="L41" s="14"/>
+      <c r="M41" s="114" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="41" spans="1:14" s="96" customFormat="1" ht="18" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="101"/>
-      <c r="B41" s="148" t="s">
+    <row r="42" spans="1:14" s="96" customFormat="1" ht="18" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="101"/>
+      <c r="B42" s="148" t="s">
         <v>169</v>
       </c>
-      <c r="C41" s="149" t="s">
+      <c r="C42" s="149" t="s">
         <v>261</v>
       </c>
-      <c r="D41" s="150">
-        <v>1</v>
-      </c>
-      <c r="E41" s="151" t="s">
+      <c r="D42" s="150">
+        <v>1</v>
+      </c>
+      <c r="E42" s="151" t="s">
         <v>22</v>
       </c>
-      <c r="F41" s="152" t="s">
+      <c r="F42" s="152" t="s">
         <v>15</v>
       </c>
-      <c r="G41" s="142" t="s">
+      <c r="G42" s="142" t="s">
         <v>317</v>
       </c>
-      <c r="H41" s="153"/>
-      <c r="I41" s="153"/>
-      <c r="J41" s="142" t="s">
+      <c r="H42" s="153"/>
+      <c r="I42" s="153"/>
+      <c r="J42" s="142" t="s">
         <v>296</v>
       </c>
-      <c r="K41" s="153"/>
-      <c r="L41" s="153"/>
-      <c r="M41" s="154" t="s">
+      <c r="K42" s="153"/>
+      <c r="L42" s="153"/>
+      <c r="M42" s="154" t="s">
         <v>199</v>
       </c>
-      <c r="N41"/>
-    </row>
-    <row r="42" spans="1:14" s="96" customFormat="1" ht="18" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="101"/>
-      <c r="B42" s="128" t="s">
-        <v>294</v>
-      </c>
-      <c r="C42" s="145" t="s">
-        <v>13</v>
-      </c>
-      <c r="D42" s="146">
-        <v>1</v>
-      </c>
-      <c r="E42" s="145" t="s">
-        <v>14</v>
-      </c>
-      <c r="F42" s="147" t="s">
-        <v>18</v>
-      </c>
-      <c r="G42" s="147"/>
-      <c r="H42" s="147"/>
-      <c r="I42" s="147"/>
-      <c r="J42" s="147"/>
-      <c r="K42" s="147"/>
-      <c r="L42" s="147"/>
-      <c r="M42" s="156" t="s">
-        <v>16</v>
-      </c>
       <c r="N42"/>
     </row>
-    <row r="43" spans="1:14" ht="17" x14ac:dyDescent="0.2">
-      <c r="A43" s="15"/>
+    <row r="43" spans="1:14" s="96" customFormat="1" ht="18" thickTop="1" x14ac:dyDescent="0.2">
+      <c r="A43" s="101"/>
       <c r="B43" s="128" t="s">
         <v>294</v>
       </c>
-      <c r="C43" s="129" t="s">
-        <v>297</v>
-      </c>
-      <c r="D43" s="130">
-        <v>1</v>
-      </c>
-      <c r="E43" s="129" t="s">
+      <c r="C43" s="145" t="s">
+        <v>13</v>
+      </c>
+      <c r="D43" s="146">
+        <v>1</v>
+      </c>
+      <c r="E43" s="145" t="s">
         <v>14</v>
       </c>
-      <c r="F43" s="131" t="s">
-        <v>18</v>
-      </c>
-      <c r="G43" s="131"/>
-      <c r="H43" s="131"/>
-      <c r="I43" s="131"/>
-      <c r="J43" s="131"/>
-      <c r="K43" s="131"/>
-      <c r="L43" s="131"/>
-      <c r="M43" s="138" t="s">
-        <v>299</v>
-      </c>
+      <c r="F43" s="147" t="s">
+        <v>18</v>
+      </c>
+      <c r="G43" s="147"/>
+      <c r="H43" s="147"/>
+      <c r="I43" s="147"/>
+      <c r="J43" s="147"/>
+      <c r="K43" s="147"/>
+      <c r="L43" s="147"/>
+      <c r="M43" s="156" t="s">
+        <v>16</v>
+      </c>
+      <c r="N43"/>
     </row>
     <row r="44" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A44" s="15"/>
@@ -3855,13 +3866,13 @@
         <v>294</v>
       </c>
       <c r="C44" s="129" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="D44" s="130">
         <v>1</v>
       </c>
       <c r="E44" s="129" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="F44" s="131" t="s">
         <v>18</v>
@@ -3873,67 +3884,64 @@
       <c r="K44" s="131"/>
       <c r="L44" s="131"/>
       <c r="M44" s="138" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="45" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A45" s="15"/>
-      <c r="B45" s="11" t="s">
+      <c r="B45" s="128" t="s">
         <v>294</v>
       </c>
-      <c r="C45" s="12" t="s">
+      <c r="C45" s="129" t="s">
+        <v>298</v>
+      </c>
+      <c r="D45" s="130">
+        <v>1</v>
+      </c>
+      <c r="E45" s="129" t="s">
+        <v>19</v>
+      </c>
+      <c r="F45" s="131" t="s">
+        <v>18</v>
+      </c>
+      <c r="G45" s="131"/>
+      <c r="H45" s="131"/>
+      <c r="I45" s="131"/>
+      <c r="J45" s="131"/>
+      <c r="K45" s="131"/>
+      <c r="L45" s="131"/>
+      <c r="M45" s="138" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="46" spans="1:14" ht="17" x14ac:dyDescent="0.2">
+      <c r="A46" s="15"/>
+      <c r="B46" s="11" t="s">
+        <v>294</v>
+      </c>
+      <c r="C46" s="12" t="s">
         <v>195</v>
       </c>
-      <c r="D45" s="13">
-        <v>1</v>
-      </c>
-      <c r="E45" s="12" t="s">
+      <c r="D46" s="13">
+        <v>1</v>
+      </c>
+      <c r="E46" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="F45" s="14" t="s">
+      <c r="F46" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="G45" s="14"/>
-      <c r="H45" s="14"/>
-      <c r="I45" s="14"/>
-      <c r="J45" s="14" t="s">
+      <c r="G46" s="14"/>
+      <c r="H46" s="14"/>
+      <c r="I46" s="14"/>
+      <c r="J46" s="14" t="s">
         <v>296</v>
       </c>
-      <c r="K45" s="14"/>
-      <c r="L45" s="14"/>
-      <c r="M45" s="117" t="s">
+      <c r="K46" s="14"/>
+      <c r="L46" s="14"/>
+      <c r="M46" s="117" t="s">
         <v>205</v>
       </c>
-    </row>
-    <row r="46" spans="1:14" s="96" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A46" s="101"/>
-      <c r="B46" s="97" t="s">
-        <v>294</v>
-      </c>
-      <c r="C46" s="102" t="s">
-        <v>163</v>
-      </c>
-      <c r="D46" s="157">
-        <v>1</v>
-      </c>
-      <c r="E46" s="102" t="s">
-        <v>14</v>
-      </c>
-      <c r="F46" s="103" t="s">
-        <v>15</v>
-      </c>
-      <c r="G46" s="103"/>
-      <c r="H46" s="103"/>
-      <c r="I46" s="103"/>
-      <c r="J46" s="103" t="s">
-        <v>296</v>
-      </c>
-      <c r="K46" s="103"/>
-      <c r="L46" s="103"/>
-      <c r="M46" s="158" t="s">
-        <v>206</v>
-      </c>
-      <c r="N46"/>
     </row>
     <row r="47" spans="1:14" s="96" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A47" s="101"/>
@@ -3941,16 +3949,16 @@
         <v>294</v>
       </c>
       <c r="C47" s="102" t="s">
-        <v>209</v>
+        <v>163</v>
       </c>
       <c r="D47" s="157">
         <v>1</v>
       </c>
       <c r="E47" s="102" t="s">
-        <v>58</v>
+        <v>14</v>
       </c>
       <c r="F47" s="103" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="G47" s="103"/>
       <c r="H47" s="103"/>
@@ -3958,43 +3966,46 @@
       <c r="J47" s="103" t="s">
         <v>296</v>
       </c>
-      <c r="K47" s="103" t="s">
+      <c r="K47" s="103"/>
+      <c r="L47" s="103"/>
+      <c r="M47" s="158" t="s">
+        <v>206</v>
+      </c>
+      <c r="N47"/>
+    </row>
+    <row r="48" spans="1:14" s="96" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A48" s="101"/>
+      <c r="B48" s="97" t="s">
+        <v>294</v>
+      </c>
+      <c r="C48" s="102" t="s">
+        <v>209</v>
+      </c>
+      <c r="D48" s="157">
+        <v>1</v>
+      </c>
+      <c r="E48" s="102" t="s">
+        <v>58</v>
+      </c>
+      <c r="F48" s="103" t="s">
+        <v>18</v>
+      </c>
+      <c r="G48" s="103"/>
+      <c r="H48" s="103"/>
+      <c r="I48" s="103"/>
+      <c r="J48" s="103" t="s">
+        <v>296</v>
+      </c>
+      <c r="K48" s="103" t="s">
         <v>21</v>
       </c>
-      <c r="L47" s="103" t="s">
+      <c r="L48" s="103" t="s">
         <v>234</v>
       </c>
-      <c r="M47" s="158" t="s">
+      <c r="M48" s="158" t="s">
         <v>208</v>
       </c>
-      <c r="N47"/>
-    </row>
-    <row r="48" spans="1:14" ht="17" x14ac:dyDescent="0.2">
-      <c r="A48" s="15"/>
-      <c r="B48" s="11" t="s">
-        <v>294</v>
-      </c>
-      <c r="C48" s="12" t="s">
-        <v>282</v>
-      </c>
-      <c r="D48" s="13">
-        <v>1</v>
-      </c>
-      <c r="E48" s="12" t="s">
-        <v>49</v>
-      </c>
-      <c r="F48" s="14" t="s">
-        <v>15</v>
-      </c>
-      <c r="G48" s="14"/>
-      <c r="H48" s="14"/>
-      <c r="I48" s="14"/>
-      <c r="J48" s="14"/>
-      <c r="K48" s="14"/>
-      <c r="L48" s="14"/>
-      <c r="M48" s="112" t="s">
-        <v>307</v>
-      </c>
+      <c r="N48"/>
     </row>
     <row r="49" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A49" s="15"/>
@@ -4002,13 +4013,13 @@
         <v>294</v>
       </c>
       <c r="C49" s="12" t="s">
-        <v>305</v>
+        <v>282</v>
       </c>
       <c r="D49" s="13">
         <v>1</v>
       </c>
       <c r="E49" s="12" t="s">
-        <v>161</v>
+        <v>49</v>
       </c>
       <c r="F49" s="14" t="s">
         <v>15</v>
@@ -4016,13 +4027,11 @@
       <c r="G49" s="14"/>
       <c r="H49" s="14"/>
       <c r="I49" s="14"/>
-      <c r="J49" s="14" t="s">
-        <v>296</v>
-      </c>
+      <c r="J49" s="14"/>
       <c r="K49" s="14"/>
       <c r="L49" s="14"/>
       <c r="M49" s="112" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
     </row>
     <row r="50" spans="1:14" ht="17" x14ac:dyDescent="0.2">
@@ -4031,16 +4040,16 @@
         <v>294</v>
       </c>
       <c r="C50" s="12" t="s">
-        <v>237</v>
+        <v>305</v>
       </c>
       <c r="D50" s="13">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E50" s="12" t="s">
-        <v>14</v>
+        <v>161</v>
       </c>
       <c r="F50" s="14" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="G50" s="14"/>
       <c r="H50" s="14"/>
@@ -4051,22 +4060,22 @@
       <c r="K50" s="14"/>
       <c r="L50" s="14"/>
       <c r="M50" s="112" t="s">
-        <v>308</v>
-      </c>
-    </row>
-    <row r="51" spans="1:14" s="96" customFormat="1" x14ac:dyDescent="0.2">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="51" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A51" s="15"/>
       <c r="B51" s="11" t="s">
         <v>294</v>
       </c>
       <c r="C51" s="12" t="s">
-        <v>262</v>
+        <v>237</v>
       </c>
       <c r="D51" s="13">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E51" s="12" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="F51" s="14" t="s">
         <v>18</v>
@@ -4079,27 +4088,26 @@
       </c>
       <c r="K51" s="14"/>
       <c r="L51" s="14"/>
-      <c r="M51" s="118" t="s">
-        <v>207</v>
-      </c>
-      <c r="N51"/>
-    </row>
-    <row r="52" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="M51" s="112" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="52" spans="1:14" s="96" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A52" s="15"/>
       <c r="B52" s="11" t="s">
         <v>294</v>
       </c>
       <c r="C52" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="D52" s="13" t="s">
-        <v>314</v>
+        <v>262</v>
+      </c>
+      <c r="D52" s="13">
+        <v>1</v>
       </c>
       <c r="E52" s="12" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="F52" s="14" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="G52" s="14"/>
       <c r="H52" s="14"/>
@@ -4110,68 +4118,68 @@
       <c r="K52" s="14"/>
       <c r="L52" s="14"/>
       <c r="M52" s="118" t="s">
-        <v>309</v>
-      </c>
+        <v>207</v>
+      </c>
+      <c r="N52"/>
     </row>
     <row r="53" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A53" s="96"/>
+      <c r="A53" s="15"/>
       <c r="B53" s="11" t="s">
         <v>294</v>
       </c>
-      <c r="C53" s="98" t="s">
-        <v>263</v>
-      </c>
-      <c r="D53" s="99">
-        <v>1</v>
-      </c>
-      <c r="E53" s="98" t="s">
-        <v>22</v>
-      </c>
-      <c r="F53" s="100" t="s">
-        <v>18</v>
-      </c>
-      <c r="G53" s="100" t="s">
-        <v>318</v>
-      </c>
-      <c r="H53" s="100"/>
-      <c r="I53" s="100"/>
+      <c r="C53" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="D53" s="13" t="s">
+        <v>314</v>
+      </c>
+      <c r="E53" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="F53" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="G53" s="14"/>
+      <c r="H53" s="14"/>
+      <c r="I53" s="14"/>
       <c r="J53" s="14" t="s">
         <v>296</v>
       </c>
-      <c r="K53" s="100"/>
-      <c r="L53" s="100"/>
-      <c r="M53" s="119" t="s">
-        <v>200</v>
+      <c r="K53" s="14"/>
+      <c r="L53" s="14"/>
+      <c r="M53" s="118" t="s">
+        <v>309</v>
       </c>
     </row>
     <row r="54" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A54" s="96"/>
       <c r="B54" s="11" t="s">
         <v>294</v>
       </c>
-      <c r="C54" s="12" t="s">
-        <v>264</v>
-      </c>
-      <c r="D54" s="13">
-        <v>1</v>
-      </c>
-      <c r="E54" s="12" t="s">
+      <c r="C54" s="98" t="s">
+        <v>263</v>
+      </c>
+      <c r="D54" s="99">
+        <v>1</v>
+      </c>
+      <c r="E54" s="98" t="s">
         <v>22</v>
       </c>
-      <c r="F54" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="G54" s="14" t="s">
+      <c r="F54" s="100" t="s">
+        <v>18</v>
+      </c>
+      <c r="G54" s="100" t="s">
         <v>318</v>
       </c>
-      <c r="H54" s="14"/>
-      <c r="I54" s="14"/>
+      <c r="H54" s="100"/>
+      <c r="I54" s="100"/>
       <c r="J54" s="14" t="s">
         <v>296</v>
       </c>
-      <c r="K54" s="14"/>
-      <c r="L54" s="14"/>
-      <c r="M54" s="120" t="s">
-        <v>201</v>
+      <c r="K54" s="100"/>
+      <c r="L54" s="100"/>
+      <c r="M54" s="119" t="s">
+        <v>200</v>
       </c>
     </row>
     <row r="55" spans="1:14" x14ac:dyDescent="0.2">
@@ -4179,7 +4187,7 @@
         <v>294</v>
       </c>
       <c r="C55" s="12" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D55" s="13">
         <v>1</v>
@@ -4191,7 +4199,7 @@
         <v>18</v>
       </c>
       <c r="G55" s="14" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="H55" s="14"/>
       <c r="I55" s="14"/>
@@ -4200,148 +4208,151 @@
       </c>
       <c r="K55" s="14"/>
       <c r="L55" s="14"/>
-      <c r="M55" s="111" t="s">
+      <c r="M55" s="120" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="56" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B56" s="11" t="s">
+        <v>294</v>
+      </c>
+      <c r="C56" s="12" t="s">
+        <v>265</v>
+      </c>
+      <c r="D56" s="13">
+        <v>1</v>
+      </c>
+      <c r="E56" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="F56" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="G56" s="14" t="s">
+        <v>319</v>
+      </c>
+      <c r="H56" s="14"/>
+      <c r="I56" s="14"/>
+      <c r="J56" s="14" t="s">
+        <v>296</v>
+      </c>
+      <c r="K56" s="14"/>
+      <c r="L56" s="14"/>
+      <c r="M56" s="111" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="56" spans="1:14" s="96" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B56" s="97" t="s">
+    <row r="57" spans="1:14" s="96" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B57" s="97" t="s">
         <v>294</v>
       </c>
-      <c r="C56" s="102" t="s">
+      <c r="C57" s="102" t="s">
         <v>266</v>
       </c>
-      <c r="D56" s="157">
-        <v>1</v>
-      </c>
-      <c r="E56" s="102" t="s">
+      <c r="D57" s="157">
+        <v>1</v>
+      </c>
+      <c r="E57" s="102" t="s">
         <v>22</v>
       </c>
-      <c r="F56" s="103" t="s">
-        <v>18</v>
-      </c>
-      <c r="G56" s="103" t="s">
+      <c r="F57" s="103" t="s">
+        <v>18</v>
+      </c>
+      <c r="G57" s="103" t="s">
         <v>319</v>
       </c>
-      <c r="H56" s="103"/>
-      <c r="I56" s="103"/>
-      <c r="J56" s="103" t="s">
+      <c r="H57" s="103"/>
+      <c r="I57" s="103"/>
+      <c r="J57" s="103" t="s">
         <v>296</v>
       </c>
-      <c r="K56" s="103"/>
-      <c r="L56" s="103"/>
-      <c r="M56" s="159" t="s">
+      <c r="K57" s="103"/>
+      <c r="L57" s="103"/>
+      <c r="M57" s="159" t="s">
         <v>203</v>
       </c>
-      <c r="N56"/>
-    </row>
-    <row r="57" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="B57" s="11" t="s">
+      <c r="N57"/>
+    </row>
+    <row r="58" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B58" s="11" t="s">
         <v>294</v>
       </c>
-      <c r="C57" s="12" t="s">
+      <c r="C58" s="12" t="s">
         <v>267</v>
       </c>
-      <c r="D57" s="13">
-        <v>1</v>
-      </c>
-      <c r="E57" s="12" t="s">
+      <c r="D58" s="13">
+        <v>1</v>
+      </c>
+      <c r="E58" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="F57" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="G57" s="14"/>
-      <c r="H57" s="14"/>
-      <c r="I57" s="14" t="s">
+      <c r="F58" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="G58" s="14"/>
+      <c r="H58" s="14"/>
+      <c r="I58" s="14" t="s">
         <v>170</v>
       </c>
-      <c r="J57" s="14"/>
-      <c r="K57" s="14"/>
-      <c r="L57" s="14"/>
-      <c r="M57" s="121" t="s">
+      <c r="J58" s="14"/>
+      <c r="K58" s="14"/>
+      <c r="L58" s="14"/>
+      <c r="M58" s="121" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="58" spans="1:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="96"/>
-      <c r="B58" s="139" t="s">
+    <row r="59" spans="1:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A59" s="96"/>
+      <c r="B59" s="139" t="s">
         <v>294</v>
       </c>
-      <c r="C58" s="140" t="s">
+      <c r="C59" s="140" t="s">
         <v>280</v>
       </c>
-      <c r="D58" s="141">
-        <v>1</v>
-      </c>
-      <c r="E58" s="140" t="s">
+      <c r="D59" s="141">
+        <v>1</v>
+      </c>
+      <c r="E59" s="140" t="s">
         <v>49</v>
       </c>
-      <c r="F58" s="142" t="s">
-        <v>18</v>
-      </c>
-      <c r="G58" s="142"/>
-      <c r="H58" s="142"/>
-      <c r="I58" s="142"/>
-      <c r="J58" s="142"/>
-      <c r="K58" s="142"/>
-      <c r="L58" s="142"/>
-      <c r="M58" s="155" t="s">
+      <c r="F59" s="142" t="s">
+        <v>18</v>
+      </c>
+      <c r="G59" s="142"/>
+      <c r="H59" s="142"/>
+      <c r="I59" s="142"/>
+      <c r="J59" s="142"/>
+      <c r="K59" s="142"/>
+      <c r="L59" s="142"/>
+      <c r="M59" s="155" t="s">
         <v>281</v>
       </c>
     </row>
-    <row r="59" spans="1:14" ht="18" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A59" s="101"/>
-      <c r="B59" s="128" t="s">
-        <v>170</v>
-      </c>
-      <c r="C59" s="145" t="s">
-        <v>13</v>
-      </c>
-      <c r="D59" s="146">
-        <v>1</v>
-      </c>
-      <c r="E59" s="145" t="s">
-        <v>14</v>
-      </c>
-      <c r="F59" s="147" t="s">
-        <v>18</v>
-      </c>
-      <c r="G59" s="147"/>
-      <c r="H59" s="147"/>
-      <c r="I59" s="147"/>
-      <c r="J59" s="147"/>
-      <c r="K59" s="147"/>
-      <c r="L59" s="147"/>
-      <c r="M59" s="156" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="60" spans="1:14" ht="17" x14ac:dyDescent="0.2">
-      <c r="A60" s="15"/>
+    <row r="60" spans="1:14" ht="18" thickTop="1" x14ac:dyDescent="0.2">
+      <c r="A60" s="101"/>
       <c r="B60" s="128" t="s">
         <v>170</v>
       </c>
-      <c r="C60" s="129" t="s">
-        <v>297</v>
-      </c>
-      <c r="D60" s="130">
-        <v>1</v>
-      </c>
-      <c r="E60" s="129" t="s">
+      <c r="C60" s="145" t="s">
+        <v>13</v>
+      </c>
+      <c r="D60" s="146">
+        <v>1</v>
+      </c>
+      <c r="E60" s="145" t="s">
         <v>14</v>
       </c>
-      <c r="F60" s="131" t="s">
-        <v>18</v>
-      </c>
-      <c r="G60" s="131"/>
-      <c r="H60" s="131"/>
-      <c r="I60" s="131"/>
-      <c r="J60" s="131"/>
-      <c r="K60" s="131"/>
-      <c r="L60" s="131"/>
-      <c r="M60" s="138" t="s">
-        <v>299</v>
+      <c r="F60" s="147" t="s">
+        <v>18</v>
+      </c>
+      <c r="G60" s="147"/>
+      <c r="H60" s="147"/>
+      <c r="I60" s="147"/>
+      <c r="J60" s="147"/>
+      <c r="K60" s="147"/>
+      <c r="L60" s="147"/>
+      <c r="M60" s="156" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="61" spans="1:14" ht="17" x14ac:dyDescent="0.2">
@@ -4350,13 +4361,13 @@
         <v>170</v>
       </c>
       <c r="C61" s="129" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="D61" s="130">
         <v>1</v>
       </c>
       <c r="E61" s="129" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="F61" s="131" t="s">
         <v>18</v>
@@ -4368,35 +4379,34 @@
       <c r="K61" s="131"/>
       <c r="L61" s="131"/>
       <c r="M61" s="138" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="62" spans="1:14" ht="17" x14ac:dyDescent="0.2">
+      <c r="A62" s="15"/>
+      <c r="B62" s="128" t="s">
+        <v>170</v>
+      </c>
+      <c r="C62" s="129" t="s">
+        <v>298</v>
+      </c>
+      <c r="D62" s="130">
+        <v>1</v>
+      </c>
+      <c r="E62" s="129" t="s">
+        <v>19</v>
+      </c>
+      <c r="F62" s="131" t="s">
+        <v>18</v>
+      </c>
+      <c r="G62" s="131"/>
+      <c r="H62" s="131"/>
+      <c r="I62" s="131"/>
+      <c r="J62" s="131"/>
+      <c r="K62" s="131"/>
+      <c r="L62" s="131"/>
+      <c r="M62" s="138" t="s">
         <v>300</v>
-      </c>
-    </row>
-    <row r="62" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="B62" s="11" t="s">
-        <v>170</v>
-      </c>
-      <c r="C62" s="12" t="s">
-        <v>210</v>
-      </c>
-      <c r="D62" s="13">
-        <v>1</v>
-      </c>
-      <c r="E62" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="F62" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="G62" s="14"/>
-      <c r="H62" s="14"/>
-      <c r="I62" s="14"/>
-      <c r="J62" s="14" t="s">
-        <v>296</v>
-      </c>
-      <c r="K62" s="14"/>
-      <c r="L62" s="14"/>
-      <c r="M62" s="111" t="s">
-        <v>211</v>
       </c>
     </row>
     <row r="63" spans="1:14" x14ac:dyDescent="0.2">
@@ -4404,7 +4414,7 @@
         <v>170</v>
       </c>
       <c r="C63" s="12" t="s">
-        <v>194</v>
+        <v>210</v>
       </c>
       <c r="D63" s="13">
         <v>1</v>
@@ -4423,8 +4433,8 @@
       </c>
       <c r="K63" s="14"/>
       <c r="L63" s="14"/>
-      <c r="M63" s="121" t="s">
-        <v>212</v>
+      <c r="M63" s="111" t="s">
+        <v>211</v>
       </c>
     </row>
     <row r="64" spans="1:14" x14ac:dyDescent="0.2">
@@ -4432,25 +4442,27 @@
         <v>170</v>
       </c>
       <c r="C64" s="12" t="s">
-        <v>283</v>
+        <v>194</v>
       </c>
       <c r="D64" s="13">
         <v>1</v>
       </c>
       <c r="E64" s="12" t="s">
-        <v>49</v>
+        <v>14</v>
       </c>
       <c r="F64" s="14" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="G64" s="14"/>
       <c r="H64" s="14"/>
       <c r="I64" s="14"/>
-      <c r="J64" s="14"/>
+      <c r="J64" s="14" t="s">
+        <v>296</v>
+      </c>
       <c r="K64" s="14"/>
       <c r="L64" s="14"/>
-      <c r="M64" s="159" t="s">
-        <v>285</v>
+      <c r="M64" s="121" t="s">
+        <v>212</v>
       </c>
     </row>
     <row r="65" spans="1:14" x14ac:dyDescent="0.2">
@@ -4458,31 +4470,25 @@
         <v>170</v>
       </c>
       <c r="C65" s="12" t="s">
-        <v>268</v>
+        <v>283</v>
       </c>
       <c r="D65" s="13">
         <v>1</v>
       </c>
       <c r="E65" s="12" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="F65" s="14" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="G65" s="14"/>
       <c r="H65" s="14"/>
       <c r="I65" s="14"/>
-      <c r="J65" s="14" t="s">
-        <v>284</v>
-      </c>
-      <c r="K65" s="14" t="s">
-        <v>21</v>
-      </c>
-      <c r="L65" s="14" t="s">
-        <v>310</v>
-      </c>
-      <c r="M65" s="111" t="s">
-        <v>213</v>
+      <c r="J65" s="14"/>
+      <c r="K65" s="14"/>
+      <c r="L65" s="14"/>
+      <c r="M65" s="159" t="s">
+        <v>285</v>
       </c>
     </row>
     <row r="66" spans="1:14" x14ac:dyDescent="0.2">
@@ -4490,16 +4496,16 @@
         <v>170</v>
       </c>
       <c r="C66" s="12" t="s">
-        <v>171</v>
+        <v>268</v>
       </c>
       <c r="D66" s="13">
         <v>1</v>
       </c>
-      <c r="E66" s="102" t="s">
-        <v>25</v>
+      <c r="E66" s="12" t="s">
+        <v>58</v>
       </c>
       <c r="F66" s="14" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="G66" s="14"/>
       <c r="H66" s="14"/>
@@ -4507,10 +4513,14 @@
       <c r="J66" s="14" t="s">
         <v>284</v>
       </c>
-      <c r="K66" s="14"/>
-      <c r="L66" s="14"/>
-      <c r="M66" s="122" t="s">
-        <v>214</v>
+      <c r="K66" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="L66" s="14" t="s">
+        <v>310</v>
+      </c>
+      <c r="M66" s="111" t="s">
+        <v>213</v>
       </c>
     </row>
     <row r="67" spans="1:14" x14ac:dyDescent="0.2">
@@ -4518,20 +4528,18 @@
         <v>170</v>
       </c>
       <c r="C67" s="12" t="s">
-        <v>269</v>
+        <v>171</v>
       </c>
       <c r="D67" s="13">
         <v>1</v>
       </c>
-      <c r="E67" s="12" t="s">
-        <v>22</v>
+      <c r="E67" s="102" t="s">
+        <v>25</v>
       </c>
       <c r="F67" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="G67" s="14" t="s">
-        <v>320</v>
-      </c>
+      <c r="G67" s="14"/>
       <c r="H67" s="14"/>
       <c r="I67" s="14"/>
       <c r="J67" s="14" t="s">
@@ -4539,8 +4547,8 @@
       </c>
       <c r="K67" s="14"/>
       <c r="L67" s="14"/>
-      <c r="M67" s="111" t="s">
-        <v>215</v>
+      <c r="M67" s="122" t="s">
+        <v>214</v>
       </c>
     </row>
     <row r="68" spans="1:14" x14ac:dyDescent="0.2">
@@ -4548,13 +4556,13 @@
         <v>170</v>
       </c>
       <c r="C68" s="12" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="D68" s="13">
         <v>1</v>
       </c>
       <c r="E68" s="12" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F68" s="14" t="s">
         <v>15</v>
@@ -4569,73 +4577,75 @@
       </c>
       <c r="K68" s="14"/>
       <c r="L68" s="14"/>
-      <c r="M68" s="121" t="s">
+      <c r="M68" s="111" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="69" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B69" s="11" t="s">
+        <v>170</v>
+      </c>
+      <c r="C69" s="12" t="s">
+        <v>270</v>
+      </c>
+      <c r="D69" s="13">
+        <v>1</v>
+      </c>
+      <c r="E69" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="F69" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="G69" s="14" t="s">
+        <v>320</v>
+      </c>
+      <c r="H69" s="14"/>
+      <c r="I69" s="14"/>
+      <c r="J69" s="14" t="s">
+        <v>284</v>
+      </c>
+      <c r="K69" s="14"/>
+      <c r="L69" s="14"/>
+      <c r="M69" s="121" t="s">
         <v>216</v>
       </c>
     </row>
-    <row r="69" spans="1:14" s="96" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B69" s="97" t="s">
+    <row r="70" spans="1:14" s="96" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B70" s="97" t="s">
         <v>170</v>
       </c>
-      <c r="C69" s="102" t="s">
+      <c r="C70" s="102" t="s">
         <v>172</v>
       </c>
-      <c r="D69" s="157">
-        <v>1</v>
-      </c>
-      <c r="E69" s="102" t="s">
-        <v>25</v>
-      </c>
-      <c r="F69" s="103" t="s">
-        <v>15</v>
-      </c>
-      <c r="G69" s="103"/>
-      <c r="H69" s="103"/>
-      <c r="I69" s="103"/>
-      <c r="J69" s="103" t="s">
-        <v>284</v>
-      </c>
-      <c r="K69" s="103"/>
-      <c r="L69" s="103"/>
-      <c r="M69" s="161" t="s">
-        <v>217</v>
-      </c>
-      <c r="N69"/>
-    </row>
-    <row r="70" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="B70" s="11" t="s">
-        <v>170</v>
-      </c>
-      <c r="C70" s="12" t="s">
-        <v>173</v>
-      </c>
-      <c r="D70" s="13">
+      <c r="D70" s="157">
         <v>1</v>
       </c>
       <c r="E70" s="102" t="s">
         <v>25</v>
       </c>
-      <c r="F70" s="14" t="s">
+      <c r="F70" s="103" t="s">
         <v>15</v>
       </c>
-      <c r="G70" s="14"/>
-      <c r="H70" s="14"/>
-      <c r="I70" s="14"/>
-      <c r="J70" s="14" t="s">
+      <c r="G70" s="103"/>
+      <c r="H70" s="103"/>
+      <c r="I70" s="103"/>
+      <c r="J70" s="103" t="s">
         <v>284</v>
       </c>
-      <c r="K70" s="14"/>
-      <c r="L70" s="14"/>
-      <c r="M70" s="121" t="s">
-        <v>220</v>
-      </c>
+      <c r="K70" s="103"/>
+      <c r="L70" s="103"/>
+      <c r="M70" s="161" t="s">
+        <v>217</v>
+      </c>
+      <c r="N70"/>
     </row>
     <row r="71" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B71" s="11" t="s">
         <v>170</v>
       </c>
       <c r="C71" s="12" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D71" s="13">
         <v>1</v>
@@ -4654,8 +4664,8 @@
       </c>
       <c r="K71" s="14"/>
       <c r="L71" s="14"/>
-      <c r="M71" s="111" t="s">
-        <v>221</v>
+      <c r="M71" s="121" t="s">
+        <v>220</v>
       </c>
     </row>
     <row r="72" spans="1:14" x14ac:dyDescent="0.2">
@@ -4663,20 +4673,18 @@
         <v>170</v>
       </c>
       <c r="C72" s="12" t="s">
-        <v>271</v>
+        <v>174</v>
       </c>
       <c r="D72" s="13">
         <v>1</v>
       </c>
-      <c r="E72" s="12" t="s">
-        <v>22</v>
+      <c r="E72" s="102" t="s">
+        <v>25</v>
       </c>
       <c r="F72" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="G72" s="14" t="s">
-        <v>320</v>
-      </c>
+      <c r="G72" s="14"/>
       <c r="H72" s="14"/>
       <c r="I72" s="14"/>
       <c r="J72" s="14" t="s">
@@ -4685,91 +4693,94 @@
       <c r="K72" s="14"/>
       <c r="L72" s="14"/>
       <c r="M72" s="111" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="73" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B73" s="11" t="s">
+        <v>170</v>
+      </c>
+      <c r="C73" s="12" t="s">
+        <v>271</v>
+      </c>
+      <c r="D73" s="13">
+        <v>1</v>
+      </c>
+      <c r="E73" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="F73" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="G73" s="14" t="s">
+        <v>320</v>
+      </c>
+      <c r="H73" s="14"/>
+      <c r="I73" s="14"/>
+      <c r="J73" s="14" t="s">
+        <v>284</v>
+      </c>
+      <c r="K73" s="14"/>
+      <c r="L73" s="14"/>
+      <c r="M73" s="111" t="s">
         <v>218</v>
       </c>
     </row>
-    <row r="73" spans="1:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B73" s="139" t="s">
+    <row r="74" spans="1:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B74" s="139" t="s">
         <v>170</v>
       </c>
-      <c r="C73" s="140" t="s">
+      <c r="C74" s="140" t="s">
         <v>272</v>
       </c>
-      <c r="D73" s="141">
-        <v>1</v>
-      </c>
-      <c r="E73" s="140" t="s">
+      <c r="D74" s="141">
+        <v>1</v>
+      </c>
+      <c r="E74" s="140" t="s">
         <v>22</v>
       </c>
-      <c r="F73" s="142" t="s">
+      <c r="F74" s="142" t="s">
         <v>15</v>
       </c>
-      <c r="G73" s="142" t="s">
+      <c r="G74" s="142" t="s">
         <v>321</v>
       </c>
-      <c r="H73" s="142"/>
-      <c r="I73" s="142"/>
-      <c r="J73" s="142" t="s">
+      <c r="H74" s="142"/>
+      <c r="I74" s="142"/>
+      <c r="J74" s="142" t="s">
         <v>284</v>
       </c>
-      <c r="K73" s="142"/>
-      <c r="L73" s="142"/>
-      <c r="M73" s="160" t="s">
+      <c r="K74" s="142"/>
+      <c r="L74" s="142"/>
+      <c r="M74" s="160" t="s">
         <v>219</v>
       </c>
     </row>
-    <row r="74" spans="1:14" ht="18" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A74" s="96"/>
-      <c r="B74" s="128" t="s">
-        <v>175</v>
-      </c>
-      <c r="C74" s="145" t="s">
-        <v>13</v>
-      </c>
-      <c r="D74" s="146">
-        <v>1</v>
-      </c>
-      <c r="E74" s="145" t="s">
-        <v>14</v>
-      </c>
-      <c r="F74" s="147" t="s">
-        <v>15</v>
-      </c>
-      <c r="G74" s="147"/>
-      <c r="H74" s="147"/>
-      <c r="I74" s="147"/>
-      <c r="J74" s="147"/>
-      <c r="K74" s="147"/>
-      <c r="L74" s="147"/>
-      <c r="M74" s="138" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="75" spans="1:14" ht="17" x14ac:dyDescent="0.2">
-      <c r="A75" s="101"/>
+    <row r="75" spans="1:14" ht="18" thickTop="1" x14ac:dyDescent="0.2">
+      <c r="A75" s="96"/>
       <c r="B75" s="128" t="s">
         <v>175</v>
       </c>
-      <c r="C75" s="129" t="s">
-        <v>297</v>
-      </c>
-      <c r="D75" s="130">
-        <v>1</v>
-      </c>
-      <c r="E75" s="129" t="s">
+      <c r="C75" s="145" t="s">
+        <v>13</v>
+      </c>
+      <c r="D75" s="146">
+        <v>1</v>
+      </c>
+      <c r="E75" s="145" t="s">
         <v>14</v>
       </c>
-      <c r="F75" s="131" t="s">
-        <v>18</v>
-      </c>
-      <c r="G75" s="131"/>
-      <c r="H75" s="131"/>
-      <c r="I75" s="131"/>
-      <c r="J75" s="131"/>
-      <c r="K75" s="131"/>
-      <c r="L75" s="131"/>
+      <c r="F75" s="147" t="s">
+        <v>15</v>
+      </c>
+      <c r="G75" s="147"/>
+      <c r="H75" s="147"/>
+      <c r="I75" s="147"/>
+      <c r="J75" s="147"/>
+      <c r="K75" s="147"/>
+      <c r="L75" s="147"/>
       <c r="M75" s="138" t="s">
-        <v>299</v>
+        <v>16</v>
       </c>
     </row>
     <row r="76" spans="1:14" ht="17" x14ac:dyDescent="0.2">
@@ -4778,13 +4789,13 @@
         <v>175</v>
       </c>
       <c r="C76" s="129" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="D76" s="130">
         <v>1</v>
       </c>
       <c r="E76" s="129" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="F76" s="131" t="s">
         <v>18</v>
@@ -4796,44 +4807,43 @@
       <c r="K76" s="131"/>
       <c r="L76" s="131"/>
       <c r="M76" s="138" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="77" spans="1:14" ht="17" x14ac:dyDescent="0.2">
+      <c r="A77" s="101"/>
+      <c r="B77" s="128" t="s">
+        <v>175</v>
+      </c>
+      <c r="C77" s="129" t="s">
+        <v>298</v>
+      </c>
+      <c r="D77" s="130">
+        <v>1</v>
+      </c>
+      <c r="E77" s="129" t="s">
+        <v>19</v>
+      </c>
+      <c r="F77" s="131" t="s">
+        <v>18</v>
+      </c>
+      <c r="G77" s="131"/>
+      <c r="H77" s="131"/>
+      <c r="I77" s="131"/>
+      <c r="J77" s="131"/>
+      <c r="K77" s="131"/>
+      <c r="L77" s="131"/>
+      <c r="M77" s="138" t="s">
         <v>300</v>
       </c>
     </row>
-    <row r="77" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A77" s="96"/>
-      <c r="B77" s="11" t="s">
-        <v>175</v>
-      </c>
-      <c r="C77" s="12" t="s">
-        <v>176</v>
-      </c>
-      <c r="D77" s="13">
-        <v>1</v>
-      </c>
-      <c r="E77" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="F77" s="14" t="s">
-        <v>15</v>
-      </c>
-      <c r="G77" s="14"/>
-      <c r="H77" s="14"/>
-      <c r="I77" s="14"/>
-      <c r="J77" s="14" t="s">
-        <v>290</v>
-      </c>
-      <c r="K77" s="14"/>
-      <c r="L77" s="14"/>
-      <c r="M77" s="121" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="78" spans="1:14" s="96" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A78" s="96"/>
       <c r="B78" s="11" t="s">
         <v>175</v>
       </c>
       <c r="C78" s="12" t="s">
-        <v>12</v>
+        <v>176</v>
       </c>
       <c r="D78" s="13">
         <v>1</v>
@@ -4852,184 +4862,185 @@
       </c>
       <c r="K78" s="14"/>
       <c r="L78" s="14"/>
-      <c r="M78" s="111" t="s">
-        <v>226</v>
-      </c>
-      <c r="N78"/>
-    </row>
-    <row r="79" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A79" s="96"/>
+      <c r="M78" s="121" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="79" spans="1:14" s="96" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B79" s="11" t="s">
         <v>175</v>
       </c>
       <c r="C79" s="12" t="s">
-        <v>273</v>
+        <v>12</v>
       </c>
       <c r="D79" s="13">
         <v>1</v>
       </c>
       <c r="E79" s="12" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="F79" s="14" t="s">
         <v>15</v>
       </c>
       <c r="G79" s="14"/>
       <c r="H79" s="14"/>
-      <c r="I79" s="14" t="s">
-        <v>295</v>
-      </c>
-      <c r="J79" s="14"/>
+      <c r="I79" s="14"/>
+      <c r="J79" s="14" t="s">
+        <v>290</v>
+      </c>
       <c r="K79" s="14"/>
       <c r="L79" s="14"/>
       <c r="M79" s="111" t="s">
-        <v>227</v>
-      </c>
+        <v>226</v>
+      </c>
+      <c r="N79"/>
     </row>
     <row r="80" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A80" s="96"/>
-      <c r="B80" s="97" t="s">
+      <c r="B80" s="11" t="s">
         <v>175</v>
       </c>
-      <c r="C80" s="102" t="s">
-        <v>274</v>
-      </c>
-      <c r="D80" s="157">
-        <v>1</v>
-      </c>
-      <c r="E80" s="102" t="s">
-        <v>58</v>
-      </c>
-      <c r="F80" s="103" t="s">
+      <c r="C80" s="12" t="s">
+        <v>273</v>
+      </c>
+      <c r="D80" s="13">
+        <v>1</v>
+      </c>
+      <c r="E80" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="F80" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="G80" s="103"/>
-      <c r="H80" s="103"/>
-      <c r="I80" s="103"/>
-      <c r="J80" s="103" t="s">
-        <v>290</v>
-      </c>
-      <c r="K80" s="103" t="s">
-        <v>21</v>
-      </c>
-      <c r="L80" s="103" t="s">
-        <v>233</v>
-      </c>
-      <c r="M80" s="161" t="s">
-        <v>228</v>
+      <c r="G80" s="14"/>
+      <c r="H80" s="14"/>
+      <c r="I80" s="14" t="s">
+        <v>295</v>
+      </c>
+      <c r="J80" s="14"/>
+      <c r="K80" s="14"/>
+      <c r="L80" s="14"/>
+      <c r="M80" s="111" t="s">
+        <v>227</v>
       </c>
     </row>
     <row r="81" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A81" s="96"/>
-      <c r="B81" s="11" t="s">
+      <c r="B81" s="97" t="s">
         <v>175</v>
       </c>
-      <c r="C81" s="12" t="s">
+      <c r="C81" s="102" t="s">
+        <v>274</v>
+      </c>
+      <c r="D81" s="157">
+        <v>1</v>
+      </c>
+      <c r="E81" s="102" t="s">
+        <v>58</v>
+      </c>
+      <c r="F81" s="103" t="s">
+        <v>15</v>
+      </c>
+      <c r="G81" s="103"/>
+      <c r="H81" s="103"/>
+      <c r="I81" s="103"/>
+      <c r="J81" s="103" t="s">
+        <v>290</v>
+      </c>
+      <c r="K81" s="103" t="s">
+        <v>21</v>
+      </c>
+      <c r="L81" s="103" t="s">
+        <v>233</v>
+      </c>
+      <c r="M81" s="161" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="82" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A82" s="96"/>
+      <c r="B82" s="11" t="s">
+        <v>175</v>
+      </c>
+      <c r="C82" s="12" t="s">
         <v>275</v>
       </c>
-      <c r="D81" s="13">
-        <v>1</v>
-      </c>
-      <c r="E81" s="102" t="s">
+      <c r="D82" s="13">
+        <v>1</v>
+      </c>
+      <c r="E82" s="102" t="s">
         <v>25</v>
       </c>
-      <c r="F81" s="14" t="s">
+      <c r="F82" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="G81" s="14"/>
-      <c r="H81" s="14"/>
-      <c r="I81" s="14"/>
-      <c r="J81" s="14" t="s">
+      <c r="G82" s="14"/>
+      <c r="H82" s="14"/>
+      <c r="I82" s="14"/>
+      <c r="J82" s="14" t="s">
         <v>290</v>
       </c>
-      <c r="K81" s="14"/>
-      <c r="L81" s="14"/>
-      <c r="M81" s="121" t="s">
+      <c r="K82" s="14"/>
+      <c r="L82" s="14"/>
+      <c r="M82" s="121" t="s">
         <v>229</v>
       </c>
     </row>
-    <row r="82" spans="1:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A82" s="96"/>
-      <c r="B82" s="139" t="s">
+    <row r="83" spans="1:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A83" s="96"/>
+      <c r="B83" s="139" t="s">
         <v>175</v>
       </c>
-      <c r="C82" s="140" t="s">
+      <c r="C83" s="140" t="s">
         <v>283</v>
       </c>
-      <c r="D82" s="141">
-        <v>1</v>
-      </c>
-      <c r="E82" s="140" t="s">
+      <c r="D83" s="141">
+        <v>1</v>
+      </c>
+      <c r="E83" s="140" t="s">
         <v>49</v>
       </c>
-      <c r="F82" s="142" t="s">
-        <v>18</v>
-      </c>
-      <c r="G82" s="142"/>
-      <c r="H82" s="142" t="s">
+      <c r="F83" s="142" t="s">
+        <v>18</v>
+      </c>
+      <c r="G83" s="142"/>
+      <c r="H83" s="142" t="s">
         <v>289</v>
       </c>
-      <c r="I82" s="142"/>
-      <c r="J82" s="142"/>
-      <c r="K82" s="142"/>
-      <c r="L82" s="142"/>
-      <c r="M82" s="160" t="s">
+      <c r="I83" s="142"/>
+      <c r="J83" s="142"/>
+      <c r="K83" s="142"/>
+      <c r="L83" s="142"/>
+      <c r="M83" s="160" t="s">
         <v>311</v>
       </c>
     </row>
-    <row r="83" spans="1:14" s="96" customFormat="1" ht="18" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="B83" s="128" t="s">
-        <v>286</v>
-      </c>
-      <c r="C83" s="145" t="s">
-        <v>13</v>
-      </c>
-      <c r="D83" s="146">
-        <v>1</v>
-      </c>
-      <c r="E83" s="145" t="s">
-        <v>14</v>
-      </c>
-      <c r="F83" s="147" t="s">
-        <v>15</v>
-      </c>
-      <c r="G83" s="147"/>
-      <c r="H83" s="147"/>
-      <c r="I83" s="147"/>
-      <c r="J83" s="147"/>
-      <c r="K83" s="147"/>
-      <c r="L83" s="147"/>
-      <c r="M83" s="138" t="s">
-        <v>16</v>
-      </c>
-      <c r="N83"/>
-    </row>
-    <row r="84" spans="1:14" ht="17" x14ac:dyDescent="0.2">
-      <c r="A84" s="15"/>
+    <row r="84" spans="1:14" s="96" customFormat="1" ht="18" thickTop="1" x14ac:dyDescent="0.2">
       <c r="B84" s="128" t="s">
         <v>286</v>
       </c>
-      <c r="C84" s="129" t="s">
-        <v>297</v>
-      </c>
-      <c r="D84" s="130">
-        <v>1</v>
-      </c>
-      <c r="E84" s="129" t="s">
+      <c r="C84" s="145" t="s">
+        <v>13</v>
+      </c>
+      <c r="D84" s="146">
+        <v>1</v>
+      </c>
+      <c r="E84" s="145" t="s">
         <v>14</v>
       </c>
-      <c r="F84" s="131" t="s">
-        <v>18</v>
-      </c>
-      <c r="G84" s="131"/>
-      <c r="H84" s="131"/>
-      <c r="I84" s="131"/>
-      <c r="J84" s="131"/>
-      <c r="K84" s="131"/>
-      <c r="L84" s="131"/>
+      <c r="F84" s="147" t="s">
+        <v>15</v>
+      </c>
+      <c r="G84" s="147"/>
+      <c r="H84" s="147"/>
+      <c r="I84" s="147"/>
+      <c r="J84" s="147"/>
+      <c r="K84" s="147"/>
+      <c r="L84" s="147"/>
       <c r="M84" s="138" t="s">
-        <v>299</v>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="N84"/>
     </row>
     <row r="85" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A85" s="15"/>
@@ -5037,13 +5048,13 @@
         <v>286</v>
       </c>
       <c r="C85" s="129" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="D85" s="130">
         <v>1</v>
       </c>
       <c r="E85" s="129" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="F85" s="131" t="s">
         <v>18</v>
@@ -5055,92 +5066,91 @@
       <c r="K85" s="131"/>
       <c r="L85" s="131"/>
       <c r="M85" s="138" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="86" spans="1:14" ht="17" x14ac:dyDescent="0.2">
+      <c r="A86" s="15"/>
+      <c r="B86" s="128" t="s">
+        <v>286</v>
+      </c>
+      <c r="C86" s="129" t="s">
+        <v>298</v>
+      </c>
+      <c r="D86" s="130">
+        <v>1</v>
+      </c>
+      <c r="E86" s="129" t="s">
+        <v>19</v>
+      </c>
+      <c r="F86" s="131" t="s">
+        <v>18</v>
+      </c>
+      <c r="G86" s="131"/>
+      <c r="H86" s="131"/>
+      <c r="I86" s="131"/>
+      <c r="J86" s="131"/>
+      <c r="K86" s="131"/>
+      <c r="L86" s="131"/>
+      <c r="M86" s="138" t="s">
         <v>300</v>
       </c>
     </row>
-    <row r="86" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="B86" s="97" t="s">
-        <v>286</v>
-      </c>
-      <c r="C86" s="12" t="s">
-        <v>276</v>
-      </c>
-      <c r="D86" s="13">
-        <v>1</v>
-      </c>
-      <c r="E86" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="F86" s="14" t="s">
-        <v>15</v>
-      </c>
-      <c r="G86" s="14"/>
-      <c r="H86" s="14"/>
-      <c r="I86" s="14" t="s">
-        <v>55</v>
-      </c>
-      <c r="J86" s="14"/>
-      <c r="K86" s="14"/>
-      <c r="L86" s="14"/>
-      <c r="M86" s="111" t="s">
-        <v>230</v>
-      </c>
-    </row>
     <row r="87" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A87" s="96"/>
       <c r="B87" s="97" t="s">
         <v>286</v>
       </c>
-      <c r="C87" s="102" t="s">
-        <v>277</v>
-      </c>
-      <c r="D87" s="157">
-        <v>1</v>
-      </c>
-      <c r="E87" s="102" t="s">
+      <c r="C87" s="12" t="s">
+        <v>276</v>
+      </c>
+      <c r="D87" s="13">
+        <v>1</v>
+      </c>
+      <c r="E87" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="F87" s="103" t="s">
+      <c r="F87" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="G87" s="103"/>
-      <c r="H87" s="103"/>
-      <c r="I87" s="103" t="s">
-        <v>175</v>
-      </c>
-      <c r="J87" s="103"/>
-      <c r="K87" s="103"/>
-      <c r="L87" s="103"/>
-      <c r="M87" s="161" t="s">
-        <v>231</v>
+      <c r="G87" s="14"/>
+      <c r="H87" s="14"/>
+      <c r="I87" s="14" t="s">
+        <v>55</v>
+      </c>
+      <c r="J87" s="14"/>
+      <c r="K87" s="14"/>
+      <c r="L87" s="14"/>
+      <c r="M87" s="111" t="s">
+        <v>230</v>
       </c>
     </row>
     <row r="88" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A88" s="96"/>
       <c r="B88" s="97" t="s">
         <v>286</v>
       </c>
-      <c r="C88" s="12" t="s">
-        <v>287</v>
-      </c>
-      <c r="D88" s="13">
-        <v>1</v>
-      </c>
-      <c r="E88" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="F88" s="14" t="s">
+      <c r="C88" s="102" t="s">
+        <v>277</v>
+      </c>
+      <c r="D88" s="157">
+        <v>1</v>
+      </c>
+      <c r="E88" s="102" t="s">
+        <v>20</v>
+      </c>
+      <c r="F88" s="103" t="s">
         <v>15</v>
       </c>
-      <c r="G88" s="14"/>
-      <c r="H88" s="14"/>
-      <c r="I88" s="14"/>
-      <c r="J88" s="14" t="s">
-        <v>291</v>
-      </c>
-      <c r="K88" s="14"/>
-      <c r="L88" s="14"/>
-      <c r="M88" s="111" t="s">
-        <v>288</v>
+      <c r="G88" s="103"/>
+      <c r="H88" s="103"/>
+      <c r="I88" s="103" t="s">
+        <v>175</v>
+      </c>
+      <c r="J88" s="103"/>
+      <c r="K88" s="103"/>
+      <c r="L88" s="103"/>
+      <c r="M88" s="161" t="s">
+        <v>231</v>
       </c>
     </row>
     <row r="89" spans="1:14" x14ac:dyDescent="0.2">
@@ -5148,7 +5158,7 @@
         <v>286</v>
       </c>
       <c r="C89" s="12" t="s">
-        <v>177</v>
+        <v>287</v>
       </c>
       <c r="D89" s="13">
         <v>1</v>
@@ -5167,90 +5177,91 @@
       </c>
       <c r="K89" s="14"/>
       <c r="L89" s="14"/>
-      <c r="M89" s="121" t="s">
+      <c r="M89" s="111" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="90" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B90" s="97" t="s">
+        <v>286</v>
+      </c>
+      <c r="C90" s="12" t="s">
+        <v>177</v>
+      </c>
+      <c r="D90" s="13">
+        <v>1</v>
+      </c>
+      <c r="E90" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="F90" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="G90" s="14"/>
+      <c r="H90" s="14"/>
+      <c r="I90" s="14"/>
+      <c r="J90" s="14" t="s">
+        <v>291</v>
+      </c>
+      <c r="K90" s="14"/>
+      <c r="L90" s="14"/>
+      <c r="M90" s="121" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="90" spans="1:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B90" s="148" t="s">
+    <row r="91" spans="1:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B91" s="148" t="s">
         <v>286</v>
       </c>
-      <c r="C90" s="140" t="s">
+      <c r="C91" s="140" t="s">
         <v>283</v>
       </c>
-      <c r="D90" s="141">
-        <v>1</v>
-      </c>
-      <c r="E90" s="140" t="s">
+      <c r="D91" s="141">
+        <v>1</v>
+      </c>
+      <c r="E91" s="140" t="s">
         <v>49</v>
       </c>
-      <c r="F90" s="142" t="s">
-        <v>18</v>
-      </c>
-      <c r="G90" s="142"/>
-      <c r="H90" s="142" t="s">
+      <c r="F91" s="142" t="s">
+        <v>18</v>
+      </c>
+      <c r="G91" s="142"/>
+      <c r="H91" s="142" t="s">
         <v>289</v>
       </c>
-      <c r="I90" s="142"/>
-      <c r="J90" s="142"/>
-      <c r="K90" s="142"/>
-      <c r="L90" s="142"/>
-      <c r="M90" s="160" t="s">
+      <c r="I91" s="142"/>
+      <c r="J91" s="142"/>
+      <c r="K91" s="142"/>
+      <c r="L91" s="142"/>
+      <c r="M91" s="160" t="s">
         <v>312</v>
       </c>
     </row>
-    <row r="91" spans="1:14" ht="17" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A91" s="104"/>
-      <c r="B91" s="128" t="s">
-        <v>295</v>
-      </c>
-      <c r="C91" s="145" t="s">
-        <v>13</v>
-      </c>
-      <c r="D91" s="146">
-        <v>1</v>
-      </c>
-      <c r="E91" s="145" t="s">
-        <v>14</v>
-      </c>
-      <c r="F91" s="147" t="s">
-        <v>15</v>
-      </c>
-      <c r="G91" s="147"/>
-      <c r="H91" s="147"/>
-      <c r="I91" s="147"/>
-      <c r="J91" s="147"/>
-      <c r="K91" s="147"/>
-      <c r="L91" s="147"/>
-      <c r="M91" s="132" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="92" spans="1:14" ht="17" x14ac:dyDescent="0.2">
-      <c r="A92" s="15"/>
+    <row r="92" spans="1:14" ht="17" thickTop="1" x14ac:dyDescent="0.2">
+      <c r="A92" s="104"/>
       <c r="B92" s="128" t="s">
         <v>295</v>
       </c>
-      <c r="C92" s="129" t="s">
-        <v>297</v>
-      </c>
-      <c r="D92" s="130">
-        <v>1</v>
-      </c>
-      <c r="E92" s="129" t="s">
+      <c r="C92" s="145" t="s">
+        <v>13</v>
+      </c>
+      <c r="D92" s="146">
+        <v>1</v>
+      </c>
+      <c r="E92" s="145" t="s">
         <v>14</v>
       </c>
-      <c r="F92" s="131" t="s">
-        <v>18</v>
-      </c>
-      <c r="G92" s="131"/>
-      <c r="H92" s="131"/>
-      <c r="I92" s="131"/>
-      <c r="J92" s="131"/>
-      <c r="K92" s="131"/>
-      <c r="L92" s="131"/>
-      <c r="M92" s="138" t="s">
-        <v>299</v>
+      <c r="F92" s="147" t="s">
+        <v>15</v>
+      </c>
+      <c r="G92" s="147"/>
+      <c r="H92" s="147"/>
+      <c r="I92" s="147"/>
+      <c r="J92" s="147"/>
+      <c r="K92" s="147"/>
+      <c r="L92" s="147"/>
+      <c r="M92" s="132" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="93" spans="1:14" ht="17" x14ac:dyDescent="0.2">
@@ -5259,13 +5270,13 @@
         <v>295</v>
       </c>
       <c r="C93" s="129" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="D93" s="130">
         <v>1</v>
       </c>
       <c r="E93" s="129" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="F93" s="131" t="s">
         <v>18</v>
@@ -5277,35 +5288,34 @@
       <c r="K93" s="131"/>
       <c r="L93" s="131"/>
       <c r="M93" s="138" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="94" spans="1:14" ht="17" x14ac:dyDescent="0.2">
+      <c r="A94" s="15"/>
+      <c r="B94" s="128" t="s">
+        <v>295</v>
+      </c>
+      <c r="C94" s="129" t="s">
+        <v>298</v>
+      </c>
+      <c r="D94" s="130">
+        <v>1</v>
+      </c>
+      <c r="E94" s="129" t="s">
+        <v>19</v>
+      </c>
+      <c r="F94" s="131" t="s">
+        <v>18</v>
+      </c>
+      <c r="G94" s="131"/>
+      <c r="H94" s="131"/>
+      <c r="I94" s="131"/>
+      <c r="J94" s="131"/>
+      <c r="K94" s="131"/>
+      <c r="L94" s="131"/>
+      <c r="M94" s="138" t="s">
         <v>300</v>
-      </c>
-    </row>
-    <row r="94" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="B94" s="11" t="s">
-        <v>295</v>
-      </c>
-      <c r="C94" s="12" t="s">
-        <v>210</v>
-      </c>
-      <c r="D94" s="13">
-        <v>1</v>
-      </c>
-      <c r="E94" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="F94" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="G94" s="14"/>
-      <c r="H94" s="14"/>
-      <c r="I94" s="14"/>
-      <c r="J94" s="14" t="s">
-        <v>296</v>
-      </c>
-      <c r="K94" s="14"/>
-      <c r="L94" s="14"/>
-      <c r="M94" s="111" t="s">
-        <v>222</v>
       </c>
     </row>
     <row r="95" spans="1:14" x14ac:dyDescent="0.2">
@@ -5313,7 +5323,7 @@
         <v>295</v>
       </c>
       <c r="C95" s="12" t="s">
-        <v>194</v>
+        <v>210</v>
       </c>
       <c r="D95" s="13">
         <v>1</v>
@@ -5322,7 +5332,7 @@
         <v>14</v>
       </c>
       <c r="F95" s="14" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="G95" s="14"/>
       <c r="H95" s="14"/>
@@ -5333,7 +5343,7 @@
       <c r="K95" s="14"/>
       <c r="L95" s="14"/>
       <c r="M95" s="111" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="96" spans="1:14" x14ac:dyDescent="0.2">
@@ -5341,7 +5351,7 @@
         <v>295</v>
       </c>
       <c r="C96" s="12" t="s">
-        <v>278</v>
+        <v>194</v>
       </c>
       <c r="D96" s="13">
         <v>1</v>
@@ -5361,34 +5371,62 @@
       <c r="K96" s="14"/>
       <c r="L96" s="14"/>
       <c r="M96" s="111" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="97" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B97" s="11" t="s">
+        <v>295</v>
+      </c>
+      <c r="C97" s="12" t="s">
+        <v>278</v>
+      </c>
+      <c r="D97" s="13">
+        <v>1</v>
+      </c>
+      <c r="E97" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="F97" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="G97" s="14"/>
+      <c r="H97" s="14"/>
+      <c r="I97" s="14"/>
+      <c r="J97" s="14" t="s">
+        <v>296</v>
+      </c>
+      <c r="K97" s="14"/>
+      <c r="L97" s="14"/>
+      <c r="M97" s="111" t="s">
         <v>279</v>
       </c>
     </row>
-    <row r="97" spans="2:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B97" s="123" t="s">
+    <row r="98" spans="2:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B98" s="123" t="s">
         <v>295</v>
       </c>
-      <c r="C97" s="124" t="s">
+      <c r="C98" s="124" t="s">
         <v>161</v>
       </c>
-      <c r="D97" s="125">
-        <v>1</v>
-      </c>
-      <c r="E97" s="124" t="s">
+      <c r="D98" s="125">
+        <v>1</v>
+      </c>
+      <c r="E98" s="124" t="s">
         <v>14</v>
       </c>
-      <c r="F97" s="126" t="s">
+      <c r="F98" s="126" t="s">
         <v>15</v>
       </c>
-      <c r="G97" s="126"/>
-      <c r="H97" s="126"/>
-      <c r="I97" s="126"/>
-      <c r="J97" s="126" t="s">
+      <c r="G98" s="126"/>
+      <c r="H98" s="126"/>
+      <c r="I98" s="126"/>
+      <c r="J98" s="126" t="s">
         <v>296</v>
       </c>
-      <c r="K97" s="126"/>
-      <c r="L97" s="126"/>
-      <c r="M97" s="127" t="s">
+      <c r="K98" s="126"/>
+      <c r="L98" s="126"/>
+      <c r="M98" s="127" t="s">
         <v>224</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Pretrained changed to pretrainedVersion
</commit_message>
<xml_diff>
--- a/Schema/DB_scheme.xlsx
+++ b/Schema/DB_scheme.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aksam432/Documents/GitHub/WP3/Schema/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D71973B3-3252-2C4F-A288-93CF822A0E52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFD1274B-58E3-694E-96A8-5B8913019332}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38400" yWindow="500" windowWidth="21600" windowHeight="37900" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -745,9 +745,6 @@
     <t>["training","test","val"]</t>
   </si>
   <si>
-    <t>The category of pre-trained model ( type &amp; size )</t>
-  </si>
-  <si>
     <t>The test set details</t>
   </si>
   <si>
@@ -757,9 +754,6 @@
     <t>The model has electrostatics taken into account</t>
   </si>
   <si>
-    <t>pretrained</t>
-  </si>
-  <si>
     <t>noOfElements</t>
   </si>
   <si>
@@ -1019,6 +1013,12 @@
   </si>
   <si>
     <t>The number of parameters in the model</t>
+  </si>
+  <si>
+    <t>pretrainedVersion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The name of the parent model on which finetuned </t>
   </si>
 </sst>
 </file>
@@ -2711,7 +2711,7 @@
       </c>
       <c r="C2" s="169"/>
       <c r="D2" s="170" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="E2" s="170"/>
       <c r="F2" s="170"/>
@@ -2792,7 +2792,7 @@
         <v>55</v>
       </c>
       <c r="C7" s="129" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="D7" s="130">
         <v>1</v>
@@ -2810,7 +2810,7 @@
       <c r="K7" s="131"/>
       <c r="L7" s="131"/>
       <c r="M7" s="132" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
     </row>
     <row r="8" spans="2:14" x14ac:dyDescent="0.2">
@@ -2818,7 +2818,7 @@
         <v>55</v>
       </c>
       <c r="C8" s="129" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="D8" s="130">
         <v>1</v>
@@ -2836,7 +2836,7 @@
       <c r="K8" s="131"/>
       <c r="L8" s="131"/>
       <c r="M8" s="132" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
     </row>
     <row r="9" spans="2:14" x14ac:dyDescent="0.2">
@@ -2859,7 +2859,7 @@
       <c r="H9" s="14"/>
       <c r="I9" s="14"/>
       <c r="J9" s="14" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="K9" s="14"/>
       <c r="L9" s="14"/>
@@ -2887,7 +2887,7 @@
       <c r="H10" s="14"/>
       <c r="I10" s="14"/>
       <c r="J10" s="14" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="K10" s="14"/>
       <c r="L10" s="14"/>
@@ -2915,13 +2915,13 @@
       <c r="H11" s="14"/>
       <c r="I11" s="14"/>
       <c r="J11" s="14" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="K11" s="14" t="s">
         <v>21</v>
       </c>
       <c r="L11" s="14" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="M11" s="112" t="s">
         <v>165</v>
@@ -2933,7 +2933,7 @@
         <v>55</v>
       </c>
       <c r="C12" s="93" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="D12" s="94">
         <v>1</v>
@@ -2948,7 +2948,7 @@
       <c r="H12" s="95"/>
       <c r="I12" s="95"/>
       <c r="J12" s="14" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="K12" s="95"/>
       <c r="L12" s="95"/>
@@ -2961,7 +2961,7 @@
         <v>55</v>
       </c>
       <c r="C13" s="93" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="D13" s="94">
         <v>1</v>
@@ -2976,13 +2976,13 @@
       <c r="H13" s="95"/>
       <c r="I13" s="95"/>
       <c r="J13" s="14" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="K13" s="95" t="s">
         <v>21</v>
       </c>
       <c r="L13" s="95" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="M13" s="113" t="s">
         <v>184</v>
@@ -2994,7 +2994,7 @@
         <v>55</v>
       </c>
       <c r="C14" s="93" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="D14" s="94">
         <v>1</v>
@@ -3009,12 +3009,12 @@
       <c r="H14" s="95"/>
       <c r="I14" s="95"/>
       <c r="J14" s="14" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="K14" s="95"/>
       <c r="L14" s="95"/>
       <c r="M14" s="113" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="N14" s="178"/>
     </row>
@@ -3023,7 +3023,7 @@
         <v>55</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="D15" s="13">
         <v>1</v>
@@ -3038,13 +3038,13 @@
       <c r="H15" s="14"/>
       <c r="I15" s="12"/>
       <c r="J15" s="14" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="K15" s="14" t="s">
         <v>21</v>
       </c>
       <c r="L15" s="14" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="M15" s="111" t="s">
         <v>178</v>
@@ -3055,13 +3055,13 @@
         <v>55</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>239</v>
+        <v>325</v>
       </c>
       <c r="D16" s="13">
         <v>1</v>
       </c>
       <c r="E16" s="12" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="F16" s="14" t="s">
         <v>15</v>
@@ -3070,12 +3070,12 @@
       <c r="H16" s="14"/>
       <c r="I16" s="12"/>
       <c r="J16" s="14" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="K16" s="14"/>
       <c r="L16" s="14"/>
       <c r="M16" s="111" t="s">
-        <v>235</v>
+        <v>326</v>
       </c>
       <c r="N16" s="167"/>
     </row>
@@ -3084,7 +3084,7 @@
         <v>55</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="D17" s="13">
         <v>1</v>
@@ -3099,12 +3099,12 @@
       <c r="H17" s="14"/>
       <c r="I17" s="12"/>
       <c r="J17" s="14" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="K17" s="14"/>
       <c r="L17" s="14"/>
       <c r="M17" s="111" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="N17" s="168"/>
     </row>
@@ -3113,7 +3113,7 @@
         <v>55</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="D18" s="13">
         <v>1</v>
@@ -3128,7 +3128,7 @@
       <c r="H18" s="14"/>
       <c r="I18" s="14"/>
       <c r="J18" s="14" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="K18" s="14"/>
       <c r="L18" s="14"/>
@@ -3141,7 +3141,7 @@
         <v>55</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="D19" s="13">
         <v>1</v>
@@ -3156,7 +3156,7 @@
       <c r="H19" s="14"/>
       <c r="I19" s="12"/>
       <c r="J19" s="14" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="K19" s="14"/>
       <c r="L19" s="14"/>
@@ -3169,7 +3169,7 @@
         <v>55</v>
       </c>
       <c r="C20" s="12" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="D20" s="13">
         <v>1</v>
@@ -3184,7 +3184,7 @@
       <c r="H20" s="14"/>
       <c r="I20" s="14"/>
       <c r="J20" s="14" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="K20" s="14"/>
       <c r="L20" s="14"/>
@@ -3197,7 +3197,7 @@
         <v>55</v>
       </c>
       <c r="C21" s="163" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="D21" s="164">
         <v>1</v>
@@ -3223,7 +3223,7 @@
         <v>55</v>
       </c>
       <c r="C22" s="12" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="D22" s="13">
         <v>1</v>
@@ -3252,7 +3252,7 @@
         <v>55</v>
       </c>
       <c r="C23" s="98" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="D23" s="99">
         <v>1</v>
@@ -3267,13 +3267,13 @@
       <c r="H23" s="100"/>
       <c r="I23" s="100"/>
       <c r="J23" s="14" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="K23" s="100" t="s">
         <v>21</v>
       </c>
       <c r="L23" s="105" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="M23" s="115" t="s">
         <v>183</v>
@@ -3300,7 +3300,7 @@
       <c r="H24" s="14"/>
       <c r="I24" s="14"/>
       <c r="J24" s="14" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="K24" s="14" t="s">
         <v>21</v>
@@ -3317,7 +3317,7 @@
         <v>55</v>
       </c>
       <c r="C25" s="12" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="D25" s="13">
         <v>1</v>
@@ -3331,7 +3331,7 @@
       <c r="G25" s="14"/>
       <c r="H25" s="14"/>
       <c r="I25" s="14" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="J25" s="14"/>
       <c r="K25" s="14"/>
@@ -3345,7 +3345,7 @@
         <v>55</v>
       </c>
       <c r="C26" s="12" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="D26" s="13">
         <v>1</v>
@@ -3359,13 +3359,13 @@
       <c r="G26" s="14"/>
       <c r="H26" s="14"/>
       <c r="I26" s="14" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="J26" s="14"/>
       <c r="K26" s="14"/>
       <c r="L26" s="14"/>
       <c r="M26" s="114" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="27" spans="1:14" ht="17" x14ac:dyDescent="0.2">
@@ -3373,7 +3373,7 @@
         <v>55</v>
       </c>
       <c r="C27" s="12" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="D27" s="13">
         <v>1</v>
@@ -3387,7 +3387,7 @@
       <c r="G27" s="14"/>
       <c r="H27" s="14"/>
       <c r="I27" s="14" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="J27" s="14"/>
       <c r="K27" s="14"/>
@@ -3401,7 +3401,7 @@
         <v>55</v>
       </c>
       <c r="C28" s="12" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="D28" s="13">
         <v>1</v>
@@ -3416,7 +3416,7 @@
       <c r="H28" s="14"/>
       <c r="I28" s="14"/>
       <c r="J28" s="14" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="K28" s="14" t="s">
         <v>21</v>
@@ -3433,7 +3433,7 @@
         <v>55</v>
       </c>
       <c r="C29" s="12" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="D29" s="13">
         <v>10</v>
@@ -3448,7 +3448,7 @@
       <c r="H29" s="14"/>
       <c r="I29" s="14"/>
       <c r="J29" s="14" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="K29" s="14"/>
       <c r="L29" s="14"/>
@@ -3461,7 +3461,7 @@
         <v>55</v>
       </c>
       <c r="C30" s="134" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="D30" s="135">
         <v>1</v>
@@ -3474,7 +3474,7 @@
       </c>
       <c r="G30" s="136"/>
       <c r="H30" s="136" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="I30" s="136"/>
       <c r="J30" s="136"/>
@@ -3489,7 +3489,7 @@
         <v>55</v>
       </c>
       <c r="C31" s="140" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="D31" s="141">
         <v>10</v>
@@ -3503,7 +3503,7 @@
       <c r="G31" s="142"/>
       <c r="H31" s="142"/>
       <c r="I31" s="142" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="J31" s="142"/>
       <c r="K31" s="142"/>
@@ -3545,7 +3545,7 @@
         <v>169</v>
       </c>
       <c r="C33" s="129" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="D33" s="130">
         <v>1</v>
@@ -3563,7 +3563,7 @@
       <c r="K33" s="131"/>
       <c r="L33" s="131"/>
       <c r="M33" s="138" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
     </row>
     <row r="34" spans="1:14" ht="17" x14ac:dyDescent="0.2">
@@ -3572,7 +3572,7 @@
         <v>169</v>
       </c>
       <c r="C34" s="129" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="D34" s="130">
         <v>1</v>
@@ -3590,7 +3590,7 @@
       <c r="K34" s="131"/>
       <c r="L34" s="131"/>
       <c r="M34" s="138" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
     </row>
     <row r="35" spans="1:14" ht="17" x14ac:dyDescent="0.2">
@@ -3614,7 +3614,7 @@
       <c r="H35" s="14"/>
       <c r="I35" s="16"/>
       <c r="J35" s="14" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="K35" s="14"/>
       <c r="L35" s="14"/>
@@ -3628,7 +3628,7 @@
         <v>169</v>
       </c>
       <c r="C36" s="12" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="D36" s="13">
         <v>1</v>
@@ -3646,7 +3646,7 @@
       <c r="K36" s="14"/>
       <c r="L36" s="14"/>
       <c r="M36" s="112" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
     </row>
     <row r="37" spans="1:14" ht="17" x14ac:dyDescent="0.2">
@@ -3655,7 +3655,7 @@
         <v>169</v>
       </c>
       <c r="C37" s="12" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="D37" s="13">
         <v>1</v>
@@ -3673,7 +3673,7 @@
       <c r="K37" s="14"/>
       <c r="L37" s="14"/>
       <c r="M37" s="112" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
     </row>
     <row r="38" spans="1:14" ht="17" x14ac:dyDescent="0.2">
@@ -3682,7 +3682,7 @@
         <v>169</v>
       </c>
       <c r="C38" s="12" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="D38" s="13">
         <v>1</v>
@@ -3694,12 +3694,12 @@
         <v>18</v>
       </c>
       <c r="G38" s="14" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="H38" s="14"/>
       <c r="I38" s="16"/>
       <c r="J38" s="14" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="K38" s="14"/>
       <c r="L38" s="14"/>
@@ -3713,7 +3713,7 @@
         <v>169</v>
       </c>
       <c r="C39" s="116" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="D39" s="13">
         <v>1</v>
@@ -3725,12 +3725,12 @@
         <v>18</v>
       </c>
       <c r="G39" s="14" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="H39" s="14"/>
       <c r="I39" s="16"/>
       <c r="J39" s="14" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="K39" s="14"/>
       <c r="L39" s="14"/>
@@ -3744,7 +3744,7 @@
         <v>169</v>
       </c>
       <c r="C40" s="144" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="D40" s="13">
         <v>1</v>
@@ -3756,12 +3756,12 @@
         <v>18</v>
       </c>
       <c r="G40" s="14" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="H40" s="14"/>
       <c r="I40" s="14"/>
       <c r="J40" s="14" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="K40" s="14"/>
       <c r="L40" s="14"/>
@@ -3775,7 +3775,7 @@
         <v>169</v>
       </c>
       <c r="C41" s="12" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="D41" s="13">
         <v>1</v>
@@ -3787,12 +3787,12 @@
         <v>15</v>
       </c>
       <c r="G41" s="14" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="H41" s="14"/>
       <c r="I41" s="14"/>
       <c r="J41" s="14" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="K41" s="14"/>
       <c r="L41" s="14"/>
@@ -3806,7 +3806,7 @@
         <v>169</v>
       </c>
       <c r="C42" s="149" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="D42" s="150">
         <v>1</v>
@@ -3818,12 +3818,12 @@
         <v>15</v>
       </c>
       <c r="G42" s="142" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="H42" s="153"/>
       <c r="I42" s="153"/>
       <c r="J42" s="142" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="K42" s="153"/>
       <c r="L42" s="153"/>
@@ -3835,7 +3835,7 @@
     <row r="43" spans="1:14" s="96" customFormat="1" ht="18" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A43" s="101"/>
       <c r="B43" s="128" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="C43" s="145" t="s">
         <v>13</v>
@@ -3863,10 +3863,10 @@
     <row r="44" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A44" s="15"/>
       <c r="B44" s="128" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="C44" s="129" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="D44" s="130">
         <v>1</v>
@@ -3884,16 +3884,16 @@
       <c r="K44" s="131"/>
       <c r="L44" s="131"/>
       <c r="M44" s="138" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
     </row>
     <row r="45" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A45" s="15"/>
       <c r="B45" s="128" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="C45" s="129" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="D45" s="130">
         <v>1</v>
@@ -3911,13 +3911,13 @@
       <c r="K45" s="131"/>
       <c r="L45" s="131"/>
       <c r="M45" s="138" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
     </row>
     <row r="46" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A46" s="15"/>
       <c r="B46" s="11" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="C46" s="12" t="s">
         <v>195</v>
@@ -3935,7 +3935,7 @@
       <c r="H46" s="14"/>
       <c r="I46" s="14"/>
       <c r="J46" s="14" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="K46" s="14"/>
       <c r="L46" s="14"/>
@@ -3946,7 +3946,7 @@
     <row r="47" spans="1:14" s="96" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A47" s="101"/>
       <c r="B47" s="97" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="C47" s="102" t="s">
         <v>163</v>
@@ -3964,7 +3964,7 @@
       <c r="H47" s="103"/>
       <c r="I47" s="103"/>
       <c r="J47" s="103" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="K47" s="103"/>
       <c r="L47" s="103"/>
@@ -3976,7 +3976,7 @@
     <row r="48" spans="1:14" s="96" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A48" s="101"/>
       <c r="B48" s="97" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="C48" s="102" t="s">
         <v>209</v>
@@ -3994,7 +3994,7 @@
       <c r="H48" s="103"/>
       <c r="I48" s="103"/>
       <c r="J48" s="103" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="K48" s="103" t="s">
         <v>21</v>
@@ -4010,10 +4010,10 @@
     <row r="49" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A49" s="15"/>
       <c r="B49" s="11" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="C49" s="12" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="D49" s="13">
         <v>1</v>
@@ -4031,16 +4031,16 @@
       <c r="K49" s="14"/>
       <c r="L49" s="14"/>
       <c r="M49" s="112" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
     </row>
     <row r="50" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A50" s="15"/>
       <c r="B50" s="11" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="C50" s="12" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="D50" s="13">
         <v>1</v>
@@ -4055,21 +4055,21 @@
       <c r="H50" s="14"/>
       <c r="I50" s="14"/>
       <c r="J50" s="14" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="K50" s="14"/>
       <c r="L50" s="14"/>
       <c r="M50" s="112" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
     </row>
     <row r="51" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A51" s="15"/>
       <c r="B51" s="11" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="C51" s="12" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="D51" s="13">
         <v>5</v>
@@ -4084,21 +4084,21 @@
       <c r="H51" s="14"/>
       <c r="I51" s="14"/>
       <c r="J51" s="14" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="K51" s="14"/>
       <c r="L51" s="14"/>
       <c r="M51" s="112" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
     </row>
     <row r="52" spans="1:14" s="96" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A52" s="15"/>
       <c r="B52" s="11" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="C52" s="12" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="D52" s="13">
         <v>1</v>
@@ -4113,7 +4113,7 @@
       <c r="H52" s="14"/>
       <c r="I52" s="14"/>
       <c r="J52" s="14" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="K52" s="14"/>
       <c r="L52" s="14"/>
@@ -4125,13 +4125,13 @@
     <row r="53" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A53" s="15"/>
       <c r="B53" s="11" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="C53" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D53" s="13" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="E53" s="12" t="s">
         <v>14</v>
@@ -4143,21 +4143,21 @@
       <c r="H53" s="14"/>
       <c r="I53" s="14"/>
       <c r="J53" s="14" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="K53" s="14"/>
       <c r="L53" s="14"/>
       <c r="M53" s="118" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="54" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A54" s="96"/>
       <c r="B54" s="11" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="C54" s="98" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="D54" s="99">
         <v>1</v>
@@ -4169,12 +4169,12 @@
         <v>18</v>
       </c>
       <c r="G54" s="100" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="H54" s="100"/>
       <c r="I54" s="100"/>
       <c r="J54" s="14" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="K54" s="100"/>
       <c r="L54" s="100"/>
@@ -4184,10 +4184,10 @@
     </row>
     <row r="55" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B55" s="11" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="C55" s="12" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="D55" s="13">
         <v>1</v>
@@ -4199,12 +4199,12 @@
         <v>18</v>
       </c>
       <c r="G55" s="14" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="H55" s="14"/>
       <c r="I55" s="14"/>
       <c r="J55" s="14" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="K55" s="14"/>
       <c r="L55" s="14"/>
@@ -4214,10 +4214,10 @@
     </row>
     <row r="56" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B56" s="11" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="C56" s="12" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="D56" s="13">
         <v>1</v>
@@ -4229,12 +4229,12 @@
         <v>18</v>
       </c>
       <c r="G56" s="14" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="H56" s="14"/>
       <c r="I56" s="14"/>
       <c r="J56" s="14" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="K56" s="14"/>
       <c r="L56" s="14"/>
@@ -4244,10 +4244,10 @@
     </row>
     <row r="57" spans="1:14" s="96" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B57" s="97" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="C57" s="102" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="D57" s="157">
         <v>1</v>
@@ -4259,12 +4259,12 @@
         <v>18</v>
       </c>
       <c r="G57" s="103" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="H57" s="103"/>
       <c r="I57" s="103"/>
       <c r="J57" s="103" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="K57" s="103"/>
       <c r="L57" s="103"/>
@@ -4275,10 +4275,10 @@
     </row>
     <row r="58" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B58" s="11" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="C58" s="12" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="D58" s="13">
         <v>1</v>
@@ -4304,10 +4304,10 @@
     <row r="59" spans="1:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A59" s="96"/>
       <c r="B59" s="139" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="C59" s="140" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="D59" s="141">
         <v>1</v>
@@ -4325,7 +4325,7 @@
       <c r="K59" s="142"/>
       <c r="L59" s="142"/>
       <c r="M59" s="155" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
     </row>
     <row r="60" spans="1:14" ht="18" thickTop="1" x14ac:dyDescent="0.2">
@@ -4361,7 +4361,7 @@
         <v>170</v>
       </c>
       <c r="C61" s="129" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="D61" s="130">
         <v>1</v>
@@ -4379,7 +4379,7 @@
       <c r="K61" s="131"/>
       <c r="L61" s="131"/>
       <c r="M61" s="138" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
     </row>
     <row r="62" spans="1:14" ht="17" x14ac:dyDescent="0.2">
@@ -4388,7 +4388,7 @@
         <v>170</v>
       </c>
       <c r="C62" s="129" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="D62" s="130">
         <v>1</v>
@@ -4406,7 +4406,7 @@
       <c r="K62" s="131"/>
       <c r="L62" s="131"/>
       <c r="M62" s="138" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
     </row>
     <row r="63" spans="1:14" x14ac:dyDescent="0.2">
@@ -4429,7 +4429,7 @@
       <c r="H63" s="14"/>
       <c r="I63" s="14"/>
       <c r="J63" s="14" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="K63" s="14"/>
       <c r="L63" s="14"/>
@@ -4457,7 +4457,7 @@
       <c r="H64" s="14"/>
       <c r="I64" s="14"/>
       <c r="J64" s="14" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="K64" s="14"/>
       <c r="L64" s="14"/>
@@ -4470,7 +4470,7 @@
         <v>170</v>
       </c>
       <c r="C65" s="12" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="D65" s="13">
         <v>1</v>
@@ -4488,7 +4488,7 @@
       <c r="K65" s="14"/>
       <c r="L65" s="14"/>
       <c r="M65" s="159" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
     </row>
     <row r="66" spans="1:14" x14ac:dyDescent="0.2">
@@ -4496,7 +4496,7 @@
         <v>170</v>
       </c>
       <c r="C66" s="12" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="D66" s="13">
         <v>1</v>
@@ -4511,13 +4511,13 @@
       <c r="H66" s="14"/>
       <c r="I66" s="14"/>
       <c r="J66" s="14" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="K66" s="14" t="s">
         <v>21</v>
       </c>
       <c r="L66" s="14" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="M66" s="111" t="s">
         <v>213</v>
@@ -4543,7 +4543,7 @@
       <c r="H67" s="14"/>
       <c r="I67" s="14"/>
       <c r="J67" s="14" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="K67" s="14"/>
       <c r="L67" s="14"/>
@@ -4556,7 +4556,7 @@
         <v>170</v>
       </c>
       <c r="C68" s="12" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D68" s="13">
         <v>1</v>
@@ -4568,12 +4568,12 @@
         <v>15</v>
       </c>
       <c r="G68" s="14" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="H68" s="14"/>
       <c r="I68" s="14"/>
       <c r="J68" s="14" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="K68" s="14"/>
       <c r="L68" s="14"/>
@@ -4586,7 +4586,7 @@
         <v>170</v>
       </c>
       <c r="C69" s="12" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="D69" s="13">
         <v>1</v>
@@ -4598,12 +4598,12 @@
         <v>15</v>
       </c>
       <c r="G69" s="14" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="H69" s="14"/>
       <c r="I69" s="14"/>
       <c r="J69" s="14" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="K69" s="14"/>
       <c r="L69" s="14"/>
@@ -4631,7 +4631,7 @@
       <c r="H70" s="103"/>
       <c r="I70" s="103"/>
       <c r="J70" s="103" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="K70" s="103"/>
       <c r="L70" s="103"/>
@@ -4660,7 +4660,7 @@
       <c r="H71" s="14"/>
       <c r="I71" s="14"/>
       <c r="J71" s="14" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="K71" s="14"/>
       <c r="L71" s="14"/>
@@ -4688,7 +4688,7 @@
       <c r="H72" s="14"/>
       <c r="I72" s="14"/>
       <c r="J72" s="14" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="K72" s="14"/>
       <c r="L72" s="14"/>
@@ -4701,7 +4701,7 @@
         <v>170</v>
       </c>
       <c r="C73" s="12" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="D73" s="13">
         <v>1</v>
@@ -4713,12 +4713,12 @@
         <v>15</v>
       </c>
       <c r="G73" s="14" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="H73" s="14"/>
       <c r="I73" s="14"/>
       <c r="J73" s="14" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="K73" s="14"/>
       <c r="L73" s="14"/>
@@ -4731,7 +4731,7 @@
         <v>170</v>
       </c>
       <c r="C74" s="140" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="D74" s="141">
         <v>1</v>
@@ -4743,12 +4743,12 @@
         <v>15</v>
       </c>
       <c r="G74" s="142" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="H74" s="142"/>
       <c r="I74" s="142"/>
       <c r="J74" s="142" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="K74" s="142"/>
       <c r="L74" s="142"/>
@@ -4789,7 +4789,7 @@
         <v>175</v>
       </c>
       <c r="C76" s="129" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="D76" s="130">
         <v>1</v>
@@ -4807,7 +4807,7 @@
       <c r="K76" s="131"/>
       <c r="L76" s="131"/>
       <c r="M76" s="138" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
     </row>
     <row r="77" spans="1:14" ht="17" x14ac:dyDescent="0.2">
@@ -4816,7 +4816,7 @@
         <v>175</v>
       </c>
       <c r="C77" s="129" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="D77" s="130">
         <v>1</v>
@@ -4834,7 +4834,7 @@
       <c r="K77" s="131"/>
       <c r="L77" s="131"/>
       <c r="M77" s="138" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
     </row>
     <row r="78" spans="1:14" x14ac:dyDescent="0.2">
@@ -4858,7 +4858,7 @@
       <c r="H78" s="14"/>
       <c r="I78" s="14"/>
       <c r="J78" s="14" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="K78" s="14"/>
       <c r="L78" s="14"/>
@@ -4886,7 +4886,7 @@
       <c r="H79" s="14"/>
       <c r="I79" s="14"/>
       <c r="J79" s="14" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="K79" s="14"/>
       <c r="L79" s="14"/>
@@ -4901,7 +4901,7 @@
         <v>175</v>
       </c>
       <c r="C80" s="12" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="D80" s="13">
         <v>1</v>
@@ -4915,7 +4915,7 @@
       <c r="G80" s="14"/>
       <c r="H80" s="14"/>
       <c r="I80" s="14" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="J80" s="14"/>
       <c r="K80" s="14"/>
@@ -4930,7 +4930,7 @@
         <v>175</v>
       </c>
       <c r="C81" s="102" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="D81" s="157">
         <v>1</v>
@@ -4945,7 +4945,7 @@
       <c r="H81" s="103"/>
       <c r="I81" s="103"/>
       <c r="J81" s="103" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="K81" s="103" t="s">
         <v>21</v>
@@ -4963,7 +4963,7 @@
         <v>175</v>
       </c>
       <c r="C82" s="12" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="D82" s="13">
         <v>1</v>
@@ -4978,7 +4978,7 @@
       <c r="H82" s="14"/>
       <c r="I82" s="14"/>
       <c r="J82" s="14" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="K82" s="14"/>
       <c r="L82" s="14"/>
@@ -4992,7 +4992,7 @@
         <v>175</v>
       </c>
       <c r="C83" s="140" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="D83" s="141">
         <v>1</v>
@@ -5005,19 +5005,19 @@
       </c>
       <c r="G83" s="142"/>
       <c r="H83" s="142" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="I83" s="142"/>
       <c r="J83" s="142"/>
       <c r="K83" s="142"/>
       <c r="L83" s="142"/>
       <c r="M83" s="160" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
     </row>
     <row r="84" spans="1:14" s="96" customFormat="1" ht="18" thickTop="1" x14ac:dyDescent="0.2">
       <c r="B84" s="128" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="C84" s="145" t="s">
         <v>13</v>
@@ -5045,10 +5045,10 @@
     <row r="85" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A85" s="15"/>
       <c r="B85" s="128" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="C85" s="129" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="D85" s="130">
         <v>1</v>
@@ -5066,16 +5066,16 @@
       <c r="K85" s="131"/>
       <c r="L85" s="131"/>
       <c r="M85" s="138" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
     </row>
     <row r="86" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A86" s="15"/>
       <c r="B86" s="128" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="C86" s="129" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="D86" s="130">
         <v>1</v>
@@ -5093,15 +5093,15 @@
       <c r="K86" s="131"/>
       <c r="L86" s="131"/>
       <c r="M86" s="138" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
     </row>
     <row r="87" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B87" s="97" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="C87" s="12" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="D87" s="13">
         <v>1</v>
@@ -5127,10 +5127,10 @@
     <row r="88" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A88" s="96"/>
       <c r="B88" s="97" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="C88" s="102" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="D88" s="157">
         <v>1</v>
@@ -5155,10 +5155,10 @@
     </row>
     <row r="89" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B89" s="97" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="C89" s="12" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="D89" s="13">
         <v>1</v>
@@ -5173,17 +5173,17 @@
       <c r="H89" s="14"/>
       <c r="I89" s="14"/>
       <c r="J89" s="14" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="K89" s="14"/>
       <c r="L89" s="14"/>
       <c r="M89" s="111" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
     </row>
     <row r="90" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B90" s="97" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="C90" s="12" t="s">
         <v>177</v>
@@ -5201,7 +5201,7 @@
       <c r="H90" s="14"/>
       <c r="I90" s="14"/>
       <c r="J90" s="14" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="K90" s="14"/>
       <c r="L90" s="14"/>
@@ -5211,10 +5211,10 @@
     </row>
     <row r="91" spans="1:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B91" s="148" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="C91" s="140" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="D91" s="141">
         <v>1</v>
@@ -5227,20 +5227,20 @@
       </c>
       <c r="G91" s="142"/>
       <c r="H91" s="142" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="I91" s="142"/>
       <c r="J91" s="142"/>
       <c r="K91" s="142"/>
       <c r="L91" s="142"/>
       <c r="M91" s="160" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
     </row>
     <row r="92" spans="1:14" ht="17" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A92" s="104"/>
       <c r="B92" s="128" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="C92" s="145" t="s">
         <v>13</v>
@@ -5267,10 +5267,10 @@
     <row r="93" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A93" s="15"/>
       <c r="B93" s="128" t="s">
+        <v>293</v>
+      </c>
+      <c r="C93" s="129" t="s">
         <v>295</v>
-      </c>
-      <c r="C93" s="129" t="s">
-        <v>297</v>
       </c>
       <c r="D93" s="130">
         <v>1</v>
@@ -5288,16 +5288,16 @@
       <c r="K93" s="131"/>
       <c r="L93" s="131"/>
       <c r="M93" s="138" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
     </row>
     <row r="94" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A94" s="15"/>
       <c r="B94" s="128" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="C94" s="129" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="D94" s="130">
         <v>1</v>
@@ -5315,12 +5315,12 @@
       <c r="K94" s="131"/>
       <c r="L94" s="131"/>
       <c r="M94" s="138" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
     </row>
     <row r="95" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B95" s="11" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="C95" s="12" t="s">
         <v>210</v>
@@ -5338,7 +5338,7 @@
       <c r="H95" s="14"/>
       <c r="I95" s="14"/>
       <c r="J95" s="14" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="K95" s="14"/>
       <c r="L95" s="14"/>
@@ -5348,7 +5348,7 @@
     </row>
     <row r="96" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B96" s="11" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="C96" s="12" t="s">
         <v>194</v>
@@ -5366,7 +5366,7 @@
       <c r="H96" s="14"/>
       <c r="I96" s="14"/>
       <c r="J96" s="14" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="K96" s="14"/>
       <c r="L96" s="14"/>
@@ -5376,10 +5376,10 @@
     </row>
     <row r="97" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B97" s="11" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="C97" s="12" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="D97" s="13">
         <v>1</v>
@@ -5394,17 +5394,17 @@
       <c r="H97" s="14"/>
       <c r="I97" s="14"/>
       <c r="J97" s="14" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="K97" s="14"/>
       <c r="L97" s="14"/>
       <c r="M97" s="111" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="98" spans="2:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B98" s="123" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="C98" s="124" t="s">
         <v>161</v>
@@ -5422,7 +5422,7 @@
       <c r="H98" s="126"/>
       <c r="I98" s="126"/>
       <c r="J98" s="126" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="K98" s="126"/>
       <c r="L98" s="126"/>

</xml_diff>

<commit_message>
New row for Software_url
</commit_message>
<xml_diff>
--- a/Schema/DB_scheme.xlsx
+++ b/Schema/DB_scheme.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aksam432/Documents/GitHub/WP3/Schema/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C1112B4-8E3F-724D-B3E4-AE5FA083A07B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A883E7E-DDC3-BE4D-A59D-CFEF44A94EAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38400" yWindow="0" windowWidth="21600" windowHeight="38400" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="907" uniqueCount="330">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="913" uniqueCount="332">
   <si>
     <t>PROJET :</t>
   </si>
@@ -760,9 +760,6 @@
     <t>softwareVersion</t>
   </si>
   <si>
-    <t>gitURL</t>
-  </si>
-  <si>
     <t>doi</t>
   </si>
   <si>
@@ -1028,6 +1025,15 @@
   </si>
   <si>
     <t>The URL link to the checkpoint or model files.</t>
+  </si>
+  <si>
+    <t>modelVaraint</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The particular variant of the MLIP architecture </t>
+  </si>
+  <si>
+    <t>softwareUrl</t>
   </si>
 </sst>
 </file>
@@ -1753,7 +1759,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="173">
+  <cellXfs count="174">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2233,6 +2239,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2669,7 +2678,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:N99"/>
+  <dimension ref="A2:N100"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2.83203125" customWidth="1"/>
@@ -2696,7 +2705,7 @@
       </c>
       <c r="C2" s="164"/>
       <c r="D2" s="165" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="E2" s="165"/>
       <c r="F2" s="165"/>
@@ -2777,7 +2786,7 @@
         <v>54</v>
       </c>
       <c r="C7" s="129" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="D7" s="130">
         <v>1</v>
@@ -2795,7 +2804,7 @@
       <c r="K7" s="131"/>
       <c r="L7" s="131"/>
       <c r="M7" s="132" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="8" spans="2:14" x14ac:dyDescent="0.2">
@@ -2803,7 +2812,7 @@
         <v>54</v>
       </c>
       <c r="C8" s="129" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="D8" s="130">
         <v>1</v>
@@ -2821,7 +2830,7 @@
       <c r="K8" s="131"/>
       <c r="L8" s="131"/>
       <c r="M8" s="132" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="9" spans="2:14" x14ac:dyDescent="0.2">
@@ -2829,7 +2838,7 @@
         <v>54</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="D9" s="13">
         <v>1</v>
@@ -2844,7 +2853,7 @@
       <c r="H9" s="14"/>
       <c r="I9" s="14"/>
       <c r="J9" s="14" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="K9" s="14"/>
       <c r="L9" s="14"/>
@@ -2872,7 +2881,7 @@
       <c r="H10" s="14"/>
       <c r="I10" s="14"/>
       <c r="J10" s="14" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="K10" s="14"/>
       <c r="L10" s="14"/>
@@ -2900,13 +2909,13 @@
       <c r="H11" s="14"/>
       <c r="I11" s="14"/>
       <c r="J11" s="14" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="K11" s="14" t="s">
         <v>20</v>
       </c>
       <c r="L11" s="14" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="M11" s="112" t="s">
         <v>164</v>
@@ -2933,7 +2942,7 @@
       <c r="H12" s="95"/>
       <c r="I12" s="95"/>
       <c r="J12" s="14" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="K12" s="95"/>
       <c r="L12" s="95"/>
@@ -2946,7 +2955,7 @@
         <v>54</v>
       </c>
       <c r="C13" s="93" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="D13" s="94">
         <v>1</v>
@@ -2961,13 +2970,13 @@
       <c r="H13" s="95"/>
       <c r="I13" s="95"/>
       <c r="J13" s="14" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="K13" s="95" t="s">
         <v>20</v>
       </c>
       <c r="L13" s="95" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="M13" s="113" t="s">
         <v>183</v>
@@ -2979,7 +2988,7 @@
         <v>54</v>
       </c>
       <c r="C14" s="93" t="s">
-        <v>321</v>
+        <v>329</v>
       </c>
       <c r="D14" s="94">
         <v>1</v>
@@ -2988,79 +2997,80 @@
         <v>14</v>
       </c>
       <c r="F14" s="95" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="G14" s="95"/>
       <c r="H14" s="95"/>
       <c r="I14" s="95"/>
       <c r="J14" s="14" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="K14" s="95"/>
       <c r="L14" s="95"/>
       <c r="M14" s="113" t="s">
-        <v>322</v>
-      </c>
-      <c r="N14" s="163"/>
-    </row>
-    <row r="15" spans="2:14" x14ac:dyDescent="0.2">
+        <v>330</v>
+      </c>
+      <c r="N14" s="173"/>
+    </row>
+    <row r="15" spans="2:14" ht="17" x14ac:dyDescent="0.2">
       <c r="B15" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="C15" s="12" t="s">
-        <v>238</v>
-      </c>
-      <c r="D15" s="13">
-        <v>1</v>
-      </c>
-      <c r="E15" s="12" t="s">
-        <v>57</v>
-      </c>
-      <c r="F15" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="G15" s="14"/>
-      <c r="H15" s="14"/>
-      <c r="I15" s="12"/>
+      <c r="C15" s="93" t="s">
+        <v>320</v>
+      </c>
+      <c r="D15" s="94">
+        <v>1</v>
+      </c>
+      <c r="E15" s="93" t="s">
+        <v>14</v>
+      </c>
+      <c r="F15" s="95" t="s">
+        <v>15</v>
+      </c>
+      <c r="G15" s="95"/>
+      <c r="H15" s="95"/>
+      <c r="I15" s="95"/>
       <c r="J15" s="14" t="s">
-        <v>292</v>
-      </c>
-      <c r="K15" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="L15" s="14" t="s">
-        <v>319</v>
-      </c>
-      <c r="M15" s="111" t="s">
-        <v>177</v>
-      </c>
+        <v>291</v>
+      </c>
+      <c r="K15" s="95"/>
+      <c r="L15" s="95"/>
+      <c r="M15" s="113" t="s">
+        <v>321</v>
+      </c>
+      <c r="N15" s="163"/>
     </row>
     <row r="16" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B16" s="11" t="s">
         <v>54</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>325</v>
+        <v>238</v>
       </c>
       <c r="D16" s="13">
         <v>1</v>
       </c>
       <c r="E16" s="12" t="s">
-        <v>14</v>
+        <v>57</v>
       </c>
       <c r="F16" s="14" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G16" s="14"/>
       <c r="H16" s="14"/>
       <c r="I16" s="12"/>
       <c r="J16" s="14" t="s">
-        <v>326</v>
-      </c>
-      <c r="K16" s="14"/>
-      <c r="L16" s="14"/>
+        <v>291</v>
+      </c>
+      <c r="K16" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="L16" s="14" t="s">
+        <v>318</v>
+      </c>
       <c r="M16" s="111" t="s">
-        <v>327</v>
+        <v>177</v>
       </c>
     </row>
     <row r="17" spans="2:14" x14ac:dyDescent="0.2">
@@ -3068,7 +3078,7 @@
         <v>54</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="D17" s="13">
         <v>1</v>
@@ -3083,248 +3093,248 @@
       <c r="H17" s="14"/>
       <c r="I17" s="12"/>
       <c r="J17" s="14" t="s">
-        <v>292</v>
+        <v>325</v>
       </c>
       <c r="K17" s="14"/>
       <c r="L17" s="14"/>
       <c r="M17" s="111" t="s">
-        <v>324</v>
-      </c>
-      <c r="N17" s="162"/>
+        <v>326</v>
+      </c>
     </row>
     <row r="18" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B18" s="11" t="s">
         <v>54</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>237</v>
+        <v>322</v>
       </c>
       <c r="D18" s="13">
         <v>1</v>
       </c>
       <c r="E18" s="12" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="F18" s="14" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="G18" s="14"/>
       <c r="H18" s="14"/>
       <c r="I18" s="12"/>
       <c r="J18" s="14" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="K18" s="14"/>
       <c r="L18" s="14"/>
       <c r="M18" s="111" t="s">
-        <v>235</v>
-      </c>
-      <c r="N18" s="163"/>
-    </row>
-    <row r="19" spans="2:14" ht="17" x14ac:dyDescent="0.2">
+        <v>323</v>
+      </c>
+      <c r="N18" s="162"/>
+    </row>
+    <row r="19" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B19" s="11" t="s">
         <v>54</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="D19" s="13">
         <v>1</v>
       </c>
       <c r="E19" s="12" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="F19" s="14" t="s">
         <v>17</v>
       </c>
       <c r="G19" s="14"/>
       <c r="H19" s="14"/>
-      <c r="I19" s="14"/>
+      <c r="I19" s="12"/>
       <c r="J19" s="14" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="K19" s="14"/>
       <c r="L19" s="14"/>
-      <c r="M19" s="112" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="20" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="M19" s="111" t="s">
+        <v>235</v>
+      </c>
+      <c r="N19" s="163"/>
+    </row>
+    <row r="20" spans="2:14" ht="17" x14ac:dyDescent="0.2">
       <c r="B20" s="11" t="s">
         <v>54</v>
       </c>
       <c r="C20" s="12" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="D20" s="13">
         <v>1</v>
       </c>
       <c r="E20" s="12" t="s">
-        <v>160</v>
+        <v>14</v>
       </c>
       <c r="F20" s="14" t="s">
         <v>15</v>
       </c>
       <c r="G20" s="14"/>
       <c r="H20" s="14"/>
-      <c r="I20" s="12"/>
+      <c r="I20" s="14"/>
       <c r="J20" s="14" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="K20" s="14"/>
       <c r="L20" s="14"/>
-      <c r="M20" s="111" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="21" spans="2:14" ht="17" x14ac:dyDescent="0.2">
+      <c r="M20" s="112" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="21" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B21" s="11" t="s">
         <v>54</v>
       </c>
       <c r="C21" s="12" t="s">
-        <v>241</v>
+        <v>331</v>
       </c>
       <c r="D21" s="13">
         <v>1</v>
       </c>
       <c r="E21" s="12" t="s">
-        <v>14</v>
+        <v>160</v>
       </c>
       <c r="F21" s="14" t="s">
         <v>15</v>
       </c>
       <c r="G21" s="14"/>
       <c r="H21" s="14"/>
-      <c r="I21" s="14"/>
+      <c r="I21" s="12"/>
       <c r="J21" s="14" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="K21" s="14"/>
       <c r="L21" s="14"/>
-      <c r="M21" s="114" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="22" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="M21" s="111" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="22" spans="2:14" ht="17" x14ac:dyDescent="0.2">
       <c r="B22" s="11" t="s">
         <v>54</v>
       </c>
       <c r="C22" s="12" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="D22" s="13">
         <v>1</v>
       </c>
       <c r="E22" s="12" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="F22" s="14" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="G22" s="14"/>
       <c r="H22" s="14"/>
-      <c r="I22" s="14" t="s">
-        <v>168</v>
-      </c>
-      <c r="J22" s="14"/>
+      <c r="I22" s="14"/>
+      <c r="J22" s="14" t="s">
+        <v>291</v>
+      </c>
       <c r="K22" s="14"/>
       <c r="L22" s="14"/>
-      <c r="M22" s="111" t="s">
+      <c r="M22" s="114" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="23" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B23" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="C23" s="12" t="s">
+        <v>242</v>
+      </c>
+      <c r="D23" s="13">
+        <v>1</v>
+      </c>
+      <c r="E23" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="F23" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="G23" s="14"/>
+      <c r="H23" s="14"/>
+      <c r="I23" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="J23" s="14"/>
+      <c r="K23" s="14"/>
+      <c r="L23" s="14"/>
+      <c r="M23" s="111" t="s">
         <v>181</v>
       </c>
-      <c r="N22" s="162"/>
-    </row>
-    <row r="23" spans="2:14" s="96" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="B23" s="97" t="s">
+      <c r="N23" s="162"/>
+    </row>
+    <row r="24" spans="2:14" s="96" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="B24" s="97" t="s">
         <v>54</v>
       </c>
-      <c r="C23" s="98" t="s">
-        <v>244</v>
-      </c>
-      <c r="D23" s="99">
-        <v>1</v>
-      </c>
-      <c r="E23" s="98" t="s">
+      <c r="C24" s="98" t="s">
+        <v>243</v>
+      </c>
+      <c r="D24" s="99">
+        <v>1</v>
+      </c>
+      <c r="E24" s="98" t="s">
         <v>57</v>
       </c>
-      <c r="F23" s="100" t="s">
+      <c r="F24" s="100" t="s">
         <v>15</v>
       </c>
-      <c r="G23" s="100"/>
-      <c r="H23" s="100"/>
-      <c r="I23" s="100"/>
-      <c r="J23" s="14" t="s">
-        <v>292</v>
-      </c>
-      <c r="K23" s="100" t="s">
+      <c r="G24" s="100"/>
+      <c r="H24" s="100"/>
+      <c r="I24" s="100"/>
+      <c r="J24" s="14" t="s">
+        <v>291</v>
+      </c>
+      <c r="K24" s="100" t="s">
         <v>20</v>
       </c>
-      <c r="L23" s="105" t="s">
-        <v>289</v>
-      </c>
-      <c r="M23" s="115" t="s">
+      <c r="L24" s="105" t="s">
+        <v>288</v>
+      </c>
+      <c r="M24" s="115" t="s">
         <v>182</v>
       </c>
-      <c r="N23"/>
-    </row>
-    <row r="24" spans="2:14" ht="17" x14ac:dyDescent="0.2">
-      <c r="B24" s="11" t="s">
-        <v>54</v>
-      </c>
-      <c r="C24" s="12" t="s">
-        <v>178</v>
-      </c>
-      <c r="D24" s="13">
-        <v>1</v>
-      </c>
-      <c r="E24" s="12" t="s">
-        <v>57</v>
-      </c>
-      <c r="F24" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="G24" s="14"/>
-      <c r="H24" s="14"/>
-      <c r="I24" s="14"/>
-      <c r="J24" s="14" t="s">
-        <v>292</v>
-      </c>
-      <c r="K24" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="L24" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="M24" s="112" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="25" spans="2:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="N24"/>
+    </row>
+    <row r="25" spans="2:14" ht="17" x14ac:dyDescent="0.2">
       <c r="B25" s="11" t="s">
         <v>54</v>
       </c>
       <c r="C25" s="12" t="s">
-        <v>245</v>
+        <v>178</v>
       </c>
       <c r="D25" s="13">
         <v>1</v>
       </c>
       <c r="E25" s="12" t="s">
-        <v>19</v>
+        <v>57</v>
       </c>
       <c r="F25" s="14" t="s">
         <v>17</v>
       </c>
       <c r="G25" s="14"/>
       <c r="H25" s="14"/>
-      <c r="I25" s="14" t="s">
-        <v>290</v>
-      </c>
-      <c r="J25" s="14"/>
-      <c r="K25" s="14"/>
-      <c r="L25" s="14"/>
-      <c r="M25" s="114" t="s">
-        <v>186</v>
+      <c r="I25" s="14"/>
+      <c r="J25" s="14" t="s">
+        <v>291</v>
+      </c>
+      <c r="K25" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="L25" s="14" t="s">
+        <v>179</v>
+      </c>
+      <c r="M25" s="112" t="s">
+        <v>185</v>
       </c>
     </row>
     <row r="26" spans="2:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -3332,7 +3342,7 @@
         <v>54</v>
       </c>
       <c r="C26" s="12" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="D26" s="13">
         <v>1</v>
@@ -3341,26 +3351,26 @@
         <v>19</v>
       </c>
       <c r="F26" s="14" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G26" s="14"/>
       <c r="H26" s="14"/>
       <c r="I26" s="14" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="J26" s="14"/>
       <c r="K26" s="14"/>
       <c r="L26" s="14"/>
       <c r="M26" s="114" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="27" spans="2:14" ht="17" x14ac:dyDescent="0.2">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="27" spans="2:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B27" s="11" t="s">
         <v>54</v>
       </c>
       <c r="C27" s="12" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="D27" s="13">
         <v>1</v>
@@ -3374,13 +3384,13 @@
       <c r="G27" s="14"/>
       <c r="H27" s="14"/>
       <c r="I27" s="14" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="J27" s="14"/>
       <c r="K27" s="14"/>
       <c r="L27" s="14"/>
       <c r="M27" s="114" t="s">
-        <v>187</v>
+        <v>233</v>
       </c>
     </row>
     <row r="28" spans="2:14" ht="17" x14ac:dyDescent="0.2">
@@ -3388,31 +3398,27 @@
         <v>54</v>
       </c>
       <c r="C28" s="12" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="D28" s="13">
         <v>1</v>
       </c>
       <c r="E28" s="12" t="s">
-        <v>57</v>
+        <v>19</v>
       </c>
       <c r="F28" s="14" t="s">
         <v>15</v>
       </c>
       <c r="G28" s="14"/>
       <c r="H28" s="14"/>
-      <c r="I28" s="14"/>
-      <c r="J28" s="14" t="s">
-        <v>292</v>
-      </c>
-      <c r="K28" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="L28" s="14" t="s">
-        <v>180</v>
-      </c>
-      <c r="M28" s="112" t="s">
-        <v>188</v>
+      <c r="I28" s="14" t="s">
+        <v>289</v>
+      </c>
+      <c r="J28" s="14"/>
+      <c r="K28" s="14"/>
+      <c r="L28" s="14"/>
+      <c r="M28" s="114" t="s">
+        <v>187</v>
       </c>
     </row>
     <row r="29" spans="2:14" ht="17" x14ac:dyDescent="0.2">
@@ -3420,13 +3426,13 @@
         <v>54</v>
       </c>
       <c r="C29" s="12" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="D29" s="13">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="E29" s="12" t="s">
-        <v>14</v>
+        <v>57</v>
       </c>
       <c r="F29" s="14" t="s">
         <v>15</v>
@@ -3435,12 +3441,16 @@
       <c r="H29" s="14"/>
       <c r="I29" s="14"/>
       <c r="J29" s="14" t="s">
-        <v>292</v>
-      </c>
-      <c r="K29" s="14"/>
-      <c r="L29" s="14"/>
+        <v>291</v>
+      </c>
+      <c r="K29" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="L29" s="14" t="s">
+        <v>180</v>
+      </c>
       <c r="M29" s="112" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="30" spans="2:14" ht="17" x14ac:dyDescent="0.2">
@@ -3448,13 +3458,13 @@
         <v>54</v>
       </c>
       <c r="C30" s="12" t="s">
-        <v>328</v>
+        <v>248</v>
       </c>
       <c r="D30" s="13">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="E30" s="12" t="s">
-        <v>160</v>
+        <v>14</v>
       </c>
       <c r="F30" s="14" t="s">
         <v>15</v>
@@ -3463,104 +3473,105 @@
       <c r="H30" s="14"/>
       <c r="I30" s="14"/>
       <c r="J30" s="14" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="K30" s="14"/>
       <c r="L30" s="14"/>
       <c r="M30" s="112" t="s">
-        <v>329</v>
+        <v>189</v>
       </c>
     </row>
     <row r="31" spans="2:14" ht="17" x14ac:dyDescent="0.2">
-      <c r="B31" s="133" t="s">
+      <c r="B31" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="C31" s="134" t="s">
+      <c r="C31" s="12" t="s">
+        <v>327</v>
+      </c>
+      <c r="D31" s="13">
+        <v>1</v>
+      </c>
+      <c r="E31" s="12" t="s">
+        <v>160</v>
+      </c>
+      <c r="F31" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="G31" s="14"/>
+      <c r="H31" s="14"/>
+      <c r="I31" s="14"/>
+      <c r="J31" s="14" t="s">
+        <v>291</v>
+      </c>
+      <c r="K31" s="14"/>
+      <c r="L31" s="14"/>
+      <c r="M31" s="112" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="32" spans="2:14" ht="17" x14ac:dyDescent="0.2">
+      <c r="B32" s="133" t="s">
+        <v>54</v>
+      </c>
+      <c r="C32" s="134" t="s">
+        <v>249</v>
+      </c>
+      <c r="D32" s="135">
+        <v>1</v>
+      </c>
+      <c r="E32" s="134" t="s">
+        <v>48</v>
+      </c>
+      <c r="F32" s="136" t="s">
+        <v>17</v>
+      </c>
+      <c r="G32" s="136"/>
+      <c r="H32" s="136" t="s">
+        <v>251</v>
+      </c>
+      <c r="I32" s="136"/>
+      <c r="J32" s="136"/>
+      <c r="K32" s="136"/>
+      <c r="L32" s="136"/>
+      <c r="M32" s="137" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="33" spans="1:14" ht="18" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B33" s="139" t="s">
+        <v>54</v>
+      </c>
+      <c r="C33" s="140" t="s">
         <v>250</v>
       </c>
-      <c r="D31" s="135">
-        <v>1</v>
-      </c>
-      <c r="E31" s="134" t="s">
-        <v>48</v>
-      </c>
-      <c r="F31" s="136" t="s">
-        <v>17</v>
-      </c>
-      <c r="G31" s="136"/>
-      <c r="H31" s="136" t="s">
-        <v>252</v>
-      </c>
-      <c r="I31" s="136"/>
-      <c r="J31" s="136"/>
-      <c r="K31" s="136"/>
-      <c r="L31" s="136"/>
-      <c r="M31" s="137" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="32" spans="2:14" ht="18" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B32" s="139" t="s">
-        <v>54</v>
-      </c>
-      <c r="C32" s="140" t="s">
-        <v>251</v>
-      </c>
-      <c r="D32" s="141">
+      <c r="D33" s="141">
         <v>10</v>
       </c>
-      <c r="E32" s="140" t="s">
+      <c r="E33" s="140" t="s">
         <v>19</v>
       </c>
-      <c r="F32" s="142" t="s">
-        <v>17</v>
-      </c>
-      <c r="G32" s="142"/>
-      <c r="H32" s="142"/>
-      <c r="I32" s="142" t="s">
-        <v>291</v>
-      </c>
-      <c r="J32" s="142"/>
-      <c r="K32" s="142"/>
-      <c r="L32" s="142"/>
-      <c r="M32" s="143" t="s">
+      <c r="F33" s="142" t="s">
+        <v>15</v>
+      </c>
+      <c r="G33" s="142"/>
+      <c r="H33" s="142"/>
+      <c r="I33" s="142" t="s">
+        <v>290</v>
+      </c>
+      <c r="J33" s="142"/>
+      <c r="K33" s="142"/>
+      <c r="L33" s="142"/>
+      <c r="M33" s="143" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="33" spans="1:14" ht="18" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="15"/>
-      <c r="B33" s="128" t="s">
-        <v>168</v>
-      </c>
-      <c r="C33" s="129" t="s">
-        <v>13</v>
-      </c>
-      <c r="D33" s="130">
-        <v>1</v>
-      </c>
-      <c r="E33" s="129" t="s">
-        <v>14</v>
-      </c>
-      <c r="F33" s="131" t="s">
-        <v>17</v>
-      </c>
-      <c r="G33" s="131"/>
-      <c r="H33" s="131"/>
-      <c r="I33" s="131"/>
-      <c r="J33" s="131"/>
-      <c r="K33" s="131"/>
-      <c r="L33" s="131"/>
-      <c r="M33" s="138" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="34" spans="1:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:14" ht="18" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A34" s="15"/>
       <c r="B34" s="128" t="s">
         <v>168</v>
       </c>
       <c r="C34" s="129" t="s">
-        <v>293</v>
+        <v>13</v>
       </c>
       <c r="D34" s="130">
         <v>1</v>
@@ -3578,7 +3589,7 @@
       <c r="K34" s="131"/>
       <c r="L34" s="131"/>
       <c r="M34" s="138" t="s">
-        <v>295</v>
+        <v>16</v>
       </c>
     </row>
     <row r="35" spans="1:14" ht="17" x14ac:dyDescent="0.2">
@@ -3587,13 +3598,13 @@
         <v>168</v>
       </c>
       <c r="C35" s="129" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="D35" s="130">
         <v>1</v>
       </c>
       <c r="E35" s="129" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="F35" s="131" t="s">
         <v>17</v>
@@ -3605,36 +3616,34 @@
       <c r="K35" s="131"/>
       <c r="L35" s="131"/>
       <c r="M35" s="138" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
     </row>
     <row r="36" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A36" s="15"/>
-      <c r="B36" s="11" t="s">
+      <c r="B36" s="128" t="s">
         <v>168</v>
       </c>
-      <c r="C36" s="12" t="s">
-        <v>162</v>
-      </c>
-      <c r="D36" s="13">
-        <v>1</v>
-      </c>
-      <c r="E36" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="F36" s="14" t="s">
-        <v>15</v>
-      </c>
-      <c r="G36" s="14"/>
-      <c r="H36" s="14"/>
-      <c r="I36" s="16"/>
-      <c r="J36" s="14" t="s">
-        <v>292</v>
-      </c>
-      <c r="K36" s="14"/>
-      <c r="L36" s="14"/>
-      <c r="M36" s="112" t="s">
-        <v>194</v>
+      <c r="C36" s="129" t="s">
+        <v>293</v>
+      </c>
+      <c r="D36" s="130">
+        <v>1</v>
+      </c>
+      <c r="E36" s="129" t="s">
+        <v>18</v>
+      </c>
+      <c r="F36" s="131" t="s">
+        <v>17</v>
+      </c>
+      <c r="G36" s="131"/>
+      <c r="H36" s="131"/>
+      <c r="I36" s="131"/>
+      <c r="J36" s="131"/>
+      <c r="K36" s="131"/>
+      <c r="L36" s="131"/>
+      <c r="M36" s="138" t="s">
+        <v>295</v>
       </c>
     </row>
     <row r="37" spans="1:14" ht="17" x14ac:dyDescent="0.2">
@@ -3643,13 +3652,13 @@
         <v>168</v>
       </c>
       <c r="C37" s="12" t="s">
-        <v>300</v>
+        <v>162</v>
       </c>
       <c r="D37" s="13">
         <v>1</v>
       </c>
       <c r="E37" s="12" t="s">
-        <v>48</v>
+        <v>14</v>
       </c>
       <c r="F37" s="14" t="s">
         <v>15</v>
@@ -3657,11 +3666,13 @@
       <c r="G37" s="14"/>
       <c r="H37" s="14"/>
       <c r="I37" s="16"/>
-      <c r="J37" s="14"/>
+      <c r="J37" s="14" t="s">
+        <v>291</v>
+      </c>
       <c r="K37" s="14"/>
       <c r="L37" s="14"/>
       <c r="M37" s="112" t="s">
-        <v>299</v>
+        <v>194</v>
       </c>
     </row>
     <row r="38" spans="1:14" ht="17" x14ac:dyDescent="0.2">
@@ -3670,13 +3681,13 @@
         <v>168</v>
       </c>
       <c r="C38" s="12" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="D38" s="13">
         <v>1</v>
       </c>
       <c r="E38" s="12" t="s">
-        <v>160</v>
+        <v>48</v>
       </c>
       <c r="F38" s="14" t="s">
         <v>15</v>
@@ -3697,29 +3708,25 @@
         <v>168</v>
       </c>
       <c r="C39" s="12" t="s">
-        <v>253</v>
+        <v>296</v>
       </c>
       <c r="D39" s="13">
         <v>1</v>
       </c>
       <c r="E39" s="12" t="s">
-        <v>21</v>
+        <v>160</v>
       </c>
       <c r="F39" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="G39" s="14" t="s">
-        <v>311</v>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="G39" s="14"/>
       <c r="H39" s="14"/>
       <c r="I39" s="16"/>
-      <c r="J39" s="14" t="s">
-        <v>292</v>
-      </c>
+      <c r="J39" s="14"/>
       <c r="K39" s="14"/>
       <c r="L39" s="14"/>
       <c r="M39" s="112" t="s">
-        <v>195</v>
+        <v>297</v>
       </c>
     </row>
     <row r="40" spans="1:14" ht="17" x14ac:dyDescent="0.2">
@@ -3727,8 +3734,8 @@
       <c r="B40" s="11" t="s">
         <v>168</v>
       </c>
-      <c r="C40" s="116" t="s">
-        <v>254</v>
+      <c r="C40" s="12" t="s">
+        <v>252</v>
       </c>
       <c r="D40" s="13">
         <v>1</v>
@@ -3740,17 +3747,17 @@
         <v>17</v>
       </c>
       <c r="G40" s="14" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="H40" s="14"/>
       <c r="I40" s="16"/>
       <c r="J40" s="14" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="K40" s="14"/>
       <c r="L40" s="14"/>
       <c r="M40" s="112" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="41" spans="1:14" ht="17" x14ac:dyDescent="0.2">
@@ -3758,8 +3765,8 @@
       <c r="B41" s="11" t="s">
         <v>168</v>
       </c>
-      <c r="C41" s="144" t="s">
-        <v>255</v>
+      <c r="C41" s="116" t="s">
+        <v>253</v>
       </c>
       <c r="D41" s="13">
         <v>1</v>
@@ -3771,16 +3778,16 @@
         <v>17</v>
       </c>
       <c r="G41" s="14" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="H41" s="14"/>
-      <c r="I41" s="14"/>
+      <c r="I41" s="16"/>
       <c r="J41" s="14" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="K41" s="14"/>
       <c r="L41" s="14"/>
-      <c r="M41" s="114" t="s">
+      <c r="M41" s="112" t="s">
         <v>196</v>
       </c>
     </row>
@@ -3789,8 +3796,8 @@
       <c r="B42" s="11" t="s">
         <v>168</v>
       </c>
-      <c r="C42" s="12" t="s">
-        <v>256</v>
+      <c r="C42" s="144" t="s">
+        <v>254</v>
       </c>
       <c r="D42" s="13">
         <v>1</v>
@@ -3799,122 +3806,126 @@
         <v>21</v>
       </c>
       <c r="F42" s="14" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G42" s="14" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="H42" s="14"/>
       <c r="I42" s="14"/>
       <c r="J42" s="14" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="K42" s="14"/>
       <c r="L42" s="14"/>
       <c r="M42" s="114" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="43" spans="1:14" ht="17" x14ac:dyDescent="0.2">
+      <c r="A43" s="15"/>
+      <c r="B43" s="11" t="s">
+        <v>168</v>
+      </c>
+      <c r="C43" s="12" t="s">
+        <v>255</v>
+      </c>
+      <c r="D43" s="13">
+        <v>1</v>
+      </c>
+      <c r="E43" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="F43" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="G43" s="14" t="s">
+        <v>312</v>
+      </c>
+      <c r="H43" s="14"/>
+      <c r="I43" s="14"/>
+      <c r="J43" s="14" t="s">
+        <v>291</v>
+      </c>
+      <c r="K43" s="14"/>
+      <c r="L43" s="14"/>
+      <c r="M43" s="114" t="s">
         <v>197</v>
       </c>
     </row>
-    <row r="43" spans="1:14" s="96" customFormat="1" ht="18" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="101"/>
-      <c r="B43" s="148" t="s">
+    <row r="44" spans="1:14" s="96" customFormat="1" ht="18" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="101"/>
+      <c r="B44" s="148" t="s">
         <v>168</v>
       </c>
-      <c r="C43" s="149" t="s">
-        <v>257</v>
-      </c>
-      <c r="D43" s="150">
-        <v>1</v>
-      </c>
-      <c r="E43" s="151" t="s">
+      <c r="C44" s="149" t="s">
+        <v>256</v>
+      </c>
+      <c r="D44" s="150">
+        <v>1</v>
+      </c>
+      <c r="E44" s="151" t="s">
         <v>21</v>
       </c>
-      <c r="F43" s="152" t="s">
+      <c r="F44" s="152" t="s">
         <v>15</v>
       </c>
-      <c r="G43" s="142" t="s">
-        <v>313</v>
-      </c>
-      <c r="H43" s="153"/>
-      <c r="I43" s="153"/>
-      <c r="J43" s="142" t="s">
-        <v>292</v>
-      </c>
-      <c r="K43" s="153"/>
-      <c r="L43" s="153"/>
-      <c r="M43" s="154" t="s">
+      <c r="G44" s="142" t="s">
+        <v>312</v>
+      </c>
+      <c r="H44" s="153"/>
+      <c r="I44" s="153"/>
+      <c r="J44" s="142" t="s">
+        <v>291</v>
+      </c>
+      <c r="K44" s="153"/>
+      <c r="L44" s="153"/>
+      <c r="M44" s="154" t="s">
         <v>197</v>
       </c>
-      <c r="N43"/>
-    </row>
-    <row r="44" spans="1:14" s="96" customFormat="1" ht="18" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="101"/>
-      <c r="B44" s="128" t="s">
-        <v>290</v>
-      </c>
-      <c r="C44" s="145" t="s">
+      <c r="N44"/>
+    </row>
+    <row r="45" spans="1:14" s="96" customFormat="1" ht="18" thickTop="1" x14ac:dyDescent="0.2">
+      <c r="A45" s="101"/>
+      <c r="B45" s="128" t="s">
+        <v>289</v>
+      </c>
+      <c r="C45" s="145" t="s">
         <v>13</v>
       </c>
-      <c r="D44" s="146">
-        <v>1</v>
-      </c>
-      <c r="E44" s="145" t="s">
+      <c r="D45" s="146">
+        <v>1</v>
+      </c>
+      <c r="E45" s="145" t="s">
         <v>14</v>
       </c>
-      <c r="F44" s="147" t="s">
-        <v>17</v>
-      </c>
-      <c r="G44" s="147"/>
-      <c r="H44" s="147"/>
-      <c r="I44" s="147"/>
-      <c r="J44" s="147"/>
-      <c r="K44" s="147"/>
-      <c r="L44" s="147"/>
-      <c r="M44" s="156" t="s">
+      <c r="F45" s="147" t="s">
+        <v>17</v>
+      </c>
+      <c r="G45" s="147"/>
+      <c r="H45" s="147"/>
+      <c r="I45" s="147"/>
+      <c r="J45" s="147"/>
+      <c r="K45" s="147"/>
+      <c r="L45" s="147"/>
+      <c r="M45" s="156" t="s">
         <v>16</v>
       </c>
-      <c r="N44"/>
-    </row>
-    <row r="45" spans="1:14" ht="17" x14ac:dyDescent="0.2">
-      <c r="A45" s="15"/>
-      <c r="B45" s="128" t="s">
-        <v>290</v>
-      </c>
-      <c r="C45" s="129" t="s">
-        <v>293</v>
-      </c>
-      <c r="D45" s="130">
-        <v>1</v>
-      </c>
-      <c r="E45" s="129" t="s">
-        <v>14</v>
-      </c>
-      <c r="F45" s="131" t="s">
-        <v>17</v>
-      </c>
-      <c r="G45" s="131"/>
-      <c r="H45" s="131"/>
-      <c r="I45" s="131"/>
-      <c r="J45" s="131"/>
-      <c r="K45" s="131"/>
-      <c r="L45" s="131"/>
-      <c r="M45" s="138" t="s">
-        <v>295</v>
-      </c>
+      <c r="N45"/>
     </row>
     <row r="46" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A46" s="15"/>
       <c r="B46" s="128" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="C46" s="129" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="D46" s="130">
         <v>1</v>
       </c>
       <c r="E46" s="129" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="F46" s="131" t="s">
         <v>17</v>
@@ -3926,142 +3937,142 @@
       <c r="K46" s="131"/>
       <c r="L46" s="131"/>
       <c r="M46" s="138" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
     </row>
     <row r="47" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A47" s="15"/>
-      <c r="B47" s="11" t="s">
-        <v>290</v>
-      </c>
-      <c r="C47" s="12" t="s">
+      <c r="B47" s="128" t="s">
+        <v>289</v>
+      </c>
+      <c r="C47" s="129" t="s">
+        <v>293</v>
+      </c>
+      <c r="D47" s="130">
+        <v>1</v>
+      </c>
+      <c r="E47" s="129" t="s">
+        <v>18</v>
+      </c>
+      <c r="F47" s="131" t="s">
+        <v>17</v>
+      </c>
+      <c r="G47" s="131"/>
+      <c r="H47" s="131"/>
+      <c r="I47" s="131"/>
+      <c r="J47" s="131"/>
+      <c r="K47" s="131"/>
+      <c r="L47" s="131"/>
+      <c r="M47" s="138" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="48" spans="1:14" ht="17" x14ac:dyDescent="0.2">
+      <c r="A48" s="15"/>
+      <c r="B48" s="11" t="s">
+        <v>289</v>
+      </c>
+      <c r="C48" s="12" t="s">
         <v>193</v>
       </c>
-      <c r="D47" s="13">
-        <v>1</v>
-      </c>
-      <c r="E47" s="12" t="s">
+      <c r="D48" s="13">
+        <v>1</v>
+      </c>
+      <c r="E48" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="F47" s="14" t="s">
+      <c r="F48" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="G47" s="14"/>
-      <c r="H47" s="14"/>
-      <c r="I47" s="14"/>
-      <c r="J47" s="14" t="s">
-        <v>292</v>
-      </c>
-      <c r="K47" s="14"/>
-      <c r="L47" s="14"/>
-      <c r="M47" s="117" t="s">
+      <c r="G48" s="14"/>
+      <c r="H48" s="14"/>
+      <c r="I48" s="14"/>
+      <c r="J48" s="14" t="s">
+        <v>291</v>
+      </c>
+      <c r="K48" s="14"/>
+      <c r="L48" s="14"/>
+      <c r="M48" s="117" t="s">
         <v>203</v>
       </c>
-    </row>
-    <row r="48" spans="1:14" s="96" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A48" s="101"/>
-      <c r="B48" s="97" t="s">
-        <v>290</v>
-      </c>
-      <c r="C48" s="102" t="s">
-        <v>162</v>
-      </c>
-      <c r="D48" s="157">
-        <v>1</v>
-      </c>
-      <c r="E48" s="102" t="s">
-        <v>14</v>
-      </c>
-      <c r="F48" s="103" t="s">
-        <v>15</v>
-      </c>
-      <c r="G48" s="103"/>
-      <c r="H48" s="103"/>
-      <c r="I48" s="103"/>
-      <c r="J48" s="103" t="s">
-        <v>292</v>
-      </c>
-      <c r="K48" s="103"/>
-      <c r="L48" s="103"/>
-      <c r="M48" s="158" t="s">
-        <v>204</v>
-      </c>
-      <c r="N48"/>
     </row>
     <row r="49" spans="1:14" s="96" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A49" s="101"/>
       <c r="B49" s="97" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="C49" s="102" t="s">
-        <v>207</v>
+        <v>162</v>
       </c>
       <c r="D49" s="157">
         <v>1</v>
       </c>
       <c r="E49" s="102" t="s">
-        <v>57</v>
+        <v>14</v>
       </c>
       <c r="F49" s="103" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="G49" s="103"/>
       <c r="H49" s="103"/>
       <c r="I49" s="103"/>
       <c r="J49" s="103" t="s">
-        <v>292</v>
-      </c>
-      <c r="K49" s="103" t="s">
+        <v>291</v>
+      </c>
+      <c r="K49" s="103"/>
+      <c r="L49" s="103"/>
+      <c r="M49" s="158" t="s">
+        <v>204</v>
+      </c>
+      <c r="N49"/>
+    </row>
+    <row r="50" spans="1:14" s="96" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A50" s="101"/>
+      <c r="B50" s="97" t="s">
+        <v>289</v>
+      </c>
+      <c r="C50" s="102" t="s">
+        <v>207</v>
+      </c>
+      <c r="D50" s="157">
+        <v>1</v>
+      </c>
+      <c r="E50" s="102" t="s">
+        <v>57</v>
+      </c>
+      <c r="F50" s="103" t="s">
+        <v>17</v>
+      </c>
+      <c r="G50" s="103"/>
+      <c r="H50" s="103"/>
+      <c r="I50" s="103"/>
+      <c r="J50" s="103" t="s">
+        <v>291</v>
+      </c>
+      <c r="K50" s="103" t="s">
         <v>20</v>
       </c>
-      <c r="L49" s="103" t="s">
+      <c r="L50" s="103" t="s">
         <v>232</v>
       </c>
-      <c r="M49" s="158" t="s">
+      <c r="M50" s="158" t="s">
         <v>206</v>
       </c>
-      <c r="N49"/>
-    </row>
-    <row r="50" spans="1:14" ht="17" x14ac:dyDescent="0.2">
-      <c r="A50" s="15"/>
-      <c r="B50" s="11" t="s">
-        <v>290</v>
-      </c>
-      <c r="C50" s="12" t="s">
-        <v>278</v>
-      </c>
-      <c r="D50" s="13">
-        <v>1</v>
-      </c>
-      <c r="E50" s="12" t="s">
-        <v>48</v>
-      </c>
-      <c r="F50" s="14" t="s">
-        <v>15</v>
-      </c>
-      <c r="G50" s="14"/>
-      <c r="H50" s="14"/>
-      <c r="I50" s="14"/>
-      <c r="J50" s="14"/>
-      <c r="K50" s="14"/>
-      <c r="L50" s="14"/>
-      <c r="M50" s="112" t="s">
-        <v>303</v>
-      </c>
+      <c r="N50"/>
     </row>
     <row r="51" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A51" s="15"/>
       <c r="B51" s="11" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="C51" s="12" t="s">
-        <v>301</v>
+        <v>277</v>
       </c>
       <c r="D51" s="13">
         <v>1</v>
       </c>
       <c r="E51" s="12" t="s">
-        <v>160</v>
+        <v>48</v>
       </c>
       <c r="F51" s="14" t="s">
         <v>15</v>
@@ -4069,9 +4080,7 @@
       <c r="G51" s="14"/>
       <c r="H51" s="14"/>
       <c r="I51" s="14"/>
-      <c r="J51" s="14" t="s">
-        <v>292</v>
-      </c>
+      <c r="J51" s="14"/>
       <c r="K51" s="14"/>
       <c r="L51" s="14"/>
       <c r="M51" s="112" t="s">
@@ -4081,45 +4090,45 @@
     <row r="52" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A52" s="15"/>
       <c r="B52" s="11" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="C52" s="12" t="s">
-        <v>234</v>
+        <v>300</v>
       </c>
       <c r="D52" s="13">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E52" s="12" t="s">
-        <v>14</v>
+        <v>160</v>
       </c>
       <c r="F52" s="14" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="G52" s="14"/>
       <c r="H52" s="14"/>
       <c r="I52" s="14"/>
       <c r="J52" s="14" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="K52" s="14"/>
       <c r="L52" s="14"/>
       <c r="M52" s="112" t="s">
-        <v>304</v>
-      </c>
-    </row>
-    <row r="53" spans="1:14" s="96" customFormat="1" x14ac:dyDescent="0.2">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="53" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A53" s="15"/>
       <c r="B53" s="11" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="C53" s="12" t="s">
-        <v>258</v>
+        <v>234</v>
       </c>
       <c r="D53" s="13">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E53" s="12" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="F53" s="14" t="s">
         <v>17</v>
@@ -4128,111 +4137,110 @@
       <c r="H53" s="14"/>
       <c r="I53" s="14"/>
       <c r="J53" s="14" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="K53" s="14"/>
       <c r="L53" s="14"/>
-      <c r="M53" s="118" t="s">
-        <v>205</v>
-      </c>
-      <c r="N53"/>
-    </row>
-    <row r="54" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="M53" s="112" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="54" spans="1:14" s="96" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A54" s="15"/>
       <c r="B54" s="11" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="C54" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="D54" s="13" t="s">
-        <v>310</v>
+        <v>257</v>
+      </c>
+      <c r="D54" s="13">
+        <v>1</v>
       </c>
       <c r="E54" s="12" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="F54" s="14" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G54" s="14"/>
       <c r="H54" s="14"/>
       <c r="I54" s="14"/>
       <c r="J54" s="14" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="K54" s="14"/>
       <c r="L54" s="14"/>
       <c r="M54" s="118" t="s">
-        <v>305</v>
-      </c>
+        <v>205</v>
+      </c>
+      <c r="N54"/>
     </row>
     <row r="55" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A55" s="96"/>
+      <c r="A55" s="15"/>
       <c r="B55" s="11" t="s">
-        <v>290</v>
-      </c>
-      <c r="C55" s="98" t="s">
-        <v>259</v>
-      </c>
-      <c r="D55" s="99">
-        <v>1</v>
-      </c>
-      <c r="E55" s="98" t="s">
+        <v>289</v>
+      </c>
+      <c r="C55" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="D55" s="13" t="s">
+        <v>309</v>
+      </c>
+      <c r="E55" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="F55" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="G55" s="14"/>
+      <c r="H55" s="14"/>
+      <c r="I55" s="14"/>
+      <c r="J55" s="14" t="s">
+        <v>291</v>
+      </c>
+      <c r="K55" s="14"/>
+      <c r="L55" s="14"/>
+      <c r="M55" s="118" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="56" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A56" s="96"/>
+      <c r="B56" s="11" t="s">
+        <v>289</v>
+      </c>
+      <c r="C56" s="98" t="s">
+        <v>258</v>
+      </c>
+      <c r="D56" s="99">
+        <v>1</v>
+      </c>
+      <c r="E56" s="98" t="s">
         <v>21</v>
       </c>
-      <c r="F55" s="100" t="s">
-        <v>17</v>
-      </c>
-      <c r="G55" s="100" t="s">
-        <v>314</v>
-      </c>
-      <c r="H55" s="100"/>
-      <c r="I55" s="100"/>
-      <c r="J55" s="14" t="s">
-        <v>292</v>
-      </c>
-      <c r="K55" s="100"/>
-      <c r="L55" s="100"/>
-      <c r="M55" s="119" t="s">
+      <c r="F56" s="100" t="s">
+        <v>17</v>
+      </c>
+      <c r="G56" s="100" t="s">
+        <v>313</v>
+      </c>
+      <c r="H56" s="100"/>
+      <c r="I56" s="100"/>
+      <c r="J56" s="14" t="s">
+        <v>291</v>
+      </c>
+      <c r="K56" s="100"/>
+      <c r="L56" s="100"/>
+      <c r="M56" s="119" t="s">
         <v>198</v>
-      </c>
-    </row>
-    <row r="56" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="B56" s="11" t="s">
-        <v>290</v>
-      </c>
-      <c r="C56" s="12" t="s">
-        <v>260</v>
-      </c>
-      <c r="D56" s="13">
-        <v>1</v>
-      </c>
-      <c r="E56" s="12" t="s">
-        <v>21</v>
-      </c>
-      <c r="F56" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="G56" s="14" t="s">
-        <v>314</v>
-      </c>
-      <c r="H56" s="14"/>
-      <c r="I56" s="14"/>
-      <c r="J56" s="14" t="s">
-        <v>292</v>
-      </c>
-      <c r="K56" s="14"/>
-      <c r="L56" s="14"/>
-      <c r="M56" s="120" t="s">
-        <v>199</v>
       </c>
     </row>
     <row r="57" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B57" s="11" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="C57" s="12" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="D57" s="13">
         <v>1</v>
@@ -4244,157 +4252,160 @@
         <v>17</v>
       </c>
       <c r="G57" s="14" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="H57" s="14"/>
       <c r="I57" s="14"/>
       <c r="J57" s="14" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="K57" s="14"/>
       <c r="L57" s="14"/>
-      <c r="M57" s="111" t="s">
+      <c r="M57" s="120" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="58" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B58" s="11" t="s">
+        <v>289</v>
+      </c>
+      <c r="C58" s="12" t="s">
+        <v>260</v>
+      </c>
+      <c r="D58" s="13">
+        <v>1</v>
+      </c>
+      <c r="E58" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="F58" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="G58" s="14" t="s">
+        <v>314</v>
+      </c>
+      <c r="H58" s="14"/>
+      <c r="I58" s="14"/>
+      <c r="J58" s="14" t="s">
+        <v>291</v>
+      </c>
+      <c r="K58" s="14"/>
+      <c r="L58" s="14"/>
+      <c r="M58" s="111" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="58" spans="1:14" s="96" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B58" s="97" t="s">
-        <v>290</v>
-      </c>
-      <c r="C58" s="102" t="s">
+    <row r="59" spans="1:14" s="96" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B59" s="97" t="s">
+        <v>289</v>
+      </c>
+      <c r="C59" s="102" t="s">
+        <v>261</v>
+      </c>
+      <c r="D59" s="157">
+        <v>1</v>
+      </c>
+      <c r="E59" s="102" t="s">
+        <v>21</v>
+      </c>
+      <c r="F59" s="103" t="s">
+        <v>17</v>
+      </c>
+      <c r="G59" s="103" t="s">
+        <v>314</v>
+      </c>
+      <c r="H59" s="103"/>
+      <c r="I59" s="103"/>
+      <c r="J59" s="103" t="s">
+        <v>291</v>
+      </c>
+      <c r="K59" s="103"/>
+      <c r="L59" s="103"/>
+      <c r="M59" s="159" t="s">
+        <v>201</v>
+      </c>
+      <c r="N59"/>
+    </row>
+    <row r="60" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B60" s="11" t="s">
+        <v>289</v>
+      </c>
+      <c r="C60" s="12" t="s">
         <v>262</v>
       </c>
-      <c r="D58" s="157">
-        <v>1</v>
-      </c>
-      <c r="E58" s="102" t="s">
-        <v>21</v>
-      </c>
-      <c r="F58" s="103" t="s">
-        <v>17</v>
-      </c>
-      <c r="G58" s="103" t="s">
-        <v>315</v>
-      </c>
-      <c r="H58" s="103"/>
-      <c r="I58" s="103"/>
-      <c r="J58" s="103" t="s">
-        <v>292</v>
-      </c>
-      <c r="K58" s="103"/>
-      <c r="L58" s="103"/>
-      <c r="M58" s="159" t="s">
-        <v>201</v>
-      </c>
-      <c r="N58"/>
-    </row>
-    <row r="59" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="B59" s="11" t="s">
-        <v>290</v>
-      </c>
-      <c r="C59" s="12" t="s">
-        <v>263</v>
-      </c>
-      <c r="D59" s="13">
-        <v>1</v>
-      </c>
-      <c r="E59" s="12" t="s">
+      <c r="D60" s="13">
+        <v>1</v>
+      </c>
+      <c r="E60" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="F59" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="G59" s="14"/>
-      <c r="H59" s="14"/>
-      <c r="I59" s="14" t="s">
+      <c r="F60" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="G60" s="14"/>
+      <c r="H60" s="14"/>
+      <c r="I60" s="14" t="s">
         <v>169</v>
       </c>
-      <c r="J59" s="14"/>
-      <c r="K59" s="14"/>
-      <c r="L59" s="14"/>
-      <c r="M59" s="121" t="s">
+      <c r="J60" s="14"/>
+      <c r="K60" s="14"/>
+      <c r="L60" s="14"/>
+      <c r="M60" s="121" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="60" spans="1:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="96"/>
-      <c r="B60" s="139" t="s">
-        <v>290</v>
-      </c>
-      <c r="C60" s="140" t="s">
+    <row r="61" spans="1:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A61" s="96"/>
+      <c r="B61" s="139" t="s">
+        <v>289</v>
+      </c>
+      <c r="C61" s="140" t="s">
+        <v>275</v>
+      </c>
+      <c r="D61" s="141">
+        <v>1</v>
+      </c>
+      <c r="E61" s="140" t="s">
+        <v>48</v>
+      </c>
+      <c r="F61" s="142" t="s">
+        <v>17</v>
+      </c>
+      <c r="G61" s="142"/>
+      <c r="H61" s="142"/>
+      <c r="I61" s="142"/>
+      <c r="J61" s="142"/>
+      <c r="K61" s="142"/>
+      <c r="L61" s="142"/>
+      <c r="M61" s="155" t="s">
         <v>276</v>
       </c>
-      <c r="D60" s="141">
-        <v>1</v>
-      </c>
-      <c r="E60" s="140" t="s">
-        <v>48</v>
-      </c>
-      <c r="F60" s="142" t="s">
-        <v>17</v>
-      </c>
-      <c r="G60" s="142"/>
-      <c r="H60" s="142"/>
-      <c r="I60" s="142"/>
-      <c r="J60" s="142"/>
-      <c r="K60" s="142"/>
-      <c r="L60" s="142"/>
-      <c r="M60" s="155" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="61" spans="1:14" ht="18" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A61" s="101"/>
-      <c r="B61" s="128" t="s">
-        <v>169</v>
-      </c>
-      <c r="C61" s="145" t="s">
-        <v>13</v>
-      </c>
-      <c r="D61" s="146">
-        <v>1</v>
-      </c>
-      <c r="E61" s="145" t="s">
-        <v>14</v>
-      </c>
-      <c r="F61" s="147" t="s">
-        <v>17</v>
-      </c>
-      <c r="G61" s="147"/>
-      <c r="H61" s="147"/>
-      <c r="I61" s="147"/>
-      <c r="J61" s="147"/>
-      <c r="K61" s="147"/>
-      <c r="L61" s="147"/>
-      <c r="M61" s="156" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="62" spans="1:14" ht="17" x14ac:dyDescent="0.2">
-      <c r="A62" s="15"/>
+    </row>
+    <row r="62" spans="1:14" ht="18" thickTop="1" x14ac:dyDescent="0.2">
+      <c r="A62" s="101"/>
       <c r="B62" s="128" t="s">
         <v>169</v>
       </c>
-      <c r="C62" s="129" t="s">
-        <v>293</v>
-      </c>
-      <c r="D62" s="130">
-        <v>1</v>
-      </c>
-      <c r="E62" s="129" t="s">
+      <c r="C62" s="145" t="s">
+        <v>13</v>
+      </c>
+      <c r="D62" s="146">
+        <v>1</v>
+      </c>
+      <c r="E62" s="145" t="s">
         <v>14</v>
       </c>
-      <c r="F62" s="131" t="s">
-        <v>17</v>
-      </c>
-      <c r="G62" s="131"/>
-      <c r="H62" s="131"/>
-      <c r="I62" s="131"/>
-      <c r="J62" s="131"/>
-      <c r="K62" s="131"/>
-      <c r="L62" s="131"/>
-      <c r="M62" s="138" t="s">
-        <v>295</v>
+      <c r="F62" s="147" t="s">
+        <v>17</v>
+      </c>
+      <c r="G62" s="147"/>
+      <c r="H62" s="147"/>
+      <c r="I62" s="147"/>
+      <c r="J62" s="147"/>
+      <c r="K62" s="147"/>
+      <c r="L62" s="147"/>
+      <c r="M62" s="156" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="63" spans="1:14" ht="17" x14ac:dyDescent="0.2">
@@ -4403,13 +4414,13 @@
         <v>169</v>
       </c>
       <c r="C63" s="129" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="D63" s="130">
         <v>1</v>
       </c>
       <c r="E63" s="129" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="F63" s="131" t="s">
         <v>17</v>
@@ -4421,35 +4432,34 @@
       <c r="K63" s="131"/>
       <c r="L63" s="131"/>
       <c r="M63" s="138" t="s">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="64" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="B64" s="11" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="64" spans="1:14" ht="17" x14ac:dyDescent="0.2">
+      <c r="A64" s="15"/>
+      <c r="B64" s="128" t="s">
         <v>169</v>
       </c>
-      <c r="C64" s="12" t="s">
-        <v>208</v>
-      </c>
-      <c r="D64" s="13">
-        <v>1</v>
-      </c>
-      <c r="E64" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="F64" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="G64" s="14"/>
-      <c r="H64" s="14"/>
-      <c r="I64" s="14"/>
-      <c r="J64" s="14" t="s">
-        <v>292</v>
-      </c>
-      <c r="K64" s="14"/>
-      <c r="L64" s="14"/>
-      <c r="M64" s="111" t="s">
-        <v>209</v>
+      <c r="C64" s="129" t="s">
+        <v>293</v>
+      </c>
+      <c r="D64" s="130">
+        <v>1</v>
+      </c>
+      <c r="E64" s="129" t="s">
+        <v>18</v>
+      </c>
+      <c r="F64" s="131" t="s">
+        <v>17</v>
+      </c>
+      <c r="G64" s="131"/>
+      <c r="H64" s="131"/>
+      <c r="I64" s="131"/>
+      <c r="J64" s="131"/>
+      <c r="K64" s="131"/>
+      <c r="L64" s="131"/>
+      <c r="M64" s="138" t="s">
+        <v>295</v>
       </c>
     </row>
     <row r="65" spans="1:14" x14ac:dyDescent="0.2">
@@ -4457,7 +4467,7 @@
         <v>169</v>
       </c>
       <c r="C65" s="12" t="s">
-        <v>192</v>
+        <v>208</v>
       </c>
       <c r="D65" s="13">
         <v>1</v>
@@ -4472,12 +4482,12 @@
       <c r="H65" s="14"/>
       <c r="I65" s="14"/>
       <c r="J65" s="14" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="K65" s="14"/>
       <c r="L65" s="14"/>
-      <c r="M65" s="121" t="s">
-        <v>210</v>
+      <c r="M65" s="111" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="66" spans="1:14" x14ac:dyDescent="0.2">
@@ -4485,25 +4495,27 @@
         <v>169</v>
       </c>
       <c r="C66" s="12" t="s">
-        <v>279</v>
+        <v>192</v>
       </c>
       <c r="D66" s="13">
         <v>1</v>
       </c>
       <c r="E66" s="12" t="s">
-        <v>48</v>
+        <v>14</v>
       </c>
       <c r="F66" s="14" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G66" s="14"/>
       <c r="H66" s="14"/>
       <c r="I66" s="14"/>
-      <c r="J66" s="14"/>
+      <c r="J66" s="14" t="s">
+        <v>291</v>
+      </c>
       <c r="K66" s="14"/>
       <c r="L66" s="14"/>
-      <c r="M66" s="159" t="s">
-        <v>281</v>
+      <c r="M66" s="121" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="67" spans="1:14" x14ac:dyDescent="0.2">
@@ -4511,31 +4523,25 @@
         <v>169</v>
       </c>
       <c r="C67" s="12" t="s">
-        <v>264</v>
+        <v>278</v>
       </c>
       <c r="D67" s="13">
         <v>1</v>
       </c>
       <c r="E67" s="12" t="s">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="F67" s="14" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="G67" s="14"/>
       <c r="H67" s="14"/>
       <c r="I67" s="14"/>
-      <c r="J67" s="14" t="s">
+      <c r="J67" s="14"/>
+      <c r="K67" s="14"/>
+      <c r="L67" s="14"/>
+      <c r="M67" s="159" t="s">
         <v>280</v>
-      </c>
-      <c r="K67" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="L67" s="14" t="s">
-        <v>306</v>
-      </c>
-      <c r="M67" s="111" t="s">
-        <v>211</v>
       </c>
     </row>
     <row r="68" spans="1:14" x14ac:dyDescent="0.2">
@@ -4543,27 +4549,31 @@
         <v>169</v>
       </c>
       <c r="C68" s="12" t="s">
-        <v>170</v>
+        <v>263</v>
       </c>
       <c r="D68" s="13">
         <v>1</v>
       </c>
-      <c r="E68" s="102" t="s">
-        <v>24</v>
+      <c r="E68" s="12" t="s">
+        <v>57</v>
       </c>
       <c r="F68" s="14" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G68" s="14"/>
       <c r="H68" s="14"/>
       <c r="I68" s="14"/>
       <c r="J68" s="14" t="s">
-        <v>280</v>
-      </c>
-      <c r="K68" s="14"/>
-      <c r="L68" s="14"/>
-      <c r="M68" s="122" t="s">
-        <v>212</v>
+        <v>279</v>
+      </c>
+      <c r="K68" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="L68" s="14" t="s">
+        <v>305</v>
+      </c>
+      <c r="M68" s="111" t="s">
+        <v>211</v>
       </c>
     </row>
     <row r="69" spans="1:14" x14ac:dyDescent="0.2">
@@ -4571,29 +4581,27 @@
         <v>169</v>
       </c>
       <c r="C69" s="12" t="s">
-        <v>265</v>
+        <v>170</v>
       </c>
       <c r="D69" s="13">
         <v>1</v>
       </c>
-      <c r="E69" s="12" t="s">
-        <v>21</v>
+      <c r="E69" s="102" t="s">
+        <v>24</v>
       </c>
       <c r="F69" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="G69" s="14" t="s">
-        <v>316</v>
-      </c>
+      <c r="G69" s="14"/>
       <c r="H69" s="14"/>
       <c r="I69" s="14"/>
       <c r="J69" s="14" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="K69" s="14"/>
       <c r="L69" s="14"/>
-      <c r="M69" s="111" t="s">
-        <v>213</v>
+      <c r="M69" s="122" t="s">
+        <v>212</v>
       </c>
     </row>
     <row r="70" spans="1:14" x14ac:dyDescent="0.2">
@@ -4601,94 +4609,96 @@
         <v>169</v>
       </c>
       <c r="C70" s="12" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="D70" s="13">
         <v>1</v>
       </c>
       <c r="E70" s="12" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F70" s="14" t="s">
         <v>15</v>
       </c>
       <c r="G70" s="14" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="H70" s="14"/>
       <c r="I70" s="14"/>
       <c r="J70" s="14" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="K70" s="14"/>
       <c r="L70" s="14"/>
-      <c r="M70" s="121" t="s">
+      <c r="M70" s="111" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="71" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B71" s="11" t="s">
+        <v>169</v>
+      </c>
+      <c r="C71" s="12" t="s">
+        <v>265</v>
+      </c>
+      <c r="D71" s="13">
+        <v>1</v>
+      </c>
+      <c r="E71" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="F71" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="G71" s="14" t="s">
+        <v>315</v>
+      </c>
+      <c r="H71" s="14"/>
+      <c r="I71" s="14"/>
+      <c r="J71" s="14" t="s">
+        <v>279</v>
+      </c>
+      <c r="K71" s="14"/>
+      <c r="L71" s="14"/>
+      <c r="M71" s="121" t="s">
         <v>214</v>
       </c>
     </row>
-    <row r="71" spans="1:14" s="96" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B71" s="97" t="s">
+    <row r="72" spans="1:14" s="96" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B72" s="97" t="s">
         <v>169</v>
       </c>
-      <c r="C71" s="102" t="s">
+      <c r="C72" s="102" t="s">
         <v>171</v>
       </c>
-      <c r="D71" s="157">
-        <v>1</v>
-      </c>
-      <c r="E71" s="102" t="s">
-        <v>24</v>
-      </c>
-      <c r="F71" s="103" t="s">
-        <v>15</v>
-      </c>
-      <c r="G71" s="103"/>
-      <c r="H71" s="103"/>
-      <c r="I71" s="103"/>
-      <c r="J71" s="103" t="s">
-        <v>280</v>
-      </c>
-      <c r="K71" s="103"/>
-      <c r="L71" s="103"/>
-      <c r="M71" s="161" t="s">
-        <v>215</v>
-      </c>
-      <c r="N71"/>
-    </row>
-    <row r="72" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="B72" s="11" t="s">
-        <v>169</v>
-      </c>
-      <c r="C72" s="12" t="s">
-        <v>172</v>
-      </c>
-      <c r="D72" s="13">
+      <c r="D72" s="157">
         <v>1</v>
       </c>
       <c r="E72" s="102" t="s">
         <v>24</v>
       </c>
-      <c r="F72" s="14" t="s">
+      <c r="F72" s="103" t="s">
         <v>15</v>
       </c>
-      <c r="G72" s="14"/>
-      <c r="H72" s="14"/>
-      <c r="I72" s="14"/>
-      <c r="J72" s="14" t="s">
-        <v>280</v>
-      </c>
-      <c r="K72" s="14"/>
-      <c r="L72" s="14"/>
-      <c r="M72" s="121" t="s">
-        <v>218</v>
-      </c>
+      <c r="G72" s="103"/>
+      <c r="H72" s="103"/>
+      <c r="I72" s="103"/>
+      <c r="J72" s="103" t="s">
+        <v>279</v>
+      </c>
+      <c r="K72" s="103"/>
+      <c r="L72" s="103"/>
+      <c r="M72" s="161" t="s">
+        <v>215</v>
+      </c>
+      <c r="N72"/>
     </row>
     <row r="73" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B73" s="11" t="s">
         <v>169</v>
       </c>
       <c r="C73" s="12" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D73" s="13">
         <v>1</v>
@@ -4703,12 +4713,12 @@
       <c r="H73" s="14"/>
       <c r="I73" s="14"/>
       <c r="J73" s="14" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="K73" s="14"/>
       <c r="L73" s="14"/>
-      <c r="M73" s="111" t="s">
-        <v>219</v>
+      <c r="M73" s="121" t="s">
+        <v>218</v>
       </c>
     </row>
     <row r="74" spans="1:14" x14ac:dyDescent="0.2">
@@ -4716,113 +4726,114 @@
         <v>169</v>
       </c>
       <c r="C74" s="12" t="s">
-        <v>267</v>
+        <v>173</v>
       </c>
       <c r="D74" s="13">
         <v>1</v>
       </c>
-      <c r="E74" s="12" t="s">
-        <v>21</v>
+      <c r="E74" s="102" t="s">
+        <v>24</v>
       </c>
       <c r="F74" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="G74" s="14" t="s">
-        <v>316</v>
-      </c>
+      <c r="G74" s="14"/>
       <c r="H74" s="14"/>
       <c r="I74" s="14"/>
       <c r="J74" s="14" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="K74" s="14"/>
       <c r="L74" s="14"/>
       <c r="M74" s="111" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="75" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B75" s="11" t="s">
+        <v>169</v>
+      </c>
+      <c r="C75" s="12" t="s">
+        <v>266</v>
+      </c>
+      <c r="D75" s="13">
+        <v>1</v>
+      </c>
+      <c r="E75" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="F75" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="G75" s="14" t="s">
+        <v>315</v>
+      </c>
+      <c r="H75" s="14"/>
+      <c r="I75" s="14"/>
+      <c r="J75" s="14" t="s">
+        <v>279</v>
+      </c>
+      <c r="K75" s="14"/>
+      <c r="L75" s="14"/>
+      <c r="M75" s="111" t="s">
         <v>216</v>
       </c>
     </row>
-    <row r="75" spans="1:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B75" s="139" t="s">
+    <row r="76" spans="1:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B76" s="139" t="s">
         <v>169</v>
       </c>
-      <c r="C75" s="140" t="s">
-        <v>268</v>
-      </c>
-      <c r="D75" s="141">
-        <v>1</v>
-      </c>
-      <c r="E75" s="140" t="s">
+      <c r="C76" s="140" t="s">
+        <v>267</v>
+      </c>
+      <c r="D76" s="141">
+        <v>1</v>
+      </c>
+      <c r="E76" s="140" t="s">
         <v>21</v>
       </c>
-      <c r="F75" s="142" t="s">
+      <c r="F76" s="142" t="s">
         <v>15</v>
       </c>
-      <c r="G75" s="142" t="s">
-        <v>317</v>
-      </c>
-      <c r="H75" s="142"/>
-      <c r="I75" s="142"/>
-      <c r="J75" s="142" t="s">
-        <v>280</v>
-      </c>
-      <c r="K75" s="142"/>
-      <c r="L75" s="142"/>
-      <c r="M75" s="160" t="s">
+      <c r="G76" s="142" t="s">
+        <v>316</v>
+      </c>
+      <c r="H76" s="142"/>
+      <c r="I76" s="142"/>
+      <c r="J76" s="142" t="s">
+        <v>279</v>
+      </c>
+      <c r="K76" s="142"/>
+      <c r="L76" s="142"/>
+      <c r="M76" s="160" t="s">
         <v>217</v>
       </c>
     </row>
-    <row r="76" spans="1:14" ht="18" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A76" s="96"/>
-      <c r="B76" s="128" t="s">
-        <v>174</v>
-      </c>
-      <c r="C76" s="145" t="s">
-        <v>13</v>
-      </c>
-      <c r="D76" s="146">
-        <v>1</v>
-      </c>
-      <c r="E76" s="145" t="s">
-        <v>14</v>
-      </c>
-      <c r="F76" s="147" t="s">
-        <v>15</v>
-      </c>
-      <c r="G76" s="147"/>
-      <c r="H76" s="147"/>
-      <c r="I76" s="147"/>
-      <c r="J76" s="147"/>
-      <c r="K76" s="147"/>
-      <c r="L76" s="147"/>
-      <c r="M76" s="138" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="77" spans="1:14" ht="17" x14ac:dyDescent="0.2">
-      <c r="A77" s="101"/>
+    <row r="77" spans="1:14" ht="18" thickTop="1" x14ac:dyDescent="0.2">
+      <c r="A77" s="96"/>
       <c r="B77" s="128" t="s">
         <v>174</v>
       </c>
-      <c r="C77" s="129" t="s">
-        <v>293</v>
-      </c>
-      <c r="D77" s="130">
-        <v>1</v>
-      </c>
-      <c r="E77" s="129" t="s">
+      <c r="C77" s="145" t="s">
+        <v>13</v>
+      </c>
+      <c r="D77" s="146">
+        <v>1</v>
+      </c>
+      <c r="E77" s="145" t="s">
         <v>14</v>
       </c>
-      <c r="F77" s="131" t="s">
-        <v>17</v>
-      </c>
-      <c r="G77" s="131"/>
-      <c r="H77" s="131"/>
-      <c r="I77" s="131"/>
-      <c r="J77" s="131"/>
-      <c r="K77" s="131"/>
-      <c r="L77" s="131"/>
+      <c r="F77" s="147" t="s">
+        <v>15</v>
+      </c>
+      <c r="G77" s="147"/>
+      <c r="H77" s="147"/>
+      <c r="I77" s="147"/>
+      <c r="J77" s="147"/>
+      <c r="K77" s="147"/>
+      <c r="L77" s="147"/>
       <c r="M77" s="138" t="s">
-        <v>295</v>
+        <v>16</v>
       </c>
     </row>
     <row r="78" spans="1:14" ht="17" x14ac:dyDescent="0.2">
@@ -4831,13 +4842,13 @@
         <v>174</v>
       </c>
       <c r="C78" s="129" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="D78" s="130">
         <v>1</v>
       </c>
       <c r="E78" s="129" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="F78" s="131" t="s">
         <v>17</v>
@@ -4849,44 +4860,43 @@
       <c r="K78" s="131"/>
       <c r="L78" s="131"/>
       <c r="M78" s="138" t="s">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="79" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A79" s="96"/>
-      <c r="B79" s="11" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="79" spans="1:14" ht="17" x14ac:dyDescent="0.2">
+      <c r="A79" s="101"/>
+      <c r="B79" s="128" t="s">
         <v>174</v>
       </c>
-      <c r="C79" s="12" t="s">
-        <v>175</v>
-      </c>
-      <c r="D79" s="13">
-        <v>1</v>
-      </c>
-      <c r="E79" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="F79" s="14" t="s">
-        <v>15</v>
-      </c>
-      <c r="G79" s="14"/>
-      <c r="H79" s="14"/>
-      <c r="I79" s="14"/>
-      <c r="J79" s="14" t="s">
-        <v>286</v>
-      </c>
-      <c r="K79" s="14"/>
-      <c r="L79" s="14"/>
-      <c r="M79" s="121" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="80" spans="1:14" s="96" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="C79" s="129" t="s">
+        <v>293</v>
+      </c>
+      <c r="D79" s="130">
+        <v>1</v>
+      </c>
+      <c r="E79" s="129" t="s">
+        <v>18</v>
+      </c>
+      <c r="F79" s="131" t="s">
+        <v>17</v>
+      </c>
+      <c r="G79" s="131"/>
+      <c r="H79" s="131"/>
+      <c r="I79" s="131"/>
+      <c r="J79" s="131"/>
+      <c r="K79" s="131"/>
+      <c r="L79" s="131"/>
+      <c r="M79" s="138" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="80" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A80" s="96"/>
       <c r="B80" s="11" t="s">
         <v>174</v>
       </c>
       <c r="C80" s="12" t="s">
-        <v>12</v>
+        <v>175</v>
       </c>
       <c r="D80" s="13">
         <v>1</v>
@@ -4901,202 +4911,203 @@
       <c r="H80" s="14"/>
       <c r="I80" s="14"/>
       <c r="J80" s="14" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="K80" s="14"/>
       <c r="L80" s="14"/>
-      <c r="M80" s="111" t="s">
-        <v>224</v>
-      </c>
-      <c r="N80"/>
-    </row>
-    <row r="81" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A81" s="96"/>
+      <c r="M80" s="121" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="81" spans="1:14" s="96" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B81" s="11" t="s">
         <v>174</v>
       </c>
       <c r="C81" s="12" t="s">
-        <v>269</v>
+        <v>12</v>
       </c>
       <c r="D81" s="13">
         <v>1</v>
       </c>
       <c r="E81" s="12" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="F81" s="14" t="s">
         <v>15</v>
       </c>
       <c r="G81" s="14"/>
       <c r="H81" s="14"/>
-      <c r="I81" s="14" t="s">
-        <v>291</v>
-      </c>
-      <c r="J81" s="14"/>
+      <c r="I81" s="14"/>
+      <c r="J81" s="14" t="s">
+        <v>285</v>
+      </c>
       <c r="K81" s="14"/>
       <c r="L81" s="14"/>
       <c r="M81" s="111" t="s">
-        <v>225</v>
-      </c>
+        <v>224</v>
+      </c>
+      <c r="N81"/>
     </row>
     <row r="82" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A82" s="96"/>
-      <c r="B82" s="97" t="s">
+      <c r="B82" s="11" t="s">
         <v>174</v>
       </c>
-      <c r="C82" s="102" t="s">
-        <v>270</v>
-      </c>
-      <c r="D82" s="157">
-        <v>1</v>
-      </c>
-      <c r="E82" s="102" t="s">
-        <v>57</v>
-      </c>
-      <c r="F82" s="103" t="s">
+      <c r="C82" s="12" t="s">
+        <v>268</v>
+      </c>
+      <c r="D82" s="13">
+        <v>1</v>
+      </c>
+      <c r="E82" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="F82" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="G82" s="103"/>
-      <c r="H82" s="103"/>
-      <c r="I82" s="103"/>
-      <c r="J82" s="103" t="s">
-        <v>286</v>
-      </c>
-      <c r="K82" s="103" t="s">
-        <v>20</v>
-      </c>
-      <c r="L82" s="103" t="s">
-        <v>231</v>
-      </c>
-      <c r="M82" s="161" t="s">
-        <v>226</v>
+      <c r="G82" s="14"/>
+      <c r="H82" s="14"/>
+      <c r="I82" s="14" t="s">
+        <v>290</v>
+      </c>
+      <c r="J82" s="14"/>
+      <c r="K82" s="14"/>
+      <c r="L82" s="14"/>
+      <c r="M82" s="111" t="s">
+        <v>225</v>
       </c>
     </row>
     <row r="83" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A83" s="96"/>
-      <c r="B83" s="11" t="s">
+      <c r="B83" s="97" t="s">
         <v>174</v>
       </c>
-      <c r="C83" s="12" t="s">
-        <v>271</v>
-      </c>
-      <c r="D83" s="13">
+      <c r="C83" s="102" t="s">
+        <v>269</v>
+      </c>
+      <c r="D83" s="157">
         <v>1</v>
       </c>
       <c r="E83" s="102" t="s">
+        <v>57</v>
+      </c>
+      <c r="F83" s="103" t="s">
+        <v>15</v>
+      </c>
+      <c r="G83" s="103"/>
+      <c r="H83" s="103"/>
+      <c r="I83" s="103"/>
+      <c r="J83" s="103" t="s">
+        <v>285</v>
+      </c>
+      <c r="K83" s="103" t="s">
+        <v>20</v>
+      </c>
+      <c r="L83" s="103" t="s">
+        <v>231</v>
+      </c>
+      <c r="M83" s="161" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="84" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A84" s="96"/>
+      <c r="B84" s="11" t="s">
+        <v>174</v>
+      </c>
+      <c r="C84" s="12" t="s">
+        <v>270</v>
+      </c>
+      <c r="D84" s="13">
+        <v>1</v>
+      </c>
+      <c r="E84" s="102" t="s">
         <v>24</v>
       </c>
-      <c r="F83" s="14" t="s">
+      <c r="F84" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="G83" s="14"/>
-      <c r="H83" s="14"/>
-      <c r="I83" s="14"/>
-      <c r="J83" s="14" t="s">
-        <v>286</v>
-      </c>
-      <c r="K83" s="14"/>
-      <c r="L83" s="14"/>
-      <c r="M83" s="121" t="s">
+      <c r="G84" s="14"/>
+      <c r="H84" s="14"/>
+      <c r="I84" s="14"/>
+      <c r="J84" s="14" t="s">
+        <v>285</v>
+      </c>
+      <c r="K84" s="14"/>
+      <c r="L84" s="14"/>
+      <c r="M84" s="121" t="s">
         <v>227</v>
       </c>
     </row>
-    <row r="84" spans="1:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A84" s="96"/>
-      <c r="B84" s="139" t="s">
+    <row r="85" spans="1:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A85" s="96"/>
+      <c r="B85" s="139" t="s">
         <v>174</v>
       </c>
-      <c r="C84" s="140" t="s">
-        <v>279</v>
-      </c>
-      <c r="D84" s="141">
-        <v>1</v>
-      </c>
-      <c r="E84" s="140" t="s">
+      <c r="C85" s="140" t="s">
+        <v>278</v>
+      </c>
+      <c r="D85" s="141">
+        <v>1</v>
+      </c>
+      <c r="E85" s="140" t="s">
         <v>48</v>
       </c>
-      <c r="F84" s="142" t="s">
-        <v>17</v>
-      </c>
-      <c r="G84" s="142"/>
-      <c r="H84" s="142" t="s">
-        <v>285</v>
-      </c>
-      <c r="I84" s="142"/>
-      <c r="J84" s="142"/>
-      <c r="K84" s="142"/>
-      <c r="L84" s="142"/>
-      <c r="M84" s="160" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="85" spans="1:14" s="96" customFormat="1" ht="18" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="B85" s="128" t="s">
-        <v>282</v>
-      </c>
-      <c r="C85" s="145" t="s">
+      <c r="F85" s="142" t="s">
+        <v>17</v>
+      </c>
+      <c r="G85" s="142"/>
+      <c r="H85" s="142" t="s">
+        <v>284</v>
+      </c>
+      <c r="I85" s="142"/>
+      <c r="J85" s="142"/>
+      <c r="K85" s="142"/>
+      <c r="L85" s="142"/>
+      <c r="M85" s="160" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="86" spans="1:14" s="96" customFormat="1" ht="18" thickTop="1" x14ac:dyDescent="0.2">
+      <c r="B86" s="128" t="s">
+        <v>281</v>
+      </c>
+      <c r="C86" s="145" t="s">
         <v>13</v>
       </c>
-      <c r="D85" s="146">
-        <v>1</v>
-      </c>
-      <c r="E85" s="145" t="s">
+      <c r="D86" s="146">
+        <v>1</v>
+      </c>
+      <c r="E86" s="145" t="s">
         <v>14</v>
       </c>
-      <c r="F85" s="147" t="s">
+      <c r="F86" s="147" t="s">
         <v>15</v>
       </c>
-      <c r="G85" s="147"/>
-      <c r="H85" s="147"/>
-      <c r="I85" s="147"/>
-      <c r="J85" s="147"/>
-      <c r="K85" s="147"/>
-      <c r="L85" s="147"/>
-      <c r="M85" s="138" t="s">
+      <c r="G86" s="147"/>
+      <c r="H86" s="147"/>
+      <c r="I86" s="147"/>
+      <c r="J86" s="147"/>
+      <c r="K86" s="147"/>
+      <c r="L86" s="147"/>
+      <c r="M86" s="138" t="s">
         <v>16</v>
       </c>
-      <c r="N85"/>
-    </row>
-    <row r="86" spans="1:14" ht="17" x14ac:dyDescent="0.2">
-      <c r="A86" s="15"/>
-      <c r="B86" s="128" t="s">
-        <v>282</v>
-      </c>
-      <c r="C86" s="129" t="s">
-        <v>293</v>
-      </c>
-      <c r="D86" s="130">
-        <v>1</v>
-      </c>
-      <c r="E86" s="129" t="s">
-        <v>14</v>
-      </c>
-      <c r="F86" s="131" t="s">
-        <v>17</v>
-      </c>
-      <c r="G86" s="131"/>
-      <c r="H86" s="131"/>
-      <c r="I86" s="131"/>
-      <c r="J86" s="131"/>
-      <c r="K86" s="131"/>
-      <c r="L86" s="131"/>
-      <c r="M86" s="138" t="s">
-        <v>295</v>
-      </c>
+      <c r="N86"/>
     </row>
     <row r="87" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A87" s="15"/>
       <c r="B87" s="128" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="C87" s="129" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="D87" s="130">
         <v>1</v>
       </c>
       <c r="E87" s="129" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="F87" s="131" t="s">
         <v>17</v>
@@ -5108,100 +5119,99 @@
       <c r="K87" s="131"/>
       <c r="L87" s="131"/>
       <c r="M87" s="138" t="s">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="88" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="B88" s="97" t="s">
-        <v>282</v>
-      </c>
-      <c r="C88" s="12" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="88" spans="1:14" ht="17" x14ac:dyDescent="0.2">
+      <c r="A88" s="15"/>
+      <c r="B88" s="128" t="s">
+        <v>281</v>
+      </c>
+      <c r="C88" s="129" t="s">
+        <v>293</v>
+      </c>
+      <c r="D88" s="130">
+        <v>1</v>
+      </c>
+      <c r="E88" s="129" t="s">
+        <v>18</v>
+      </c>
+      <c r="F88" s="131" t="s">
+        <v>17</v>
+      </c>
+      <c r="G88" s="131"/>
+      <c r="H88" s="131"/>
+      <c r="I88" s="131"/>
+      <c r="J88" s="131"/>
+      <c r="K88" s="131"/>
+      <c r="L88" s="131"/>
+      <c r="M88" s="138" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="89" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B89" s="97" t="s">
+        <v>281</v>
+      </c>
+      <c r="C89" s="12" t="s">
+        <v>271</v>
+      </c>
+      <c r="D89" s="13">
+        <v>1</v>
+      </c>
+      <c r="E89" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="F89" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="G89" s="14"/>
+      <c r="H89" s="14"/>
+      <c r="I89" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="J89" s="14"/>
+      <c r="K89" s="14"/>
+      <c r="L89" s="14"/>
+      <c r="M89" s="111" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="90" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A90" s="96"/>
+      <c r="B90" s="97" t="s">
+        <v>281</v>
+      </c>
+      <c r="C90" s="102" t="s">
         <v>272</v>
       </c>
-      <c r="D88" s="13">
-        <v>1</v>
-      </c>
-      <c r="E88" s="12" t="s">
+      <c r="D90" s="157">
+        <v>1</v>
+      </c>
+      <c r="E90" s="102" t="s">
         <v>19</v>
       </c>
-      <c r="F88" s="14" t="s">
+      <c r="F90" s="103" t="s">
         <v>15</v>
       </c>
-      <c r="G88" s="14"/>
-      <c r="H88" s="14"/>
-      <c r="I88" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="J88" s="14"/>
-      <c r="K88" s="14"/>
-      <c r="L88" s="14"/>
-      <c r="M88" s="111" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="89" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A89" s="96"/>
-      <c r="B89" s="97" t="s">
-        <v>282</v>
-      </c>
-      <c r="C89" s="102" t="s">
-        <v>273</v>
-      </c>
-      <c r="D89" s="157">
-        <v>1</v>
-      </c>
-      <c r="E89" s="102" t="s">
-        <v>19</v>
-      </c>
-      <c r="F89" s="103" t="s">
-        <v>15</v>
-      </c>
-      <c r="G89" s="103"/>
-      <c r="H89" s="103"/>
-      <c r="I89" s="103" t="s">
+      <c r="G90" s="103"/>
+      <c r="H90" s="103"/>
+      <c r="I90" s="103" t="s">
         <v>174</v>
       </c>
-      <c r="J89" s="103"/>
-      <c r="K89" s="103"/>
-      <c r="L89" s="103"/>
-      <c r="M89" s="161" t="s">
+      <c r="J90" s="103"/>
+      <c r="K90" s="103"/>
+      <c r="L90" s="103"/>
+      <c r="M90" s="161" t="s">
         <v>229</v>
-      </c>
-    </row>
-    <row r="90" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="B90" s="97" t="s">
-        <v>282</v>
-      </c>
-      <c r="C90" s="12" t="s">
-        <v>283</v>
-      </c>
-      <c r="D90" s="13">
-        <v>1</v>
-      </c>
-      <c r="E90" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="F90" s="14" t="s">
-        <v>15</v>
-      </c>
-      <c r="G90" s="14"/>
-      <c r="H90" s="14"/>
-      <c r="I90" s="14"/>
-      <c r="J90" s="14" t="s">
-        <v>287</v>
-      </c>
-      <c r="K90" s="14"/>
-      <c r="L90" s="14"/>
-      <c r="M90" s="111" t="s">
-        <v>284</v>
       </c>
     </row>
     <row r="91" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B91" s="97" t="s">
+        <v>281</v>
+      </c>
+      <c r="C91" s="12" t="s">
         <v>282</v>
-      </c>
-      <c r="C91" s="12" t="s">
-        <v>176</v>
       </c>
       <c r="D91" s="13">
         <v>1</v>
@@ -5216,109 +5226,110 @@
       <c r="H91" s="14"/>
       <c r="I91" s="14"/>
       <c r="J91" s="14" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="K91" s="14"/>
       <c r="L91" s="14"/>
-      <c r="M91" s="121" t="s">
+      <c r="M91" s="111" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="92" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B92" s="97" t="s">
+        <v>281</v>
+      </c>
+      <c r="C92" s="12" t="s">
+        <v>176</v>
+      </c>
+      <c r="D92" s="13">
+        <v>1</v>
+      </c>
+      <c r="E92" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="F92" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="G92" s="14"/>
+      <c r="H92" s="14"/>
+      <c r="I92" s="14"/>
+      <c r="J92" s="14" t="s">
+        <v>286</v>
+      </c>
+      <c r="K92" s="14"/>
+      <c r="L92" s="14"/>
+      <c r="M92" s="121" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="92" spans="1:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B92" s="148" t="s">
-        <v>282</v>
-      </c>
-      <c r="C92" s="140" t="s">
-        <v>279</v>
-      </c>
-      <c r="D92" s="141">
-        <v>1</v>
-      </c>
-      <c r="E92" s="140" t="s">
+    <row r="93" spans="1:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B93" s="148" t="s">
+        <v>281</v>
+      </c>
+      <c r="C93" s="140" t="s">
+        <v>278</v>
+      </c>
+      <c r="D93" s="141">
+        <v>1</v>
+      </c>
+      <c r="E93" s="140" t="s">
         <v>48</v>
       </c>
-      <c r="F92" s="142" t="s">
-        <v>17</v>
-      </c>
-      <c r="G92" s="142"/>
-      <c r="H92" s="142" t="s">
-        <v>285</v>
-      </c>
-      <c r="I92" s="142"/>
-      <c r="J92" s="142"/>
-      <c r="K92" s="142"/>
-      <c r="L92" s="142"/>
-      <c r="M92" s="160" t="s">
-        <v>308</v>
-      </c>
-    </row>
-    <row r="93" spans="1:14" ht="17" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A93" s="104"/>
-      <c r="B93" s="128" t="s">
-        <v>291</v>
-      </c>
-      <c r="C93" s="145" t="s">
+      <c r="F93" s="142" t="s">
+        <v>17</v>
+      </c>
+      <c r="G93" s="142"/>
+      <c r="H93" s="142" t="s">
+        <v>284</v>
+      </c>
+      <c r="I93" s="142"/>
+      <c r="J93" s="142"/>
+      <c r="K93" s="142"/>
+      <c r="L93" s="142"/>
+      <c r="M93" s="160" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="94" spans="1:14" ht="17" thickTop="1" x14ac:dyDescent="0.2">
+      <c r="A94" s="104"/>
+      <c r="B94" s="128" t="s">
+        <v>290</v>
+      </c>
+      <c r="C94" s="145" t="s">
         <v>13</v>
       </c>
-      <c r="D93" s="146">
-        <v>1</v>
-      </c>
-      <c r="E93" s="145" t="s">
+      <c r="D94" s="146">
+        <v>1</v>
+      </c>
+      <c r="E94" s="145" t="s">
         <v>14</v>
       </c>
-      <c r="F93" s="147" t="s">
+      <c r="F94" s="147" t="s">
         <v>15</v>
       </c>
-      <c r="G93" s="147"/>
-      <c r="H93" s="147"/>
-      <c r="I93" s="147"/>
-      <c r="J93" s="147"/>
-      <c r="K93" s="147"/>
-      <c r="L93" s="147"/>
-      <c r="M93" s="132" t="s">
+      <c r="G94" s="147"/>
+      <c r="H94" s="147"/>
+      <c r="I94" s="147"/>
+      <c r="J94" s="147"/>
+      <c r="K94" s="147"/>
+      <c r="L94" s="147"/>
+      <c r="M94" s="132" t="s">
         <v>16</v>
-      </c>
-    </row>
-    <row r="94" spans="1:14" ht="17" x14ac:dyDescent="0.2">
-      <c r="A94" s="15"/>
-      <c r="B94" s="128" t="s">
-        <v>291</v>
-      </c>
-      <c r="C94" s="129" t="s">
-        <v>293</v>
-      </c>
-      <c r="D94" s="130">
-        <v>1</v>
-      </c>
-      <c r="E94" s="129" t="s">
-        <v>14</v>
-      </c>
-      <c r="F94" s="131" t="s">
-        <v>17</v>
-      </c>
-      <c r="G94" s="131"/>
-      <c r="H94" s="131"/>
-      <c r="I94" s="131"/>
-      <c r="J94" s="131"/>
-      <c r="K94" s="131"/>
-      <c r="L94" s="131"/>
-      <c r="M94" s="138" t="s">
-        <v>295</v>
       </c>
     </row>
     <row r="95" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A95" s="15"/>
       <c r="B95" s="128" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="C95" s="129" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="D95" s="130">
         <v>1</v>
       </c>
       <c r="E95" s="129" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="F95" s="131" t="s">
         <v>17</v>
@@ -5330,43 +5341,42 @@
       <c r="K95" s="131"/>
       <c r="L95" s="131"/>
       <c r="M95" s="138" t="s">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="96" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="B96" s="11" t="s">
-        <v>291</v>
-      </c>
-      <c r="C96" s="12" t="s">
-        <v>208</v>
-      </c>
-      <c r="D96" s="13">
-        <v>1</v>
-      </c>
-      <c r="E96" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="F96" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="G96" s="14"/>
-      <c r="H96" s="14"/>
-      <c r="I96" s="14"/>
-      <c r="J96" s="14" t="s">
-        <v>292</v>
-      </c>
-      <c r="K96" s="14"/>
-      <c r="L96" s="14"/>
-      <c r="M96" s="111" t="s">
-        <v>220</v>
+        <v>294</v>
+      </c>
+    </row>
+    <row r="96" spans="1:14" ht="17" x14ac:dyDescent="0.2">
+      <c r="A96" s="15"/>
+      <c r="B96" s="128" t="s">
+        <v>290</v>
+      </c>
+      <c r="C96" s="129" t="s">
+        <v>293</v>
+      </c>
+      <c r="D96" s="130">
+        <v>1</v>
+      </c>
+      <c r="E96" s="129" t="s">
+        <v>18</v>
+      </c>
+      <c r="F96" s="131" t="s">
+        <v>17</v>
+      </c>
+      <c r="G96" s="131"/>
+      <c r="H96" s="131"/>
+      <c r="I96" s="131"/>
+      <c r="J96" s="131"/>
+      <c r="K96" s="131"/>
+      <c r="L96" s="131"/>
+      <c r="M96" s="138" t="s">
+        <v>295</v>
       </c>
     </row>
     <row r="97" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B97" s="11" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="C97" s="12" t="s">
-        <v>192</v>
+        <v>208</v>
       </c>
       <c r="D97" s="13">
         <v>1</v>
@@ -5375,26 +5385,26 @@
         <v>14</v>
       </c>
       <c r="F97" s="14" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G97" s="14"/>
       <c r="H97" s="14"/>
       <c r="I97" s="14"/>
       <c r="J97" s="14" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="K97" s="14"/>
       <c r="L97" s="14"/>
       <c r="M97" s="111" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="98" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B98" s="11" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="C98" s="12" t="s">
-        <v>274</v>
+        <v>192</v>
       </c>
       <c r="D98" s="13">
         <v>1</v>
@@ -5409,39 +5419,67 @@
       <c r="H98" s="14"/>
       <c r="I98" s="14"/>
       <c r="J98" s="14" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="K98" s="14"/>
       <c r="L98" s="14"/>
       <c r="M98" s="111" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="99" spans="2:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B99" s="123" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="99" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B99" s="11" t="s">
+        <v>290</v>
+      </c>
+      <c r="C99" s="12" t="s">
+        <v>273</v>
+      </c>
+      <c r="D99" s="13">
+        <v>1</v>
+      </c>
+      <c r="E99" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="F99" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="G99" s="14"/>
+      <c r="H99" s="14"/>
+      <c r="I99" s="14"/>
+      <c r="J99" s="14" t="s">
         <v>291</v>
       </c>
-      <c r="C99" s="124" t="s">
+      <c r="K99" s="14"/>
+      <c r="L99" s="14"/>
+      <c r="M99" s="111" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="100" spans="2:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B100" s="123" t="s">
+        <v>290</v>
+      </c>
+      <c r="C100" s="124" t="s">
         <v>160</v>
       </c>
-      <c r="D99" s="125">
-        <v>1</v>
-      </c>
-      <c r="E99" s="124" t="s">
+      <c r="D100" s="125">
+        <v>1</v>
+      </c>
+      <c r="E100" s="124" t="s">
         <v>14</v>
       </c>
-      <c r="F99" s="126" t="s">
+      <c r="F100" s="126" t="s">
         <v>15</v>
       </c>
-      <c r="G99" s="126"/>
-      <c r="H99" s="126"/>
-      <c r="I99" s="126"/>
-      <c r="J99" s="126" t="s">
-        <v>292</v>
-      </c>
-      <c r="K99" s="126"/>
-      <c r="L99" s="126"/>
-      <c r="M99" s="127" t="s">
+      <c r="G100" s="126"/>
+      <c r="H100" s="126"/>
+      <c r="I100" s="126"/>
+      <c r="J100" s="126" t="s">
+        <v>291</v>
+      </c>
+      <c r="K100" s="126"/>
+      <c r="L100" s="126"/>
+      <c r="M100" s="127" t="s">
         <v>222</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Change attribute targetedSystem to targetSystem
</commit_message>
<xml_diff>
--- a/Schema/DB_scheme.xlsx
+++ b/Schema/DB_scheme.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aksam432/Documents/GitHub/WP3/Schema/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A883E7E-DDC3-BE4D-A59D-CFEF44A94EAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D39673A8-7D95-C346-8A93-9B57D03688E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38400" yWindow="0" windowWidth="21600" windowHeight="38400" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -781,9 +781,6 @@
     <t>validationSet</t>
   </si>
   <si>
-    <t>targetedSystem</t>
-  </si>
-  <si>
     <t>targetProperties</t>
   </si>
   <si>
@@ -1034,6 +1031,9 @@
   </si>
   <si>
     <t>softwareUrl</t>
+  </si>
+  <si>
+    <t>targetSystem</t>
   </si>
 </sst>
 </file>
@@ -2705,7 +2705,7 @@
       </c>
       <c r="C2" s="164"/>
       <c r="D2" s="165" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="E2" s="165"/>
       <c r="F2" s="165"/>
@@ -2786,7 +2786,7 @@
         <v>54</v>
       </c>
       <c r="C7" s="129" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="D7" s="130">
         <v>1</v>
@@ -2804,7 +2804,7 @@
       <c r="K7" s="131"/>
       <c r="L7" s="131"/>
       <c r="M7" s="132" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="8" spans="2:14" x14ac:dyDescent="0.2">
@@ -2812,7 +2812,7 @@
         <v>54</v>
       </c>
       <c r="C8" s="129" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="D8" s="130">
         <v>1</v>
@@ -2830,7 +2830,7 @@
       <c r="K8" s="131"/>
       <c r="L8" s="131"/>
       <c r="M8" s="132" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="9" spans="2:14" x14ac:dyDescent="0.2">
@@ -2853,7 +2853,7 @@
       <c r="H9" s="14"/>
       <c r="I9" s="14"/>
       <c r="J9" s="14" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="K9" s="14"/>
       <c r="L9" s="14"/>
@@ -2881,7 +2881,7 @@
       <c r="H10" s="14"/>
       <c r="I10" s="14"/>
       <c r="J10" s="14" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="K10" s="14"/>
       <c r="L10" s="14"/>
@@ -2909,13 +2909,13 @@
       <c r="H11" s="14"/>
       <c r="I11" s="14"/>
       <c r="J11" s="14" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="K11" s="14" t="s">
         <v>20</v>
       </c>
       <c r="L11" s="14" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="M11" s="112" t="s">
         <v>164</v>
@@ -2942,7 +2942,7 @@
       <c r="H12" s="95"/>
       <c r="I12" s="95"/>
       <c r="J12" s="14" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="K12" s="95"/>
       <c r="L12" s="95"/>
@@ -2955,7 +2955,7 @@
         <v>54</v>
       </c>
       <c r="C13" s="93" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="D13" s="94">
         <v>1</v>
@@ -2970,13 +2970,13 @@
       <c r="H13" s="95"/>
       <c r="I13" s="95"/>
       <c r="J13" s="14" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="K13" s="95" t="s">
         <v>20</v>
       </c>
       <c r="L13" s="95" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="M13" s="113" t="s">
         <v>183</v>
@@ -2988,7 +2988,7 @@
         <v>54</v>
       </c>
       <c r="C14" s="93" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="D14" s="94">
         <v>1</v>
@@ -3003,12 +3003,12 @@
       <c r="H14" s="95"/>
       <c r="I14" s="95"/>
       <c r="J14" s="14" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="K14" s="95"/>
       <c r="L14" s="95"/>
       <c r="M14" s="113" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="N14" s="173"/>
     </row>
@@ -3017,7 +3017,7 @@
         <v>54</v>
       </c>
       <c r="C15" s="93" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="D15" s="94">
         <v>1</v>
@@ -3032,12 +3032,12 @@
       <c r="H15" s="95"/>
       <c r="I15" s="95"/>
       <c r="J15" s="14" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="K15" s="95"/>
       <c r="L15" s="95"/>
       <c r="M15" s="113" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="N15" s="163"/>
     </row>
@@ -3061,13 +3061,13 @@
       <c r="H16" s="14"/>
       <c r="I16" s="12"/>
       <c r="J16" s="14" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="K16" s="14" t="s">
         <v>20</v>
       </c>
       <c r="L16" s="14" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="M16" s="111" t="s">
         <v>177</v>
@@ -3078,7 +3078,7 @@
         <v>54</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="D17" s="13">
         <v>1</v>
@@ -3087,18 +3087,18 @@
         <v>14</v>
       </c>
       <c r="F17" s="14" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G17" s="14"/>
       <c r="H17" s="14"/>
       <c r="I17" s="12"/>
       <c r="J17" s="14" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="K17" s="14"/>
       <c r="L17" s="14"/>
       <c r="M17" s="111" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="18" spans="2:14" x14ac:dyDescent="0.2">
@@ -3106,7 +3106,7 @@
         <v>54</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="D18" s="13">
         <v>1</v>
@@ -3121,12 +3121,12 @@
       <c r="H18" s="14"/>
       <c r="I18" s="12"/>
       <c r="J18" s="14" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="K18" s="14"/>
       <c r="L18" s="14"/>
       <c r="M18" s="111" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="N18" s="162"/>
     </row>
@@ -3150,7 +3150,7 @@
       <c r="H19" s="14"/>
       <c r="I19" s="12"/>
       <c r="J19" s="14" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="K19" s="14"/>
       <c r="L19" s="14"/>
@@ -3179,7 +3179,7 @@
       <c r="H20" s="14"/>
       <c r="I20" s="14"/>
       <c r="J20" s="14" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="K20" s="14"/>
       <c r="L20" s="14"/>
@@ -3192,7 +3192,7 @@
         <v>54</v>
       </c>
       <c r="C21" s="12" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="D21" s="13">
         <v>1</v>
@@ -3207,7 +3207,7 @@
       <c r="H21" s="14"/>
       <c r="I21" s="12"/>
       <c r="J21" s="14" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="K21" s="14"/>
       <c r="L21" s="14"/>
@@ -3235,7 +3235,7 @@
       <c r="H22" s="14"/>
       <c r="I22" s="14"/>
       <c r="J22" s="14" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="K22" s="14"/>
       <c r="L22" s="14"/>
@@ -3292,13 +3292,13 @@
       <c r="H24" s="100"/>
       <c r="I24" s="100"/>
       <c r="J24" s="14" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="K24" s="100" t="s">
         <v>20</v>
       </c>
       <c r="L24" s="105" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="M24" s="115" t="s">
         <v>182</v>
@@ -3325,7 +3325,7 @@
       <c r="H25" s="14"/>
       <c r="I25" s="14"/>
       <c r="J25" s="14" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="K25" s="14" t="s">
         <v>20</v>
@@ -3356,7 +3356,7 @@
       <c r="G26" s="14"/>
       <c r="H26" s="14"/>
       <c r="I26" s="14" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="J26" s="14"/>
       <c r="K26" s="14"/>
@@ -3384,7 +3384,7 @@
       <c r="G27" s="14"/>
       <c r="H27" s="14"/>
       <c r="I27" s="14" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="J27" s="14"/>
       <c r="K27" s="14"/>
@@ -3412,7 +3412,7 @@
       <c r="G28" s="14"/>
       <c r="H28" s="14"/>
       <c r="I28" s="14" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="J28" s="14"/>
       <c r="K28" s="14"/>
@@ -3426,7 +3426,7 @@
         <v>54</v>
       </c>
       <c r="C29" s="12" t="s">
-        <v>247</v>
+        <v>331</v>
       </c>
       <c r="D29" s="13">
         <v>1</v>
@@ -3441,7 +3441,7 @@
       <c r="H29" s="14"/>
       <c r="I29" s="14"/>
       <c r="J29" s="14" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="K29" s="14" t="s">
         <v>20</v>
@@ -3458,7 +3458,7 @@
         <v>54</v>
       </c>
       <c r="C30" s="12" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="D30" s="13">
         <v>10</v>
@@ -3473,7 +3473,7 @@
       <c r="H30" s="14"/>
       <c r="I30" s="14"/>
       <c r="J30" s="14" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="K30" s="14"/>
       <c r="L30" s="14"/>
@@ -3486,7 +3486,7 @@
         <v>54</v>
       </c>
       <c r="C31" s="12" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="D31" s="13">
         <v>1</v>
@@ -3501,12 +3501,12 @@
       <c r="H31" s="14"/>
       <c r="I31" s="14"/>
       <c r="J31" s="14" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="K31" s="14"/>
       <c r="L31" s="14"/>
       <c r="M31" s="112" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="32" spans="2:14" ht="17" x14ac:dyDescent="0.2">
@@ -3514,7 +3514,7 @@
         <v>54</v>
       </c>
       <c r="C32" s="134" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D32" s="135">
         <v>1</v>
@@ -3527,7 +3527,7 @@
       </c>
       <c r="G32" s="136"/>
       <c r="H32" s="136" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="I32" s="136"/>
       <c r="J32" s="136"/>
@@ -3542,7 +3542,7 @@
         <v>54</v>
       </c>
       <c r="C33" s="140" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="D33" s="141">
         <v>10</v>
@@ -3556,7 +3556,7 @@
       <c r="G33" s="142"/>
       <c r="H33" s="142"/>
       <c r="I33" s="142" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="J33" s="142"/>
       <c r="K33" s="142"/>
@@ -3598,7 +3598,7 @@
         <v>168</v>
       </c>
       <c r="C35" s="129" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="D35" s="130">
         <v>1</v>
@@ -3616,7 +3616,7 @@
       <c r="K35" s="131"/>
       <c r="L35" s="131"/>
       <c r="M35" s="138" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="36" spans="1:14" ht="17" x14ac:dyDescent="0.2">
@@ -3625,7 +3625,7 @@
         <v>168</v>
       </c>
       <c r="C36" s="129" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="D36" s="130">
         <v>1</v>
@@ -3643,7 +3643,7 @@
       <c r="K36" s="131"/>
       <c r="L36" s="131"/>
       <c r="M36" s="138" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="37" spans="1:14" ht="17" x14ac:dyDescent="0.2">
@@ -3667,7 +3667,7 @@
       <c r="H37" s="14"/>
       <c r="I37" s="16"/>
       <c r="J37" s="14" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="K37" s="14"/>
       <c r="L37" s="14"/>
@@ -3681,7 +3681,7 @@
         <v>168</v>
       </c>
       <c r="C38" s="12" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D38" s="13">
         <v>1</v>
@@ -3699,7 +3699,7 @@
       <c r="K38" s="14"/>
       <c r="L38" s="14"/>
       <c r="M38" s="112" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="39" spans="1:14" ht="17" x14ac:dyDescent="0.2">
@@ -3708,7 +3708,7 @@
         <v>168</v>
       </c>
       <c r="C39" s="12" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="D39" s="13">
         <v>1</v>
@@ -3726,7 +3726,7 @@
       <c r="K39" s="14"/>
       <c r="L39" s="14"/>
       <c r="M39" s="112" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="40" spans="1:14" ht="17" x14ac:dyDescent="0.2">
@@ -3735,7 +3735,7 @@
         <v>168</v>
       </c>
       <c r="C40" s="12" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="D40" s="13">
         <v>1</v>
@@ -3747,12 +3747,12 @@
         <v>17</v>
       </c>
       <c r="G40" s="14" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="H40" s="14"/>
       <c r="I40" s="16"/>
       <c r="J40" s="14" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="K40" s="14"/>
       <c r="L40" s="14"/>
@@ -3766,7 +3766,7 @@
         <v>168</v>
       </c>
       <c r="C41" s="116" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D41" s="13">
         <v>1</v>
@@ -3778,12 +3778,12 @@
         <v>17</v>
       </c>
       <c r="G41" s="14" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="H41" s="14"/>
       <c r="I41" s="16"/>
       <c r="J41" s="14" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="K41" s="14"/>
       <c r="L41" s="14"/>
@@ -3797,7 +3797,7 @@
         <v>168</v>
       </c>
       <c r="C42" s="144" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="D42" s="13">
         <v>1</v>
@@ -3809,12 +3809,12 @@
         <v>17</v>
       </c>
       <c r="G42" s="14" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="H42" s="14"/>
       <c r="I42" s="14"/>
       <c r="J42" s="14" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="K42" s="14"/>
       <c r="L42" s="14"/>
@@ -3828,7 +3828,7 @@
         <v>168</v>
       </c>
       <c r="C43" s="12" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="D43" s="13">
         <v>1</v>
@@ -3840,12 +3840,12 @@
         <v>15</v>
       </c>
       <c r="G43" s="14" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="H43" s="14"/>
       <c r="I43" s="14"/>
       <c r="J43" s="14" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="K43" s="14"/>
       <c r="L43" s="14"/>
@@ -3859,7 +3859,7 @@
         <v>168</v>
       </c>
       <c r="C44" s="149" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="D44" s="150">
         <v>1</v>
@@ -3871,12 +3871,12 @@
         <v>15</v>
       </c>
       <c r="G44" s="142" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="H44" s="153"/>
       <c r="I44" s="153"/>
       <c r="J44" s="142" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="K44" s="153"/>
       <c r="L44" s="153"/>
@@ -3888,7 +3888,7 @@
     <row r="45" spans="1:14" s="96" customFormat="1" ht="18" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A45" s="101"/>
       <c r="B45" s="128" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C45" s="145" t="s">
         <v>13</v>
@@ -3916,10 +3916,10 @@
     <row r="46" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A46" s="15"/>
       <c r="B46" s="128" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C46" s="129" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="D46" s="130">
         <v>1</v>
@@ -3937,16 +3937,16 @@
       <c r="K46" s="131"/>
       <c r="L46" s="131"/>
       <c r="M46" s="138" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="47" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A47" s="15"/>
       <c r="B47" s="128" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C47" s="129" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="D47" s="130">
         <v>1</v>
@@ -3964,13 +3964,13 @@
       <c r="K47" s="131"/>
       <c r="L47" s="131"/>
       <c r="M47" s="138" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="48" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A48" s="15"/>
       <c r="B48" s="11" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C48" s="12" t="s">
         <v>193</v>
@@ -3988,7 +3988,7 @@
       <c r="H48" s="14"/>
       <c r="I48" s="14"/>
       <c r="J48" s="14" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="K48" s="14"/>
       <c r="L48" s="14"/>
@@ -3999,7 +3999,7 @@
     <row r="49" spans="1:14" s="96" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A49" s="101"/>
       <c r="B49" s="97" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C49" s="102" t="s">
         <v>162</v>
@@ -4017,7 +4017,7 @@
       <c r="H49" s="103"/>
       <c r="I49" s="103"/>
       <c r="J49" s="103" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="K49" s="103"/>
       <c r="L49" s="103"/>
@@ -4029,7 +4029,7 @@
     <row r="50" spans="1:14" s="96" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A50" s="101"/>
       <c r="B50" s="97" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C50" s="102" t="s">
         <v>207</v>
@@ -4047,7 +4047,7 @@
       <c r="H50" s="103"/>
       <c r="I50" s="103"/>
       <c r="J50" s="103" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="K50" s="103" t="s">
         <v>20</v>
@@ -4063,10 +4063,10 @@
     <row r="51" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A51" s="15"/>
       <c r="B51" s="11" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C51" s="12" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="D51" s="13">
         <v>1</v>
@@ -4084,16 +4084,16 @@
       <c r="K51" s="14"/>
       <c r="L51" s="14"/>
       <c r="M51" s="112" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="52" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A52" s="15"/>
       <c r="B52" s="11" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C52" s="12" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="D52" s="13">
         <v>1</v>
@@ -4108,18 +4108,18 @@
       <c r="H52" s="14"/>
       <c r="I52" s="14"/>
       <c r="J52" s="14" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="K52" s="14"/>
       <c r="L52" s="14"/>
       <c r="M52" s="112" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="53" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A53" s="15"/>
       <c r="B53" s="11" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C53" s="12" t="s">
         <v>234</v>
@@ -4137,21 +4137,21 @@
       <c r="H53" s="14"/>
       <c r="I53" s="14"/>
       <c r="J53" s="14" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="K53" s="14"/>
       <c r="L53" s="14"/>
       <c r="M53" s="112" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="54" spans="1:14" s="96" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A54" s="15"/>
       <c r="B54" s="11" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C54" s="12" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="D54" s="13">
         <v>1</v>
@@ -4166,7 +4166,7 @@
       <c r="H54" s="14"/>
       <c r="I54" s="14"/>
       <c r="J54" s="14" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="K54" s="14"/>
       <c r="L54" s="14"/>
@@ -4178,13 +4178,13 @@
     <row r="55" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A55" s="15"/>
       <c r="B55" s="11" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C55" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D55" s="13" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="E55" s="12" t="s">
         <v>14</v>
@@ -4196,21 +4196,21 @@
       <c r="H55" s="14"/>
       <c r="I55" s="14"/>
       <c r="J55" s="14" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="K55" s="14"/>
       <c r="L55" s="14"/>
       <c r="M55" s="118" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="56" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A56" s="96"/>
       <c r="B56" s="11" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C56" s="98" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="D56" s="99">
         <v>1</v>
@@ -4222,12 +4222,12 @@
         <v>17</v>
       </c>
       <c r="G56" s="100" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="H56" s="100"/>
       <c r="I56" s="100"/>
       <c r="J56" s="14" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="K56" s="100"/>
       <c r="L56" s="100"/>
@@ -4237,10 +4237,10 @@
     </row>
     <row r="57" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B57" s="11" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C57" s="12" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="D57" s="13">
         <v>1</v>
@@ -4252,12 +4252,12 @@
         <v>17</v>
       </c>
       <c r="G57" s="14" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="H57" s="14"/>
       <c r="I57" s="14"/>
       <c r="J57" s="14" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="K57" s="14"/>
       <c r="L57" s="14"/>
@@ -4267,10 +4267,10 @@
     </row>
     <row r="58" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B58" s="11" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C58" s="12" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="D58" s="13">
         <v>1</v>
@@ -4282,12 +4282,12 @@
         <v>17</v>
       </c>
       <c r="G58" s="14" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="H58" s="14"/>
       <c r="I58" s="14"/>
       <c r="J58" s="14" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="K58" s="14"/>
       <c r="L58" s="14"/>
@@ -4297,10 +4297,10 @@
     </row>
     <row r="59" spans="1:14" s="96" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B59" s="97" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C59" s="102" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="D59" s="157">
         <v>1</v>
@@ -4312,12 +4312,12 @@
         <v>17</v>
       </c>
       <c r="G59" s="103" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="H59" s="103"/>
       <c r="I59" s="103"/>
       <c r="J59" s="103" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="K59" s="103"/>
       <c r="L59" s="103"/>
@@ -4328,10 +4328,10 @@
     </row>
     <row r="60" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B60" s="11" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C60" s="12" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="D60" s="13">
         <v>1</v>
@@ -4357,10 +4357,10 @@
     <row r="61" spans="1:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A61" s="96"/>
       <c r="B61" s="139" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C61" s="140" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="D61" s="141">
         <v>1</v>
@@ -4378,7 +4378,7 @@
       <c r="K61" s="142"/>
       <c r="L61" s="142"/>
       <c r="M61" s="155" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="62" spans="1:14" ht="18" thickTop="1" x14ac:dyDescent="0.2">
@@ -4414,7 +4414,7 @@
         <v>169</v>
       </c>
       <c r="C63" s="129" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="D63" s="130">
         <v>1</v>
@@ -4432,7 +4432,7 @@
       <c r="K63" s="131"/>
       <c r="L63" s="131"/>
       <c r="M63" s="138" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="64" spans="1:14" ht="17" x14ac:dyDescent="0.2">
@@ -4441,7 +4441,7 @@
         <v>169</v>
       </c>
       <c r="C64" s="129" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="D64" s="130">
         <v>1</v>
@@ -4459,7 +4459,7 @@
       <c r="K64" s="131"/>
       <c r="L64" s="131"/>
       <c r="M64" s="138" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="65" spans="1:14" x14ac:dyDescent="0.2">
@@ -4482,7 +4482,7 @@
       <c r="H65" s="14"/>
       <c r="I65" s="14"/>
       <c r="J65" s="14" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="K65" s="14"/>
       <c r="L65" s="14"/>
@@ -4510,7 +4510,7 @@
       <c r="H66" s="14"/>
       <c r="I66" s="14"/>
       <c r="J66" s="14" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="K66" s="14"/>
       <c r="L66" s="14"/>
@@ -4523,7 +4523,7 @@
         <v>169</v>
       </c>
       <c r="C67" s="12" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="D67" s="13">
         <v>1</v>
@@ -4541,7 +4541,7 @@
       <c r="K67" s="14"/>
       <c r="L67" s="14"/>
       <c r="M67" s="159" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="68" spans="1:14" x14ac:dyDescent="0.2">
@@ -4549,7 +4549,7 @@
         <v>169</v>
       </c>
       <c r="C68" s="12" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="D68" s="13">
         <v>1</v>
@@ -4564,13 +4564,13 @@
       <c r="H68" s="14"/>
       <c r="I68" s="14"/>
       <c r="J68" s="14" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="K68" s="14" t="s">
         <v>20</v>
       </c>
       <c r="L68" s="14" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="M68" s="111" t="s">
         <v>211</v>
@@ -4596,7 +4596,7 @@
       <c r="H69" s="14"/>
       <c r="I69" s="14"/>
       <c r="J69" s="14" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="K69" s="14"/>
       <c r="L69" s="14"/>
@@ -4609,7 +4609,7 @@
         <v>169</v>
       </c>
       <c r="C70" s="12" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D70" s="13">
         <v>1</v>
@@ -4621,12 +4621,12 @@
         <v>15</v>
       </c>
       <c r="G70" s="14" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="H70" s="14"/>
       <c r="I70" s="14"/>
       <c r="J70" s="14" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="K70" s="14"/>
       <c r="L70" s="14"/>
@@ -4639,7 +4639,7 @@
         <v>169</v>
       </c>
       <c r="C71" s="12" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D71" s="13">
         <v>1</v>
@@ -4651,12 +4651,12 @@
         <v>15</v>
       </c>
       <c r="G71" s="14" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="H71" s="14"/>
       <c r="I71" s="14"/>
       <c r="J71" s="14" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="K71" s="14"/>
       <c r="L71" s="14"/>
@@ -4684,7 +4684,7 @@
       <c r="H72" s="103"/>
       <c r="I72" s="103"/>
       <c r="J72" s="103" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="K72" s="103"/>
       <c r="L72" s="103"/>
@@ -4713,7 +4713,7 @@
       <c r="H73" s="14"/>
       <c r="I73" s="14"/>
       <c r="J73" s="14" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="K73" s="14"/>
       <c r="L73" s="14"/>
@@ -4741,7 +4741,7 @@
       <c r="H74" s="14"/>
       <c r="I74" s="14"/>
       <c r="J74" s="14" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="K74" s="14"/>
       <c r="L74" s="14"/>
@@ -4754,7 +4754,7 @@
         <v>169</v>
       </c>
       <c r="C75" s="12" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D75" s="13">
         <v>1</v>
@@ -4766,12 +4766,12 @@
         <v>15</v>
       </c>
       <c r="G75" s="14" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="H75" s="14"/>
       <c r="I75" s="14"/>
       <c r="J75" s="14" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="K75" s="14"/>
       <c r="L75" s="14"/>
@@ -4784,7 +4784,7 @@
         <v>169</v>
       </c>
       <c r="C76" s="140" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D76" s="141">
         <v>1</v>
@@ -4796,12 +4796,12 @@
         <v>15</v>
       </c>
       <c r="G76" s="142" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="H76" s="142"/>
       <c r="I76" s="142"/>
       <c r="J76" s="142" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="K76" s="142"/>
       <c r="L76" s="142"/>
@@ -4842,7 +4842,7 @@
         <v>174</v>
       </c>
       <c r="C78" s="129" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="D78" s="130">
         <v>1</v>
@@ -4860,7 +4860,7 @@
       <c r="K78" s="131"/>
       <c r="L78" s="131"/>
       <c r="M78" s="138" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="79" spans="1:14" ht="17" x14ac:dyDescent="0.2">
@@ -4869,7 +4869,7 @@
         <v>174</v>
       </c>
       <c r="C79" s="129" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="D79" s="130">
         <v>1</v>
@@ -4887,7 +4887,7 @@
       <c r="K79" s="131"/>
       <c r="L79" s="131"/>
       <c r="M79" s="138" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="80" spans="1:14" x14ac:dyDescent="0.2">
@@ -4911,7 +4911,7 @@
       <c r="H80" s="14"/>
       <c r="I80" s="14"/>
       <c r="J80" s="14" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="K80" s="14"/>
       <c r="L80" s="14"/>
@@ -4939,7 +4939,7 @@
       <c r="H81" s="14"/>
       <c r="I81" s="14"/>
       <c r="J81" s="14" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="K81" s="14"/>
       <c r="L81" s="14"/>
@@ -4954,7 +4954,7 @@
         <v>174</v>
       </c>
       <c r="C82" s="12" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D82" s="13">
         <v>1</v>
@@ -4968,7 +4968,7 @@
       <c r="G82" s="14"/>
       <c r="H82" s="14"/>
       <c r="I82" s="14" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="J82" s="14"/>
       <c r="K82" s="14"/>
@@ -4983,7 +4983,7 @@
         <v>174</v>
       </c>
       <c r="C83" s="102" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="D83" s="157">
         <v>1</v>
@@ -4998,7 +4998,7 @@
       <c r="H83" s="103"/>
       <c r="I83" s="103"/>
       <c r="J83" s="103" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="K83" s="103" t="s">
         <v>20</v>
@@ -5016,7 +5016,7 @@
         <v>174</v>
       </c>
       <c r="C84" s="12" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="D84" s="13">
         <v>1</v>
@@ -5031,7 +5031,7 @@
       <c r="H84" s="14"/>
       <c r="I84" s="14"/>
       <c r="J84" s="14" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="K84" s="14"/>
       <c r="L84" s="14"/>
@@ -5045,7 +5045,7 @@
         <v>174</v>
       </c>
       <c r="C85" s="140" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="D85" s="141">
         <v>1</v>
@@ -5058,19 +5058,19 @@
       </c>
       <c r="G85" s="142"/>
       <c r="H85" s="142" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="I85" s="142"/>
       <c r="J85" s="142"/>
       <c r="K85" s="142"/>
       <c r="L85" s="142"/>
       <c r="M85" s="160" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="86" spans="1:14" s="96" customFormat="1" ht="18" thickTop="1" x14ac:dyDescent="0.2">
       <c r="B86" s="128" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C86" s="145" t="s">
         <v>13</v>
@@ -5098,10 +5098,10 @@
     <row r="87" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A87" s="15"/>
       <c r="B87" s="128" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C87" s="129" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="D87" s="130">
         <v>1</v>
@@ -5119,16 +5119,16 @@
       <c r="K87" s="131"/>
       <c r="L87" s="131"/>
       <c r="M87" s="138" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="88" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A88" s="15"/>
       <c r="B88" s="128" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C88" s="129" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="D88" s="130">
         <v>1</v>
@@ -5146,15 +5146,15 @@
       <c r="K88" s="131"/>
       <c r="L88" s="131"/>
       <c r="M88" s="138" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="89" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B89" s="97" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C89" s="12" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="D89" s="13">
         <v>1</v>
@@ -5180,10 +5180,10 @@
     <row r="90" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A90" s="96"/>
       <c r="B90" s="97" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C90" s="102" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="D90" s="157">
         <v>1</v>
@@ -5208,10 +5208,10 @@
     </row>
     <row r="91" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B91" s="97" t="s">
+        <v>280</v>
+      </c>
+      <c r="C91" s="12" t="s">
         <v>281</v>
-      </c>
-      <c r="C91" s="12" t="s">
-        <v>282</v>
       </c>
       <c r="D91" s="13">
         <v>1</v>
@@ -5226,17 +5226,17 @@
       <c r="H91" s="14"/>
       <c r="I91" s="14"/>
       <c r="J91" s="14" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="K91" s="14"/>
       <c r="L91" s="14"/>
       <c r="M91" s="111" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="92" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B92" s="97" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C92" s="12" t="s">
         <v>176</v>
@@ -5254,7 +5254,7 @@
       <c r="H92" s="14"/>
       <c r="I92" s="14"/>
       <c r="J92" s="14" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="K92" s="14"/>
       <c r="L92" s="14"/>
@@ -5264,10 +5264,10 @@
     </row>
     <row r="93" spans="1:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B93" s="148" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C93" s="140" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="D93" s="141">
         <v>1</v>
@@ -5280,20 +5280,20 @@
       </c>
       <c r="G93" s="142"/>
       <c r="H93" s="142" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="I93" s="142"/>
       <c r="J93" s="142"/>
       <c r="K93" s="142"/>
       <c r="L93" s="142"/>
       <c r="M93" s="160" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="94" spans="1:14" ht="17" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A94" s="104"/>
       <c r="B94" s="128" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="C94" s="145" t="s">
         <v>13</v>
@@ -5320,10 +5320,10 @@
     <row r="95" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A95" s="15"/>
       <c r="B95" s="128" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="C95" s="129" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="D95" s="130">
         <v>1</v>
@@ -5341,16 +5341,16 @@
       <c r="K95" s="131"/>
       <c r="L95" s="131"/>
       <c r="M95" s="138" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="96" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A96" s="15"/>
       <c r="B96" s="128" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="C96" s="129" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="D96" s="130">
         <v>1</v>
@@ -5368,12 +5368,12 @@
       <c r="K96" s="131"/>
       <c r="L96" s="131"/>
       <c r="M96" s="138" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="97" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B97" s="11" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="C97" s="12" t="s">
         <v>208</v>
@@ -5391,7 +5391,7 @@
       <c r="H97" s="14"/>
       <c r="I97" s="14"/>
       <c r="J97" s="14" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="K97" s="14"/>
       <c r="L97" s="14"/>
@@ -5401,7 +5401,7 @@
     </row>
     <row r="98" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B98" s="11" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="C98" s="12" t="s">
         <v>192</v>
@@ -5419,7 +5419,7 @@
       <c r="H98" s="14"/>
       <c r="I98" s="14"/>
       <c r="J98" s="14" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="K98" s="14"/>
       <c r="L98" s="14"/>
@@ -5429,10 +5429,10 @@
     </row>
     <row r="99" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B99" s="11" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="C99" s="12" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="D99" s="13">
         <v>1</v>
@@ -5447,17 +5447,17 @@
       <c r="H99" s="14"/>
       <c r="I99" s="14"/>
       <c r="J99" s="14" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="K99" s="14"/>
       <c r="L99" s="14"/>
       <c r="M99" s="111" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="100" spans="2:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B100" s="123" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="C100" s="124" t="s">
         <v>160</v>
@@ -5475,7 +5475,7 @@
       <c r="H100" s="126"/>
       <c r="I100" s="126"/>
       <c r="J100" s="126" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="K100" s="126"/>
       <c r="L100" s="126"/>

</xml_diff>

<commit_message>
Functinal and theory level to be provide din userform
</commit_message>
<xml_diff>
--- a/Schema/DB_scheme.xlsx
+++ b/Schema/DB_scheme.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aksam432/Documents/GitHub/WP3/Schema/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C0436E3-E0D1-CF47-89F9-F17FADE47BA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{780307DE-8835-3D44-94E0-66A539085B5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38400" yWindow="0" windowWidth="21600" windowHeight="38400" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38400" yWindow="5400" windowWidth="21600" windowHeight="20160" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Schéma à compléter" sheetId="1" r:id="rId1"/>
@@ -4564,7 +4564,7 @@
       <c r="H68" s="14"/>
       <c r="I68" s="14"/>
       <c r="J68" s="14" t="s">
-        <v>278</v>
+        <v>289</v>
       </c>
       <c r="K68" s="14" t="s">
         <v>20</v>
@@ -4587,16 +4587,16 @@
         <v>1</v>
       </c>
       <c r="E69" s="102" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F69" s="14" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G69" s="14"/>
       <c r="H69" s="14"/>
       <c r="I69" s="14"/>
       <c r="J69" s="14" t="s">
-        <v>278</v>
+        <v>289</v>
       </c>
       <c r="K69" s="14"/>
       <c r="L69" s="14"/>

</xml_diff>